<commit_message>
bench: run 2026-06-25 01:56 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,9 +557,6 @@
       <c r="I2" t="n">
         <v>429</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>205</v>
       </c>
@@ -572,8 +569,6 @@
       <c r="P2" t="n">
         <v>3</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -622,9 +617,6 @@
       <c r="I3" t="n">
         <v>429</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>217</v>
       </c>
@@ -637,8 +629,6 @@
       <c r="P3" t="n">
         <v>3</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -687,9 +677,6 @@
       <c r="I4" t="n">
         <v>429</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>400</v>
       </c>
@@ -702,8 +689,6 @@
       <c r="P4" t="n">
         <v>3</v>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -752,9 +737,6 @@
       <c r="I5" t="n">
         <v>429</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>766</v>
       </c>
@@ -767,8 +749,6 @@
       <c r="P5" t="n">
         <v>3</v>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -843,8 +823,6 @@
           <t>responses/20260625T004409Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -914,8 +892,6 @@
           <t>responses/20260625T004409Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -980,9 +956,6 @@
       <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1052,8 +1025,546 @@
           <t>responses/20260625T004409Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>429</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>237</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>429</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>280</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>429</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>344</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>429</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>276</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>200</v>
+      </c>
+      <c r="J14" t="n">
+        <v>668</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3667</v>
+      </c>
+      <c r="L14" t="n">
+        <v>4335</v>
+      </c>
+      <c r="M14" t="n">
+        <v>33903</v>
+      </c>
+      <c r="N14" t="n">
+        <v>14881</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1591</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>200</v>
+      </c>
+      <c r="J15" t="n">
+        <v>668</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2048</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2716</v>
+      </c>
+      <c r="M15" t="n">
+        <v>45811</v>
+      </c>
+      <c r="N15" t="n">
+        <v>8741</v>
+      </c>
+      <c r="O15" t="n">
+        <v>839</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>200</v>
+      </c>
+      <c r="J16" t="n">
+        <v>606</v>
+      </c>
+      <c r="K16" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L16" t="n">
+        <v>6606</v>
+      </c>
+      <c r="M16" t="n">
+        <v>54378</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Design and implement a **self‑contained Java class** that provides a **concurren</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>200</v>
+      </c>
+      <c r="J17" t="n">
+        <v>688</v>
+      </c>
+      <c r="K17" t="n">
+        <v>2616</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3304</v>
+      </c>
+      <c r="M17" t="n">
+        <v>143845</v>
+      </c>
+      <c r="N17" t="n">
+        <v>12939</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1251</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1066,7 +1577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1208,9 +1719,6 @@
       <c r="I2" t="n">
         <v>429</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>240</v>
       </c>
@@ -1223,8 +1731,6 @@
       <c r="P2" t="n">
         <v>3</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -1273,9 +1779,6 @@
       <c r="I3" t="n">
         <v>429</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>280</v>
       </c>
@@ -1288,8 +1791,6 @@
       <c r="P3" t="n">
         <v>3</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -1364,8 +1865,6 @@
           <t>responses/20260625T004409Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1435,8 +1934,6 @@
           <t>responses/20260625T004409Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1506,8 +2003,6 @@
           <t>responses/20260625T004409Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1577,8 +2072,6 @@
           <t>responses/20260625T004409Z/text/qwen_qwen3-next-80b-a3b-instruct_free.md</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1648,8 +2141,6 @@
           <t>responses/20260625T004409Z/text/nousresearch_hermes-3-llama-3.1-405b_free.md</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1719,8 +2210,550 @@
           <t>responses/20260625T004409Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>429</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>280</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>429</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>333</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>200</v>
+      </c>
+      <c r="J12" t="n">
+        <v>905</v>
+      </c>
+      <c r="K12" t="n">
+        <v>536</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1441</v>
+      </c>
+      <c r="M12" t="n">
+        <v>5790</v>
+      </c>
+      <c r="N12" t="n">
+        <v>650</v>
+      </c>
+      <c r="O12" t="n">
+        <v>108</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>429</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>298</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>429</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>1144</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>200</v>
+      </c>
+      <c r="J15" t="n">
+        <v>762</v>
+      </c>
+      <c r="K15" t="n">
+        <v>7998</v>
+      </c>
+      <c r="L15" t="n">
+        <v>8760</v>
+      </c>
+      <c r="M15" t="n">
+        <v>57317</v>
+      </c>
+      <c r="N15" t="n">
+        <v>33252</v>
+      </c>
+      <c r="O15" t="n">
+        <v>4172</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>200</v>
+      </c>
+      <c r="J16" t="n">
+        <v>836</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5645</v>
+      </c>
+      <c r="L16" t="n">
+        <v>6481</v>
+      </c>
+      <c r="M16" t="n">
+        <v>125834</v>
+      </c>
+      <c r="N16" t="n">
+        <v>24792</v>
+      </c>
+      <c r="O16" t="n">
+        <v>3558</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Write a thorough, approximately 1000‑line (≈12,000‑15,000‑word) article that ser</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>200</v>
+      </c>
+      <c r="J17" t="n">
+        <v>861</v>
+      </c>
+      <c r="K17" t="n">
+        <v>6886</v>
+      </c>
+      <c r="L17" t="n">
+        <v>7747</v>
+      </c>
+      <c r="M17" t="n">
+        <v>236232</v>
+      </c>
+      <c r="N17" t="n">
+        <v>29207</v>
+      </c>
+      <c r="O17" t="n">
+        <v>3857</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1733,7 +2766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1875,9 +2908,6 @@
       <c r="I2" t="n">
         <v>429</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>286</v>
       </c>
@@ -1890,8 +2920,6 @@
       <c r="P2" t="n">
         <v>3</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -1966,8 +2994,6 @@
           <t>responses/20260625T004409Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2011,9 +3037,6 @@
       <c r="I4" t="n">
         <v>429</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>225</v>
       </c>
@@ -2026,8 +3049,6 @@
       <c r="P4" t="n">
         <v>3</v>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -2102,8 +3123,6 @@
           <t>responses/20260625T004409Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2173,8 +3192,6 @@
           <t>responses/20260625T004409Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2218,9 +3235,6 @@
       <c r="I7" t="n">
         <v>429</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>219</v>
       </c>
@@ -2233,8 +3247,6 @@
       <c r="P7" t="n">
         <v>3</v>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -2283,9 +3295,6 @@
       <c r="I8" t="n">
         <v>429</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>233</v>
       </c>
@@ -2298,8 +3307,6 @@
       <c r="P8" t="n">
         <v>3</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -2374,8 +3381,550 @@
           <t>responses/20260625T004409Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>429</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>258</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>200</v>
+      </c>
+      <c r="J11" t="n">
+        <v>611</v>
+      </c>
+      <c r="K11" t="n">
+        <v>832</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1443</v>
+      </c>
+      <c r="M11" t="n">
+        <v>7029</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3671</v>
+      </c>
+      <c r="O11" t="n">
+        <v>519</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>429</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>358</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>429</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>275</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>200</v>
+      </c>
+      <c r="J14" t="n">
+        <v>604</v>
+      </c>
+      <c r="K14" t="n">
+        <v>522</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1126</v>
+      </c>
+      <c r="M14" t="n">
+        <v>19547</v>
+      </c>
+      <c r="N14" t="n">
+        <v>2635</v>
+      </c>
+      <c r="O14" t="n">
+        <v>385</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>429</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>296</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>200</v>
+      </c>
+      <c r="J16" t="n">
+        <v>539</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1336</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1875</v>
+      </c>
+      <c r="M16" t="n">
+        <v>19295</v>
+      </c>
+      <c r="N16" t="n">
+        <v>3564</v>
+      </c>
+      <c r="O16" t="n">
+        <v>499</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20260625T015001Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-25T01:50:01.633689+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry About Co‑Funding Opportunities for the “Youth Tech Labs” Initia</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>200</v>
+      </c>
+      <c r="J17" t="n">
+        <v>613</v>
+      </c>
+      <c r="K17" t="n">
+        <v>888</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1501</v>
+      </c>
+      <c r="M17" t="n">
+        <v>49948</v>
+      </c>
+      <c r="N17" t="n">
+        <v>4301</v>
+      </c>
+      <c r="O17" t="n">
+        <v>618</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>responses/20260625T015001Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-06-25 02:13 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1068,9 +1068,6 @@
       <c r="I10" t="n">
         <v>429</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>237</v>
       </c>
@@ -1083,8 +1080,6 @@
       <c r="P10" t="n">
         <v>3</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -1133,9 +1128,6 @@
       <c r="I11" t="n">
         <v>429</v>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>280</v>
       </c>
@@ -1148,8 +1140,6 @@
       <c r="P11" t="n">
         <v>3</v>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -1198,9 +1188,6 @@
       <c r="I12" t="n">
         <v>429</v>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>344</v>
       </c>
@@ -1213,8 +1200,6 @@
       <c r="P12" t="n">
         <v>3</v>
       </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -1263,9 +1248,6 @@
       <c r="I13" t="n">
         <v>429</v>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>276</v>
       </c>
@@ -1278,8 +1260,6 @@
       <c r="P13" t="n">
         <v>3</v>
       </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -1354,8 +1334,6 @@
           <t>responses/20260625T015001Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1425,8 +1403,6 @@
           <t>responses/20260625T015001Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1491,9 +1467,6 @@
       <c r="P16" t="n">
         <v>1</v>
       </c>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1563,8 +1536,558 @@
           <t>responses/20260625T015001Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>200</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1177</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1424</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2601</v>
+      </c>
+      <c r="M18" t="n">
+        <v>14024</v>
+      </c>
+      <c r="N18" t="n">
+        <v>5241</v>
+      </c>
+      <c r="O18" t="n">
+        <v>761</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>429</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>98</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>429</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>102</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>200</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1097</v>
+      </c>
+      <c r="K21" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L21" t="n">
+        <v>7097</v>
+      </c>
+      <c r="M21" t="n">
+        <v>36940</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>200</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1146</v>
+      </c>
+      <c r="K22" t="n">
+        <v>3779</v>
+      </c>
+      <c r="L22" t="n">
+        <v>4925</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29262</v>
+      </c>
+      <c r="N22" t="n">
+        <v>17758</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1698</v>
+      </c>
+      <c r="P22" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/code/qwen_qwen3-next-80b-a3b-instruct_free.java</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>200</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1208</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2564</v>
+      </c>
+      <c r="L23" t="n">
+        <v>3772</v>
+      </c>
+      <c r="M23" t="n">
+        <v>59527</v>
+      </c>
+      <c r="N23" t="n">
+        <v>9546</v>
+      </c>
+      <c r="O23" t="n">
+        <v>968</v>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>200</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1135</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1106</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2241</v>
+      </c>
+      <c r="M24" t="n">
+        <v>68022</v>
+      </c>
+      <c r="N24" t="n">
+        <v>4893</v>
+      </c>
+      <c r="O24" t="n">
+        <v>695</v>
+      </c>
+      <c r="P24" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/code/nousresearch_hermes-3-llama-3.1-405b_free.java</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a **single, self‑contained Java program** that implements a **concurrent, </t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>200</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1192</v>
+      </c>
+      <c r="K25" t="n">
+        <v>3148</v>
+      </c>
+      <c r="L25" t="n">
+        <v>4340</v>
+      </c>
+      <c r="M25" t="n">
+        <v>131483</v>
+      </c>
+      <c r="N25" t="n">
+        <v>14242</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1448</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1577,7 +2100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2253,9 +2776,6 @@
       <c r="I10" t="n">
         <v>429</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>280</v>
       </c>
@@ -2268,8 +2788,6 @@
       <c r="P10" t="n">
         <v>3</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -2318,9 +2836,6 @@
       <c r="I11" t="n">
         <v>429</v>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>333</v>
       </c>
@@ -2333,8 +2848,6 @@
       <c r="P11" t="n">
         <v>3</v>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -2409,8 +2922,6 @@
           <t>responses/20260625T015001Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2454,9 +2965,6 @@
       <c r="I13" t="n">
         <v>429</v>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>298</v>
       </c>
@@ -2469,8 +2977,6 @@
       <c r="P13" t="n">
         <v>3</v>
       </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -2519,9 +3025,6 @@
       <c r="I14" t="n">
         <v>429</v>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
         <v>1144</v>
       </c>
@@ -2534,8 +3037,6 @@
       <c r="P14" t="n">
         <v>3</v>
       </c>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -2610,8 +3111,6 @@
           <t>responses/20260625T015001Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2681,8 +3180,6 @@
           <t>responses/20260625T015001Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2752,8 +3249,540 @@
           <t>responses/20260625T015001Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>429</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>134</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>429</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>176</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>429</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>132</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>429</v>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>117</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>200</v>
+      </c>
+      <c r="J22" t="n">
+        <v>908</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7997</v>
+      </c>
+      <c r="L22" t="n">
+        <v>8905</v>
+      </c>
+      <c r="M22" t="n">
+        <v>53958</v>
+      </c>
+      <c r="N22" t="n">
+        <v>19708</v>
+      </c>
+      <c r="O22" t="n">
+        <v>2477</v>
+      </c>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>200</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1041</v>
+      </c>
+      <c r="K23" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L23" t="n">
+        <v>9041</v>
+      </c>
+      <c r="M23" t="n">
+        <v>100360</v>
+      </c>
+      <c r="N23" t="n">
+        <v>30432</v>
+      </c>
+      <c r="O23" t="n">
+        <v>3840</v>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>JSONDecodeError: Expecting value: line 497 column 1 (char 2728)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Write a comprehensive, approximately 1000‑line (≈12,000‑15,000‑word) article tit</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>200</v>
+      </c>
+      <c r="J25" t="n">
+        <v>992</v>
+      </c>
+      <c r="K25" t="n">
+        <v>8192</v>
+      </c>
+      <c r="L25" t="n">
+        <v>9184</v>
+      </c>
+      <c r="M25" t="n">
+        <v>375489</v>
+      </c>
+      <c r="N25" t="n">
+        <v>34488</v>
+      </c>
+      <c r="O25" t="n">
+        <v>4336</v>
+      </c>
+      <c r="P25" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2766,7 +3795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3424,9 +4453,6 @@
       <c r="I10" t="n">
         <v>429</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>258</v>
       </c>
@@ -3439,8 +4465,6 @@
       <c r="P10" t="n">
         <v>3</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -3515,8 +4539,6 @@
           <t>responses/20260625T015001Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3560,9 +4582,6 @@
       <c r="I12" t="n">
         <v>429</v>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>358</v>
       </c>
@@ -3575,8 +4594,6 @@
       <c r="P12" t="n">
         <v>3</v>
       </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -3625,9 +4642,6 @@
       <c r="I13" t="n">
         <v>429</v>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>275</v>
       </c>
@@ -3640,8 +4654,6 @@
       <c r="P13" t="n">
         <v>3</v>
       </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -3716,8 +4728,6 @@
           <t>responses/20260625T015001Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3761,9 +4771,6 @@
       <c r="I15" t="n">
         <v>429</v>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
         <v>296</v>
       </c>
@@ -3776,8 +4783,6 @@
       <c r="P15" t="n">
         <v>3</v>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -3852,8 +4857,6 @@
           <t>responses/20260625T015001Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3923,8 +4926,556 @@
           <t>responses/20260625T015001Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>429</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>122</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>429</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>149</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>200</v>
+      </c>
+      <c r="J20" t="n">
+        <v>739</v>
+      </c>
+      <c r="K20" t="n">
+        <v>885</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1624</v>
+      </c>
+      <c r="M20" t="n">
+        <v>7983</v>
+      </c>
+      <c r="N20" t="n">
+        <v>3726</v>
+      </c>
+      <c r="O20" t="n">
+        <v>550</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>200</v>
+      </c>
+      <c r="J21" t="n">
+        <v>666</v>
+      </c>
+      <c r="K21" t="n">
+        <v>919</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1585</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4823</v>
+      </c>
+      <c r="N21" t="n">
+        <v>4532</v>
+      </c>
+      <c r="O21" t="n">
+        <v>659</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>200</v>
+      </c>
+      <c r="J22" t="n">
+        <v>742</v>
+      </c>
+      <c r="K22" t="n">
+        <v>573</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1315</v>
+      </c>
+      <c r="M22" t="n">
+        <v>15489</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2910</v>
+      </c>
+      <c r="O22" t="n">
+        <v>438</v>
+      </c>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>429</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>98</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>200</v>
+      </c>
+      <c r="J24" t="n">
+        <v>727</v>
+      </c>
+      <c r="K24" t="n">
+        <v>811</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1538</v>
+      </c>
+      <c r="M24" t="n">
+        <v>7186</v>
+      </c>
+      <c r="N24" t="n">
+        <v>4031</v>
+      </c>
+      <c r="O24" t="n">
+        <v>575</v>
+      </c>
+      <c r="P24" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/email/qwen_qwen3-next-80b-a3b-instruct_free.md</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20260625T020407Z</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-25T02:04:07.384927+00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Request for Clarification on Eligibility Criteria for the Rural Health </t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>200</v>
+      </c>
+      <c r="J25" t="n">
+        <v>744</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1001</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1745</v>
+      </c>
+      <c r="M25" t="n">
+        <v>47955</v>
+      </c>
+      <c r="N25" t="n">
+        <v>4570</v>
+      </c>
+      <c r="O25" t="n">
+        <v>706</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>responses/20260625T020407Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-06-26 13:14 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1605,8 +1605,6 @@
           <t>responses/20260625T020407Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1650,9 +1648,6 @@
       <c r="I19" t="n">
         <v>429</v>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>98</v>
       </c>
@@ -1665,8 +1660,6 @@
       <c r="P19" t="n">
         <v>3</v>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -1715,9 +1708,6 @@
       <c r="I20" t="n">
         <v>429</v>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>102</v>
       </c>
@@ -1730,8 +1720,6 @@
       <c r="P20" t="n">
         <v>3</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -1801,9 +1789,6 @@
       <c r="P21" t="n">
         <v>1</v>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1873,8 +1858,6 @@
           <t>responses/20260625T020407Z/code/qwen_qwen3-next-80b-a3b-instruct_free.java</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1944,8 +1927,6 @@
           <t>responses/20260625T020407Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2015,8 +1996,6 @@
           <t>responses/20260625T020407Z/code/nousresearch_hermes-3-llama-3.1-405b_free.java</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2086,8 +2065,1114 @@
           <t>responses/20260625T020407Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>200</v>
+      </c>
+      <c r="J26" t="n">
+        <v>444</v>
+      </c>
+      <c r="K26" t="n">
+        <v>870</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1314</v>
+      </c>
+      <c r="M26" t="n">
+        <v>11230</v>
+      </c>
+      <c r="N26" t="n">
+        <v>2880</v>
+      </c>
+      <c r="O26" t="n">
+        <v>389</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>429</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>149</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>429</v>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>176</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>429</v>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>585</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>200</v>
+      </c>
+      <c r="J30" t="n">
+        <v>444</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1309</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1753</v>
+      </c>
+      <c r="M30" t="n">
+        <v>5524</v>
+      </c>
+      <c r="N30" t="n">
+        <v>3244</v>
+      </c>
+      <c r="O30" t="n">
+        <v>460</v>
+      </c>
+      <c r="P30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>429</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>217</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>200</v>
+      </c>
+      <c r="J32" t="n">
+        <v>452</v>
+      </c>
+      <c r="K32" t="n">
+        <v>517</v>
+      </c>
+      <c r="L32" t="n">
+        <v>969</v>
+      </c>
+      <c r="M32" t="n">
+        <v>13378</v>
+      </c>
+      <c r="N32" t="n">
+        <v>2255</v>
+      </c>
+      <c r="O32" t="n">
+        <v>313</v>
+      </c>
+      <c r="P32" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>200</v>
+      </c>
+      <c r="J33" t="n">
+        <v>491</v>
+      </c>
+      <c r="K33" t="n">
+        <v>783</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1274</v>
+      </c>
+      <c r="M33" t="n">
+        <v>11680</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2034</v>
+      </c>
+      <c r="O33" t="n">
+        <v>301</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>200</v>
+      </c>
+      <c r="J34" t="n">
+        <v>416</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1116</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1532</v>
+      </c>
+      <c r="M34" t="n">
+        <v>18012</v>
+      </c>
+      <c r="N34" t="n">
+        <v>811</v>
+      </c>
+      <c r="O34" t="n">
+        <v>131</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>200</v>
+      </c>
+      <c r="J35" t="n">
+        <v>453</v>
+      </c>
+      <c r="K35" t="n">
+        <v>617</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1070</v>
+      </c>
+      <c r="M35" t="n">
+        <v>45458</v>
+      </c>
+      <c r="N35" t="n">
+        <v>2593</v>
+      </c>
+      <c r="O35" t="n">
+        <v>351</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>200</v>
+      </c>
+      <c r="J36" t="n">
+        <v>489</v>
+      </c>
+      <c r="K36" t="n">
+        <v>816</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1305</v>
+      </c>
+      <c r="M36" t="n">
+        <v>46552</v>
+      </c>
+      <c r="N36" t="n">
+        <v>3426</v>
+      </c>
+      <c r="O36" t="n">
+        <v>483</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>200</v>
+      </c>
+      <c r="J37" t="n">
+        <v>446</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1691</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2137</v>
+      </c>
+      <c r="M37" t="n">
+        <v>45461</v>
+      </c>
+      <c r="N37" t="n">
+        <v>7717</v>
+      </c>
+      <c r="O37" t="n">
+        <v>729</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>200</v>
+      </c>
+      <c r="J38" t="n">
+        <v>482</v>
+      </c>
+      <c r="K38" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L38" t="n">
+        <v>6482</v>
+      </c>
+      <c r="M38" t="n">
+        <v>118064</v>
+      </c>
+      <c r="N38" t="n">
+        <v>22537</v>
+      </c>
+      <c r="O38" t="n">
+        <v>2077</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>200</v>
+      </c>
+      <c r="J39" t="n">
+        <v>440</v>
+      </c>
+      <c r="K39" t="n">
+        <v>5809</v>
+      </c>
+      <c r="L39" t="n">
+        <v>6249</v>
+      </c>
+      <c r="M39" t="n">
+        <v>118556</v>
+      </c>
+      <c r="N39" t="n">
+        <v>8174</v>
+      </c>
+      <c r="O39" t="n">
+        <v>847</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>200</v>
+      </c>
+      <c r="J40" t="n">
+        <v>444</v>
+      </c>
+      <c r="K40" t="n">
+        <v>816</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1260</v>
+      </c>
+      <c r="M40" t="n">
+        <v>195012</v>
+      </c>
+      <c r="N40" t="n">
+        <v>2215</v>
+      </c>
+      <c r="O40" t="n">
+        <v>320</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>You are tasked with writing a self‑contained Java program that implements a **co</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>200</v>
+      </c>
+      <c r="J41" t="n">
+        <v>445</v>
+      </c>
+      <c r="K41" t="n">
+        <v>2639</v>
+      </c>
+      <c r="L41" t="n">
+        <v>3084</v>
+      </c>
+      <c r="M41" t="n">
+        <v>600348</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2100,7 +3185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3292,9 +4377,6 @@
       <c r="I18" t="n">
         <v>429</v>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
         <v>134</v>
       </c>
@@ -3307,8 +4389,6 @@
       <c r="P18" t="n">
         <v>3</v>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -3357,9 +4437,6 @@
       <c r="I19" t="n">
         <v>429</v>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>176</v>
       </c>
@@ -3372,8 +4449,6 @@
       <c r="P19" t="n">
         <v>3</v>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -3422,9 +4497,6 @@
       <c r="I20" t="n">
         <v>429</v>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>132</v>
       </c>
@@ -3437,8 +4509,6 @@
       <c r="P20" t="n">
         <v>3</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -3487,9 +4557,6 @@
       <c r="I21" t="n">
         <v>429</v>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
         <v>117</v>
       </c>
@@ -3502,8 +4569,6 @@
       <c r="P21" t="n">
         <v>3</v>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -3578,8 +4643,6 @@
           <t>responses/20260625T020407Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3649,8 +4712,6 @@
           <t>responses/20260625T020407Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3691,11 +4752,6 @@
           <t>error</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
         <v>0</v>
       </c>
@@ -3705,8 +4761,6 @@
       <c r="P24" t="n">
         <v>3</v>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
           <t>JSONDecodeError: Expecting value: line 497 column 1 (char 2728)</t>
@@ -3781,8 +4835,1108 @@
           <t>responses/20260625T020407Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>429</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>134</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>429</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>156</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>429</v>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>133</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>200</v>
+      </c>
+      <c r="J29" t="n">
+        <v>486</v>
+      </c>
+      <c r="K29" t="n">
+        <v>2303</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2789</v>
+      </c>
+      <c r="M29" t="n">
+        <v>32592</v>
+      </c>
+      <c r="N29" t="n">
+        <v>9663</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1241</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>429</v>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>247</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>200</v>
+      </c>
+      <c r="J31" t="n">
+        <v>509</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1127</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1636</v>
+      </c>
+      <c r="M31" t="n">
+        <v>48297</v>
+      </c>
+      <c r="N31" t="n">
+        <v>5005</v>
+      </c>
+      <c r="O31" t="n">
+        <v>599</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>200</v>
+      </c>
+      <c r="J32" t="n">
+        <v>486</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1472</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1958</v>
+      </c>
+      <c r="M32" t="n">
+        <v>6559</v>
+      </c>
+      <c r="N32" t="n">
+        <v>4632</v>
+      </c>
+      <c r="O32" t="n">
+        <v>627</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>200</v>
+      </c>
+      <c r="J33" t="n">
+        <v>511</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1043</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1554</v>
+      </c>
+      <c r="M33" t="n">
+        <v>11866</v>
+      </c>
+      <c r="N33" t="n">
+        <v>3836</v>
+      </c>
+      <c r="O33" t="n">
+        <v>545</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>200</v>
+      </c>
+      <c r="J34" t="n">
+        <v>486</v>
+      </c>
+      <c r="K34" t="n">
+        <v>787</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1273</v>
+      </c>
+      <c r="M34" t="n">
+        <v>78215</v>
+      </c>
+      <c r="N34" t="n">
+        <v>2886</v>
+      </c>
+      <c r="O34" t="n">
+        <v>388</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>200</v>
+      </c>
+      <c r="J35" t="n">
+        <v>432</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1619</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2051</v>
+      </c>
+      <c r="M35" t="n">
+        <v>21267</v>
+      </c>
+      <c r="N35" t="n">
+        <v>6817</v>
+      </c>
+      <c r="O35" t="n">
+        <v>820</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>200</v>
+      </c>
+      <c r="J36" t="n">
+        <v>468</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1272</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1740</v>
+      </c>
+      <c r="M36" t="n">
+        <v>41336</v>
+      </c>
+      <c r="N36" t="n">
+        <v>5664</v>
+      </c>
+      <c r="O36" t="n">
+        <v>786</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>200</v>
+      </c>
+      <c r="J37" t="n">
+        <v>530</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1299</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1829</v>
+      </c>
+      <c r="M37" t="n">
+        <v>40065</v>
+      </c>
+      <c r="N37" t="n">
+        <v>5049</v>
+      </c>
+      <c r="O37" t="n">
+        <v>680</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>200</v>
+      </c>
+      <c r="J38" t="n">
+        <v>482</v>
+      </c>
+      <c r="K38" t="n">
+        <v>2509</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2991</v>
+      </c>
+      <c r="M38" t="n">
+        <v>62113</v>
+      </c>
+      <c r="N38" t="n">
+        <v>6343</v>
+      </c>
+      <c r="O38" t="n">
+        <v>824</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>200</v>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>120324</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>200</v>
+      </c>
+      <c r="J40" t="n">
+        <v>469</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1503</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1972</v>
+      </c>
+      <c r="M40" t="n">
+        <v>252270</v>
+      </c>
+      <c r="N40" t="n">
+        <v>6304</v>
+      </c>
+      <c r="O40" t="n">
+        <v>940</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article (roughly 12,</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>200</v>
+      </c>
+      <c r="J41" t="n">
+        <v>493</v>
+      </c>
+      <c r="K41" t="n">
+        <v>2710</v>
+      </c>
+      <c r="L41" t="n">
+        <v>3203</v>
+      </c>
+      <c r="M41" t="n">
+        <v>600228</v>
+      </c>
+      <c r="N41" t="n">
+        <v>5386</v>
+      </c>
+      <c r="O41" t="n">
+        <v>677</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3795,7 +5949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4969,9 +7123,6 @@
       <c r="I18" t="n">
         <v>429</v>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
         <v>122</v>
       </c>
@@ -4984,8 +7135,6 @@
       <c r="P18" t="n">
         <v>3</v>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -5034,9 +7183,6 @@
       <c r="I19" t="n">
         <v>429</v>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>149</v>
       </c>
@@ -5049,8 +7195,6 @@
       <c r="P19" t="n">
         <v>3</v>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -5125,8 +7269,6 @@
           <t>responses/20260625T020407Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5196,8 +7338,6 @@
           <t>responses/20260625T020407Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5267,8 +7407,6 @@
           <t>responses/20260625T020407Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5312,9 +7450,6 @@
       <c r="I23" t="n">
         <v>429</v>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>98</v>
       </c>
@@ -5327,8 +7462,6 @@
       <c r="P23" t="n">
         <v>3</v>
       </c>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -5403,8 +7536,6 @@
           <t>responses/20260625T020407Z/email/qwen_qwen3-next-80b-a3b-instruct_free.md</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5474,8 +7605,1098 @@
           <t>responses/20260625T020407Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>200</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>20722</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>429</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>191</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>200</v>
+      </c>
+      <c r="J28" t="n">
+        <v>571</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1085</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1656</v>
+      </c>
+      <c r="M28" t="n">
+        <v>14423</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4018</v>
+      </c>
+      <c r="O28" t="n">
+        <v>610</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>429</v>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>171</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>429</v>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>124</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>429</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>168</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>200</v>
+      </c>
+      <c r="J32" t="n">
+        <v>571</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1116</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1687</v>
+      </c>
+      <c r="M32" t="n">
+        <v>4034</v>
+      </c>
+      <c r="N32" t="n">
+        <v>4176</v>
+      </c>
+      <c r="O32" t="n">
+        <v>630</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>200</v>
+      </c>
+      <c r="J33" t="n">
+        <v>558</v>
+      </c>
+      <c r="K33" t="n">
+        <v>503</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1061</v>
+      </c>
+      <c r="M33" t="n">
+        <v>20394</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2546</v>
+      </c>
+      <c r="O33" t="n">
+        <v>391</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>200</v>
+      </c>
+      <c r="J34" t="n">
+        <v>575</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1063</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1638</v>
+      </c>
+      <c r="M34" t="n">
+        <v>39179</v>
+      </c>
+      <c r="N34" t="n">
+        <v>4814</v>
+      </c>
+      <c r="O34" t="n">
+        <v>747</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>200</v>
+      </c>
+      <c r="J35" t="n">
+        <v>577</v>
+      </c>
+      <c r="K35" t="n">
+        <v>851</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1428</v>
+      </c>
+      <c r="M35" t="n">
+        <v>11263</v>
+      </c>
+      <c r="N35" t="n">
+        <v>3643</v>
+      </c>
+      <c r="O35" t="n">
+        <v>540</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>200</v>
+      </c>
+      <c r="J36" t="n">
+        <v>501</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1467</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1968</v>
+      </c>
+      <c r="M36" t="n">
+        <v>16689</v>
+      </c>
+      <c r="N36" t="n">
+        <v>5857</v>
+      </c>
+      <c r="O36" t="n">
+        <v>879</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>200</v>
+      </c>
+      <c r="J37" t="n">
+        <v>607</v>
+      </c>
+      <c r="K37" t="n">
+        <v>661</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1268</v>
+      </c>
+      <c r="M37" t="n">
+        <v>18505</v>
+      </c>
+      <c r="N37" t="n">
+        <v>2070</v>
+      </c>
+      <c r="O37" t="n">
+        <v>292</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>200</v>
+      </c>
+      <c r="J38" t="n">
+        <v>567</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1775</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2342</v>
+      </c>
+      <c r="M38" t="n">
+        <v>30583</v>
+      </c>
+      <c r="N38" t="n">
+        <v>5838</v>
+      </c>
+      <c r="O38" t="n">
+        <v>858</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>200</v>
+      </c>
+      <c r="J39" t="n">
+        <v>559</v>
+      </c>
+      <c r="K39" t="n">
+        <v>608</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1167</v>
+      </c>
+      <c r="M39" t="n">
+        <v>67314</v>
+      </c>
+      <c r="N39" t="n">
+        <v>3011</v>
+      </c>
+      <c r="O39" t="n">
+        <v>453</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>200</v>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>120471</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20260626T130153Z</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-26T13:01:53.339120+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Subject: Clarification Needed on Indirect Cost Rate Allocation for Our Upcoming </t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>200</v>
+      </c>
+      <c r="J41" t="n">
+        <v>570</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1649</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2219</v>
+      </c>
+      <c r="M41" t="n">
+        <v>375080</v>
+      </c>
+      <c r="N41" t="n">
+        <v>3557</v>
+      </c>
+      <c r="O41" t="n">
+        <v>511</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>responses/20260626T130153Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-06-27 18:12 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2134,8 +2134,6 @@
           <t>responses/20260626T130153Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2179,9 +2177,6 @@
       <c r="I27" t="n">
         <v>429</v>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
         <v>149</v>
       </c>
@@ -2194,8 +2189,6 @@
       <c r="P27" t="n">
         <v>3</v>
       </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -2244,9 +2237,6 @@
       <c r="I28" t="n">
         <v>429</v>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
         <v>176</v>
       </c>
@@ -2259,8 +2249,6 @@
       <c r="P28" t="n">
         <v>3</v>
       </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -2309,9 +2297,6 @@
       <c r="I29" t="n">
         <v>429</v>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
         <v>585</v>
       </c>
@@ -2324,8 +2309,6 @@
       <c r="P29" t="n">
         <v>3</v>
       </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -2400,8 +2383,6 @@
           <t>responses/20260626T130153Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2445,9 +2426,6 @@
       <c r="I31" t="n">
         <v>429</v>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
         <v>217</v>
       </c>
@@ -2460,8 +2438,6 @@
       <c r="P31" t="n">
         <v>3</v>
       </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -2536,8 +2512,6 @@
           <t>responses/20260626T130153Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2607,8 +2581,6 @@
           <t>responses/20260626T130153Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2678,8 +2650,6 @@
           <t>responses/20260626T130153Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2749,8 +2719,6 @@
           <t>responses/20260626T130153Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2820,8 +2788,6 @@
           <t>responses/20260626T130153Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2891,8 +2857,6 @@
           <t>responses/20260626T130153Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2962,8 +2926,6 @@
           <t>responses/20260626T130153Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3033,8 +2995,6 @@
           <t>responses/20260626T130153Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3104,8 +3064,6 @@
           <t>responses/20260626T130153Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3170,9 +3128,1110 @@
       <c r="P41" t="n">
         <v>1</v>
       </c>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>200</v>
+      </c>
+      <c r="J42" t="n">
+        <v>442</v>
+      </c>
+      <c r="K42" t="n">
+        <v>111</v>
+      </c>
+      <c r="L42" t="n">
+        <v>553</v>
+      </c>
+      <c r="M42" t="n">
+        <v>3839</v>
+      </c>
+      <c r="N42" t="n">
+        <v>243</v>
+      </c>
+      <c r="O42" t="n">
+        <v>39</v>
+      </c>
+      <c r="P42" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>429</v>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="n">
+        <v>101</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>429</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>120</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>429</v>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>106</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>429</v>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>656</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>200</v>
+      </c>
+      <c r="J47" t="n">
+        <v>405</v>
+      </c>
+      <c r="K47" t="n">
+        <v>985</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1390</v>
+      </c>
+      <c r="M47" t="n">
+        <v>7306</v>
+      </c>
+      <c r="N47" t="n">
+        <v>2200</v>
+      </c>
+      <c r="O47" t="n">
+        <v>316</v>
+      </c>
+      <c r="P47" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>200</v>
+      </c>
+      <c r="J48" t="n">
+        <v>422</v>
+      </c>
+      <c r="K48" t="n">
+        <v>752</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1174</v>
+      </c>
+      <c r="M48" t="n">
+        <v>23728</v>
+      </c>
+      <c r="N48" t="n">
+        <v>3274</v>
+      </c>
+      <c r="O48" t="n">
+        <v>421</v>
+      </c>
+      <c r="P48" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>200</v>
+      </c>
+      <c r="J49" t="n">
+        <v>444</v>
+      </c>
+      <c r="K49" t="n">
+        <v>646</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1090</v>
+      </c>
+      <c r="M49" t="n">
+        <v>8298</v>
+      </c>
+      <c r="N49" t="n">
+        <v>1750</v>
+      </c>
+      <c r="O49" t="n">
+        <v>254</v>
+      </c>
+      <c r="P49" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>200</v>
+      </c>
+      <c r="J50" t="n">
+        <v>405</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1511</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1916</v>
+      </c>
+      <c r="M50" t="n">
+        <v>24835</v>
+      </c>
+      <c r="N50" t="n">
+        <v>5950</v>
+      </c>
+      <c r="O50" t="n">
+        <v>844</v>
+      </c>
+      <c r="P50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>200</v>
+      </c>
+      <c r="J51" t="n">
+        <v>399</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1663</v>
+      </c>
+      <c r="L51" t="n">
+        <v>2062</v>
+      </c>
+      <c r="M51" t="n">
+        <v>31270</v>
+      </c>
+      <c r="N51" t="n">
+        <v>8020</v>
+      </c>
+      <c r="O51" t="n">
+        <v>630</v>
+      </c>
+      <c r="P51" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>200</v>
+      </c>
+      <c r="J52" t="n">
+        <v>445</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1915</v>
+      </c>
+      <c r="L52" t="n">
+        <v>2360</v>
+      </c>
+      <c r="M52" t="n">
+        <v>33103</v>
+      </c>
+      <c r="N52" t="n">
+        <v>195</v>
+      </c>
+      <c r="O52" t="n">
+        <v>24</v>
+      </c>
+      <c r="P52" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>200</v>
+      </c>
+      <c r="J53" t="n">
+        <v>405</v>
+      </c>
+      <c r="K53" t="n">
+        <v>1225</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1630</v>
+      </c>
+      <c r="M53" t="n">
+        <v>56243</v>
+      </c>
+      <c r="N53" t="n">
+        <v>4465</v>
+      </c>
+      <c r="O53" t="n">
+        <v>601</v>
+      </c>
+      <c r="P53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>200</v>
+      </c>
+      <c r="J54" t="n">
+        <v>423</v>
+      </c>
+      <c r="K54" t="n">
+        <v>913</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1336</v>
+      </c>
+      <c r="M54" t="n">
+        <v>60613</v>
+      </c>
+      <c r="N54" t="n">
+        <v>3921</v>
+      </c>
+      <c r="O54" t="n">
+        <v>540</v>
+      </c>
+      <c r="P54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>200</v>
+      </c>
+      <c r="J55" t="n">
+        <v>372</v>
+      </c>
+      <c r="K55" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L55" t="n">
+        <v>6372</v>
+      </c>
+      <c r="M55" t="n">
+        <v>85807</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>200</v>
+      </c>
+      <c r="J56" t="n">
+        <v>401</v>
+      </c>
+      <c r="K56" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L56" t="n">
+        <v>6401</v>
+      </c>
+      <c r="M56" t="n">
+        <v>149617</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a sophisticated mult</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>200</v>
+      </c>
+      <c r="J57" t="n">
+        <v>408</v>
+      </c>
+      <c r="K57" t="n">
+        <v>5333</v>
+      </c>
+      <c r="L57" t="n">
+        <v>5741</v>
+      </c>
+      <c r="M57" t="n">
+        <v>209527</v>
+      </c>
+      <c r="N57" t="n">
+        <v>1894</v>
+      </c>
+      <c r="O57" t="n">
+        <v>247</v>
+      </c>
+      <c r="P57" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/code/poolside_laguna-m.1_free.java</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3185,7 +4244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4878,9 +5937,6 @@
       <c r="I26" t="n">
         <v>429</v>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
         <v>134</v>
       </c>
@@ -4893,8 +5949,6 @@
       <c r="P26" t="n">
         <v>3</v>
       </c>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -4943,9 +5997,6 @@
       <c r="I27" t="n">
         <v>429</v>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
         <v>156</v>
       </c>
@@ -4958,8 +6009,6 @@
       <c r="P27" t="n">
         <v>3</v>
       </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -5008,9 +6057,6 @@
       <c r="I28" t="n">
         <v>429</v>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
         <v>133</v>
       </c>
@@ -5023,8 +6069,6 @@
       <c r="P28" t="n">
         <v>3</v>
       </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -5099,8 +6143,6 @@
           <t>responses/20260626T130153Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5144,9 +6186,6 @@
       <c r="I30" t="n">
         <v>429</v>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
         <v>247</v>
       </c>
@@ -5159,8 +6198,6 @@
       <c r="P30" t="n">
         <v>3</v>
       </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -5235,8 +6272,6 @@
           <t>responses/20260626T130153Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5306,8 +6341,6 @@
           <t>responses/20260626T130153Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5377,8 +6410,6 @@
           <t>responses/20260626T130153Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5448,8 +6479,6 @@
           <t>responses/20260626T130153Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5519,8 +6548,6 @@
           <t>responses/20260626T130153Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5590,8 +6617,6 @@
           <t>responses/20260626T130153Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5661,8 +6686,6 @@
           <t>responses/20260626T130153Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5732,8 +6755,6 @@
           <t>responses/20260626T130153Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5777,9 +6798,6 @@
       <c r="I39" t="n">
         <v>200</v>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="n">
         <v>120324</v>
       </c>
@@ -5792,9 +6810,6 @@
       <c r="P39" t="n">
         <v>1</v>
       </c>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5864,8 +6879,6 @@
           <t>responses/20260626T130153Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5935,8 +6948,1112 @@
           <t>responses/20260626T130153Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>429</v>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>91</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>200</v>
+      </c>
+      <c r="J43" t="n">
+        <v>366</v>
+      </c>
+      <c r="K43" t="n">
+        <v>606</v>
+      </c>
+      <c r="L43" t="n">
+        <v>972</v>
+      </c>
+      <c r="M43" t="n">
+        <v>13957</v>
+      </c>
+      <c r="N43" t="n">
+        <v>1930</v>
+      </c>
+      <c r="O43" t="n">
+        <v>245</v>
+      </c>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>429</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>94</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>429</v>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>92</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>429</v>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>870</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>429</v>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="n">
+        <v>263</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>200</v>
+      </c>
+      <c r="J48" t="n">
+        <v>366</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2184</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2550</v>
+      </c>
+      <c r="M48" t="n">
+        <v>9005</v>
+      </c>
+      <c r="N48" t="n">
+        <v>7047</v>
+      </c>
+      <c r="O48" t="n">
+        <v>932</v>
+      </c>
+      <c r="P48" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>200</v>
+      </c>
+      <c r="J49" t="n">
+        <v>407</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1517</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1924</v>
+      </c>
+      <c r="M49" t="n">
+        <v>63563</v>
+      </c>
+      <c r="N49" t="n">
+        <v>6801</v>
+      </c>
+      <c r="O49" t="n">
+        <v>812</v>
+      </c>
+      <c r="P49" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>200</v>
+      </c>
+      <c r="J50" t="n">
+        <v>409</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1306</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1715</v>
+      </c>
+      <c r="M50" t="n">
+        <v>19325</v>
+      </c>
+      <c r="N50" t="n">
+        <v>4594</v>
+      </c>
+      <c r="O50" t="n">
+        <v>568</v>
+      </c>
+      <c r="P50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>200</v>
+      </c>
+      <c r="J51" t="n">
+        <v>331</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1593</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1924</v>
+      </c>
+      <c r="M51" t="n">
+        <v>27032</v>
+      </c>
+      <c r="N51" t="n">
+        <v>6880</v>
+      </c>
+      <c r="O51" t="n">
+        <v>838</v>
+      </c>
+      <c r="P51" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>200</v>
+      </c>
+      <c r="J52" t="n">
+        <v>414</v>
+      </c>
+      <c r="K52" t="n">
+        <v>2116</v>
+      </c>
+      <c r="L52" t="n">
+        <v>2530</v>
+      </c>
+      <c r="M52" t="n">
+        <v>27109</v>
+      </c>
+      <c r="N52" t="n">
+        <v>5196</v>
+      </c>
+      <c r="O52" t="n">
+        <v>667</v>
+      </c>
+      <c r="P52" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>200</v>
+      </c>
+      <c r="J53" t="n">
+        <v>364</v>
+      </c>
+      <c r="K53" t="n">
+        <v>875</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1239</v>
+      </c>
+      <c r="M53" t="n">
+        <v>20957</v>
+      </c>
+      <c r="N53" t="n">
+        <v>4089</v>
+      </c>
+      <c r="O53" t="n">
+        <v>467</v>
+      </c>
+      <c r="P53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>200</v>
+      </c>
+      <c r="J54" t="n">
+        <v>366</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1905</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2271</v>
+      </c>
+      <c r="M54" t="n">
+        <v>100909</v>
+      </c>
+      <c r="N54" t="n">
+        <v>7378</v>
+      </c>
+      <c r="O54" t="n">
+        <v>900</v>
+      </c>
+      <c r="P54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>200</v>
+      </c>
+      <c r="J55" t="n">
+        <v>377</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1805</v>
+      </c>
+      <c r="L55" t="n">
+        <v>2182</v>
+      </c>
+      <c r="M55" t="n">
+        <v>81197</v>
+      </c>
+      <c r="N55" t="n">
+        <v>6352</v>
+      </c>
+      <c r="O55" t="n">
+        <v>785</v>
+      </c>
+      <c r="P55" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>200</v>
+      </c>
+      <c r="J56" t="n">
+        <v>362</v>
+      </c>
+      <c r="K56" t="n">
+        <v>2610</v>
+      </c>
+      <c r="L56" t="n">
+        <v>2972</v>
+      </c>
+      <c r="M56" t="n">
+        <v>66952</v>
+      </c>
+      <c r="N56" t="n">
+        <v>7800</v>
+      </c>
+      <c r="O56" t="n">
+        <v>969</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Na</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>200</v>
+      </c>
+      <c r="J57" t="n">
+        <v>361</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1201</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1562</v>
+      </c>
+      <c r="M57" t="n">
+        <v>101917</v>
+      </c>
+      <c r="N57" t="n">
+        <v>5402</v>
+      </c>
+      <c r="O57" t="n">
+        <v>699</v>
+      </c>
+      <c r="P57" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5949,7 +8066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7648,9 +9765,6 @@
       <c r="I26" t="n">
         <v>200</v>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
         <v>20722</v>
       </c>
@@ -7663,9 +9777,6 @@
       <c r="P26" t="n">
         <v>1</v>
       </c>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7709,9 +9820,6 @@
       <c r="I27" t="n">
         <v>429</v>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
         <v>191</v>
       </c>
@@ -7724,8 +9832,6 @@
       <c r="P27" t="n">
         <v>3</v>
       </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -7800,8 +9906,6 @@
           <t>responses/20260626T130153Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7845,9 +9949,6 @@
       <c r="I29" t="n">
         <v>429</v>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
         <v>171</v>
       </c>
@@ -7860,8 +9961,6 @@
       <c r="P29" t="n">
         <v>3</v>
       </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -7910,9 +10009,6 @@
       <c r="I30" t="n">
         <v>429</v>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
         <v>124</v>
       </c>
@@ -7925,8 +10021,6 @@
       <c r="P30" t="n">
         <v>3</v>
       </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -7975,9 +10069,6 @@
       <c r="I31" t="n">
         <v>429</v>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
         <v>168</v>
       </c>
@@ -7990,8 +10081,6 @@
       <c r="P31" t="n">
         <v>3</v>
       </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -8066,8 +10155,6 @@
           <t>responses/20260626T130153Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8137,8 +10224,6 @@
           <t>responses/20260626T130153Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8208,8 +10293,6 @@
           <t>responses/20260626T130153Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8279,8 +10362,6 @@
           <t>responses/20260626T130153Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8350,8 +10431,6 @@
           <t>responses/20260626T130153Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8421,8 +10500,6 @@
           <t>responses/20260626T130153Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8492,8 +10569,6 @@
           <t>responses/20260626T130153Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8563,8 +10638,6 @@
           <t>responses/20260626T130153Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8608,9 +10681,6 @@
       <c r="I40" t="n">
         <v>200</v>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
         <v>120471</v>
       </c>
@@ -8623,9 +10693,6 @@
       <c r="P40" t="n">
         <v>1</v>
       </c>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8695,8 +10762,1106 @@
           <t>responses/20260626T130153Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>429</v>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>92</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>200</v>
+      </c>
+      <c r="J43" t="n">
+        <v>606</v>
+      </c>
+      <c r="K43" t="n">
+        <v>802</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1408</v>
+      </c>
+      <c r="M43" t="n">
+        <v>7522</v>
+      </c>
+      <c r="N43" t="n">
+        <v>3060</v>
+      </c>
+      <c r="O43" t="n">
+        <v>432</v>
+      </c>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>429</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>297</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>200</v>
+      </c>
+      <c r="J45" t="n">
+        <v>606</v>
+      </c>
+      <c r="K45" t="n">
+        <v>925</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1531</v>
+      </c>
+      <c r="M45" t="n">
+        <v>28913</v>
+      </c>
+      <c r="N45" t="n">
+        <v>3193</v>
+      </c>
+      <c r="O45" t="n">
+        <v>448</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>429</v>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>108</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>429</v>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="n">
+        <v>108</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>429</v>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="n">
+        <v>95</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>200</v>
+      </c>
+      <c r="J49" t="n">
+        <v>606</v>
+      </c>
+      <c r="K49" t="n">
+        <v>795</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1401</v>
+      </c>
+      <c r="M49" t="n">
+        <v>3023</v>
+      </c>
+      <c r="N49" t="n">
+        <v>3429</v>
+      </c>
+      <c r="O49" t="n">
+        <v>499</v>
+      </c>
+      <c r="P49" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>429</v>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="n">
+        <v>354</v>
+      </c>
+      <c r="N50" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>200</v>
+      </c>
+      <c r="J51" t="n">
+        <v>615</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1104</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1719</v>
+      </c>
+      <c r="M51" t="n">
+        <v>12984</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3296</v>
+      </c>
+      <c r="O51" t="n">
+        <v>494</v>
+      </c>
+      <c r="P51" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>200</v>
+      </c>
+      <c r="J52" t="n">
+        <v>648</v>
+      </c>
+      <c r="K52" t="n">
+        <v>775</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1423</v>
+      </c>
+      <c r="M52" t="n">
+        <v>7631</v>
+      </c>
+      <c r="N52" t="n">
+        <v>2605</v>
+      </c>
+      <c r="O52" t="n">
+        <v>365</v>
+      </c>
+      <c r="P52" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>200</v>
+      </c>
+      <c r="J53" t="n">
+        <v>599</v>
+      </c>
+      <c r="K53" t="n">
+        <v>475</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1074</v>
+      </c>
+      <c r="M53" t="n">
+        <v>29429</v>
+      </c>
+      <c r="N53" t="n">
+        <v>2470</v>
+      </c>
+      <c r="O53" t="n">
+        <v>361</v>
+      </c>
+      <c r="P53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>200</v>
+      </c>
+      <c r="J54" t="n">
+        <v>595</v>
+      </c>
+      <c r="K54" t="n">
+        <v>712</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1307</v>
+      </c>
+      <c r="M54" t="n">
+        <v>22019</v>
+      </c>
+      <c r="N54" t="n">
+        <v>3545</v>
+      </c>
+      <c r="O54" t="n">
+        <v>484</v>
+      </c>
+      <c r="P54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>200</v>
+      </c>
+      <c r="J55" t="n">
+        <v>539</v>
+      </c>
+      <c r="K55" t="n">
+        <v>924</v>
+      </c>
+      <c r="L55" t="n">
+        <v>1463</v>
+      </c>
+      <c r="M55" t="n">
+        <v>42477</v>
+      </c>
+      <c r="N55" t="n">
+        <v>4243</v>
+      </c>
+      <c r="O55" t="n">
+        <v>604</v>
+      </c>
+      <c r="P55" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>200</v>
+      </c>
+      <c r="J56" t="n">
+        <v>611</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1146</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1757</v>
+      </c>
+      <c r="M56" t="n">
+        <v>60881</v>
+      </c>
+      <c r="N56" t="n">
+        <v>2960</v>
+      </c>
+      <c r="O56" t="n">
+        <v>419</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>20260627T180804Z</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-06-27T18:08:04.915149+00:00</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Budget Amendment – “Solar Harvest Initiative”</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>200</v>
+      </c>
+      <c r="J57" t="n">
+        <v>602</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1332</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1934</v>
+      </c>
+      <c r="M57" t="n">
+        <v>45989</v>
+      </c>
+      <c r="N57" t="n">
+        <v>4285</v>
+      </c>
+      <c r="O57" t="n">
+        <v>577</v>
+      </c>
+      <c r="P57" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>responses/20260627T180804Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-06-28 06:28 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S57"/>
+  <dimension ref="A1:S73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3197,8 +3197,6 @@
           <t>responses/20260627T180804Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3242,9 +3240,6 @@
       <c r="I43" t="n">
         <v>429</v>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">
         <v>101</v>
       </c>
@@ -3257,8 +3252,6 @@
       <c r="P43" t="n">
         <v>3</v>
       </c>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -3307,9 +3300,6 @@
       <c r="I44" t="n">
         <v>429</v>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>120</v>
       </c>
@@ -3322,8 +3312,6 @@
       <c r="P44" t="n">
         <v>3</v>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -3372,9 +3360,6 @@
       <c r="I45" t="n">
         <v>429</v>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" t="n">
         <v>106</v>
       </c>
@@ -3387,8 +3372,6 @@
       <c r="P45" t="n">
         <v>3</v>
       </c>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -3437,9 +3420,6 @@
       <c r="I46" t="n">
         <v>429</v>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
         <v>656</v>
       </c>
@@ -3452,8 +3432,6 @@
       <c r="P46" t="n">
         <v>3</v>
       </c>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -3528,8 +3506,6 @@
           <t>responses/20260627T180804Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3599,8 +3575,6 @@
           <t>responses/20260627T180804Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3670,8 +3644,6 @@
           <t>responses/20260627T180804Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3741,8 +3713,6 @@
           <t>responses/20260627T180804Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3812,8 +3782,6 @@
           <t>responses/20260627T180804Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3883,8 +3851,6 @@
           <t>responses/20260627T180804Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3954,8 +3920,6 @@
           <t>responses/20260627T180804Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4025,8 +3989,6 @@
           <t>responses/20260627T180804Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4091,9 +4053,6 @@
       <c r="P55" t="n">
         <v>1</v>
       </c>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4158,9 +4117,6 @@
       <c r="P56" t="n">
         <v>1</v>
       </c>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4230,8 +4186,1094 @@
           <t>responses/20260627T180804Z/code/poolside_laguna-m.1_free.java</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>200</v>
+      </c>
+      <c r="J58" t="n">
+        <v>330</v>
+      </c>
+      <c r="K58" t="n">
+        <v>52</v>
+      </c>
+      <c r="L58" t="n">
+        <v>382</v>
+      </c>
+      <c r="M58" t="n">
+        <v>5605</v>
+      </c>
+      <c r="N58" t="n">
+        <v>295</v>
+      </c>
+      <c r="O58" t="n">
+        <v>41</v>
+      </c>
+      <c r="P58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>5</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>200</v>
+      </c>
+      <c r="J59" t="n">
+        <v>323</v>
+      </c>
+      <c r="K59" t="n">
+        <v>308</v>
+      </c>
+      <c r="L59" t="n">
+        <v>631</v>
+      </c>
+      <c r="M59" t="n">
+        <v>11907</v>
+      </c>
+      <c r="N59" t="n">
+        <v>48</v>
+      </c>
+      <c r="O59" t="n">
+        <v>9</v>
+      </c>
+      <c r="P59" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>200</v>
+      </c>
+      <c r="J60" t="n">
+        <v>323</v>
+      </c>
+      <c r="K60" t="n">
+        <v>2129</v>
+      </c>
+      <c r="L60" t="n">
+        <v>2452</v>
+      </c>
+      <c r="M60" t="n">
+        <v>7339</v>
+      </c>
+      <c r="N60" t="n">
+        <v>8954</v>
+      </c>
+      <c r="O60" t="n">
+        <v>1217</v>
+      </c>
+      <c r="P60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>429</v>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="n">
+        <v>97</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>429</v>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="n">
+        <v>97</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>429</v>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="n">
+        <v>107</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>429</v>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="n">
+        <v>91</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>429</v>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="n">
+        <v>232</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
+      <c r="P65" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>429</v>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="n">
+        <v>263</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>200</v>
+      </c>
+      <c r="J67" t="n">
+        <v>324</v>
+      </c>
+      <c r="K67" t="n">
+        <v>1489</v>
+      </c>
+      <c r="L67" t="n">
+        <v>1813</v>
+      </c>
+      <c r="M67" t="n">
+        <v>39318</v>
+      </c>
+      <c r="N67" t="n">
+        <v>6423</v>
+      </c>
+      <c r="O67" t="n">
+        <v>655</v>
+      </c>
+      <c r="P67" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>5</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>200</v>
+      </c>
+      <c r="J68" t="n">
+        <v>373</v>
+      </c>
+      <c r="K68" t="n">
+        <v>4774</v>
+      </c>
+      <c r="L68" t="n">
+        <v>5147</v>
+      </c>
+      <c r="M68" t="n">
+        <v>59715</v>
+      </c>
+      <c r="N68" t="n">
+        <v>15624</v>
+      </c>
+      <c r="O68" t="n">
+        <v>1750</v>
+      </c>
+      <c r="P68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>200</v>
+      </c>
+      <c r="J69" t="n">
+        <v>360</v>
+      </c>
+      <c r="K69" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L69" t="n">
+        <v>6360</v>
+      </c>
+      <c r="M69" t="n">
+        <v>65322</v>
+      </c>
+      <c r="N69" t="n">
+        <v>20426</v>
+      </c>
+      <c r="O69" t="n">
+        <v>1871</v>
+      </c>
+      <c r="P69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>5</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>200</v>
+      </c>
+      <c r="J70" t="n">
+        <v>323</v>
+      </c>
+      <c r="K70" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L70" t="n">
+        <v>6323</v>
+      </c>
+      <c r="M70" t="n">
+        <v>81019</v>
+      </c>
+      <c r="N70" t="n">
+        <v>26707</v>
+      </c>
+      <c r="O70" t="n">
+        <v>3330</v>
+      </c>
+      <c r="P70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>200</v>
+      </c>
+      <c r="J71" t="n">
+        <v>296</v>
+      </c>
+      <c r="K71" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L71" t="n">
+        <v>6296</v>
+      </c>
+      <c r="M71" t="n">
+        <v>96320</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>5</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>200</v>
+      </c>
+      <c r="J72" t="n">
+        <v>323</v>
+      </c>
+      <c r="K72" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L72" t="n">
+        <v>6323</v>
+      </c>
+      <c r="M72" t="n">
+        <v>138068</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a highly concurrent,</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>200</v>
+      </c>
+      <c r="J73" t="n">
+        <v>319</v>
+      </c>
+      <c r="K73" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L73" t="n">
+        <v>6319</v>
+      </c>
+      <c r="M73" t="n">
+        <v>132541</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4244,7 +5286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S57"/>
+  <dimension ref="A1:S73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6991,9 +8033,6 @@
       <c r="I42" t="n">
         <v>429</v>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="n">
         <v>91</v>
       </c>
@@ -7006,8 +8045,6 @@
       <c r="P42" t="n">
         <v>3</v>
       </c>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -7082,8 +8119,6 @@
           <t>responses/20260627T180804Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7127,9 +8162,6 @@
       <c r="I44" t="n">
         <v>429</v>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>94</v>
       </c>
@@ -7142,8 +8174,6 @@
       <c r="P44" t="n">
         <v>3</v>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -7192,9 +8222,6 @@
       <c r="I45" t="n">
         <v>429</v>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" t="n">
         <v>92</v>
       </c>
@@ -7207,8 +8234,6 @@
       <c r="P45" t="n">
         <v>3</v>
       </c>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -7257,9 +8282,6 @@
       <c r="I46" t="n">
         <v>429</v>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
         <v>870</v>
       </c>
@@ -7272,8 +8294,6 @@
       <c r="P46" t="n">
         <v>3</v>
       </c>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -7322,9 +8342,6 @@
       <c r="I47" t="n">
         <v>429</v>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" t="n">
         <v>263</v>
       </c>
@@ -7337,8 +8354,6 @@
       <c r="P47" t="n">
         <v>3</v>
       </c>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -7413,8 +8428,6 @@
           <t>responses/20260627T180804Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7484,8 +8497,6 @@
           <t>responses/20260627T180804Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7555,8 +8566,6 @@
           <t>responses/20260627T180804Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7626,8 +8635,6 @@
           <t>responses/20260627T180804Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7697,8 +8704,6 @@
           <t>responses/20260627T180804Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7768,8 +8773,6 @@
           <t>responses/20260627T180804Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7839,8 +8842,6 @@
           <t>responses/20260627T180804Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7910,8 +8911,6 @@
           <t>responses/20260627T180804Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7981,8 +8980,6 @@
           <t>responses/20260627T180804Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8052,8 +9049,1102 @@
           <t>responses/20260627T180804Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>200</v>
+      </c>
+      <c r="J58" t="n">
+        <v>344</v>
+      </c>
+      <c r="K58" t="n">
+        <v>26</v>
+      </c>
+      <c r="L58" t="n">
+        <v>370</v>
+      </c>
+      <c r="M58" t="n">
+        <v>2043</v>
+      </c>
+      <c r="N58" t="n">
+        <v>38</v>
+      </c>
+      <c r="O58" t="n">
+        <v>8</v>
+      </c>
+      <c r="P58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>5</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>200</v>
+      </c>
+      <c r="J59" t="n">
+        <v>310</v>
+      </c>
+      <c r="K59" t="n">
+        <v>450</v>
+      </c>
+      <c r="L59" t="n">
+        <v>760</v>
+      </c>
+      <c r="M59" t="n">
+        <v>5542</v>
+      </c>
+      <c r="N59" t="n">
+        <v>166</v>
+      </c>
+      <c r="O59" t="n">
+        <v>28</v>
+      </c>
+      <c r="P59" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>429</v>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="n">
+        <v>103</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>429</v>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="n">
+        <v>104</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>429</v>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="n">
+        <v>82</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>429</v>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="n">
+        <v>107</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>429</v>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="n">
+        <v>626</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>200</v>
+      </c>
+      <c r="J65" t="n">
+        <v>310</v>
+      </c>
+      <c r="K65" t="n">
+        <v>2147</v>
+      </c>
+      <c r="L65" t="n">
+        <v>2457</v>
+      </c>
+      <c r="M65" t="n">
+        <v>11372</v>
+      </c>
+      <c r="N65" t="n">
+        <v>6339</v>
+      </c>
+      <c r="O65" t="n">
+        <v>801</v>
+      </c>
+      <c r="P65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>200</v>
+      </c>
+      <c r="J66" t="n">
+        <v>273</v>
+      </c>
+      <c r="K66" t="n">
+        <v>1659</v>
+      </c>
+      <c r="L66" t="n">
+        <v>1932</v>
+      </c>
+      <c r="M66" t="n">
+        <v>31524</v>
+      </c>
+      <c r="N66" t="n">
+        <v>3247</v>
+      </c>
+      <c r="O66" t="n">
+        <v>509</v>
+      </c>
+      <c r="P66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>200</v>
+      </c>
+      <c r="J67" t="n">
+        <v>321</v>
+      </c>
+      <c r="K67" t="n">
+        <v>2209</v>
+      </c>
+      <c r="L67" t="n">
+        <v>2530</v>
+      </c>
+      <c r="M67" t="n">
+        <v>62706</v>
+      </c>
+      <c r="N67" t="n">
+        <v>6583</v>
+      </c>
+      <c r="O67" t="n">
+        <v>837</v>
+      </c>
+      <c r="P67" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>5</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>200</v>
+      </c>
+      <c r="J68" t="n">
+        <v>346</v>
+      </c>
+      <c r="K68" t="n">
+        <v>1442</v>
+      </c>
+      <c r="L68" t="n">
+        <v>1788</v>
+      </c>
+      <c r="M68" t="n">
+        <v>53020</v>
+      </c>
+      <c r="N68" t="n">
+        <v>4618</v>
+      </c>
+      <c r="O68" t="n">
+        <v>617</v>
+      </c>
+      <c r="P68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>200</v>
+      </c>
+      <c r="J69" t="n">
+        <v>303</v>
+      </c>
+      <c r="K69" t="n">
+        <v>973</v>
+      </c>
+      <c r="L69" t="n">
+        <v>1276</v>
+      </c>
+      <c r="M69" t="n">
+        <v>92005</v>
+      </c>
+      <c r="N69" t="n">
+        <v>3983</v>
+      </c>
+      <c r="O69" t="n">
+        <v>547</v>
+      </c>
+      <c r="P69" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>5</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>200</v>
+      </c>
+      <c r="J70" t="n">
+        <v>358</v>
+      </c>
+      <c r="K70" t="n">
+        <v>7651</v>
+      </c>
+      <c r="L70" t="n">
+        <v>8009</v>
+      </c>
+      <c r="M70" t="n">
+        <v>80332</v>
+      </c>
+      <c r="N70" t="n">
+        <v>39916</v>
+      </c>
+      <c r="O70" t="n">
+        <v>5009</v>
+      </c>
+      <c r="P70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>200</v>
+      </c>
+      <c r="J71" t="n">
+        <v>310</v>
+      </c>
+      <c r="K71" t="n">
+        <v>1695</v>
+      </c>
+      <c r="L71" t="n">
+        <v>2005</v>
+      </c>
+      <c r="M71" t="n">
+        <v>147578</v>
+      </c>
+      <c r="N71" t="n">
+        <v>6144</v>
+      </c>
+      <c r="O71" t="n">
+        <v>808</v>
+      </c>
+      <c r="P71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>5</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>200</v>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="n">
+        <v>120220</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“Le</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>200</v>
+      </c>
+      <c r="J73" t="n">
+        <v>306</v>
+      </c>
+      <c r="K73" t="n">
+        <v>5212</v>
+      </c>
+      <c r="L73" t="n">
+        <v>5518</v>
+      </c>
+      <c r="M73" t="n">
+        <v>115940</v>
+      </c>
+      <c r="N73" t="n">
+        <v>16988</v>
+      </c>
+      <c r="O73" t="n">
+        <v>2184</v>
+      </c>
+      <c r="P73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8066,7 +10157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S57"/>
+  <dimension ref="A1:S73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10805,9 +12896,6 @@
       <c r="I42" t="n">
         <v>429</v>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="n">
         <v>92</v>
       </c>
@@ -10820,8 +12908,6 @@
       <c r="P42" t="n">
         <v>3</v>
       </c>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -10896,8 +12982,6 @@
           <t>responses/20260627T180804Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -10941,9 +13025,6 @@
       <c r="I44" t="n">
         <v>429</v>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>297</v>
       </c>
@@ -10956,8 +13037,6 @@
       <c r="P44" t="n">
         <v>3</v>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -11032,8 +13111,6 @@
           <t>responses/20260627T180804Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -11077,9 +13154,6 @@
       <c r="I46" t="n">
         <v>429</v>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
         <v>108</v>
       </c>
@@ -11092,8 +13166,6 @@
       <c r="P46" t="n">
         <v>3</v>
       </c>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -11142,9 +13214,6 @@
       <c r="I47" t="n">
         <v>429</v>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" t="n">
         <v>108</v>
       </c>
@@ -11157,8 +13226,6 @@
       <c r="P47" t="n">
         <v>3</v>
       </c>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -11207,9 +13274,6 @@
       <c r="I48" t="n">
         <v>429</v>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
         <v>95</v>
       </c>
@@ -11222,8 +13286,6 @@
       <c r="P48" t="n">
         <v>3</v>
       </c>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -11298,8 +13360,6 @@
           <t>responses/20260627T180804Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11343,9 +13403,6 @@
       <c r="I50" t="n">
         <v>429</v>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
       <c r="M50" t="n">
         <v>354</v>
       </c>
@@ -11358,8 +13415,6 @@
       <c r="P50" t="n">
         <v>3</v>
       </c>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -11434,8 +13489,6 @@
           <t>responses/20260627T180804Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11505,8 +13558,6 @@
           <t>responses/20260627T180804Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11576,8 +13627,6 @@
           <t>responses/20260627T180804Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -11647,8 +13696,6 @@
           <t>responses/20260627T180804Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11718,8 +13765,6 @@
           <t>responses/20260627T180804Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11789,8 +13834,6 @@
           <t>responses/20260627T180804Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11860,8 +13903,1108 @@
           <t>responses/20260627T180804Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>200</v>
+      </c>
+      <c r="J58" t="n">
+        <v>589</v>
+      </c>
+      <c r="K58" t="n">
+        <v>650</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1239</v>
+      </c>
+      <c r="M58" t="n">
+        <v>6340</v>
+      </c>
+      <c r="N58" t="n">
+        <v>2675</v>
+      </c>
+      <c r="O58" t="n">
+        <v>370</v>
+      </c>
+      <c r="P58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>5</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>429</v>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="n">
+        <v>92</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>200</v>
+      </c>
+      <c r="J60" t="n">
+        <v>589</v>
+      </c>
+      <c r="K60" t="n">
+        <v>799</v>
+      </c>
+      <c r="L60" t="n">
+        <v>1388</v>
+      </c>
+      <c r="M60" t="n">
+        <v>10604</v>
+      </c>
+      <c r="N60" t="n">
+        <v>3301</v>
+      </c>
+      <c r="O60" t="n">
+        <v>459</v>
+      </c>
+      <c r="P60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>429</v>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="n">
+        <v>82</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>429</v>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="n">
+        <v>111</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>429</v>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="n">
+        <v>88</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>200</v>
+      </c>
+      <c r="J64" t="n">
+        <v>589</v>
+      </c>
+      <c r="K64" t="n">
+        <v>853</v>
+      </c>
+      <c r="L64" t="n">
+        <v>1442</v>
+      </c>
+      <c r="M64" t="n">
+        <v>3894</v>
+      </c>
+      <c r="N64" t="n">
+        <v>3490</v>
+      </c>
+      <c r="O64" t="n">
+        <v>475</v>
+      </c>
+      <c r="P64" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>200</v>
+      </c>
+      <c r="J65" t="n">
+        <v>606</v>
+      </c>
+      <c r="K65" t="n">
+        <v>834</v>
+      </c>
+      <c r="L65" t="n">
+        <v>1440</v>
+      </c>
+      <c r="M65" t="n">
+        <v>36946</v>
+      </c>
+      <c r="N65" t="n">
+        <v>3965</v>
+      </c>
+      <c r="O65" t="n">
+        <v>567</v>
+      </c>
+      <c r="P65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>200</v>
+      </c>
+      <c r="J66" t="n">
+        <v>532</v>
+      </c>
+      <c r="K66" t="n">
+        <v>799</v>
+      </c>
+      <c r="L66" t="n">
+        <v>1331</v>
+      </c>
+      <c r="M66" t="n">
+        <v>10293</v>
+      </c>
+      <c r="N66" t="n">
+        <v>3863</v>
+      </c>
+      <c r="O66" t="n">
+        <v>545</v>
+      </c>
+      <c r="P66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>200</v>
+      </c>
+      <c r="J67" t="n">
+        <v>598</v>
+      </c>
+      <c r="K67" t="n">
+        <v>499</v>
+      </c>
+      <c r="L67" t="n">
+        <v>1097</v>
+      </c>
+      <c r="M67" t="n">
+        <v>13328</v>
+      </c>
+      <c r="N67" t="n">
+        <v>2603</v>
+      </c>
+      <c r="O67" t="n">
+        <v>374</v>
+      </c>
+      <c r="P67" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>5</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>200</v>
+      </c>
+      <c r="J68" t="n">
+        <v>635</v>
+      </c>
+      <c r="K68" t="n">
+        <v>717</v>
+      </c>
+      <c r="L68" t="n">
+        <v>1352</v>
+      </c>
+      <c r="M68" t="n">
+        <v>6967</v>
+      </c>
+      <c r="N68" t="n">
+        <v>2359</v>
+      </c>
+      <c r="O68" t="n">
+        <v>333</v>
+      </c>
+      <c r="P68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>200</v>
+      </c>
+      <c r="J69" t="n">
+        <v>608</v>
+      </c>
+      <c r="K69" t="n">
+        <v>837</v>
+      </c>
+      <c r="L69" t="n">
+        <v>1445</v>
+      </c>
+      <c r="M69" t="n">
+        <v>11824</v>
+      </c>
+      <c r="N69" t="n">
+        <v>3795</v>
+      </c>
+      <c r="O69" t="n">
+        <v>548</v>
+      </c>
+      <c r="P69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>5</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>200</v>
+      </c>
+      <c r="J70" t="n">
+        <v>598</v>
+      </c>
+      <c r="K70" t="n">
+        <v>1266</v>
+      </c>
+      <c r="L70" t="n">
+        <v>1864</v>
+      </c>
+      <c r="M70" t="n">
+        <v>29494</v>
+      </c>
+      <c r="N70" t="n">
+        <v>3882</v>
+      </c>
+      <c r="O70" t="n">
+        <v>570</v>
+      </c>
+      <c r="P70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>200</v>
+      </c>
+      <c r="J71" t="n">
+        <v>585</v>
+      </c>
+      <c r="K71" t="n">
+        <v>1815</v>
+      </c>
+      <c r="L71" t="n">
+        <v>2400</v>
+      </c>
+      <c r="M71" t="n">
+        <v>35875</v>
+      </c>
+      <c r="N71" t="n">
+        <v>5073</v>
+      </c>
+      <c r="O71" t="n">
+        <v>713</v>
+      </c>
+      <c r="P71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>5</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>200</v>
+      </c>
+      <c r="J72" t="n">
+        <v>599</v>
+      </c>
+      <c r="K72" t="n">
+        <v>529</v>
+      </c>
+      <c r="L72" t="n">
+        <v>1128</v>
+      </c>
+      <c r="M72" t="n">
+        <v>61121</v>
+      </c>
+      <c r="N72" t="n">
+        <v>2694</v>
+      </c>
+      <c r="O72" t="n">
+        <v>392</v>
+      </c>
+      <c r="P72" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>responses/20260628T062329Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>20260628T062329Z</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-06-28T06:23:29.086750+00:00</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Subject: Request for a Mid‑Project Financial Progress Report – “Clean Water Init</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>200</v>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="n">
+        <v>120487</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-06-29 12:32 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S73"/>
+  <dimension ref="A1:S89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4255,8 +4255,6 @@
           <t>responses/20260628T062329Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4326,8 +4324,6 @@
           <t>responses/20260628T062329Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4397,8 +4393,6 @@
           <t>responses/20260628T062329Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4442,9 +4436,6 @@
       <c r="I61" t="n">
         <v>429</v>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
         <v>97</v>
       </c>
@@ -4457,8 +4448,6 @@
       <c r="P61" t="n">
         <v>3</v>
       </c>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -4507,9 +4496,6 @@
       <c r="I62" t="n">
         <v>429</v>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="n">
         <v>97</v>
       </c>
@@ -4522,8 +4508,6 @@
       <c r="P62" t="n">
         <v>3</v>
       </c>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -4572,9 +4556,6 @@
       <c r="I63" t="n">
         <v>429</v>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>107</v>
       </c>
@@ -4587,8 +4568,6 @@
       <c r="P63" t="n">
         <v>3</v>
       </c>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -4637,9 +4616,6 @@
       <c r="I64" t="n">
         <v>429</v>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="n">
         <v>91</v>
       </c>
@@ -4652,8 +4628,6 @@
       <c r="P64" t="n">
         <v>3</v>
       </c>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -4702,9 +4676,6 @@
       <c r="I65" t="n">
         <v>429</v>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" t="n">
         <v>232</v>
       </c>
@@ -4717,8 +4688,6 @@
       <c r="P65" t="n">
         <v>3</v>
       </c>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -4767,9 +4736,6 @@
       <c r="I66" t="n">
         <v>429</v>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
       <c r="M66" t="n">
         <v>263</v>
       </c>
@@ -4782,8 +4748,6 @@
       <c r="P66" t="n">
         <v>3</v>
       </c>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -4858,8 +4822,6 @@
           <t>responses/20260628T062329Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4929,8 +4891,6 @@
           <t>responses/20260628T062329Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5000,8 +4960,6 @@
           <t>responses/20260628T062329Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5071,8 +5029,6 @@
           <t>responses/20260628T062329Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5137,9 +5093,6 @@
       <c r="P71" t="n">
         <v>1</v>
       </c>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5204,9 +5157,6 @@
       <c r="P72" t="n">
         <v>1</v>
       </c>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5271,9 +5221,1118 @@
       <c r="P73" t="n">
         <v>1</v>
       </c>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>200</v>
+      </c>
+      <c r="J74" t="n">
+        <v>209</v>
+      </c>
+      <c r="K74" t="n">
+        <v>1118</v>
+      </c>
+      <c r="L74" t="n">
+        <v>1327</v>
+      </c>
+      <c r="M74" t="n">
+        <v>9327</v>
+      </c>
+      <c r="N74" t="n">
+        <v>4056</v>
+      </c>
+      <c r="O74" t="n">
+        <v>580</v>
+      </c>
+      <c r="P74" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>6</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>200</v>
+      </c>
+      <c r="J75" t="n">
+        <v>203</v>
+      </c>
+      <c r="K75" t="n">
+        <v>721</v>
+      </c>
+      <c r="L75" t="n">
+        <v>924</v>
+      </c>
+      <c r="M75" t="n">
+        <v>14938</v>
+      </c>
+      <c r="N75" t="n">
+        <v>3276</v>
+      </c>
+      <c r="O75" t="n">
+        <v>445</v>
+      </c>
+      <c r="P75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>6</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>429</v>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="n">
+        <v>133</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>6</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>429</v>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="n">
+        <v>193</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>6</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>429</v>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="n">
+        <v>233</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>6</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>429</v>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="n">
+        <v>166</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>6</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>200</v>
+      </c>
+      <c r="J80" t="n">
+        <v>209</v>
+      </c>
+      <c r="K80" t="n">
+        <v>2332</v>
+      </c>
+      <c r="L80" t="n">
+        <v>2541</v>
+      </c>
+      <c r="M80" t="n">
+        <v>12681</v>
+      </c>
+      <c r="N80" t="n">
+        <v>7466</v>
+      </c>
+      <c r="O80" t="n">
+        <v>1044</v>
+      </c>
+      <c r="P80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>200</v>
+      </c>
+      <c r="J81" t="n">
+        <v>250</v>
+      </c>
+      <c r="K81" t="n">
+        <v>857</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1107</v>
+      </c>
+      <c r="M81" t="n">
+        <v>13421</v>
+      </c>
+      <c r="N81" t="n">
+        <v>2664</v>
+      </c>
+      <c r="O81" t="n">
+        <v>393</v>
+      </c>
+      <c r="P81" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>6</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>200</v>
+      </c>
+      <c r="J82" t="n">
+        <v>248</v>
+      </c>
+      <c r="K82" t="n">
+        <v>1174</v>
+      </c>
+      <c r="L82" t="n">
+        <v>1422</v>
+      </c>
+      <c r="M82" t="n">
+        <v>29180</v>
+      </c>
+      <c r="N82" t="n">
+        <v>5391</v>
+      </c>
+      <c r="O82" t="n">
+        <v>763</v>
+      </c>
+      <c r="P82" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>6</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>200</v>
+      </c>
+      <c r="J83" t="n">
+        <v>236</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1142</v>
+      </c>
+      <c r="L83" t="n">
+        <v>1378</v>
+      </c>
+      <c r="M83" t="n">
+        <v>19797</v>
+      </c>
+      <c r="N83" t="n">
+        <v>4068</v>
+      </c>
+      <c r="O83" t="n">
+        <v>557</v>
+      </c>
+      <c r="P83" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>6</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>200</v>
+      </c>
+      <c r="J84" t="n">
+        <v>207</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1301</v>
+      </c>
+      <c r="L84" t="n">
+        <v>1508</v>
+      </c>
+      <c r="M84" t="n">
+        <v>25566</v>
+      </c>
+      <c r="N84" t="n">
+        <v>5695</v>
+      </c>
+      <c r="O84" t="n">
+        <v>683</v>
+      </c>
+      <c r="P84" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>6</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>200</v>
+      </c>
+      <c r="J85" t="n">
+        <v>204</v>
+      </c>
+      <c r="K85" t="n">
+        <v>787</v>
+      </c>
+      <c r="L85" t="n">
+        <v>991</v>
+      </c>
+      <c r="M85" t="n">
+        <v>53125</v>
+      </c>
+      <c r="N85" t="n">
+        <v>3406</v>
+      </c>
+      <c r="O85" t="n">
+        <v>470</v>
+      </c>
+      <c r="P85" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>6</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>200</v>
+      </c>
+      <c r="J86" t="n">
+        <v>205</v>
+      </c>
+      <c r="K86" t="n">
+        <v>2125</v>
+      </c>
+      <c r="L86" t="n">
+        <v>2330</v>
+      </c>
+      <c r="M86" t="n">
+        <v>41458</v>
+      </c>
+      <c r="N86" t="n">
+        <v>2190</v>
+      </c>
+      <c r="O86" t="n">
+        <v>279</v>
+      </c>
+      <c r="P86" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>6</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>200</v>
+      </c>
+      <c r="J87" t="n">
+        <v>209</v>
+      </c>
+      <c r="K87" t="n">
+        <v>522</v>
+      </c>
+      <c r="L87" t="n">
+        <v>731</v>
+      </c>
+      <c r="M87" t="n">
+        <v>85137</v>
+      </c>
+      <c r="N87" t="n">
+        <v>1775</v>
+      </c>
+      <c r="O87" t="n">
+        <v>240</v>
+      </c>
+      <c r="P87" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>6</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>200</v>
+      </c>
+      <c r="J88" t="n">
+        <v>177</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1938</v>
+      </c>
+      <c r="L88" t="n">
+        <v>2115</v>
+      </c>
+      <c r="M88" t="n">
+        <v>104548</v>
+      </c>
+      <c r="N88" t="n">
+        <v>7153</v>
+      </c>
+      <c r="O88" t="n">
+        <v>973</v>
+      </c>
+      <c r="P88" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>6</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Write a self-contained Java program that implements a highly concurrent token‑bu</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>200</v>
+      </c>
+      <c r="J89" t="n">
+        <v>199</v>
+      </c>
+      <c r="K89" t="n">
+        <v>2292</v>
+      </c>
+      <c r="L89" t="n">
+        <v>2491</v>
+      </c>
+      <c r="M89" t="n">
+        <v>129489</v>
+      </c>
+      <c r="N89" t="n">
+        <v>2619</v>
+      </c>
+      <c r="O89" t="n">
+        <v>342</v>
+      </c>
+      <c r="P89" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/code/poolside_laguna-m.1_free.java</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5286,7 +6345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S73"/>
+  <dimension ref="A1:S89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9118,8 +10177,6 @@
           <t>responses/20260628T062329Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9189,8 +10246,6 @@
           <t>responses/20260628T062329Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9234,9 +10289,6 @@
       <c r="I60" t="n">
         <v>429</v>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
       <c r="M60" t="n">
         <v>103</v>
       </c>
@@ -9249,8 +10301,6 @@
       <c r="P60" t="n">
         <v>3</v>
       </c>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -9299,9 +10349,6 @@
       <c r="I61" t="n">
         <v>429</v>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
         <v>104</v>
       </c>
@@ -9314,8 +10361,6 @@
       <c r="P61" t="n">
         <v>3</v>
       </c>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -9364,9 +10409,6 @@
       <c r="I62" t="n">
         <v>429</v>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="n">
         <v>82</v>
       </c>
@@ -9379,8 +10421,6 @@
       <c r="P62" t="n">
         <v>3</v>
       </c>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -9429,9 +10469,6 @@
       <c r="I63" t="n">
         <v>429</v>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>107</v>
       </c>
@@ -9444,8 +10481,6 @@
       <c r="P63" t="n">
         <v>3</v>
       </c>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -9494,9 +10529,6 @@
       <c r="I64" t="n">
         <v>429</v>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="n">
         <v>626</v>
       </c>
@@ -9509,8 +10541,6 @@
       <c r="P64" t="n">
         <v>3</v>
       </c>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -9585,8 +10615,6 @@
           <t>responses/20260628T062329Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -9656,8 +10684,6 @@
           <t>responses/20260628T062329Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9727,8 +10753,6 @@
           <t>responses/20260628T062329Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9798,8 +10822,6 @@
           <t>responses/20260628T062329Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9869,8 +10891,6 @@
           <t>responses/20260628T062329Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9940,8 +10960,6 @@
           <t>responses/20260628T062329Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10011,8 +11029,6 @@
           <t>responses/20260628T062329Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10056,9 +11072,6 @@
       <c r="I72" t="n">
         <v>200</v>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
       <c r="M72" t="n">
         <v>120220</v>
       </c>
@@ -10071,9 +11084,6 @@
       <c r="P72" t="n">
         <v>1</v>
       </c>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10143,8 +11153,1112 @@
           <t>responses/20260628T062329Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>429</v>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="n">
+        <v>188</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>6</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>429</v>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="n">
+        <v>632</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>6</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>429</v>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="n">
+        <v>169</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>6</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>429</v>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="n">
+        <v>168</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>6</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>200</v>
+      </c>
+      <c r="J78" t="n">
+        <v>170</v>
+      </c>
+      <c r="K78" t="n">
+        <v>1883</v>
+      </c>
+      <c r="L78" t="n">
+        <v>2053</v>
+      </c>
+      <c r="M78" t="n">
+        <v>27661</v>
+      </c>
+      <c r="N78" t="n">
+        <v>7411</v>
+      </c>
+      <c r="O78" t="n">
+        <v>928</v>
+      </c>
+      <c r="P78" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>6</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>200</v>
+      </c>
+      <c r="J79" t="n">
+        <v>170</v>
+      </c>
+      <c r="K79" t="n">
+        <v>1223</v>
+      </c>
+      <c r="L79" t="n">
+        <v>1393</v>
+      </c>
+      <c r="M79" t="n">
+        <v>43944</v>
+      </c>
+      <c r="N79" t="n">
+        <v>4605</v>
+      </c>
+      <c r="O79" t="n">
+        <v>558</v>
+      </c>
+      <c r="P79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>6</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>429</v>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="n">
+        <v>135</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>200</v>
+      </c>
+      <c r="J81" t="n">
+        <v>170</v>
+      </c>
+      <c r="K81" t="n">
+        <v>1906</v>
+      </c>
+      <c r="L81" t="n">
+        <v>2076</v>
+      </c>
+      <c r="M81" t="n">
+        <v>17002</v>
+      </c>
+      <c r="N81" t="n">
+        <v>5729</v>
+      </c>
+      <c r="O81" t="n">
+        <v>741</v>
+      </c>
+      <c r="P81" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>6</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>200</v>
+      </c>
+      <c r="J82" t="n">
+        <v>208</v>
+      </c>
+      <c r="K82" t="n">
+        <v>1176</v>
+      </c>
+      <c r="L82" t="n">
+        <v>1384</v>
+      </c>
+      <c r="M82" t="n">
+        <v>12366</v>
+      </c>
+      <c r="N82" t="n">
+        <v>4478</v>
+      </c>
+      <c r="O82" t="n">
+        <v>607</v>
+      </c>
+      <c r="P82" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>6</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>200</v>
+      </c>
+      <c r="J83" t="n">
+        <v>161</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1177</v>
+      </c>
+      <c r="L83" t="n">
+        <v>1338</v>
+      </c>
+      <c r="M83" t="n">
+        <v>29253</v>
+      </c>
+      <c r="N83" t="n">
+        <v>4903</v>
+      </c>
+      <c r="O83" t="n">
+        <v>692</v>
+      </c>
+      <c r="P83" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>6</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>200</v>
+      </c>
+      <c r="J84" t="n">
+        <v>213</v>
+      </c>
+      <c r="K84" t="n">
+        <v>667</v>
+      </c>
+      <c r="L84" t="n">
+        <v>880</v>
+      </c>
+      <c r="M84" t="n">
+        <v>18641</v>
+      </c>
+      <c r="N84" t="n">
+        <v>2672</v>
+      </c>
+      <c r="O84" t="n">
+        <v>367</v>
+      </c>
+      <c r="P84" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>6</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>200</v>
+      </c>
+      <c r="J85" t="n">
+        <v>143</v>
+      </c>
+      <c r="K85" t="n">
+        <v>1662</v>
+      </c>
+      <c r="L85" t="n">
+        <v>1805</v>
+      </c>
+      <c r="M85" t="n">
+        <v>29847</v>
+      </c>
+      <c r="N85" t="n">
+        <v>6219</v>
+      </c>
+      <c r="O85" t="n">
+        <v>861</v>
+      </c>
+      <c r="P85" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>6</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>200</v>
+      </c>
+      <c r="J86" t="n">
+        <v>168</v>
+      </c>
+      <c r="K86" t="n">
+        <v>997</v>
+      </c>
+      <c r="L86" t="n">
+        <v>1165</v>
+      </c>
+      <c r="M86" t="n">
+        <v>18806</v>
+      </c>
+      <c r="N86" t="n">
+        <v>4296</v>
+      </c>
+      <c r="O86" t="n">
+        <v>533</v>
+      </c>
+      <c r="P86" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>6</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>200</v>
+      </c>
+      <c r="J87" t="n">
+        <v>166</v>
+      </c>
+      <c r="K87" t="n">
+        <v>2460</v>
+      </c>
+      <c r="L87" t="n">
+        <v>2626</v>
+      </c>
+      <c r="M87" t="n">
+        <v>43387</v>
+      </c>
+      <c r="N87" t="n">
+        <v>6549</v>
+      </c>
+      <c r="O87" t="n">
+        <v>797</v>
+      </c>
+      <c r="P87" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>6</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>200</v>
+      </c>
+      <c r="J88" t="n">
+        <v>162</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1064</v>
+      </c>
+      <c r="L88" t="n">
+        <v>1226</v>
+      </c>
+      <c r="M88" t="n">
+        <v>74887</v>
+      </c>
+      <c r="N88" t="n">
+        <v>4657</v>
+      </c>
+      <c r="O88" t="n">
+        <v>647</v>
+      </c>
+      <c r="P88" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>6</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Compose an in‑depth, approximately 1000‑line article titled "Leveraging European</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>200</v>
+      </c>
+      <c r="J89" t="n">
+        <v>171</v>
+      </c>
+      <c r="K89" t="n">
+        <v>2078</v>
+      </c>
+      <c r="L89" t="n">
+        <v>2249</v>
+      </c>
+      <c r="M89" t="n">
+        <v>95147</v>
+      </c>
+      <c r="N89" t="n">
+        <v>6237</v>
+      </c>
+      <c r="O89" t="n">
+        <v>784</v>
+      </c>
+      <c r="P89" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10157,7 +12271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S73"/>
+  <dimension ref="A1:S89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13972,8 +16086,6 @@
           <t>responses/20260628T062329Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -14017,9 +16129,6 @@
       <c r="I59" t="n">
         <v>429</v>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
       <c r="M59" t="n">
         <v>92</v>
       </c>
@@ -14032,8 +16141,6 @@
       <c r="P59" t="n">
         <v>3</v>
       </c>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -14108,8 +16215,6 @@
           <t>responses/20260628T062329Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -14153,9 +16258,6 @@
       <c r="I61" t="n">
         <v>429</v>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
         <v>82</v>
       </c>
@@ -14168,8 +16270,6 @@
       <c r="P61" t="n">
         <v>3</v>
       </c>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -14218,9 +16318,6 @@
       <c r="I62" t="n">
         <v>429</v>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="n">
         <v>111</v>
       </c>
@@ -14233,8 +16330,6 @@
       <c r="P62" t="n">
         <v>3</v>
       </c>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -14283,9 +16378,6 @@
       <c r="I63" t="n">
         <v>429</v>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>88</v>
       </c>
@@ -14298,8 +16390,6 @@
       <c r="P63" t="n">
         <v>3</v>
       </c>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -14374,8 +16464,6 @@
           <t>responses/20260628T062329Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -14445,8 +16533,6 @@
           <t>responses/20260628T062329Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -14516,8 +16602,6 @@
           <t>responses/20260628T062329Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -14587,8 +16671,6 @@
           <t>responses/20260628T062329Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -14658,8 +16740,6 @@
           <t>responses/20260628T062329Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -14729,8 +16809,6 @@
           <t>responses/20260628T062329Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -14800,8 +16878,6 @@
           <t>responses/20260628T062329Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -14871,8 +16947,6 @@
           <t>responses/20260628T062329Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -14942,8 +17016,6 @@
           <t>responses/20260628T062329Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -14987,9 +17059,6 @@
       <c r="I73" t="n">
         <v>200</v>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
       <c r="M73" t="n">
         <v>120487</v>
       </c>
@@ -15002,9 +17071,1108 @@
       <c r="P73" t="n">
         <v>1</v>
       </c>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>429</v>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="n">
+        <v>171</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>6</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>200</v>
+      </c>
+      <c r="J75" t="n">
+        <v>525</v>
+      </c>
+      <c r="K75" t="n">
+        <v>1170</v>
+      </c>
+      <c r="L75" t="n">
+        <v>1695</v>
+      </c>
+      <c r="M75" t="n">
+        <v>10980</v>
+      </c>
+      <c r="N75" t="n">
+        <v>4661</v>
+      </c>
+      <c r="O75" t="n">
+        <v>653</v>
+      </c>
+      <c r="P75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>6</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>429</v>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="n">
+        <v>184</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>6</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>429</v>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="n">
+        <v>122</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>6</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>429</v>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="n">
+        <v>179</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>6</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>200</v>
+      </c>
+      <c r="J79" t="n">
+        <v>525</v>
+      </c>
+      <c r="K79" t="n">
+        <v>871</v>
+      </c>
+      <c r="L79" t="n">
+        <v>1396</v>
+      </c>
+      <c r="M79" t="n">
+        <v>40569</v>
+      </c>
+      <c r="N79" t="n">
+        <v>3799</v>
+      </c>
+      <c r="O79" t="n">
+        <v>530</v>
+      </c>
+      <c r="P79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>6</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>200</v>
+      </c>
+      <c r="J80" t="n">
+        <v>525</v>
+      </c>
+      <c r="K80" t="n">
+        <v>1029</v>
+      </c>
+      <c r="L80" t="n">
+        <v>1554</v>
+      </c>
+      <c r="M80" t="n">
+        <v>7630</v>
+      </c>
+      <c r="N80" t="n">
+        <v>4483</v>
+      </c>
+      <c r="O80" t="n">
+        <v>599</v>
+      </c>
+      <c r="P80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>200</v>
+      </c>
+      <c r="J81" t="n">
+        <v>570</v>
+      </c>
+      <c r="K81" t="n">
+        <v>751</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1321</v>
+      </c>
+      <c r="M81" t="n">
+        <v>7334</v>
+      </c>
+      <c r="N81" t="n">
+        <v>3269</v>
+      </c>
+      <c r="O81" t="n">
+        <v>438</v>
+      </c>
+      <c r="P81" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>6</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>200</v>
+      </c>
+      <c r="J82" t="n">
+        <v>541</v>
+      </c>
+      <c r="K82" t="n">
+        <v>819</v>
+      </c>
+      <c r="L82" t="n">
+        <v>1360</v>
+      </c>
+      <c r="M82" t="n">
+        <v>12399</v>
+      </c>
+      <c r="N82" t="n">
+        <v>3193</v>
+      </c>
+      <c r="O82" t="n">
+        <v>440</v>
+      </c>
+      <c r="P82" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>6</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>200</v>
+      </c>
+      <c r="J83" t="n">
+        <v>515</v>
+      </c>
+      <c r="K83" t="n">
+        <v>603</v>
+      </c>
+      <c r="L83" t="n">
+        <v>1118</v>
+      </c>
+      <c r="M83" t="n">
+        <v>22235</v>
+      </c>
+      <c r="N83" t="n">
+        <v>3131</v>
+      </c>
+      <c r="O83" t="n">
+        <v>449</v>
+      </c>
+      <c r="P83" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>6</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>200</v>
+      </c>
+      <c r="J84" t="n">
+        <v>466</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1334</v>
+      </c>
+      <c r="L84" t="n">
+        <v>1800</v>
+      </c>
+      <c r="M84" t="n">
+        <v>23005</v>
+      </c>
+      <c r="N84" t="n">
+        <v>6398</v>
+      </c>
+      <c r="O84" t="n">
+        <v>870</v>
+      </c>
+      <c r="P84" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>6</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>200</v>
+      </c>
+      <c r="J85" t="n">
+        <v>539</v>
+      </c>
+      <c r="K85" t="n">
+        <v>1015</v>
+      </c>
+      <c r="L85" t="n">
+        <v>1554</v>
+      </c>
+      <c r="M85" t="n">
+        <v>55764</v>
+      </c>
+      <c r="N85" t="n">
+        <v>4944</v>
+      </c>
+      <c r="O85" t="n">
+        <v>696</v>
+      </c>
+      <c r="P85" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>6</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>200</v>
+      </c>
+      <c r="J86" t="n">
+        <v>533</v>
+      </c>
+      <c r="K86" t="n">
+        <v>1034</v>
+      </c>
+      <c r="L86" t="n">
+        <v>1567</v>
+      </c>
+      <c r="M86" t="n">
+        <v>40840</v>
+      </c>
+      <c r="N86" t="n">
+        <v>3479</v>
+      </c>
+      <c r="O86" t="n">
+        <v>489</v>
+      </c>
+      <c r="P86" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>6</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>200</v>
+      </c>
+      <c r="J87" t="n">
+        <v>521</v>
+      </c>
+      <c r="K87" t="n">
+        <v>1676</v>
+      </c>
+      <c r="L87" t="n">
+        <v>2197</v>
+      </c>
+      <c r="M87" t="n">
+        <v>55571</v>
+      </c>
+      <c r="N87" t="n">
+        <v>5342</v>
+      </c>
+      <c r="O87" t="n">
+        <v>762</v>
+      </c>
+      <c r="P87" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>6</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>200</v>
+      </c>
+      <c r="J88" t="n">
+        <v>516</v>
+      </c>
+      <c r="K88" t="n">
+        <v>569</v>
+      </c>
+      <c r="L88" t="n">
+        <v>1085</v>
+      </c>
+      <c r="M88" t="n">
+        <v>73796</v>
+      </c>
+      <c r="N88" t="n">
+        <v>3029</v>
+      </c>
+      <c r="O88" t="n">
+        <v>436</v>
+      </c>
+      <c r="P88" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>responses/20260629T122741Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>20260629T122741Z</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-06-29T12:27:41.985967+00:00</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>6</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Subject: Inquiry Regarding Eligibility and Co‑Funding Options for the "Rural Ren</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>200</v>
+      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="n">
+        <v>120419</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q89" t="inlineStr"/>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-06-30 16:33 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S89"/>
+  <dimension ref="A1:S105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5290,8 +5290,6 @@
           <t>responses/20260629T122741Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R74" t="inlineStr"/>
-      <c r="S74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5361,8 +5359,6 @@
           <t>responses/20260629T122741Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R75" t="inlineStr"/>
-      <c r="S75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5406,9 +5402,6 @@
       <c r="I76" t="n">
         <v>429</v>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" t="n">
         <v>133</v>
       </c>
@@ -5421,8 +5414,6 @@
       <c r="P76" t="n">
         <v>3</v>
       </c>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -5471,9 +5462,6 @@
       <c r="I77" t="n">
         <v>429</v>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="n">
         <v>193</v>
       </c>
@@ -5486,8 +5474,6 @@
       <c r="P77" t="n">
         <v>3</v>
       </c>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -5536,9 +5522,6 @@
       <c r="I78" t="n">
         <v>429</v>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="n">
         <v>233</v>
       </c>
@@ -5551,8 +5534,6 @@
       <c r="P78" t="n">
         <v>3</v>
       </c>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -5601,9 +5582,6 @@
       <c r="I79" t="n">
         <v>429</v>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
       <c r="M79" t="n">
         <v>166</v>
       </c>
@@ -5616,8 +5594,6 @@
       <c r="P79" t="n">
         <v>3</v>
       </c>
-      <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -5692,8 +5668,6 @@
           <t>responses/20260629T122741Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5763,8 +5737,6 @@
           <t>responses/20260629T122741Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5834,8 +5806,6 @@
           <t>responses/20260629T122741Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5905,8 +5875,6 @@
           <t>responses/20260629T122741Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5976,8 +5944,6 @@
           <t>responses/20260629T122741Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6047,8 +6013,6 @@
           <t>responses/20260629T122741Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6118,8 +6082,6 @@
           <t>responses/20260629T122741Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr"/>
-      <c r="S86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6189,8 +6151,6 @@
           <t>responses/20260629T122741Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6260,8 +6220,6 @@
           <t>responses/20260629T122741Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6331,8 +6289,1102 @@
           <t>responses/20260629T122741Z/code/poolside_laguna-m.1_free.java</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>200</v>
+      </c>
+      <c r="J90" t="n">
+        <v>228</v>
+      </c>
+      <c r="K90" t="n">
+        <v>981</v>
+      </c>
+      <c r="L90" t="n">
+        <v>1209</v>
+      </c>
+      <c r="M90" t="n">
+        <v>15442</v>
+      </c>
+      <c r="N90" t="n">
+        <v>3650</v>
+      </c>
+      <c r="O90" t="n">
+        <v>488</v>
+      </c>
+      <c r="P90" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>7</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>429</v>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="n">
+        <v>395</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>7</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>429</v>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="n">
+        <v>413</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>7</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>429</v>
+      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="n">
+        <v>398</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>7</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>429</v>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="n">
+        <v>491</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>7</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>429</v>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="n">
+        <v>385</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>7</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>200</v>
+      </c>
+      <c r="J96" t="n">
+        <v>230</v>
+      </c>
+      <c r="K96" t="n">
+        <v>538</v>
+      </c>
+      <c r="L96" t="n">
+        <v>768</v>
+      </c>
+      <c r="M96" t="n">
+        <v>13644</v>
+      </c>
+      <c r="N96" t="n">
+        <v>2372</v>
+      </c>
+      <c r="O96" t="n">
+        <v>320</v>
+      </c>
+      <c r="P96" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>7</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>200</v>
+      </c>
+      <c r="J97" t="n">
+        <v>228</v>
+      </c>
+      <c r="K97" t="n">
+        <v>1437</v>
+      </c>
+      <c r="L97" t="n">
+        <v>1665</v>
+      </c>
+      <c r="M97" t="n">
+        <v>9540</v>
+      </c>
+      <c r="N97" t="n">
+        <v>5248</v>
+      </c>
+      <c r="O97" t="n">
+        <v>741</v>
+      </c>
+      <c r="P97" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr"/>
+      <c r="S97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>7</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>200</v>
+      </c>
+      <c r="J98" t="n">
+        <v>258</v>
+      </c>
+      <c r="K98" t="n">
+        <v>1100</v>
+      </c>
+      <c r="L98" t="n">
+        <v>1358</v>
+      </c>
+      <c r="M98" t="n">
+        <v>20246</v>
+      </c>
+      <c r="N98" t="n">
+        <v>3866</v>
+      </c>
+      <c r="O98" t="n">
+        <v>512</v>
+      </c>
+      <c r="P98" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr"/>
+      <c r="S98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>7</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>200</v>
+      </c>
+      <c r="J99" t="n">
+        <v>270</v>
+      </c>
+      <c r="K99" t="n">
+        <v>1611</v>
+      </c>
+      <c r="L99" t="n">
+        <v>1881</v>
+      </c>
+      <c r="M99" t="n">
+        <v>21377</v>
+      </c>
+      <c r="N99" t="n">
+        <v>4630</v>
+      </c>
+      <c r="O99" t="n">
+        <v>647</v>
+      </c>
+      <c r="P99" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr"/>
+      <c r="S99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>7</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>200</v>
+      </c>
+      <c r="J100" t="n">
+        <v>228</v>
+      </c>
+      <c r="K100" t="n">
+        <v>678</v>
+      </c>
+      <c r="L100" t="n">
+        <v>906</v>
+      </c>
+      <c r="M100" t="n">
+        <v>44226</v>
+      </c>
+      <c r="N100" t="n">
+        <v>2186</v>
+      </c>
+      <c r="O100" t="n">
+        <v>289</v>
+      </c>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr"/>
+      <c r="S100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>7</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>200</v>
+      </c>
+      <c r="J101" t="n">
+        <v>194</v>
+      </c>
+      <c r="K101" t="n">
+        <v>1297</v>
+      </c>
+      <c r="L101" t="n">
+        <v>1491</v>
+      </c>
+      <c r="M101" t="n">
+        <v>35721</v>
+      </c>
+      <c r="N101" t="n">
+        <v>3636</v>
+      </c>
+      <c r="O101" t="n">
+        <v>493</v>
+      </c>
+      <c r="P101" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr"/>
+      <c r="S101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>7</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>200</v>
+      </c>
+      <c r="J102" t="n">
+        <v>231</v>
+      </c>
+      <c r="K102" t="n">
+        <v>748</v>
+      </c>
+      <c r="L102" t="n">
+        <v>979</v>
+      </c>
+      <c r="M102" t="n">
+        <v>69562</v>
+      </c>
+      <c r="N102" t="n">
+        <v>3237</v>
+      </c>
+      <c r="O102" t="n">
+        <v>423</v>
+      </c>
+      <c r="P102" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>7</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>200</v>
+      </c>
+      <c r="J103" t="n">
+        <v>221</v>
+      </c>
+      <c r="K103" t="n">
+        <v>611</v>
+      </c>
+      <c r="L103" t="n">
+        <v>832</v>
+      </c>
+      <c r="M103" t="n">
+        <v>75103</v>
+      </c>
+      <c r="N103" t="n">
+        <v>1650</v>
+      </c>
+      <c r="O103" t="n">
+        <v>222</v>
+      </c>
+      <c r="P103" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/poolside_laguna-m.1_free.java</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr"/>
+      <c r="S103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>7</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>200</v>
+      </c>
+      <c r="J104" t="n">
+        <v>224</v>
+      </c>
+      <c r="K104" t="n">
+        <v>1907</v>
+      </c>
+      <c r="L104" t="n">
+        <v>2131</v>
+      </c>
+      <c r="M104" t="n">
+        <v>89441</v>
+      </c>
+      <c r="N104" t="n">
+        <v>3006</v>
+      </c>
+      <c r="O104" t="n">
+        <v>392</v>
+      </c>
+      <c r="P104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>7</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent, lock‑fr</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>200</v>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="n">
+        <v>121370</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="inlineStr"/>
+      <c r="S105" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6345,7 +7397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S89"/>
+  <dimension ref="A1:S105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11196,9 +12248,6 @@
       <c r="I74" t="n">
         <v>429</v>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" t="n">
         <v>188</v>
       </c>
@@ -11211,8 +12260,6 @@
       <c r="P74" t="n">
         <v>3</v>
       </c>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -11261,9 +12308,6 @@
       <c r="I75" t="n">
         <v>429</v>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
       <c r="M75" t="n">
         <v>632</v>
       </c>
@@ -11276,8 +12320,6 @@
       <c r="P75" t="n">
         <v>3</v>
       </c>
-      <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -11326,9 +12368,6 @@
       <c r="I76" t="n">
         <v>429</v>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" t="n">
         <v>169</v>
       </c>
@@ -11341,8 +12380,6 @@
       <c r="P76" t="n">
         <v>3</v>
       </c>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -11391,9 +12428,6 @@
       <c r="I77" t="n">
         <v>429</v>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="n">
         <v>168</v>
       </c>
@@ -11406,8 +12440,6 @@
       <c r="P77" t="n">
         <v>3</v>
       </c>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -11482,8 +12514,6 @@
           <t>responses/20260629T122741Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr"/>
-      <c r="S78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -11553,8 +12583,6 @@
           <t>responses/20260629T122741Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -11598,9 +12626,6 @@
       <c r="I80" t="n">
         <v>429</v>
       </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
       <c r="M80" t="n">
         <v>135</v>
       </c>
@@ -11613,8 +12638,6 @@
       <c r="P80" t="n">
         <v>3</v>
       </c>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -11689,8 +12712,6 @@
           <t>responses/20260629T122741Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -11760,8 +12781,6 @@
           <t>responses/20260629T122741Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -11831,8 +12850,6 @@
           <t>responses/20260629T122741Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -11902,8 +12919,6 @@
           <t>responses/20260629T122741Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -11973,8 +12988,6 @@
           <t>responses/20260629T122741Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -12044,8 +13057,6 @@
           <t>responses/20260629T122741Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr"/>
-      <c r="S86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12115,8 +13126,6 @@
           <t>responses/20260629T122741Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -12186,8 +13195,6 @@
           <t>responses/20260629T122741Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12257,8 +13264,1112 @@
           <t>responses/20260629T122741Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>200</v>
+      </c>
+      <c r="J90" t="n">
+        <v>252</v>
+      </c>
+      <c r="K90" t="n">
+        <v>185</v>
+      </c>
+      <c r="L90" t="n">
+        <v>437</v>
+      </c>
+      <c r="M90" t="n">
+        <v>1993</v>
+      </c>
+      <c r="N90" t="n">
+        <v>61</v>
+      </c>
+      <c r="O90" t="n">
+        <v>13</v>
+      </c>
+      <c r="P90" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>7</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>429</v>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="n">
+        <v>568</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>7</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>429</v>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="n">
+        <v>353</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>7</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>200</v>
+      </c>
+      <c r="J93" t="n">
+        <v>252</v>
+      </c>
+      <c r="K93" t="n">
+        <v>269</v>
+      </c>
+      <c r="L93" t="n">
+        <v>521</v>
+      </c>
+      <c r="M93" t="n">
+        <v>36645</v>
+      </c>
+      <c r="N93" t="n">
+        <v>404</v>
+      </c>
+      <c r="O93" t="n">
+        <v>69</v>
+      </c>
+      <c r="P93" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>7</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>429</v>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="n">
+        <v>355</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>7</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>429</v>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="n">
+        <v>389</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>7</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>429</v>
+      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="n">
+        <v>1212</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>7</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>200</v>
+      </c>
+      <c r="J97" t="n">
+        <v>215</v>
+      </c>
+      <c r="K97" t="n">
+        <v>88</v>
+      </c>
+      <c r="L97" t="n">
+        <v>303</v>
+      </c>
+      <c r="M97" t="n">
+        <v>13710</v>
+      </c>
+      <c r="N97" t="n">
+        <v>44</v>
+      </c>
+      <c r="O97" t="n">
+        <v>8</v>
+      </c>
+      <c r="P97" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr"/>
+      <c r="S97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>7</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>200</v>
+      </c>
+      <c r="J98" t="n">
+        <v>252</v>
+      </c>
+      <c r="K98" t="n">
+        <v>3862</v>
+      </c>
+      <c r="L98" t="n">
+        <v>4114</v>
+      </c>
+      <c r="M98" t="n">
+        <v>16785</v>
+      </c>
+      <c r="N98" t="n">
+        <v>13183</v>
+      </c>
+      <c r="O98" t="n">
+        <v>1874</v>
+      </c>
+      <c r="P98" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr"/>
+      <c r="S98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>7</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>200</v>
+      </c>
+      <c r="J99" t="n">
+        <v>292</v>
+      </c>
+      <c r="K99" t="n">
+        <v>654</v>
+      </c>
+      <c r="L99" t="n">
+        <v>946</v>
+      </c>
+      <c r="M99" t="n">
+        <v>6953</v>
+      </c>
+      <c r="N99" t="n">
+        <v>1235</v>
+      </c>
+      <c r="O99" t="n">
+        <v>187</v>
+      </c>
+      <c r="P99" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr"/>
+      <c r="S99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>7</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>200</v>
+      </c>
+      <c r="J100" t="n">
+        <v>290</v>
+      </c>
+      <c r="K100" t="n">
+        <v>3277</v>
+      </c>
+      <c r="L100" t="n">
+        <v>3567</v>
+      </c>
+      <c r="M100" t="n">
+        <v>39535</v>
+      </c>
+      <c r="N100" t="n">
+        <v>12075</v>
+      </c>
+      <c r="O100" t="n">
+        <v>1715</v>
+      </c>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr"/>
+      <c r="S100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>7</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>200</v>
+      </c>
+      <c r="J101" t="n">
+        <v>288</v>
+      </c>
+      <c r="K101" t="n">
+        <v>2505</v>
+      </c>
+      <c r="L101" t="n">
+        <v>2793</v>
+      </c>
+      <c r="M101" t="n">
+        <v>103141</v>
+      </c>
+      <c r="N101" t="n">
+        <v>10256</v>
+      </c>
+      <c r="O101" t="n">
+        <v>1430</v>
+      </c>
+      <c r="P101" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr"/>
+      <c r="S101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>7</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>200</v>
+      </c>
+      <c r="J102" t="n">
+        <v>240</v>
+      </c>
+      <c r="K102" t="n">
+        <v>1518</v>
+      </c>
+      <c r="L102" t="n">
+        <v>1758</v>
+      </c>
+      <c r="M102" t="n">
+        <v>151919</v>
+      </c>
+      <c r="N102" t="n">
+        <v>6145</v>
+      </c>
+      <c r="O102" t="n">
+        <v>839</v>
+      </c>
+      <c r="P102" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>7</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>200</v>
+      </c>
+      <c r="J103" t="n">
+        <v>250</v>
+      </c>
+      <c r="K103" t="n">
+        <v>5471</v>
+      </c>
+      <c r="L103" t="n">
+        <v>5721</v>
+      </c>
+      <c r="M103" t="n">
+        <v>136880</v>
+      </c>
+      <c r="N103" t="n">
+        <v>32477</v>
+      </c>
+      <c r="O103" t="n">
+        <v>4187</v>
+      </c>
+      <c r="P103" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr"/>
+      <c r="S103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>7</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>200</v>
+      </c>
+      <c r="J104" t="n">
+        <v>248</v>
+      </c>
+      <c r="K104" t="n">
+        <v>5729</v>
+      </c>
+      <c r="L104" t="n">
+        <v>5977</v>
+      </c>
+      <c r="M104" t="n">
+        <v>178489</v>
+      </c>
+      <c r="N104" t="n">
+        <v>30480</v>
+      </c>
+      <c r="O104" t="n">
+        <v>4007</v>
+      </c>
+      <c r="P104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>7</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>200</v>
+      </c>
+      <c r="J105" t="n">
+        <v>255</v>
+      </c>
+      <c r="K105" t="n">
+        <v>4204</v>
+      </c>
+      <c r="L105" t="n">
+        <v>4459</v>
+      </c>
+      <c r="M105" t="n">
+        <v>551604</v>
+      </c>
+      <c r="N105" t="n">
+        <v>12437</v>
+      </c>
+      <c r="O105" t="n">
+        <v>1539</v>
+      </c>
+      <c r="P105" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr"/>
+      <c r="S105" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12271,7 +14382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S89"/>
+  <dimension ref="A1:S105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17114,9 +19225,6 @@
       <c r="I74" t="n">
         <v>429</v>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" t="n">
         <v>171</v>
       </c>
@@ -17129,8 +19237,6 @@
       <c r="P74" t="n">
         <v>3</v>
       </c>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -17205,8 +19311,6 @@
           <t>responses/20260629T122741Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R75" t="inlineStr"/>
-      <c r="S75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -17250,9 +19354,6 @@
       <c r="I76" t="n">
         <v>429</v>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" t="n">
         <v>184</v>
       </c>
@@ -17265,8 +19366,6 @@
       <c r="P76" t="n">
         <v>3</v>
       </c>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -17315,9 +19414,6 @@
       <c r="I77" t="n">
         <v>429</v>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="n">
         <v>122</v>
       </c>
@@ -17330,8 +19426,6 @@
       <c r="P77" t="n">
         <v>3</v>
       </c>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -17380,9 +19474,6 @@
       <c r="I78" t="n">
         <v>429</v>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="n">
         <v>179</v>
       </c>
@@ -17395,8 +19486,6 @@
       <c r="P78" t="n">
         <v>3</v>
       </c>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -17471,8 +19560,6 @@
           <t>responses/20260629T122741Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -17542,8 +19629,6 @@
           <t>responses/20260629T122741Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -17613,8 +19698,6 @@
           <t>responses/20260629T122741Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -17684,8 +19767,6 @@
           <t>responses/20260629T122741Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -17755,8 +19836,6 @@
           <t>responses/20260629T122741Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -17826,8 +19905,6 @@
           <t>responses/20260629T122741Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -17897,8 +19974,6 @@
           <t>responses/20260629T122741Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -17968,8 +20043,6 @@
           <t>responses/20260629T122741Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr"/>
-      <c r="S86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -18039,8 +20112,6 @@
           <t>responses/20260629T122741Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -18110,8 +20181,6 @@
           <t>responses/20260629T122741Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -18155,9 +20224,6 @@
       <c r="I89" t="n">
         <v>200</v>
       </c>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
       <c r="M89" t="n">
         <v>120419</v>
       </c>
@@ -18170,9 +20236,1092 @@
       <c r="P89" t="n">
         <v>1</v>
       </c>
-      <c r="Q89" t="inlineStr"/>
-      <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>429</v>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="n">
+        <v>328</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q90" t="inlineStr"/>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>7</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>200</v>
+      </c>
+      <c r="J91" t="n">
+        <v>597</v>
+      </c>
+      <c r="K91" t="n">
+        <v>901</v>
+      </c>
+      <c r="L91" t="n">
+        <v>1498</v>
+      </c>
+      <c r="M91" t="n">
+        <v>20487</v>
+      </c>
+      <c r="N91" t="n">
+        <v>3821</v>
+      </c>
+      <c r="O91" t="n">
+        <v>562</v>
+      </c>
+      <c r="P91" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>7</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>200</v>
+      </c>
+      <c r="J92" t="n">
+        <v>597</v>
+      </c>
+      <c r="K92" t="n">
+        <v>991</v>
+      </c>
+      <c r="L92" t="n">
+        <v>1588</v>
+      </c>
+      <c r="M92" t="n">
+        <v>13252</v>
+      </c>
+      <c r="N92" t="n">
+        <v>3465</v>
+      </c>
+      <c r="O92" t="n">
+        <v>536</v>
+      </c>
+      <c r="P92" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>7</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>429</v>
+      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="n">
+        <v>1416</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>7</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>429</v>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="n">
+        <v>795</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>7</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>200</v>
+      </c>
+      <c r="J95" t="n">
+        <v>605</v>
+      </c>
+      <c r="K95" t="n">
+        <v>569</v>
+      </c>
+      <c r="L95" t="n">
+        <v>1174</v>
+      </c>
+      <c r="M95" t="n">
+        <v>11863</v>
+      </c>
+      <c r="N95" t="n">
+        <v>2878</v>
+      </c>
+      <c r="O95" t="n">
+        <v>434</v>
+      </c>
+      <c r="P95" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>7</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>429</v>
+      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="n">
+        <v>390</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>7</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>429</v>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="n">
+        <v>392</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q97" t="inlineStr"/>
+      <c r="R97" t="inlineStr"/>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>7</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>200</v>
+      </c>
+      <c r="J98" t="n">
+        <v>597</v>
+      </c>
+      <c r="K98" t="n">
+        <v>1042</v>
+      </c>
+      <c r="L98" t="n">
+        <v>1639</v>
+      </c>
+      <c r="M98" t="n">
+        <v>10588</v>
+      </c>
+      <c r="N98" t="n">
+        <v>4684</v>
+      </c>
+      <c r="O98" t="n">
+        <v>735</v>
+      </c>
+      <c r="P98" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr"/>
+      <c r="S98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>7</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>200</v>
+      </c>
+      <c r="J99" t="n">
+        <v>538</v>
+      </c>
+      <c r="K99" t="n">
+        <v>1078</v>
+      </c>
+      <c r="L99" t="n">
+        <v>1616</v>
+      </c>
+      <c r="M99" t="n">
+        <v>20472</v>
+      </c>
+      <c r="N99" t="n">
+        <v>3397</v>
+      </c>
+      <c r="O99" t="n">
+        <v>498</v>
+      </c>
+      <c r="P99" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr"/>
+      <c r="S99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>7</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>200</v>
+      </c>
+      <c r="J100" t="n">
+        <v>640</v>
+      </c>
+      <c r="K100" t="n">
+        <v>863</v>
+      </c>
+      <c r="L100" t="n">
+        <v>1503</v>
+      </c>
+      <c r="M100" t="n">
+        <v>10428</v>
+      </c>
+      <c r="N100" t="n">
+        <v>3005</v>
+      </c>
+      <c r="O100" t="n">
+        <v>432</v>
+      </c>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr"/>
+      <c r="S100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>7</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>200</v>
+      </c>
+      <c r="J101" t="n">
+        <v>614</v>
+      </c>
+      <c r="K101" t="n">
+        <v>1530</v>
+      </c>
+      <c r="L101" t="n">
+        <v>2144</v>
+      </c>
+      <c r="M101" t="n">
+        <v>18607</v>
+      </c>
+      <c r="N101" t="n">
+        <v>4609</v>
+      </c>
+      <c r="O101" t="n">
+        <v>751</v>
+      </c>
+      <c r="P101" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr"/>
+      <c r="S101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>7</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q102" t="inlineStr"/>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>JSONDecodeError: Expecting value: line 377 column 1 (char 2068)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>7</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>200</v>
+      </c>
+      <c r="J103" t="n">
+        <v>606</v>
+      </c>
+      <c r="K103" t="n">
+        <v>538</v>
+      </c>
+      <c r="L103" t="n">
+        <v>1144</v>
+      </c>
+      <c r="M103" t="n">
+        <v>80735</v>
+      </c>
+      <c r="N103" t="n">
+        <v>2841</v>
+      </c>
+      <c r="O103" t="n">
+        <v>402</v>
+      </c>
+      <c r="P103" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr"/>
+      <c r="S103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>7</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>200</v>
+      </c>
+      <c r="J104" t="n">
+        <v>593</v>
+      </c>
+      <c r="K104" t="n">
+        <v>2160</v>
+      </c>
+      <c r="L104" t="n">
+        <v>2753</v>
+      </c>
+      <c r="M104" t="n">
+        <v>93145</v>
+      </c>
+      <c r="N104" t="n">
+        <v>6330</v>
+      </c>
+      <c r="O104" t="n">
+        <v>936</v>
+      </c>
+      <c r="P104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>responses/20260630T162244Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20260630T162244Z</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-06-30T16:22:44.741466+00:00</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>7</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Indirect Cost Rate Allocation for Our Upco</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>200</v>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="n">
+        <v>120797</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="inlineStr"/>
+      <c r="S105" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-01 21:37 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S105"/>
+  <dimension ref="A1:S121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6358,8 +6358,6 @@
           <t>responses/20260630T162244Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R90" t="inlineStr"/>
-      <c r="S90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6403,9 +6401,6 @@
       <c r="I91" t="n">
         <v>429</v>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="n">
         <v>395</v>
       </c>
@@ -6418,8 +6413,6 @@
       <c r="P91" t="n">
         <v>3</v>
       </c>
-      <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
       <c r="S91" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -6468,9 +6461,6 @@
       <c r="I92" t="n">
         <v>429</v>
       </c>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
       <c r="M92" t="n">
         <v>413</v>
       </c>
@@ -6483,8 +6473,6 @@
       <c r="P92" t="n">
         <v>3</v>
       </c>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
       <c r="S92" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -6533,9 +6521,6 @@
       <c r="I93" t="n">
         <v>429</v>
       </c>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="n">
         <v>398</v>
       </c>
@@ -6548,8 +6533,6 @@
       <c r="P93" t="n">
         <v>3</v>
       </c>
-      <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
       <c r="S93" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -6598,9 +6581,6 @@
       <c r="I94" t="n">
         <v>429</v>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="n">
         <v>491</v>
       </c>
@@ -6613,8 +6593,6 @@
       <c r="P94" t="n">
         <v>3</v>
       </c>
-      <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -6663,9 +6641,6 @@
       <c r="I95" t="n">
         <v>429</v>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
       <c r="M95" t="n">
         <v>385</v>
       </c>
@@ -6678,8 +6653,6 @@
       <c r="P95" t="n">
         <v>3</v>
       </c>
-      <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="inlineStr"/>
       <c r="S95" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -6754,8 +6727,6 @@
           <t>responses/20260630T162244Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R96" t="inlineStr"/>
-      <c r="S96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6825,8 +6796,6 @@
           <t>responses/20260630T162244Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R97" t="inlineStr"/>
-      <c r="S97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6896,8 +6865,6 @@
           <t>responses/20260630T162244Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr"/>
-      <c r="S98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6967,8 +6934,6 @@
           <t>responses/20260630T162244Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R99" t="inlineStr"/>
-      <c r="S99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7038,8 +7003,6 @@
           <t>responses/20260630T162244Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R100" t="inlineStr"/>
-      <c r="S100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7109,8 +7072,6 @@
           <t>responses/20260630T162244Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr"/>
-      <c r="S101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7180,8 +7141,6 @@
           <t>responses/20260630T162244Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr"/>
-      <c r="S102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7251,8 +7210,6 @@
           <t>responses/20260630T162244Z/code/poolside_laguna-m.1_free.java</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr"/>
-      <c r="S103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7322,8 +7279,6 @@
           <t>responses/20260630T162244Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
         </is>
       </c>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7367,9 +7322,6 @@
       <c r="I105" t="n">
         <v>200</v>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" t="n">
         <v>121370</v>
       </c>
@@ -7382,9 +7334,1100 @@
       <c r="P105" t="n">
         <v>1</v>
       </c>
-      <c r="Q105" t="inlineStr"/>
-      <c r="R105" t="inlineStr"/>
-      <c r="S105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>8</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>200</v>
+      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="n">
+        <v>1205</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>8</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>200</v>
+      </c>
+      <c r="J107" t="n">
+        <v>242</v>
+      </c>
+      <c r="K107" t="n">
+        <v>1597</v>
+      </c>
+      <c r="L107" t="n">
+        <v>1839</v>
+      </c>
+      <c r="M107" t="n">
+        <v>9242</v>
+      </c>
+      <c r="N107" t="n">
+        <v>4726</v>
+      </c>
+      <c r="O107" t="n">
+        <v>673</v>
+      </c>
+      <c r="P107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr"/>
+      <c r="S107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>8</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>429</v>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="n">
+        <v>139</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>8</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>429</v>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="n">
+        <v>219</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="inlineStr"/>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>8</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>429</v>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="n">
+        <v>187</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>8</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>429</v>
+      </c>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="n">
+        <v>148</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q111" t="inlineStr"/>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>8</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>200</v>
+      </c>
+      <c r="J112" t="n">
+        <v>242</v>
+      </c>
+      <c r="K112" t="n">
+        <v>1154</v>
+      </c>
+      <c r="L112" t="n">
+        <v>1396</v>
+      </c>
+      <c r="M112" t="n">
+        <v>16508</v>
+      </c>
+      <c r="N112" t="n">
+        <v>4287</v>
+      </c>
+      <c r="O112" t="n">
+        <v>583</v>
+      </c>
+      <c r="P112" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>8</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>200</v>
+      </c>
+      <c r="J113" t="n">
+        <v>289</v>
+      </c>
+      <c r="K113" t="n">
+        <v>27</v>
+      </c>
+      <c r="L113" t="n">
+        <v>316</v>
+      </c>
+      <c r="M113" t="n">
+        <v>2299</v>
+      </c>
+      <c r="N113" t="n">
+        <v>38</v>
+      </c>
+      <c r="O113" t="n">
+        <v>8</v>
+      </c>
+      <c r="P113" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>8</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>200</v>
+      </c>
+      <c r="J114" t="n">
+        <v>218</v>
+      </c>
+      <c r="K114" t="n">
+        <v>1428</v>
+      </c>
+      <c r="L114" t="n">
+        <v>1646</v>
+      </c>
+      <c r="M114" t="n">
+        <v>11554</v>
+      </c>
+      <c r="N114" t="n">
+        <v>36</v>
+      </c>
+      <c r="O114" t="n">
+        <v>7</v>
+      </c>
+      <c r="P114" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>8</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>200</v>
+      </c>
+      <c r="J115" t="n">
+        <v>291</v>
+      </c>
+      <c r="K115" t="n">
+        <v>857</v>
+      </c>
+      <c r="L115" t="n">
+        <v>1148</v>
+      </c>
+      <c r="M115" t="n">
+        <v>11272</v>
+      </c>
+      <c r="N115" t="n">
+        <v>2253</v>
+      </c>
+      <c r="O115" t="n">
+        <v>336</v>
+      </c>
+      <c r="P115" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr"/>
+      <c r="S115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>8</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>200</v>
+      </c>
+      <c r="J116" t="n">
+        <v>244</v>
+      </c>
+      <c r="K116" t="n">
+        <v>2137</v>
+      </c>
+      <c r="L116" t="n">
+        <v>2381</v>
+      </c>
+      <c r="M116" t="n">
+        <v>56512</v>
+      </c>
+      <c r="N116" t="n">
+        <v>8595</v>
+      </c>
+      <c r="O116" t="n">
+        <v>890</v>
+      </c>
+      <c r="P116" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>8</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>200</v>
+      </c>
+      <c r="J117" t="n">
+        <v>245</v>
+      </c>
+      <c r="K117" t="n">
+        <v>2504</v>
+      </c>
+      <c r="L117" t="n">
+        <v>2749</v>
+      </c>
+      <c r="M117" t="n">
+        <v>58566</v>
+      </c>
+      <c r="N117" t="n">
+        <v>12462</v>
+      </c>
+      <c r="O117" t="n">
+        <v>1098</v>
+      </c>
+      <c r="P117" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>8</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>200</v>
+      </c>
+      <c r="J118" t="n">
+        <v>275</v>
+      </c>
+      <c r="K118" t="n">
+        <v>5759</v>
+      </c>
+      <c r="L118" t="n">
+        <v>6034</v>
+      </c>
+      <c r="M118" t="n">
+        <v>94320</v>
+      </c>
+      <c r="N118" t="n">
+        <v>22192</v>
+      </c>
+      <c r="O118" t="n">
+        <v>2049</v>
+      </c>
+      <c r="P118" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>8</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>200</v>
+      </c>
+      <c r="J119" t="n">
+        <v>238</v>
+      </c>
+      <c r="K119" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L119" t="n">
+        <v>6238</v>
+      </c>
+      <c r="M119" t="n">
+        <v>171029</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0</v>
+      </c>
+      <c r="P119" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>8</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>200</v>
+      </c>
+      <c r="J120" t="n">
+        <v>245</v>
+      </c>
+      <c r="K120" t="n">
+        <v>2699</v>
+      </c>
+      <c r="L120" t="n">
+        <v>2944</v>
+      </c>
+      <c r="M120" t="n">
+        <v>311251</v>
+      </c>
+      <c r="N120" t="n">
+        <v>11397</v>
+      </c>
+      <c r="O120" t="n">
+        <v>1271</v>
+      </c>
+      <c r="P120" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>8</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that implements a highly concurrent **work‑s</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>200</v>
+      </c>
+      <c r="J121" t="n">
+        <v>238</v>
+      </c>
+      <c r="K121" t="n">
+        <v>1476</v>
+      </c>
+      <c r="L121" t="n">
+        <v>1714</v>
+      </c>
+      <c r="M121" t="n">
+        <v>600387</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0</v>
+      </c>
+      <c r="P121" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7397,7 +8440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S105"/>
+  <dimension ref="A1:S121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13333,8 +14376,6 @@
           <t>responses/20260630T162244Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R90" t="inlineStr"/>
-      <c r="S90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -13378,9 +14419,6 @@
       <c r="I91" t="n">
         <v>429</v>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="n">
         <v>568</v>
       </c>
@@ -13393,8 +14431,6 @@
       <c r="P91" t="n">
         <v>3</v>
       </c>
-      <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
       <c r="S91" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -13443,9 +14479,6 @@
       <c r="I92" t="n">
         <v>429</v>
       </c>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
       <c r="M92" t="n">
         <v>353</v>
       </c>
@@ -13458,8 +14491,6 @@
       <c r="P92" t="n">
         <v>3</v>
       </c>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
       <c r="S92" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -13534,8 +14565,6 @@
           <t>responses/20260630T162244Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R93" t="inlineStr"/>
-      <c r="S93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13579,9 +14608,6 @@
       <c r="I94" t="n">
         <v>429</v>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="n">
         <v>355</v>
       </c>
@@ -13594,8 +14620,6 @@
       <c r="P94" t="n">
         <v>3</v>
       </c>
-      <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -13644,9 +14668,6 @@
       <c r="I95" t="n">
         <v>429</v>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
       <c r="M95" t="n">
         <v>389</v>
       </c>
@@ -13659,8 +14680,6 @@
       <c r="P95" t="n">
         <v>3</v>
       </c>
-      <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="inlineStr"/>
       <c r="S95" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -13709,9 +14728,6 @@
       <c r="I96" t="n">
         <v>429</v>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
       <c r="M96" t="n">
         <v>1212</v>
       </c>
@@ -13724,8 +14740,6 @@
       <c r="P96" t="n">
         <v>3</v>
       </c>
-      <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr"/>
       <c r="S96" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -13800,8 +14814,6 @@
           <t>responses/20260630T162244Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R97" t="inlineStr"/>
-      <c r="S97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13871,8 +14883,6 @@
           <t>responses/20260630T162244Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr"/>
-      <c r="S98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -13942,8 +14952,6 @@
           <t>responses/20260630T162244Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R99" t="inlineStr"/>
-      <c r="S99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -14013,8 +15021,6 @@
           <t>responses/20260630T162244Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R100" t="inlineStr"/>
-      <c r="S100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14084,8 +15090,6 @@
           <t>responses/20260630T162244Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr"/>
-      <c r="S101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -14155,8 +15159,6 @@
           <t>responses/20260630T162244Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr"/>
-      <c r="S102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -14226,8 +15228,6 @@
           <t>responses/20260630T162244Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr"/>
-      <c r="S103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -14297,8 +15297,6 @@
           <t>responses/20260630T162244Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -14368,8 +15366,1118 @@
           <t>responses/20260630T162244Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R105" t="inlineStr"/>
-      <c r="S105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>8</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>429</v>
+      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="n">
+        <v>163</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>8</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>200</v>
+      </c>
+      <c r="J107" t="n">
+        <v>383</v>
+      </c>
+      <c r="K107" t="n">
+        <v>2996</v>
+      </c>
+      <c r="L107" t="n">
+        <v>3379</v>
+      </c>
+      <c r="M107" t="n">
+        <v>26966</v>
+      </c>
+      <c r="N107" t="n">
+        <v>10495</v>
+      </c>
+      <c r="O107" t="n">
+        <v>1425</v>
+      </c>
+      <c r="P107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr"/>
+      <c r="S107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>8</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>429</v>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="n">
+        <v>143</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>8</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>429</v>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="n">
+        <v>145</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="inlineStr"/>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>8</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>429</v>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="n">
+        <v>151</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>8</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>200</v>
+      </c>
+      <c r="J111" t="n">
+        <v>383</v>
+      </c>
+      <c r="K111" t="n">
+        <v>3587</v>
+      </c>
+      <c r="L111" t="n">
+        <v>3970</v>
+      </c>
+      <c r="M111" t="n">
+        <v>17783</v>
+      </c>
+      <c r="N111" t="n">
+        <v>11948</v>
+      </c>
+      <c r="O111" t="n">
+        <v>1589</v>
+      </c>
+      <c r="P111" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>8</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>200</v>
+      </c>
+      <c r="J112" t="n">
+        <v>383</v>
+      </c>
+      <c r="K112" t="n">
+        <v>4108</v>
+      </c>
+      <c r="L112" t="n">
+        <v>4491</v>
+      </c>
+      <c r="M112" t="n">
+        <v>70228</v>
+      </c>
+      <c r="N112" t="n">
+        <v>15562</v>
+      </c>
+      <c r="O112" t="n">
+        <v>1900</v>
+      </c>
+      <c r="P112" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>8</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>200</v>
+      </c>
+      <c r="J113" t="n">
+        <v>410</v>
+      </c>
+      <c r="K113" t="n">
+        <v>1578</v>
+      </c>
+      <c r="L113" t="n">
+        <v>1988</v>
+      </c>
+      <c r="M113" t="n">
+        <v>73815</v>
+      </c>
+      <c r="N113" t="n">
+        <v>6872</v>
+      </c>
+      <c r="O113" t="n">
+        <v>852</v>
+      </c>
+      <c r="P113" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>8</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>200</v>
+      </c>
+      <c r="J114" t="n">
+        <v>391</v>
+      </c>
+      <c r="K114" t="n">
+        <v>2531</v>
+      </c>
+      <c r="L114" t="n">
+        <v>2922</v>
+      </c>
+      <c r="M114" t="n">
+        <v>32343</v>
+      </c>
+      <c r="N114" t="n">
+        <v>7270</v>
+      </c>
+      <c r="O114" t="n">
+        <v>894</v>
+      </c>
+      <c r="P114" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>8</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>200</v>
+      </c>
+      <c r="J115" t="n">
+        <v>376</v>
+      </c>
+      <c r="K115" t="n">
+        <v>1598</v>
+      </c>
+      <c r="L115" t="n">
+        <v>1974</v>
+      </c>
+      <c r="M115" t="n">
+        <v>47159</v>
+      </c>
+      <c r="N115" t="n">
+        <v>6989</v>
+      </c>
+      <c r="O115" t="n">
+        <v>1011</v>
+      </c>
+      <c r="P115" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr"/>
+      <c r="S115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>8</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>200</v>
+      </c>
+      <c r="J116" t="n">
+        <v>412</v>
+      </c>
+      <c r="K116" t="n">
+        <v>1564</v>
+      </c>
+      <c r="L116" t="n">
+        <v>1976</v>
+      </c>
+      <c r="M116" t="n">
+        <v>26476</v>
+      </c>
+      <c r="N116" t="n">
+        <v>5237</v>
+      </c>
+      <c r="O116" t="n">
+        <v>739</v>
+      </c>
+      <c r="P116" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>8</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>200</v>
+      </c>
+      <c r="J117" t="n">
+        <v>428</v>
+      </c>
+      <c r="K117" t="n">
+        <v>2607</v>
+      </c>
+      <c r="L117" t="n">
+        <v>3035</v>
+      </c>
+      <c r="M117" t="n">
+        <v>26115</v>
+      </c>
+      <c r="N117" t="n">
+        <v>11404</v>
+      </c>
+      <c r="O117" t="n">
+        <v>1448</v>
+      </c>
+      <c r="P117" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>8</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>200</v>
+      </c>
+      <c r="J118" t="n">
+        <v>335</v>
+      </c>
+      <c r="K118" t="n">
+        <v>2308</v>
+      </c>
+      <c r="L118" t="n">
+        <v>2643</v>
+      </c>
+      <c r="M118" t="n">
+        <v>44573</v>
+      </c>
+      <c r="N118" t="n">
+        <v>8117</v>
+      </c>
+      <c r="O118" t="n">
+        <v>1053</v>
+      </c>
+      <c r="P118" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>8</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>200</v>
+      </c>
+      <c r="J119" t="n">
+        <v>381</v>
+      </c>
+      <c r="K119" t="n">
+        <v>4026</v>
+      </c>
+      <c r="L119" t="n">
+        <v>4407</v>
+      </c>
+      <c r="M119" t="n">
+        <v>91817</v>
+      </c>
+      <c r="N119" t="n">
+        <v>17685</v>
+      </c>
+      <c r="O119" t="n">
+        <v>2155</v>
+      </c>
+      <c r="P119" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>8</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>200</v>
+      </c>
+      <c r="J120" t="n">
+        <v>377</v>
+      </c>
+      <c r="K120" t="n">
+        <v>1206</v>
+      </c>
+      <c r="L120" t="n">
+        <v>1583</v>
+      </c>
+      <c r="M120" t="n">
+        <v>144637</v>
+      </c>
+      <c r="N120" t="n">
+        <v>5022</v>
+      </c>
+      <c r="O120" t="n">
+        <v>691</v>
+      </c>
+      <c r="P120" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>8</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 word) in‑depth, well‑stru</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>200</v>
+      </c>
+      <c r="J121" t="n">
+        <v>379</v>
+      </c>
+      <c r="K121" t="n">
+        <v>3845</v>
+      </c>
+      <c r="L121" t="n">
+        <v>4224</v>
+      </c>
+      <c r="M121" t="n">
+        <v>137030</v>
+      </c>
+      <c r="N121" t="n">
+        <v>10255</v>
+      </c>
+      <c r="O121" t="n">
+        <v>1325</v>
+      </c>
+      <c r="P121" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14382,7 +16490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S105"/>
+  <dimension ref="A1:S121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20279,9 +22387,6 @@
       <c r="I90" t="n">
         <v>429</v>
       </c>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" t="n">
         <v>328</v>
       </c>
@@ -20294,8 +22399,6 @@
       <c r="P90" t="n">
         <v>3</v>
       </c>
-      <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
       <c r="S90" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -20370,8 +22473,6 @@
           <t>responses/20260630T162244Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R91" t="inlineStr"/>
-      <c r="S91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -20441,8 +22542,6 @@
           <t>responses/20260630T162244Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -20486,9 +22585,6 @@
       <c r="I93" t="n">
         <v>429</v>
       </c>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="n">
         <v>1416</v>
       </c>
@@ -20501,8 +22597,6 @@
       <c r="P93" t="n">
         <v>3</v>
       </c>
-      <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
       <c r="S93" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -20551,9 +22645,6 @@
       <c r="I94" t="n">
         <v>429</v>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="n">
         <v>795</v>
       </c>
@@ -20566,8 +22657,6 @@
       <c r="P94" t="n">
         <v>3</v>
       </c>
-      <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -20642,8 +22731,6 @@
           <t>responses/20260630T162244Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R95" t="inlineStr"/>
-      <c r="S95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -20687,9 +22774,6 @@
       <c r="I96" t="n">
         <v>429</v>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
       <c r="M96" t="n">
         <v>390</v>
       </c>
@@ -20702,8 +22786,6 @@
       <c r="P96" t="n">
         <v>3</v>
       </c>
-      <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr"/>
       <c r="S96" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -20752,9 +22834,6 @@
       <c r="I97" t="n">
         <v>429</v>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" t="n">
         <v>392</v>
       </c>
@@ -20767,8 +22846,6 @@
       <c r="P97" t="n">
         <v>3</v>
       </c>
-      <c r="Q97" t="inlineStr"/>
-      <c r="R97" t="inlineStr"/>
       <c r="S97" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -20843,8 +22920,6 @@
           <t>responses/20260630T162244Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr"/>
-      <c r="S98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -20914,8 +22989,6 @@
           <t>responses/20260630T162244Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R99" t="inlineStr"/>
-      <c r="S99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -20985,8 +23058,6 @@
           <t>responses/20260630T162244Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R100" t="inlineStr"/>
-      <c r="S100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -21056,8 +23127,6 @@
           <t>responses/20260630T162244Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr"/>
-      <c r="S101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -21098,11 +23167,6 @@
           <t>error</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
       <c r="N102" t="n">
         <v>0</v>
       </c>
@@ -21112,8 +23176,6 @@
       <c r="P102" t="n">
         <v>3</v>
       </c>
-      <c r="Q102" t="inlineStr"/>
-      <c r="R102" t="inlineStr"/>
       <c r="S102" t="inlineStr">
         <is>
           <t>JSONDecodeError: Expecting value: line 377 column 1 (char 2068)</t>
@@ -21188,8 +23250,6 @@
           <t>responses/20260630T162244Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr"/>
-      <c r="S103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -21259,8 +23319,6 @@
           <t>responses/20260630T162244Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -21304,9 +23362,6 @@
       <c r="I105" t="n">
         <v>200</v>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" t="n">
         <v>120797</v>
       </c>
@@ -21319,9 +23374,1118 @@
       <c r="P105" t="n">
         <v>1</v>
       </c>
-      <c r="Q105" t="inlineStr"/>
-      <c r="R105" t="inlineStr"/>
-      <c r="S105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>8</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>429</v>
+      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="n">
+        <v>173</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>8</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>200</v>
+      </c>
+      <c r="J107" t="n">
+        <v>566</v>
+      </c>
+      <c r="K107" t="n">
+        <v>714</v>
+      </c>
+      <c r="L107" t="n">
+        <v>1280</v>
+      </c>
+      <c r="M107" t="n">
+        <v>11345</v>
+      </c>
+      <c r="N107" t="n">
+        <v>2792</v>
+      </c>
+      <c r="O107" t="n">
+        <v>397</v>
+      </c>
+      <c r="P107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr"/>
+      <c r="S107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>8</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>429</v>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="n">
+        <v>209</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>8</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>200</v>
+      </c>
+      <c r="J109" t="n">
+        <v>582</v>
+      </c>
+      <c r="K109" t="n">
+        <v>682</v>
+      </c>
+      <c r="L109" t="n">
+        <v>1264</v>
+      </c>
+      <c r="M109" t="n">
+        <v>29066</v>
+      </c>
+      <c r="N109" t="n">
+        <v>3228</v>
+      </c>
+      <c r="O109" t="n">
+        <v>471</v>
+      </c>
+      <c r="P109" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr"/>
+      <c r="S109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>8</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>429</v>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="n">
+        <v>150</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>8</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>200</v>
+      </c>
+      <c r="J111" t="n">
+        <v>556</v>
+      </c>
+      <c r="K111" t="n">
+        <v>448</v>
+      </c>
+      <c r="L111" t="n">
+        <v>1004</v>
+      </c>
+      <c r="M111" t="n">
+        <v>9728</v>
+      </c>
+      <c r="N111" t="n">
+        <v>2269</v>
+      </c>
+      <c r="O111" t="n">
+        <v>342</v>
+      </c>
+      <c r="P111" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>8</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>429</v>
+      </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="n">
+        <v>195</v>
+      </c>
+      <c r="N112" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>8</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>200</v>
+      </c>
+      <c r="J113" t="n">
+        <v>566</v>
+      </c>
+      <c r="K113" t="n">
+        <v>823</v>
+      </c>
+      <c r="L113" t="n">
+        <v>1389</v>
+      </c>
+      <c r="M113" t="n">
+        <v>5101</v>
+      </c>
+      <c r="N113" t="n">
+        <v>3551</v>
+      </c>
+      <c r="O113" t="n">
+        <v>518</v>
+      </c>
+      <c r="P113" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>8</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>200</v>
+      </c>
+      <c r="J114" t="n">
+        <v>502</v>
+      </c>
+      <c r="K114" t="n">
+        <v>823</v>
+      </c>
+      <c r="L114" t="n">
+        <v>1325</v>
+      </c>
+      <c r="M114" t="n">
+        <v>8684</v>
+      </c>
+      <c r="N114" t="n">
+        <v>3825</v>
+      </c>
+      <c r="O114" t="n">
+        <v>557</v>
+      </c>
+      <c r="P114" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>8</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>200</v>
+      </c>
+      <c r="J115" t="n">
+        <v>614</v>
+      </c>
+      <c r="K115" t="n">
+        <v>610</v>
+      </c>
+      <c r="L115" t="n">
+        <v>1224</v>
+      </c>
+      <c r="M115" t="n">
+        <v>4841</v>
+      </c>
+      <c r="N115" t="n">
+        <v>1883</v>
+      </c>
+      <c r="O115" t="n">
+        <v>267</v>
+      </c>
+      <c r="P115" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr"/>
+      <c r="S115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>8</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>200</v>
+      </c>
+      <c r="J116" t="n">
+        <v>584</v>
+      </c>
+      <c r="K116" t="n">
+        <v>775</v>
+      </c>
+      <c r="L116" t="n">
+        <v>1359</v>
+      </c>
+      <c r="M116" t="n">
+        <v>11574</v>
+      </c>
+      <c r="N116" t="n">
+        <v>2986</v>
+      </c>
+      <c r="O116" t="n">
+        <v>462</v>
+      </c>
+      <c r="P116" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>8</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>200</v>
+      </c>
+      <c r="J117" t="n">
+        <v>557</v>
+      </c>
+      <c r="K117" t="n">
+        <v>438</v>
+      </c>
+      <c r="L117" t="n">
+        <v>995</v>
+      </c>
+      <c r="M117" t="n">
+        <v>64440</v>
+      </c>
+      <c r="N117" t="n">
+        <v>2193</v>
+      </c>
+      <c r="O117" t="n">
+        <v>315</v>
+      </c>
+      <c r="P117" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>8</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>200</v>
+      </c>
+      <c r="J118" t="n">
+        <v>562</v>
+      </c>
+      <c r="K118" t="n">
+        <v>594</v>
+      </c>
+      <c r="L118" t="n">
+        <v>1156</v>
+      </c>
+      <c r="M118" t="n">
+        <v>36834</v>
+      </c>
+      <c r="N118" t="n">
+        <v>3128</v>
+      </c>
+      <c r="O118" t="n">
+        <v>439</v>
+      </c>
+      <c r="P118" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>8</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>200</v>
+      </c>
+      <c r="J119" t="n">
+        <v>562</v>
+      </c>
+      <c r="K119" t="n">
+        <v>1467</v>
+      </c>
+      <c r="L119" t="n">
+        <v>2029</v>
+      </c>
+      <c r="M119" t="n">
+        <v>42026</v>
+      </c>
+      <c r="N119" t="n">
+        <v>4175</v>
+      </c>
+      <c r="O119" t="n">
+        <v>588</v>
+      </c>
+      <c r="P119" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>8</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>200</v>
+      </c>
+      <c r="J120" t="n">
+        <v>577</v>
+      </c>
+      <c r="K120" t="n">
+        <v>902</v>
+      </c>
+      <c r="L120" t="n">
+        <v>1479</v>
+      </c>
+      <c r="M120" t="n">
+        <v>74060</v>
+      </c>
+      <c r="N120" t="n">
+        <v>2729</v>
+      </c>
+      <c r="O120" t="n">
+        <v>408</v>
+      </c>
+      <c r="P120" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>20260701T212623Z</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-07-01T21:26:23.695256+00:00</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>8</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Southwest Co</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>200</v>
+      </c>
+      <c r="J121" t="n">
+        <v>566</v>
+      </c>
+      <c r="K121" t="n">
+        <v>826</v>
+      </c>
+      <c r="L121" t="n">
+        <v>1392</v>
+      </c>
+      <c r="M121" t="n">
+        <v>156063</v>
+      </c>
+      <c r="N121" t="n">
+        <v>2810</v>
+      </c>
+      <c r="O121" t="n">
+        <v>406</v>
+      </c>
+      <c r="P121" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>responses/20260701T212623Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-02 08:19 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S121"/>
+  <dimension ref="A1:S137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7377,9 +7377,6 @@
       <c r="I106" t="n">
         <v>200</v>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" t="n">
         <v>1205</v>
       </c>
@@ -7392,9 +7389,6 @@
       <c r="P106" t="n">
         <v>1</v>
       </c>
-      <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr"/>
-      <c r="S106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7464,8 +7458,6 @@
           <t>responses/20260701T212623Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R107" t="inlineStr"/>
-      <c r="S107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7509,9 +7501,6 @@
       <c r="I108" t="n">
         <v>429</v>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" t="n">
         <v>139</v>
       </c>
@@ -7524,8 +7513,6 @@
       <c r="P108" t="n">
         <v>3</v>
       </c>
-      <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -7574,9 +7561,6 @@
       <c r="I109" t="n">
         <v>429</v>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
       <c r="M109" t="n">
         <v>219</v>
       </c>
@@ -7589,8 +7573,6 @@
       <c r="P109" t="n">
         <v>3</v>
       </c>
-      <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr"/>
       <c r="S109" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -7639,9 +7621,6 @@
       <c r="I110" t="n">
         <v>429</v>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
       <c r="M110" t="n">
         <v>187</v>
       </c>
@@ -7654,8 +7633,6 @@
       <c r="P110" t="n">
         <v>3</v>
       </c>
-      <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -7704,9 +7681,6 @@
       <c r="I111" t="n">
         <v>429</v>
       </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
       <c r="M111" t="n">
         <v>148</v>
       </c>
@@ -7719,8 +7693,6 @@
       <c r="P111" t="n">
         <v>3</v>
       </c>
-      <c r="Q111" t="inlineStr"/>
-      <c r="R111" t="inlineStr"/>
       <c r="S111" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -7795,8 +7767,6 @@
           <t>responses/20260701T212623Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R112" t="inlineStr"/>
-      <c r="S112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7866,8 +7836,6 @@
           <t>responses/20260701T212623Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R113" t="inlineStr"/>
-      <c r="S113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7937,8 +7905,6 @@
           <t>responses/20260701T212623Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr"/>
-      <c r="S114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8008,8 +7974,6 @@
           <t>responses/20260701T212623Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R115" t="inlineStr"/>
-      <c r="S115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8079,8 +8043,6 @@
           <t>responses/20260701T212623Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R116" t="inlineStr"/>
-      <c r="S116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8150,8 +8112,6 @@
           <t>responses/20260701T212623Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R117" t="inlineStr"/>
-      <c r="S117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8221,8 +8181,6 @@
           <t>responses/20260701T212623Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R118" t="inlineStr"/>
-      <c r="S118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8287,9 +8245,6 @@
       <c r="P119" t="n">
         <v>1</v>
       </c>
-      <c r="Q119" t="inlineStr"/>
-      <c r="R119" t="inlineStr"/>
-      <c r="S119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8359,8 +8314,6 @@
           <t>responses/20260701T212623Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R120" t="inlineStr"/>
-      <c r="S120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8425,9 +8378,1088 @@
       <c r="P121" t="n">
         <v>1</v>
       </c>
-      <c r="Q121" t="inlineStr"/>
-      <c r="R121" t="inlineStr"/>
-      <c r="S121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>9</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>400</v>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="n">
+        <v>213</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0</v>
+      </c>
+      <c r="P122" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>9</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>429</v>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="n">
+        <v>179</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0</v>
+      </c>
+      <c r="P123" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>9</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>429</v>
+      </c>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="n">
+        <v>180</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>9</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>429</v>
+      </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="n">
+        <v>157</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
+      <c r="P125" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>9</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>429</v>
+      </c>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="n">
+        <v>295</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>9</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>429</v>
+      </c>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="n">
+        <v>158</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
+      <c r="P127" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>9</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>200</v>
+      </c>
+      <c r="J128" t="n">
+        <v>88</v>
+      </c>
+      <c r="K128" t="n">
+        <v>5383</v>
+      </c>
+      <c r="L128" t="n">
+        <v>5471</v>
+      </c>
+      <c r="M128" t="n">
+        <v>29517</v>
+      </c>
+      <c r="N128" t="n">
+        <v>20762</v>
+      </c>
+      <c r="O128" t="n">
+        <v>2331</v>
+      </c>
+      <c r="P128" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>9</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>200</v>
+      </c>
+      <c r="J129" t="n">
+        <v>139</v>
+      </c>
+      <c r="K129" t="n">
+        <v>4005</v>
+      </c>
+      <c r="L129" t="n">
+        <v>4144</v>
+      </c>
+      <c r="M129" t="n">
+        <v>58900</v>
+      </c>
+      <c r="N129" t="n">
+        <v>16970</v>
+      </c>
+      <c r="O129" t="n">
+        <v>1835</v>
+      </c>
+      <c r="P129" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>9</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>200</v>
+      </c>
+      <c r="J130" t="n">
+        <v>118</v>
+      </c>
+      <c r="K130" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L130" t="n">
+        <v>6118</v>
+      </c>
+      <c r="M130" t="n">
+        <v>59119</v>
+      </c>
+      <c r="N130" t="n">
+        <v>20242</v>
+      </c>
+      <c r="O130" t="n">
+        <v>1821</v>
+      </c>
+      <c r="P130" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>9</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>200</v>
+      </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="n">
+        <v>120350</v>
+      </c>
+      <c r="N131" t="n">
+        <v>0</v>
+      </c>
+      <c r="O131" t="n">
+        <v>0</v>
+      </c>
+      <c r="P131" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q131" t="inlineStr"/>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>9</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>200</v>
+      </c>
+      <c r="J132" t="n">
+        <v>84</v>
+      </c>
+      <c r="K132" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L132" t="n">
+        <v>6084</v>
+      </c>
+      <c r="M132" t="n">
+        <v>137082</v>
+      </c>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+      <c r="O132" t="n">
+        <v>0</v>
+      </c>
+      <c r="P132" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q132" t="inlineStr"/>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>9</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>200</v>
+      </c>
+      <c r="J133" t="n">
+        <v>137</v>
+      </c>
+      <c r="K133" t="n">
+        <v>5379</v>
+      </c>
+      <c r="L133" t="n">
+        <v>5516</v>
+      </c>
+      <c r="M133" t="n">
+        <v>168372</v>
+      </c>
+      <c r="N133" t="n">
+        <v>25628</v>
+      </c>
+      <c r="O133" t="n">
+        <v>2904</v>
+      </c>
+      <c r="P133" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>9</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>200</v>
+      </c>
+      <c r="J134" t="n">
+        <v>86</v>
+      </c>
+      <c r="K134" t="n">
+        <v>2534</v>
+      </c>
+      <c r="L134" t="n">
+        <v>2620</v>
+      </c>
+      <c r="M134" t="n">
+        <v>228381</v>
+      </c>
+      <c r="N134" t="n">
+        <v>10725</v>
+      </c>
+      <c r="O134" t="n">
+        <v>1036</v>
+      </c>
+      <c r="P134" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>9</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>200</v>
+      </c>
+      <c r="J135" t="n">
+        <v>66</v>
+      </c>
+      <c r="K135" t="n">
+        <v>4675</v>
+      </c>
+      <c r="L135" t="n">
+        <v>4741</v>
+      </c>
+      <c r="M135" t="n">
+        <v>215653</v>
+      </c>
+      <c r="N135" t="n">
+        <v>3558</v>
+      </c>
+      <c r="O135" t="n">
+        <v>480</v>
+      </c>
+      <c r="P135" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>9</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>200</v>
+      </c>
+      <c r="J136" t="n">
+        <v>88</v>
+      </c>
+      <c r="K136" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L136" t="n">
+        <v>6088</v>
+      </c>
+      <c r="M136" t="n">
+        <v>246792</v>
+      </c>
+      <c r="N136" t="n">
+        <v>13793</v>
+      </c>
+      <c r="O136" t="n">
+        <v>1729</v>
+      </c>
+      <c r="P136" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>9</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>200</v>
+      </c>
+      <c r="J137" t="n">
+        <v>81</v>
+      </c>
+      <c r="K137" t="n">
+        <v>1490</v>
+      </c>
+      <c r="L137" t="n">
+        <v>1571</v>
+      </c>
+      <c r="M137" t="n">
+        <v>600502</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
+      <c r="P137" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8440,7 +9472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S121"/>
+  <dimension ref="A1:S137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15409,9 +16441,6 @@
       <c r="I106" t="n">
         <v>429</v>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" t="n">
         <v>163</v>
       </c>
@@ -15424,8 +16453,6 @@
       <c r="P106" t="n">
         <v>3</v>
       </c>
-      <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr"/>
       <c r="S106" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -15500,8 +16527,6 @@
           <t>responses/20260701T212623Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R107" t="inlineStr"/>
-      <c r="S107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -15545,9 +16570,6 @@
       <c r="I108" t="n">
         <v>429</v>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" t="n">
         <v>143</v>
       </c>
@@ -15560,8 +16582,6 @@
       <c r="P108" t="n">
         <v>3</v>
       </c>
-      <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -15610,9 +16630,6 @@
       <c r="I109" t="n">
         <v>429</v>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
       <c r="M109" t="n">
         <v>145</v>
       </c>
@@ -15625,8 +16642,6 @@
       <c r="P109" t="n">
         <v>3</v>
       </c>
-      <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr"/>
       <c r="S109" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -15675,9 +16690,6 @@
       <c r="I110" t="n">
         <v>429</v>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
       <c r="M110" t="n">
         <v>151</v>
       </c>
@@ -15690,8 +16702,6 @@
       <c r="P110" t="n">
         <v>3</v>
       </c>
-      <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -15766,8 +16776,6 @@
           <t>responses/20260701T212623Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R111" t="inlineStr"/>
-      <c r="S111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -15837,8 +16845,6 @@
           <t>responses/20260701T212623Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R112" t="inlineStr"/>
-      <c r="S112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -15908,8 +16914,6 @@
           <t>responses/20260701T212623Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R113" t="inlineStr"/>
-      <c r="S113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -15979,8 +16983,6 @@
           <t>responses/20260701T212623Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr"/>
-      <c r="S114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -16050,8 +17052,6 @@
           <t>responses/20260701T212623Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R115" t="inlineStr"/>
-      <c r="S115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -16121,8 +17121,6 @@
           <t>responses/20260701T212623Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R116" t="inlineStr"/>
-      <c r="S116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -16192,8 +17190,6 @@
           <t>responses/20260701T212623Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R117" t="inlineStr"/>
-      <c r="S117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -16263,8 +17259,6 @@
           <t>responses/20260701T212623Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R118" t="inlineStr"/>
-      <c r="S118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -16334,8 +17328,6 @@
           <t>responses/20260701T212623Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R119" t="inlineStr"/>
-      <c r="S119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -16405,8 +17397,6 @@
           <t>responses/20260701T212623Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R120" t="inlineStr"/>
-      <c r="S120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -16476,8 +17466,1086 @@
           <t>responses/20260701T212623Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R121" t="inlineStr"/>
-      <c r="S121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>9</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>400</v>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="n">
+        <v>99</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0</v>
+      </c>
+      <c r="P122" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>9</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>429</v>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="n">
+        <v>137</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0</v>
+      </c>
+      <c r="P123" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>9</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>429</v>
+      </c>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="n">
+        <v>162</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>9</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>429</v>
+      </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="n">
+        <v>173</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
+      <c r="P125" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>9</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>429</v>
+      </c>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="n">
+        <v>228</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>9</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>429</v>
+      </c>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="n">
+        <v>1076</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
+      <c r="P127" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>9</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>200</v>
+      </c>
+      <c r="J128" t="n">
+        <v>73</v>
+      </c>
+      <c r="K128" t="n">
+        <v>4568</v>
+      </c>
+      <c r="L128" t="n">
+        <v>4641</v>
+      </c>
+      <c r="M128" t="n">
+        <v>19134</v>
+      </c>
+      <c r="N128" t="n">
+        <v>11955</v>
+      </c>
+      <c r="O128" t="n">
+        <v>1687</v>
+      </c>
+      <c r="P128" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>9</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>200</v>
+      </c>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="n">
+        <v>10409</v>
+      </c>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="n">
+        <v>0</v>
+      </c>
+      <c r="P129" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>9</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>200</v>
+      </c>
+      <c r="J130" t="n">
+        <v>120</v>
+      </c>
+      <c r="K130" t="n">
+        <v>5020</v>
+      </c>
+      <c r="L130" t="n">
+        <v>5140</v>
+      </c>
+      <c r="M130" t="n">
+        <v>144905</v>
+      </c>
+      <c r="N130" t="n">
+        <v>20481</v>
+      </c>
+      <c r="O130" t="n">
+        <v>3125</v>
+      </c>
+      <c r="P130" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>9</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>200</v>
+      </c>
+      <c r="J131" t="n">
+        <v>69</v>
+      </c>
+      <c r="K131" t="n">
+        <v>3607</v>
+      </c>
+      <c r="L131" t="n">
+        <v>3676</v>
+      </c>
+      <c r="M131" t="n">
+        <v>72593</v>
+      </c>
+      <c r="N131" t="n">
+        <v>12011</v>
+      </c>
+      <c r="O131" t="n">
+        <v>1713</v>
+      </c>
+      <c r="P131" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>9</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>200</v>
+      </c>
+      <c r="J132" t="n">
+        <v>73</v>
+      </c>
+      <c r="K132" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L132" t="n">
+        <v>8073</v>
+      </c>
+      <c r="M132" t="n">
+        <v>160031</v>
+      </c>
+      <c r="N132" t="n">
+        <v>29212</v>
+      </c>
+      <c r="O132" t="n">
+        <v>4025</v>
+      </c>
+      <c r="P132" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>9</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>200</v>
+      </c>
+      <c r="J133" t="n">
+        <v>70</v>
+      </c>
+      <c r="K133" t="n">
+        <v>733</v>
+      </c>
+      <c r="L133" t="n">
+        <v>803</v>
+      </c>
+      <c r="M133" t="n">
+        <v>116074</v>
+      </c>
+      <c r="N133" t="n">
+        <v>2777</v>
+      </c>
+      <c r="O133" t="n">
+        <v>452</v>
+      </c>
+      <c r="P133" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>9</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>200</v>
+      </c>
+      <c r="J134" t="n">
+        <v>106</v>
+      </c>
+      <c r="K134" t="n">
+        <v>4549</v>
+      </c>
+      <c r="L134" t="n">
+        <v>4655</v>
+      </c>
+      <c r="M134" t="n">
+        <v>72137</v>
+      </c>
+      <c r="N134" t="n">
+        <v>25356</v>
+      </c>
+      <c r="O134" t="n">
+        <v>3345</v>
+      </c>
+      <c r="P134" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>9</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>200</v>
+      </c>
+      <c r="J135" t="n">
+        <v>69</v>
+      </c>
+      <c r="K135" t="n">
+        <v>3920</v>
+      </c>
+      <c r="L135" t="n">
+        <v>3989</v>
+      </c>
+      <c r="M135" t="n">
+        <v>93352</v>
+      </c>
+      <c r="N135" t="n">
+        <v>10168</v>
+      </c>
+      <c r="O135" t="n">
+        <v>1451</v>
+      </c>
+      <c r="P135" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>9</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>200</v>
+      </c>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="n">
+        <v>120339</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+      <c r="O136" t="n">
+        <v>0</v>
+      </c>
+      <c r="P136" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q136" t="inlineStr"/>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>9</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>200</v>
+      </c>
+      <c r="J137" t="n">
+        <v>51</v>
+      </c>
+      <c r="K137" t="n">
+        <v>6350</v>
+      </c>
+      <c r="L137" t="n">
+        <v>6401</v>
+      </c>
+      <c r="M137" t="n">
+        <v>381645</v>
+      </c>
+      <c r="N137" t="n">
+        <v>25338</v>
+      </c>
+      <c r="O137" t="n">
+        <v>3409</v>
+      </c>
+      <c r="P137" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16490,7 +18558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S121"/>
+  <dimension ref="A1:S137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23417,9 +25485,6 @@
       <c r="I106" t="n">
         <v>429</v>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" t="n">
         <v>173</v>
       </c>
@@ -23432,8 +25497,6 @@
       <c r="P106" t="n">
         <v>3</v>
       </c>
-      <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr"/>
       <c r="S106" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -23508,8 +25571,6 @@
           <t>responses/20260701T212623Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R107" t="inlineStr"/>
-      <c r="S107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -23553,9 +25614,6 @@
       <c r="I108" t="n">
         <v>429</v>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" t="n">
         <v>209</v>
       </c>
@@ -23568,8 +25626,6 @@
       <c r="P108" t="n">
         <v>3</v>
       </c>
-      <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -23644,8 +25700,6 @@
           <t>responses/20260701T212623Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R109" t="inlineStr"/>
-      <c r="S109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -23689,9 +25743,6 @@
       <c r="I110" t="n">
         <v>429</v>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
       <c r="M110" t="n">
         <v>150</v>
       </c>
@@ -23704,8 +25755,6 @@
       <c r="P110" t="n">
         <v>3</v>
       </c>
-      <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -23780,8 +25829,6 @@
           <t>responses/20260701T212623Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R111" t="inlineStr"/>
-      <c r="S111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -23825,9 +25872,6 @@
       <c r="I112" t="n">
         <v>429</v>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
       <c r="M112" t="n">
         <v>195</v>
       </c>
@@ -23840,8 +25884,6 @@
       <c r="P112" t="n">
         <v>3</v>
       </c>
-      <c r="Q112" t="inlineStr"/>
-      <c r="R112" t="inlineStr"/>
       <c r="S112" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -23916,8 +25958,6 @@
           <t>responses/20260701T212623Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R113" t="inlineStr"/>
-      <c r="S113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -23987,8 +26027,6 @@
           <t>responses/20260701T212623Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr"/>
-      <c r="S114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -24058,8 +26096,6 @@
           <t>responses/20260701T212623Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R115" t="inlineStr"/>
-      <c r="S115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -24129,8 +26165,6 @@
           <t>responses/20260701T212623Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R116" t="inlineStr"/>
-      <c r="S116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -24200,8 +26234,6 @@
           <t>responses/20260701T212623Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R117" t="inlineStr"/>
-      <c r="S117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -24271,8 +26303,6 @@
           <t>responses/20260701T212623Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R118" t="inlineStr"/>
-      <c r="S118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -24342,8 +26372,6 @@
           <t>responses/20260701T212623Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R119" t="inlineStr"/>
-      <c r="S119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -24413,8 +26441,6 @@
           <t>responses/20260701T212623Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R120" t="inlineStr"/>
-      <c r="S120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -24484,8 +26510,1112 @@
           <t>responses/20260701T212623Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R121" t="inlineStr"/>
-      <c r="S121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>9</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>400</v>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="n">
+        <v>87</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0</v>
+      </c>
+      <c r="P122" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>9</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>429</v>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="n">
+        <v>151</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0</v>
+      </c>
+      <c r="P123" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>9</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>429</v>
+      </c>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="n">
+        <v>156</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>9</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>429</v>
+      </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="n">
+        <v>209</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
+      <c r="P125" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>9</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>200</v>
+      </c>
+      <c r="J126" t="n">
+        <v>292</v>
+      </c>
+      <c r="K126" t="n">
+        <v>937</v>
+      </c>
+      <c r="L126" t="n">
+        <v>1229</v>
+      </c>
+      <c r="M126" t="n">
+        <v>30873</v>
+      </c>
+      <c r="N126" t="n">
+        <v>3994</v>
+      </c>
+      <c r="O126" t="n">
+        <v>569</v>
+      </c>
+      <c r="P126" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>9</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>429</v>
+      </c>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="n">
+        <v>174</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
+      <c r="P127" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>9</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>200</v>
+      </c>
+      <c r="J128" t="n">
+        <v>292</v>
+      </c>
+      <c r="K128" t="n">
+        <v>880</v>
+      </c>
+      <c r="L128" t="n">
+        <v>1172</v>
+      </c>
+      <c r="M128" t="n">
+        <v>5562</v>
+      </c>
+      <c r="N128" t="n">
+        <v>3802</v>
+      </c>
+      <c r="O128" t="n">
+        <v>541</v>
+      </c>
+      <c r="P128" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>9</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>200</v>
+      </c>
+      <c r="J129" t="n">
+        <v>289</v>
+      </c>
+      <c r="K129" t="n">
+        <v>412</v>
+      </c>
+      <c r="L129" t="n">
+        <v>701</v>
+      </c>
+      <c r="M129" t="n">
+        <v>13545</v>
+      </c>
+      <c r="N129" t="n">
+        <v>2173</v>
+      </c>
+      <c r="O129" t="n">
+        <v>326</v>
+      </c>
+      <c r="P129" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>9</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>200</v>
+      </c>
+      <c r="J130" t="n">
+        <v>256</v>
+      </c>
+      <c r="K130" t="n">
+        <v>860</v>
+      </c>
+      <c r="L130" t="n">
+        <v>1116</v>
+      </c>
+      <c r="M130" t="n">
+        <v>10623</v>
+      </c>
+      <c r="N130" t="n">
+        <v>4167</v>
+      </c>
+      <c r="O130" t="n">
+        <v>583</v>
+      </c>
+      <c r="P130" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>9</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>200</v>
+      </c>
+      <c r="J131" t="n">
+        <v>332</v>
+      </c>
+      <c r="K131" t="n">
+        <v>699</v>
+      </c>
+      <c r="L131" t="n">
+        <v>1031</v>
+      </c>
+      <c r="M131" t="n">
+        <v>7115</v>
+      </c>
+      <c r="N131" t="n">
+        <v>3026</v>
+      </c>
+      <c r="O131" t="n">
+        <v>437</v>
+      </c>
+      <c r="P131" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>9</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>200</v>
+      </c>
+      <c r="J132" t="n">
+        <v>332</v>
+      </c>
+      <c r="K132" t="n">
+        <v>927</v>
+      </c>
+      <c r="L132" t="n">
+        <v>1259</v>
+      </c>
+      <c r="M132" t="n">
+        <v>13202</v>
+      </c>
+      <c r="N132" t="n">
+        <v>3953</v>
+      </c>
+      <c r="O132" t="n">
+        <v>580</v>
+      </c>
+      <c r="P132" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>9</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>200</v>
+      </c>
+      <c r="J133" t="n">
+        <v>330</v>
+      </c>
+      <c r="K133" t="n">
+        <v>942</v>
+      </c>
+      <c r="L133" t="n">
+        <v>1272</v>
+      </c>
+      <c r="M133" t="n">
+        <v>58608</v>
+      </c>
+      <c r="N133" t="n">
+        <v>4614</v>
+      </c>
+      <c r="O133" t="n">
+        <v>673</v>
+      </c>
+      <c r="P133" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>9</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>200</v>
+      </c>
+      <c r="J134" t="n">
+        <v>290</v>
+      </c>
+      <c r="K134" t="n">
+        <v>396</v>
+      </c>
+      <c r="L134" t="n">
+        <v>686</v>
+      </c>
+      <c r="M134" t="n">
+        <v>30469</v>
+      </c>
+      <c r="N134" t="n">
+        <v>2108</v>
+      </c>
+      <c r="O134" t="n">
+        <v>320</v>
+      </c>
+      <c r="P134" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>9</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>200</v>
+      </c>
+      <c r="J135" t="n">
+        <v>287</v>
+      </c>
+      <c r="K135" t="n">
+        <v>576</v>
+      </c>
+      <c r="L135" t="n">
+        <v>863</v>
+      </c>
+      <c r="M135" t="n">
+        <v>13624</v>
+      </c>
+      <c r="N135" t="n">
+        <v>2953</v>
+      </c>
+      <c r="O135" t="n">
+        <v>402</v>
+      </c>
+      <c r="P135" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>9</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>200</v>
+      </c>
+      <c r="J136" t="n">
+        <v>288</v>
+      </c>
+      <c r="K136" t="n">
+        <v>1537</v>
+      </c>
+      <c r="L136" t="n">
+        <v>1825</v>
+      </c>
+      <c r="M136" t="n">
+        <v>66073</v>
+      </c>
+      <c r="N136" t="n">
+        <v>4757</v>
+      </c>
+      <c r="O136" t="n">
+        <v>673</v>
+      </c>
+      <c r="P136" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>20260702T080913Z</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-07-02T08:09:13.446368+00:00</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>9</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>200</v>
+      </c>
+      <c r="J137" t="n">
+        <v>295</v>
+      </c>
+      <c r="K137" t="n">
+        <v>774</v>
+      </c>
+      <c r="L137" t="n">
+        <v>1069</v>
+      </c>
+      <c r="M137" t="n">
+        <v>171109</v>
+      </c>
+      <c r="N137" t="n">
+        <v>2431</v>
+      </c>
+      <c r="O137" t="n">
+        <v>341</v>
+      </c>
+      <c r="P137" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>responses/20260702T080913Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-03 13:01 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S137"/>
+  <dimension ref="A1:S153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8421,9 +8421,6 @@
       <c r="I122" t="n">
         <v>400</v>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
       <c r="M122" t="n">
         <v>213</v>
       </c>
@@ -8436,8 +8433,6 @@
       <c r="P122" t="n">
         <v>1</v>
       </c>
-      <c r="Q122" t="inlineStr"/>
-      <c r="R122" t="inlineStr"/>
       <c r="S122" t="inlineStr">
         <is>
           <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
@@ -8486,9 +8481,6 @@
       <c r="I123" t="n">
         <v>429</v>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
       <c r="M123" t="n">
         <v>179</v>
       </c>
@@ -8501,8 +8493,6 @@
       <c r="P123" t="n">
         <v>3</v>
       </c>
-      <c r="Q123" t="inlineStr"/>
-      <c r="R123" t="inlineStr"/>
       <c r="S123" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -8551,9 +8541,6 @@
       <c r="I124" t="n">
         <v>429</v>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
       <c r="M124" t="n">
         <v>180</v>
       </c>
@@ -8566,8 +8553,6 @@
       <c r="P124" t="n">
         <v>3</v>
       </c>
-      <c r="Q124" t="inlineStr"/>
-      <c r="R124" t="inlineStr"/>
       <c r="S124" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -8616,9 +8601,6 @@
       <c r="I125" t="n">
         <v>429</v>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
       <c r="M125" t="n">
         <v>157</v>
       </c>
@@ -8631,8 +8613,6 @@
       <c r="P125" t="n">
         <v>3</v>
       </c>
-      <c r="Q125" t="inlineStr"/>
-      <c r="R125" t="inlineStr"/>
       <c r="S125" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -8681,9 +8661,6 @@
       <c r="I126" t="n">
         <v>429</v>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
       <c r="M126" t="n">
         <v>295</v>
       </c>
@@ -8696,8 +8673,6 @@
       <c r="P126" t="n">
         <v>3</v>
       </c>
-      <c r="Q126" t="inlineStr"/>
-      <c r="R126" t="inlineStr"/>
       <c r="S126" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -8746,9 +8721,6 @@
       <c r="I127" t="n">
         <v>429</v>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
       <c r="M127" t="n">
         <v>158</v>
       </c>
@@ -8761,8 +8733,6 @@
       <c r="P127" t="n">
         <v>3</v>
       </c>
-      <c r="Q127" t="inlineStr"/>
-      <c r="R127" t="inlineStr"/>
       <c r="S127" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -8837,8 +8807,6 @@
           <t>responses/20260702T080913Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R128" t="inlineStr"/>
-      <c r="S128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8908,8 +8876,6 @@
           <t>responses/20260702T080913Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R129" t="inlineStr"/>
-      <c r="S129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8979,8 +8945,6 @@
           <t>responses/20260702T080913Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R130" t="inlineStr"/>
-      <c r="S130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9024,9 +8988,6 @@
       <c r="I131" t="n">
         <v>200</v>
       </c>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
       <c r="M131" t="n">
         <v>120350</v>
       </c>
@@ -9039,9 +9000,6 @@
       <c r="P131" t="n">
         <v>1</v>
       </c>
-      <c r="Q131" t="inlineStr"/>
-      <c r="R131" t="inlineStr"/>
-      <c r="S131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9106,9 +9064,6 @@
       <c r="P132" t="n">
         <v>1</v>
       </c>
-      <c r="Q132" t="inlineStr"/>
-      <c r="R132" t="inlineStr"/>
-      <c r="S132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9178,8 +9133,6 @@
           <t>responses/20260702T080913Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R133" t="inlineStr"/>
-      <c r="S133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9249,8 +9202,6 @@
           <t>responses/20260702T080913Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R134" t="inlineStr"/>
-      <c r="S134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9320,8 +9271,6 @@
           <t>responses/20260702T080913Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R135" t="inlineStr"/>
-      <c r="S135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9391,8 +9340,6 @@
           <t>responses/20260702T080913Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R136" t="inlineStr"/>
-      <c r="S136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9457,9 +9404,1106 @@
       <c r="P137" t="n">
         <v>1</v>
       </c>
-      <c r="Q137" t="inlineStr"/>
-      <c r="R137" t="inlineStr"/>
-      <c r="S137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>10</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>429</v>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="n">
+        <v>130</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0</v>
+      </c>
+      <c r="P138" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>10</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>429</v>
+      </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="n">
+        <v>160</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>0</v>
+      </c>
+      <c r="P139" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>10</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>429</v>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="n">
+        <v>96</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
+        <v>0</v>
+      </c>
+      <c r="P140" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>10</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>429</v>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="n">
+        <v>208</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
+      <c r="P141" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>10</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>429</v>
+      </c>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="n">
+        <v>318</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
+        <v>0</v>
+      </c>
+      <c r="P142" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>10</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>429</v>
+      </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="n">
+        <v>134</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
+      <c r="P143" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>10</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>200</v>
+      </c>
+      <c r="J144" t="n">
+        <v>81</v>
+      </c>
+      <c r="K144" t="n">
+        <v>4254</v>
+      </c>
+      <c r="L144" t="n">
+        <v>4335</v>
+      </c>
+      <c r="M144" t="n">
+        <v>25776</v>
+      </c>
+      <c r="N144" t="n">
+        <v>15651</v>
+      </c>
+      <c r="O144" t="n">
+        <v>2036</v>
+      </c>
+      <c r="P144" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>10</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>200</v>
+      </c>
+      <c r="J145" t="n">
+        <v>81</v>
+      </c>
+      <c r="K145" t="n">
+        <v>4108</v>
+      </c>
+      <c r="L145" t="n">
+        <v>4189</v>
+      </c>
+      <c r="M145" t="n">
+        <v>47260</v>
+      </c>
+      <c r="N145" t="n">
+        <v>15345</v>
+      </c>
+      <c r="O145" t="n">
+        <v>1792</v>
+      </c>
+      <c r="P145" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>200</v>
+      </c>
+      <c r="J146" t="n">
+        <v>79</v>
+      </c>
+      <c r="K146" t="n">
+        <v>1158</v>
+      </c>
+      <c r="L146" t="n">
+        <v>1237</v>
+      </c>
+      <c r="M146" t="n">
+        <v>38609</v>
+      </c>
+      <c r="N146" t="n">
+        <v>4835</v>
+      </c>
+      <c r="O146" t="n">
+        <v>549</v>
+      </c>
+      <c r="P146" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>10</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>200</v>
+      </c>
+      <c r="J147" t="n">
+        <v>131</v>
+      </c>
+      <c r="K147" t="n">
+        <v>3800</v>
+      </c>
+      <c r="L147" t="n">
+        <v>3931</v>
+      </c>
+      <c r="M147" t="n">
+        <v>77118</v>
+      </c>
+      <c r="N147" t="n">
+        <v>14941</v>
+      </c>
+      <c r="O147" t="n">
+        <v>1718</v>
+      </c>
+      <c r="P147" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>10</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>200</v>
+      </c>
+      <c r="J148" t="n">
+        <v>58</v>
+      </c>
+      <c r="K148" t="n">
+        <v>5995</v>
+      </c>
+      <c r="L148" t="n">
+        <v>6053</v>
+      </c>
+      <c r="M148" t="n">
+        <v>81012</v>
+      </c>
+      <c r="N148" t="n">
+        <v>27394</v>
+      </c>
+      <c r="O148" t="n">
+        <v>2602</v>
+      </c>
+      <c r="P148" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr"/>
+      <c r="S148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>10</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>200</v>
+      </c>
+      <c r="J149" t="n">
+        <v>75</v>
+      </c>
+      <c r="K149" t="n">
+        <v>2174</v>
+      </c>
+      <c r="L149" t="n">
+        <v>2249</v>
+      </c>
+      <c r="M149" t="n">
+        <v>131925</v>
+      </c>
+      <c r="N149" t="n">
+        <v>8440</v>
+      </c>
+      <c r="O149" t="n">
+        <v>951</v>
+      </c>
+      <c r="P149" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>10</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>200</v>
+      </c>
+      <c r="J150" t="n">
+        <v>129</v>
+      </c>
+      <c r="K150" t="n">
+        <v>3419</v>
+      </c>
+      <c r="L150" t="n">
+        <v>3548</v>
+      </c>
+      <c r="M150" t="n">
+        <v>150834</v>
+      </c>
+      <c r="N150" t="n">
+        <v>14658</v>
+      </c>
+      <c r="O150" t="n">
+        <v>1750</v>
+      </c>
+      <c r="P150" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>10</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>200</v>
+      </c>
+      <c r="J151" t="n">
+        <v>81</v>
+      </c>
+      <c r="K151" t="n">
+        <v>4362</v>
+      </c>
+      <c r="L151" t="n">
+        <v>4443</v>
+      </c>
+      <c r="M151" t="n">
+        <v>159310</v>
+      </c>
+      <c r="N151" t="n">
+        <v>14798</v>
+      </c>
+      <c r="O151" t="n">
+        <v>1618</v>
+      </c>
+      <c r="P151" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr"/>
+      <c r="S151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>10</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>200</v>
+      </c>
+      <c r="J152" t="n">
+        <v>77</v>
+      </c>
+      <c r="K152" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L152" t="n">
+        <v>6077</v>
+      </c>
+      <c r="M152" t="n">
+        <v>175692</v>
+      </c>
+      <c r="N152" t="n">
+        <v>4312</v>
+      </c>
+      <c r="O152" t="n">
+        <v>481</v>
+      </c>
+      <c r="P152" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr"/>
+      <c r="S152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>10</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>200</v>
+      </c>
+      <c r="J153" t="n">
+        <v>110</v>
+      </c>
+      <c r="K153" t="n">
+        <v>4808</v>
+      </c>
+      <c r="L153" t="n">
+        <v>4918</v>
+      </c>
+      <c r="M153" t="n">
+        <v>461890</v>
+      </c>
+      <c r="N153" t="n">
+        <v>17167</v>
+      </c>
+      <c r="O153" t="n">
+        <v>1623</v>
+      </c>
+      <c r="P153" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9472,7 +10516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S137"/>
+  <dimension ref="A1:S153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17509,9 +18553,6 @@
       <c r="I122" t="n">
         <v>400</v>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
       <c r="M122" t="n">
         <v>99</v>
       </c>
@@ -17524,8 +18565,6 @@
       <c r="P122" t="n">
         <v>1</v>
       </c>
-      <c r="Q122" t="inlineStr"/>
-      <c r="R122" t="inlineStr"/>
       <c r="S122" t="inlineStr">
         <is>
           <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
@@ -17574,9 +18613,6 @@
       <c r="I123" t="n">
         <v>429</v>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
       <c r="M123" t="n">
         <v>137</v>
       </c>
@@ -17589,8 +18625,6 @@
       <c r="P123" t="n">
         <v>3</v>
       </c>
-      <c r="Q123" t="inlineStr"/>
-      <c r="R123" t="inlineStr"/>
       <c r="S123" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -17639,9 +18673,6 @@
       <c r="I124" t="n">
         <v>429</v>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
       <c r="M124" t="n">
         <v>162</v>
       </c>
@@ -17654,8 +18685,6 @@
       <c r="P124" t="n">
         <v>3</v>
       </c>
-      <c r="Q124" t="inlineStr"/>
-      <c r="R124" t="inlineStr"/>
       <c r="S124" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -17704,9 +18733,6 @@
       <c r="I125" t="n">
         <v>429</v>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
       <c r="M125" t="n">
         <v>173</v>
       </c>
@@ -17719,8 +18745,6 @@
       <c r="P125" t="n">
         <v>3</v>
       </c>
-      <c r="Q125" t="inlineStr"/>
-      <c r="R125" t="inlineStr"/>
       <c r="S125" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -17769,9 +18793,6 @@
       <c r="I126" t="n">
         <v>429</v>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
       <c r="M126" t="n">
         <v>228</v>
       </c>
@@ -17784,8 +18805,6 @@
       <c r="P126" t="n">
         <v>3</v>
       </c>
-      <c r="Q126" t="inlineStr"/>
-      <c r="R126" t="inlineStr"/>
       <c r="S126" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -17834,9 +18853,6 @@
       <c r="I127" t="n">
         <v>429</v>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
       <c r="M127" t="n">
         <v>1076</v>
       </c>
@@ -17849,8 +18865,6 @@
       <c r="P127" t="n">
         <v>3</v>
       </c>
-      <c r="Q127" t="inlineStr"/>
-      <c r="R127" t="inlineStr"/>
       <c r="S127" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -17925,8 +18939,6 @@
           <t>responses/20260702T080913Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R128" t="inlineStr"/>
-      <c r="S128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -17970,9 +18982,6 @@
       <c r="I129" t="n">
         <v>200</v>
       </c>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
       <c r="M129" t="n">
         <v>10409</v>
       </c>
@@ -17985,9 +18994,6 @@
       <c r="P129" t="n">
         <v>1</v>
       </c>
-      <c r="Q129" t="inlineStr"/>
-      <c r="R129" t="inlineStr"/>
-      <c r="S129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -18057,8 +19063,6 @@
           <t>responses/20260702T080913Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R130" t="inlineStr"/>
-      <c r="S130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -18128,8 +19132,6 @@
           <t>responses/20260702T080913Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R131" t="inlineStr"/>
-      <c r="S131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -18199,8 +19201,6 @@
           <t>responses/20260702T080913Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R132" t="inlineStr"/>
-      <c r="S132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -18270,8 +19270,6 @@
           <t>responses/20260702T080913Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R133" t="inlineStr"/>
-      <c r="S133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -18341,8 +19339,6 @@
           <t>responses/20260702T080913Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R134" t="inlineStr"/>
-      <c r="S134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -18412,8 +19408,6 @@
           <t>responses/20260702T080913Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R135" t="inlineStr"/>
-      <c r="S135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -18457,9 +19451,6 @@
       <c r="I136" t="n">
         <v>200</v>
       </c>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
-      <c r="L136" t="inlineStr"/>
       <c r="M136" t="n">
         <v>120339</v>
       </c>
@@ -18472,9 +19463,6 @@
       <c r="P136" t="n">
         <v>1</v>
       </c>
-      <c r="Q136" t="inlineStr"/>
-      <c r="R136" t="inlineStr"/>
-      <c r="S136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -18544,8 +19532,1112 @@
           <t>responses/20260702T080913Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R137" t="inlineStr"/>
-      <c r="S137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>10</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>429</v>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="n">
+        <v>107</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0</v>
+      </c>
+      <c r="P138" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>10</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>429</v>
+      </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="n">
+        <v>97</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>0</v>
+      </c>
+      <c r="P139" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>10</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>429</v>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="n">
+        <v>116</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
+        <v>0</v>
+      </c>
+      <c r="P140" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>10</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>429</v>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="n">
+        <v>104</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
+      <c r="P141" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>10</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>200</v>
+      </c>
+      <c r="J142" t="n">
+        <v>78</v>
+      </c>
+      <c r="K142" t="n">
+        <v>5110</v>
+      </c>
+      <c r="L142" t="n">
+        <v>5188</v>
+      </c>
+      <c r="M142" t="n">
+        <v>71396</v>
+      </c>
+      <c r="N142" t="n">
+        <v>19563</v>
+      </c>
+      <c r="O142" t="n">
+        <v>2676</v>
+      </c>
+      <c r="P142" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>10</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>429</v>
+      </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="n">
+        <v>132</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
+      <c r="P143" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>10</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>200</v>
+      </c>
+      <c r="J144" t="n">
+        <v>78</v>
+      </c>
+      <c r="K144" t="n">
+        <v>6089</v>
+      </c>
+      <c r="L144" t="n">
+        <v>6167</v>
+      </c>
+      <c r="M144" t="n">
+        <v>28503</v>
+      </c>
+      <c r="N144" t="n">
+        <v>17577</v>
+      </c>
+      <c r="O144" t="n">
+        <v>2398</v>
+      </c>
+      <c r="P144" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>10</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>200</v>
+      </c>
+      <c r="J145" t="n">
+        <v>73</v>
+      </c>
+      <c r="K145" t="n">
+        <v>2415</v>
+      </c>
+      <c r="L145" t="n">
+        <v>2488</v>
+      </c>
+      <c r="M145" t="n">
+        <v>59918</v>
+      </c>
+      <c r="N145" t="n">
+        <v>10715</v>
+      </c>
+      <c r="O145" t="n">
+        <v>1654</v>
+      </c>
+      <c r="P145" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>200</v>
+      </c>
+      <c r="J146" t="n">
+        <v>125</v>
+      </c>
+      <c r="K146" t="n">
+        <v>4304</v>
+      </c>
+      <c r="L146" t="n">
+        <v>4429</v>
+      </c>
+      <c r="M146" t="n">
+        <v>137310</v>
+      </c>
+      <c r="N146" t="n">
+        <v>17241</v>
+      </c>
+      <c r="O146" t="n">
+        <v>2447</v>
+      </c>
+      <c r="P146" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>10</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>200</v>
+      </c>
+      <c r="J147" t="n">
+        <v>76</v>
+      </c>
+      <c r="K147" t="n">
+        <v>2282</v>
+      </c>
+      <c r="L147" t="n">
+        <v>2358</v>
+      </c>
+      <c r="M147" t="n">
+        <v>49228</v>
+      </c>
+      <c r="N147" t="n">
+        <v>10647</v>
+      </c>
+      <c r="O147" t="n">
+        <v>1387</v>
+      </c>
+      <c r="P147" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>10</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>200</v>
+      </c>
+      <c r="J148" t="n">
+        <v>127</v>
+      </c>
+      <c r="K148" t="n">
+        <v>5541</v>
+      </c>
+      <c r="L148" t="n">
+        <v>5668</v>
+      </c>
+      <c r="M148" t="n">
+        <v>76143</v>
+      </c>
+      <c r="N148" t="n">
+        <v>21415</v>
+      </c>
+      <c r="O148" t="n">
+        <v>3096</v>
+      </c>
+      <c r="P148" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr"/>
+      <c r="S148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>10</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>200</v>
+      </c>
+      <c r="J149" t="n">
+        <v>54</v>
+      </c>
+      <c r="K149" t="n">
+        <v>4598</v>
+      </c>
+      <c r="L149" t="n">
+        <v>4652</v>
+      </c>
+      <c r="M149" t="n">
+        <v>86685</v>
+      </c>
+      <c r="N149" t="n">
+        <v>18729</v>
+      </c>
+      <c r="O149" t="n">
+        <v>2536</v>
+      </c>
+      <c r="P149" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>10</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>200</v>
+      </c>
+      <c r="J150" t="n">
+        <v>74</v>
+      </c>
+      <c r="K150" t="n">
+        <v>4069</v>
+      </c>
+      <c r="L150" t="n">
+        <v>4143</v>
+      </c>
+      <c r="M150" t="n">
+        <v>111112</v>
+      </c>
+      <c r="N150" t="n">
+        <v>12098</v>
+      </c>
+      <c r="O150" t="n">
+        <v>1671</v>
+      </c>
+      <c r="P150" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>10</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>200</v>
+      </c>
+      <c r="J151" t="n">
+        <v>74</v>
+      </c>
+      <c r="K151" t="n">
+        <v>1806</v>
+      </c>
+      <c r="L151" t="n">
+        <v>1880</v>
+      </c>
+      <c r="M151" t="n">
+        <v>188730</v>
+      </c>
+      <c r="N151" t="n">
+        <v>8364</v>
+      </c>
+      <c r="O151" t="n">
+        <v>1266</v>
+      </c>
+      <c r="P151" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr"/>
+      <c r="S151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>10</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>200</v>
+      </c>
+      <c r="J152" t="n">
+        <v>112</v>
+      </c>
+      <c r="K152" t="n">
+        <v>4047</v>
+      </c>
+      <c r="L152" t="n">
+        <v>4159</v>
+      </c>
+      <c r="M152" t="n">
+        <v>307970</v>
+      </c>
+      <c r="N152" t="n">
+        <v>22725</v>
+      </c>
+      <c r="O152" t="n">
+        <v>2899</v>
+      </c>
+      <c r="P152" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr"/>
+      <c r="S152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>10</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>200</v>
+      </c>
+      <c r="J153" t="n">
+        <v>78</v>
+      </c>
+      <c r="K153" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L153" t="n">
+        <v>8078</v>
+      </c>
+      <c r="M153" t="n">
+        <v>623690</v>
+      </c>
+      <c r="N153" t="n">
+        <v>29801</v>
+      </c>
+      <c r="O153" t="n">
+        <v>4227</v>
+      </c>
+      <c r="P153" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18558,7 +20650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S137"/>
+  <dimension ref="A1:S153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26553,9 +28645,6 @@
       <c r="I122" t="n">
         <v>400</v>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
       <c r="M122" t="n">
         <v>87</v>
       </c>
@@ -26568,8 +28657,6 @@
       <c r="P122" t="n">
         <v>1</v>
       </c>
-      <c r="Q122" t="inlineStr"/>
-      <c r="R122" t="inlineStr"/>
       <c r="S122" t="inlineStr">
         <is>
           <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
@@ -26618,9 +28705,6 @@
       <c r="I123" t="n">
         <v>429</v>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
       <c r="M123" t="n">
         <v>151</v>
       </c>
@@ -26633,8 +28717,6 @@
       <c r="P123" t="n">
         <v>3</v>
       </c>
-      <c r="Q123" t="inlineStr"/>
-      <c r="R123" t="inlineStr"/>
       <c r="S123" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -26683,9 +28765,6 @@
       <c r="I124" t="n">
         <v>429</v>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
       <c r="M124" t="n">
         <v>156</v>
       </c>
@@ -26698,8 +28777,6 @@
       <c r="P124" t="n">
         <v>3</v>
       </c>
-      <c r="Q124" t="inlineStr"/>
-      <c r="R124" t="inlineStr"/>
       <c r="S124" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -26748,9 +28825,6 @@
       <c r="I125" t="n">
         <v>429</v>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
       <c r="M125" t="n">
         <v>209</v>
       </c>
@@ -26763,8 +28837,6 @@
       <c r="P125" t="n">
         <v>3</v>
       </c>
-      <c r="Q125" t="inlineStr"/>
-      <c r="R125" t="inlineStr"/>
       <c r="S125" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -26839,8 +28911,6 @@
           <t>responses/20260702T080913Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R126" t="inlineStr"/>
-      <c r="S126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -26884,9 +28954,6 @@
       <c r="I127" t="n">
         <v>429</v>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
       <c r="M127" t="n">
         <v>174</v>
       </c>
@@ -26899,8 +28966,6 @@
       <c r="P127" t="n">
         <v>3</v>
       </c>
-      <c r="Q127" t="inlineStr"/>
-      <c r="R127" t="inlineStr"/>
       <c r="S127" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -26975,8 +29040,6 @@
           <t>responses/20260702T080913Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R128" t="inlineStr"/>
-      <c r="S128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -27046,8 +29109,6 @@
           <t>responses/20260702T080913Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R129" t="inlineStr"/>
-      <c r="S129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -27117,8 +29178,6 @@
           <t>responses/20260702T080913Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R130" t="inlineStr"/>
-      <c r="S130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -27188,8 +29247,6 @@
           <t>responses/20260702T080913Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R131" t="inlineStr"/>
-      <c r="S131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -27259,8 +29316,6 @@
           <t>responses/20260702T080913Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R132" t="inlineStr"/>
-      <c r="S132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -27330,8 +29385,6 @@
           <t>responses/20260702T080913Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R133" t="inlineStr"/>
-      <c r="S133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -27401,8 +29454,6 @@
           <t>responses/20260702T080913Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R134" t="inlineStr"/>
-      <c r="S134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -27472,8 +29523,6 @@
           <t>responses/20260702T080913Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R135" t="inlineStr"/>
-      <c r="S135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -27543,8 +29592,6 @@
           <t>responses/20260702T080913Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R136" t="inlineStr"/>
-      <c r="S136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -27614,8 +29661,1060 @@
           <t>responses/20260702T080913Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R137" t="inlineStr"/>
-      <c r="S137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>10</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>200</v>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="n">
+        <v>328</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0</v>
+      </c>
+      <c r="P138" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>10</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>429</v>
+      </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="n">
+        <v>142</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>0</v>
+      </c>
+      <c r="P139" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>10</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>200</v>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="n">
+        <v>316</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
+        <v>0</v>
+      </c>
+      <c r="P140" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>10</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>429</v>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="n">
+        <v>287</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
+      <c r="P141" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>10</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>429</v>
+      </c>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="n">
+        <v>125</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
+        <v>0</v>
+      </c>
+      <c r="P142" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>10</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>429</v>
+      </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="n">
+        <v>99</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
+      <c r="P143" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>10</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>429</v>
+      </c>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="n">
+        <v>121</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="n">
+        <v>0</v>
+      </c>
+      <c r="P144" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>10</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>200</v>
+      </c>
+      <c r="J145" t="n">
+        <v>292</v>
+      </c>
+      <c r="K145" t="n">
+        <v>680</v>
+      </c>
+      <c r="L145" t="n">
+        <v>972</v>
+      </c>
+      <c r="M145" t="n">
+        <v>7004</v>
+      </c>
+      <c r="N145" t="n">
+        <v>2944</v>
+      </c>
+      <c r="O145" t="n">
+        <v>424</v>
+      </c>
+      <c r="P145" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>429</v>
+      </c>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="n">
+        <v>290</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="n">
+        <v>0</v>
+      </c>
+      <c r="P146" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>10</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>429</v>
+      </c>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="n">
+        <v>105</v>
+      </c>
+      <c r="N147" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0</v>
+      </c>
+      <c r="P147" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>10</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>200</v>
+      </c>
+      <c r="J148" t="n">
+        <v>332</v>
+      </c>
+      <c r="K148" t="n">
+        <v>686</v>
+      </c>
+      <c r="L148" t="n">
+        <v>1018</v>
+      </c>
+      <c r="M148" t="n">
+        <v>13599</v>
+      </c>
+      <c r="N148" t="n">
+        <v>3018</v>
+      </c>
+      <c r="O148" t="n">
+        <v>452</v>
+      </c>
+      <c r="P148" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr"/>
+      <c r="S148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>10</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>200</v>
+      </c>
+      <c r="J149" t="n">
+        <v>256</v>
+      </c>
+      <c r="K149" t="n">
+        <v>907</v>
+      </c>
+      <c r="L149" t="n">
+        <v>1163</v>
+      </c>
+      <c r="M149" t="n">
+        <v>36219</v>
+      </c>
+      <c r="N149" t="n">
+        <v>3940</v>
+      </c>
+      <c r="O149" t="n">
+        <v>569</v>
+      </c>
+      <c r="P149" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>10</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>200</v>
+      </c>
+      <c r="J150" t="n">
+        <v>288</v>
+      </c>
+      <c r="K150" t="n">
+        <v>1711</v>
+      </c>
+      <c r="L150" t="n">
+        <v>1999</v>
+      </c>
+      <c r="M150" t="n">
+        <v>41297</v>
+      </c>
+      <c r="N150" t="n">
+        <v>4583</v>
+      </c>
+      <c r="O150" t="n">
+        <v>649</v>
+      </c>
+      <c r="P150" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>10</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>200</v>
+      </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="n">
+        <v>120347</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0</v>
+      </c>
+      <c r="P151" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q151" t="inlineStr"/>
+      <c r="R151" t="inlineStr"/>
+      <c r="S151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>10</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>200</v>
+      </c>
+      <c r="J152" t="n">
+        <v>332</v>
+      </c>
+      <c r="K152" t="n">
+        <v>885</v>
+      </c>
+      <c r="L152" t="n">
+        <v>1217</v>
+      </c>
+      <c r="M152" t="n">
+        <v>125062</v>
+      </c>
+      <c r="N152" t="n">
+        <v>4070</v>
+      </c>
+      <c r="O152" t="n">
+        <v>562</v>
+      </c>
+      <c r="P152" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>responses/20260703T125036Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr"/>
+      <c r="S152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>20260703T125036Z</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-07-03T12:50:36.663948+00:00</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>10</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>200</v>
+      </c>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="n">
+        <v>300493</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="n">
+        <v>0</v>
+      </c>
+      <c r="P153" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-04 18:10 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S153"/>
+  <dimension ref="A1:S169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9447,9 +9447,6 @@
       <c r="I138" t="n">
         <v>429</v>
       </c>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
       <c r="M138" t="n">
         <v>130</v>
       </c>
@@ -9462,8 +9459,6 @@
       <c r="P138" t="n">
         <v>3</v>
       </c>
-      <c r="Q138" t="inlineStr"/>
-      <c r="R138" t="inlineStr"/>
       <c r="S138" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -9512,9 +9507,6 @@
       <c r="I139" t="n">
         <v>429</v>
       </c>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
       <c r="M139" t="n">
         <v>160</v>
       </c>
@@ -9527,8 +9519,6 @@
       <c r="P139" t="n">
         <v>3</v>
       </c>
-      <c r="Q139" t="inlineStr"/>
-      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -9577,9 +9567,6 @@
       <c r="I140" t="n">
         <v>429</v>
       </c>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
       <c r="M140" t="n">
         <v>96</v>
       </c>
@@ -9592,8 +9579,6 @@
       <c r="P140" t="n">
         <v>3</v>
       </c>
-      <c r="Q140" t="inlineStr"/>
-      <c r="R140" t="inlineStr"/>
       <c r="S140" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -9642,9 +9627,6 @@
       <c r="I141" t="n">
         <v>429</v>
       </c>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
       <c r="M141" t="n">
         <v>208</v>
       </c>
@@ -9657,8 +9639,6 @@
       <c r="P141" t="n">
         <v>3</v>
       </c>
-      <c r="Q141" t="inlineStr"/>
-      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
@@ -9707,9 +9687,6 @@
       <c r="I142" t="n">
         <v>429</v>
       </c>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
       <c r="M142" t="n">
         <v>318</v>
       </c>
@@ -9722,8 +9699,6 @@
       <c r="P142" t="n">
         <v>3</v>
       </c>
-      <c r="Q142" t="inlineStr"/>
-      <c r="R142" t="inlineStr"/>
       <c r="S142" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -9772,9 +9747,6 @@
       <c r="I143" t="n">
         <v>429</v>
       </c>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
       <c r="M143" t="n">
         <v>134</v>
       </c>
@@ -9787,8 +9759,6 @@
       <c r="P143" t="n">
         <v>3</v>
       </c>
-      <c r="Q143" t="inlineStr"/>
-      <c r="R143" t="inlineStr"/>
       <c r="S143" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -9863,8 +9833,6 @@
           <t>responses/20260703T125036Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R144" t="inlineStr"/>
-      <c r="S144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9934,8 +9902,6 @@
           <t>responses/20260703T125036Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R145" t="inlineStr"/>
-      <c r="S145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10005,8 +9971,6 @@
           <t>responses/20260703T125036Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R146" t="inlineStr"/>
-      <c r="S146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10076,8 +10040,6 @@
           <t>responses/20260703T125036Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R147" t="inlineStr"/>
-      <c r="S147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10147,8 +10109,6 @@
           <t>responses/20260703T125036Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R148" t="inlineStr"/>
-      <c r="S148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10218,8 +10178,6 @@
           <t>responses/20260703T125036Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R149" t="inlineStr"/>
-      <c r="S149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10289,8 +10247,6 @@
           <t>responses/20260703T125036Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R150" t="inlineStr"/>
-      <c r="S150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10360,8 +10316,6 @@
           <t>responses/20260703T125036Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R151" t="inlineStr"/>
-      <c r="S151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10431,8 +10385,6 @@
           <t>responses/20260703T125036Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
         </is>
       </c>
-      <c r="R152" t="inlineStr"/>
-      <c r="S152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10502,8 +10454,1082 @@
           <t>responses/20260703T125036Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R153" t="inlineStr"/>
-      <c r="S153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>11</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>200</v>
+      </c>
+      <c r="J154" t="n">
+        <v>390</v>
+      </c>
+      <c r="K154" t="n">
+        <v>537</v>
+      </c>
+      <c r="L154" t="n">
+        <v>927</v>
+      </c>
+      <c r="M154" t="n">
+        <v>4159</v>
+      </c>
+      <c r="N154" t="n">
+        <v>1853</v>
+      </c>
+      <c r="O154" t="n">
+        <v>246</v>
+      </c>
+      <c r="P154" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>11</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>200</v>
+      </c>
+      <c r="J155" t="n">
+        <v>390</v>
+      </c>
+      <c r="K155" t="n">
+        <v>855</v>
+      </c>
+      <c r="L155" t="n">
+        <v>1245</v>
+      </c>
+      <c r="M155" t="n">
+        <v>4615</v>
+      </c>
+      <c r="N155" t="n">
+        <v>2596</v>
+      </c>
+      <c r="O155" t="n">
+        <v>347</v>
+      </c>
+      <c r="P155" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>11</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>200</v>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="n">
+        <v>10707</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0</v>
+      </c>
+      <c r="P156" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="inlineStr"/>
+      <c r="S156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>11</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>200</v>
+      </c>
+      <c r="J157" t="n">
+        <v>390</v>
+      </c>
+      <c r="K157" t="n">
+        <v>604</v>
+      </c>
+      <c r="L157" t="n">
+        <v>994</v>
+      </c>
+      <c r="M157" t="n">
+        <v>14730</v>
+      </c>
+      <c r="N157" t="n">
+        <v>1806</v>
+      </c>
+      <c r="O157" t="n">
+        <v>242</v>
+      </c>
+      <c r="P157" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr"/>
+      <c r="S157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>11</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>429</v>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="n">
+        <v>235</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0</v>
+      </c>
+      <c r="P158" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="inlineStr"/>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>11</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>429</v>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="n">
+        <v>240</v>
+      </c>
+      <c r="N159" t="n">
+        <v>0</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0</v>
+      </c>
+      <c r="P159" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q159" t="inlineStr"/>
+      <c r="R159" t="inlineStr"/>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>11</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>429</v>
+      </c>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="n">
+        <v>371</v>
+      </c>
+      <c r="N160" t="n">
+        <v>0</v>
+      </c>
+      <c r="O160" t="n">
+        <v>0</v>
+      </c>
+      <c r="P160" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q160" t="inlineStr"/>
+      <c r="R160" t="inlineStr"/>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>11</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>429</v>
+      </c>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="n">
+        <v>221</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0</v>
+      </c>
+      <c r="P161" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q161" t="inlineStr"/>
+      <c r="R161" t="inlineStr"/>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>11</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>429</v>
+      </c>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="n">
+        <v>359</v>
+      </c>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+      <c r="O162" t="n">
+        <v>0</v>
+      </c>
+      <c r="P162" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q162" t="inlineStr"/>
+      <c r="R162" t="inlineStr"/>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>11</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>429</v>
+      </c>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
+      <c r="M163" t="n">
+        <v>223</v>
+      </c>
+      <c r="N163" t="n">
+        <v>0</v>
+      </c>
+      <c r="O163" t="n">
+        <v>0</v>
+      </c>
+      <c r="P163" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q163" t="inlineStr"/>
+      <c r="R163" t="inlineStr"/>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>11</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>200</v>
+      </c>
+      <c r="J164" t="n">
+        <v>376</v>
+      </c>
+      <c r="K164" t="n">
+        <v>1085</v>
+      </c>
+      <c r="L164" t="n">
+        <v>1461</v>
+      </c>
+      <c r="M164" t="n">
+        <v>21258</v>
+      </c>
+      <c r="N164" t="n">
+        <v>1816</v>
+      </c>
+      <c r="O164" t="n">
+        <v>244</v>
+      </c>
+      <c r="P164" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/poolside_laguna-m.1_free.java</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr"/>
+      <c r="S164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>11</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>200</v>
+      </c>
+      <c r="J165" t="n">
+        <v>429</v>
+      </c>
+      <c r="K165" t="n">
+        <v>519</v>
+      </c>
+      <c r="L165" t="n">
+        <v>948</v>
+      </c>
+      <c r="M165" t="n">
+        <v>12521</v>
+      </c>
+      <c r="N165" t="n">
+        <v>1807</v>
+      </c>
+      <c r="O165" t="n">
+        <v>243</v>
+      </c>
+      <c r="P165" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr"/>
+      <c r="S165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>11</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>200</v>
+      </c>
+      <c r="J166" t="n">
+        <v>413</v>
+      </c>
+      <c r="K166" t="n">
+        <v>670</v>
+      </c>
+      <c r="L166" t="n">
+        <v>1083</v>
+      </c>
+      <c r="M166" t="n">
+        <v>14010</v>
+      </c>
+      <c r="N166" t="n">
+        <v>1756</v>
+      </c>
+      <c r="O166" t="n">
+        <v>233</v>
+      </c>
+      <c r="P166" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr"/>
+      <c r="S166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>11</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>200</v>
+      </c>
+      <c r="J167" t="n">
+        <v>352</v>
+      </c>
+      <c r="K167" t="n">
+        <v>1918</v>
+      </c>
+      <c r="L167" t="n">
+        <v>2270</v>
+      </c>
+      <c r="M167" t="n">
+        <v>30936</v>
+      </c>
+      <c r="N167" t="n">
+        <v>4480</v>
+      </c>
+      <c r="O167" t="n">
+        <v>602</v>
+      </c>
+      <c r="P167" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr"/>
+      <c r="S167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>11</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>200</v>
+      </c>
+      <c r="J168" t="n">
+        <v>386</v>
+      </c>
+      <c r="K168" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L168" t="n">
+        <v>6386</v>
+      </c>
+      <c r="M168" t="n">
+        <v>118355</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+      <c r="O168" t="n">
+        <v>0</v>
+      </c>
+      <c r="P168" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q168" t="inlineStr"/>
+      <c r="R168" t="inlineStr"/>
+      <c r="S168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>11</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that implements a complex, non‑trivi</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>200</v>
+      </c>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="n">
+        <v>120624</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q169" t="inlineStr"/>
+      <c r="R169" t="inlineStr"/>
+      <c r="S169" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10516,7 +11542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S153"/>
+  <dimension ref="A1:S169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19575,9 +20601,6 @@
       <c r="I138" t="n">
         <v>429</v>
       </c>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
       <c r="M138" t="n">
         <v>107</v>
       </c>
@@ -19590,8 +20613,6 @@
       <c r="P138" t="n">
         <v>3</v>
       </c>
-      <c r="Q138" t="inlineStr"/>
-      <c r="R138" t="inlineStr"/>
       <c r="S138" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -19640,9 +20661,6 @@
       <c r="I139" t="n">
         <v>429</v>
       </c>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
       <c r="M139" t="n">
         <v>97</v>
       </c>
@@ -19655,8 +20673,6 @@
       <c r="P139" t="n">
         <v>3</v>
       </c>
-      <c r="Q139" t="inlineStr"/>
-      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -19705,9 +20721,6 @@
       <c r="I140" t="n">
         <v>429</v>
       </c>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
       <c r="M140" t="n">
         <v>116</v>
       </c>
@@ -19720,8 +20733,6 @@
       <c r="P140" t="n">
         <v>3</v>
       </c>
-      <c r="Q140" t="inlineStr"/>
-      <c r="R140" t="inlineStr"/>
       <c r="S140" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -19770,9 +20781,6 @@
       <c r="I141" t="n">
         <v>429</v>
       </c>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
       <c r="M141" t="n">
         <v>104</v>
       </c>
@@ -19785,8 +20793,6 @@
       <c r="P141" t="n">
         <v>3</v>
       </c>
-      <c r="Q141" t="inlineStr"/>
-      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -19861,8 +20867,6 @@
           <t>responses/20260703T125036Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R142" t="inlineStr"/>
-      <c r="S142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -19906,9 +20910,6 @@
       <c r="I143" t="n">
         <v>429</v>
       </c>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
       <c r="M143" t="n">
         <v>132</v>
       </c>
@@ -19921,8 +20922,6 @@
       <c r="P143" t="n">
         <v>3</v>
       </c>
-      <c r="Q143" t="inlineStr"/>
-      <c r="R143" t="inlineStr"/>
       <c r="S143" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
@@ -19997,8 +20996,6 @@
           <t>responses/20260703T125036Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R144" t="inlineStr"/>
-      <c r="S144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -20068,8 +21065,6 @@
           <t>responses/20260703T125036Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R145" t="inlineStr"/>
-      <c r="S145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -20139,8 +21134,6 @@
           <t>responses/20260703T125036Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R146" t="inlineStr"/>
-      <c r="S146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -20210,8 +21203,6 @@
           <t>responses/20260703T125036Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R147" t="inlineStr"/>
-      <c r="S147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -20281,8 +21272,6 @@
           <t>responses/20260703T125036Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R148" t="inlineStr"/>
-      <c r="S148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -20352,8 +21341,6 @@
           <t>responses/20260703T125036Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R149" t="inlineStr"/>
-      <c r="S149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -20423,8 +21410,6 @@
           <t>responses/20260703T125036Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R150" t="inlineStr"/>
-      <c r="S150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -20494,8 +21479,6 @@
           <t>responses/20260703T125036Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R151" t="inlineStr"/>
-      <c r="S151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -20565,8 +21548,6 @@
           <t>responses/20260703T125036Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R152" t="inlineStr"/>
-      <c r="S152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -20636,8 +21617,1112 @@
           <t>responses/20260703T125036Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R153" t="inlineStr"/>
-      <c r="S153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>11</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>200</v>
+      </c>
+      <c r="J154" t="n">
+        <v>407</v>
+      </c>
+      <c r="K154" t="n">
+        <v>1683</v>
+      </c>
+      <c r="L154" t="n">
+        <v>2090</v>
+      </c>
+      <c r="M154" t="n">
+        <v>14643</v>
+      </c>
+      <c r="N154" t="n">
+        <v>6531</v>
+      </c>
+      <c r="O154" t="n">
+        <v>795</v>
+      </c>
+      <c r="P154" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>11</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>429</v>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="n">
+        <v>226</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0</v>
+      </c>
+      <c r="P155" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q155" t="inlineStr"/>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>11</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>429</v>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="n">
+        <v>344</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0</v>
+      </c>
+      <c r="P156" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="inlineStr"/>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>11</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>429</v>
+      </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="n">
+        <v>363</v>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0</v>
+      </c>
+      <c r="P157" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q157" t="inlineStr"/>
+      <c r="R157" t="inlineStr"/>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>11</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>429</v>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="n">
+        <v>266</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0</v>
+      </c>
+      <c r="P158" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="inlineStr"/>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>11</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>429</v>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="n">
+        <v>215</v>
+      </c>
+      <c r="N159" t="n">
+        <v>0</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0</v>
+      </c>
+      <c r="P159" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q159" t="inlineStr"/>
+      <c r="R159" t="inlineStr"/>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>11</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>200</v>
+      </c>
+      <c r="J160" t="n">
+        <v>407</v>
+      </c>
+      <c r="K160" t="n">
+        <v>1825</v>
+      </c>
+      <c r="L160" t="n">
+        <v>2232</v>
+      </c>
+      <c r="M160" t="n">
+        <v>13787</v>
+      </c>
+      <c r="N160" t="n">
+        <v>6316</v>
+      </c>
+      <c r="O160" t="n">
+        <v>761</v>
+      </c>
+      <c r="P160" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr"/>
+      <c r="S160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>11</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>200</v>
+      </c>
+      <c r="J161" t="n">
+        <v>432</v>
+      </c>
+      <c r="K161" t="n">
+        <v>1580</v>
+      </c>
+      <c r="L161" t="n">
+        <v>2012</v>
+      </c>
+      <c r="M161" t="n">
+        <v>17684</v>
+      </c>
+      <c r="N161" t="n">
+        <v>5851</v>
+      </c>
+      <c r="O161" t="n">
+        <v>778</v>
+      </c>
+      <c r="P161" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr"/>
+      <c r="S161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>11</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>200</v>
+      </c>
+      <c r="J162" t="n">
+        <v>358</v>
+      </c>
+      <c r="K162" t="n">
+        <v>1788</v>
+      </c>
+      <c r="L162" t="n">
+        <v>2146</v>
+      </c>
+      <c r="M162" t="n">
+        <v>30382</v>
+      </c>
+      <c r="N162" t="n">
+        <v>7608</v>
+      </c>
+      <c r="O162" t="n">
+        <v>950</v>
+      </c>
+      <c r="P162" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr"/>
+      <c r="S162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>11</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>200</v>
+      </c>
+      <c r="J163" t="n">
+        <v>397</v>
+      </c>
+      <c r="K163" t="n">
+        <v>1396</v>
+      </c>
+      <c r="L163" t="n">
+        <v>1793</v>
+      </c>
+      <c r="M163" t="n">
+        <v>35245</v>
+      </c>
+      <c r="N163" t="n">
+        <v>6320</v>
+      </c>
+      <c r="O163" t="n">
+        <v>825</v>
+      </c>
+      <c r="P163" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr"/>
+      <c r="S163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>11</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>200</v>
+      </c>
+      <c r="J164" t="n">
+        <v>459</v>
+      </c>
+      <c r="K164" t="n">
+        <v>2731</v>
+      </c>
+      <c r="L164" t="n">
+        <v>3190</v>
+      </c>
+      <c r="M164" t="n">
+        <v>27500</v>
+      </c>
+      <c r="N164" t="n">
+        <v>9278</v>
+      </c>
+      <c r="O164" t="n">
+        <v>1199</v>
+      </c>
+      <c r="P164" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr"/>
+      <c r="S164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>11</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>200</v>
+      </c>
+      <c r="J165" t="n">
+        <v>404</v>
+      </c>
+      <c r="K165" t="n">
+        <v>1102</v>
+      </c>
+      <c r="L165" t="n">
+        <v>1506</v>
+      </c>
+      <c r="M165" t="n">
+        <v>30181</v>
+      </c>
+      <c r="N165" t="n">
+        <v>4573</v>
+      </c>
+      <c r="O165" t="n">
+        <v>528</v>
+      </c>
+      <c r="P165" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr"/>
+      <c r="S165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>11</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>200</v>
+      </c>
+      <c r="J166" t="n">
+        <v>422</v>
+      </c>
+      <c r="K166" t="n">
+        <v>1607</v>
+      </c>
+      <c r="L166" t="n">
+        <v>2029</v>
+      </c>
+      <c r="M166" t="n">
+        <v>39140</v>
+      </c>
+      <c r="N166" t="n">
+        <v>5347</v>
+      </c>
+      <c r="O166" t="n">
+        <v>633</v>
+      </c>
+      <c r="P166" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr"/>
+      <c r="S166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>11</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>200</v>
+      </c>
+      <c r="J167" t="n">
+        <v>403</v>
+      </c>
+      <c r="K167" t="n">
+        <v>2251</v>
+      </c>
+      <c r="L167" t="n">
+        <v>2654</v>
+      </c>
+      <c r="M167" t="n">
+        <v>49133</v>
+      </c>
+      <c r="N167" t="n">
+        <v>6334</v>
+      </c>
+      <c r="O167" t="n">
+        <v>803</v>
+      </c>
+      <c r="P167" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr"/>
+      <c r="S167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>11</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>200</v>
+      </c>
+      <c r="J168" t="n">
+        <v>407</v>
+      </c>
+      <c r="K168" t="n">
+        <v>3322</v>
+      </c>
+      <c r="L168" t="n">
+        <v>3729</v>
+      </c>
+      <c r="M168" t="n">
+        <v>106626</v>
+      </c>
+      <c r="N168" t="n">
+        <v>12200</v>
+      </c>
+      <c r="O168" t="n">
+        <v>1578</v>
+      </c>
+      <c r="P168" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr"/>
+      <c r="S168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>11</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (≈12,000‑15,000 word) in‑depth, well‑structured</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>200</v>
+      </c>
+      <c r="J169" t="n">
+        <v>398</v>
+      </c>
+      <c r="K169" t="n">
+        <v>1260</v>
+      </c>
+      <c r="L169" t="n">
+        <v>1658</v>
+      </c>
+      <c r="M169" t="n">
+        <v>171658</v>
+      </c>
+      <c r="N169" t="n">
+        <v>5428</v>
+      </c>
+      <c r="O169" t="n">
+        <v>705</v>
+      </c>
+      <c r="P169" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr"/>
+      <c r="S169" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20650,7 +22735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S153"/>
+  <dimension ref="A1:S169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29704,9 +31789,6 @@
       <c r="I138" t="n">
         <v>200</v>
       </c>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
       <c r="M138" t="n">
         <v>328</v>
       </c>
@@ -29719,9 +31801,6 @@
       <c r="P138" t="n">
         <v>1</v>
       </c>
-      <c r="Q138" t="inlineStr"/>
-      <c r="R138" t="inlineStr"/>
-      <c r="S138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -29765,9 +31844,6 @@
       <c r="I139" t="n">
         <v>429</v>
       </c>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
       <c r="M139" t="n">
         <v>142</v>
       </c>
@@ -29780,8 +31856,6 @@
       <c r="P139" t="n">
         <v>3</v>
       </c>
-      <c r="Q139" t="inlineStr"/>
-      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -29830,9 +31904,6 @@
       <c r="I140" t="n">
         <v>200</v>
       </c>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
       <c r="M140" t="n">
         <v>316</v>
       </c>
@@ -29845,9 +31916,6 @@
       <c r="P140" t="n">
         <v>1</v>
       </c>
-      <c r="Q140" t="inlineStr"/>
-      <c r="R140" t="inlineStr"/>
-      <c r="S140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -29891,9 +31959,6 @@
       <c r="I141" t="n">
         <v>429</v>
       </c>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
       <c r="M141" t="n">
         <v>287</v>
       </c>
@@ -29906,8 +31971,6 @@
       <c r="P141" t="n">
         <v>3</v>
       </c>
-      <c r="Q141" t="inlineStr"/>
-      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -29956,9 +32019,6 @@
       <c r="I142" t="n">
         <v>429</v>
       </c>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
       <c r="M142" t="n">
         <v>125</v>
       </c>
@@ -29971,8 +32031,6 @@
       <c r="P142" t="n">
         <v>3</v>
       </c>
-      <c r="Q142" t="inlineStr"/>
-      <c r="R142" t="inlineStr"/>
       <c r="S142" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -30021,9 +32079,6 @@
       <c r="I143" t="n">
         <v>429</v>
       </c>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
       <c r="M143" t="n">
         <v>99</v>
       </c>
@@ -30036,8 +32091,6 @@
       <c r="P143" t="n">
         <v>3</v>
       </c>
-      <c r="Q143" t="inlineStr"/>
-      <c r="R143" t="inlineStr"/>
       <c r="S143" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -30086,9 +32139,6 @@
       <c r="I144" t="n">
         <v>429</v>
       </c>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
       <c r="M144" t="n">
         <v>121</v>
       </c>
@@ -30101,8 +32151,6 @@
       <c r="P144" t="n">
         <v>3</v>
       </c>
-      <c r="Q144" t="inlineStr"/>
-      <c r="R144" t="inlineStr"/>
       <c r="S144" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -30177,8 +32225,6 @@
           <t>responses/20260703T125036Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R145" t="inlineStr"/>
-      <c r="S145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -30222,9 +32268,6 @@
       <c r="I146" t="n">
         <v>429</v>
       </c>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
-      <c r="L146" t="inlineStr"/>
       <c r="M146" t="n">
         <v>290</v>
       </c>
@@ -30237,8 +32280,6 @@
       <c r="P146" t="n">
         <v>3</v>
       </c>
-      <c r="Q146" t="inlineStr"/>
-      <c r="R146" t="inlineStr"/>
       <c r="S146" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -30287,9 +32328,6 @@
       <c r="I147" t="n">
         <v>429</v>
       </c>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
       <c r="M147" t="n">
         <v>105</v>
       </c>
@@ -30302,8 +32340,6 @@
       <c r="P147" t="n">
         <v>3</v>
       </c>
-      <c r="Q147" t="inlineStr"/>
-      <c r="R147" t="inlineStr"/>
       <c r="S147" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
@@ -30378,8 +32414,6 @@
           <t>responses/20260703T125036Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R148" t="inlineStr"/>
-      <c r="S148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -30449,8 +32483,6 @@
           <t>responses/20260703T125036Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R149" t="inlineStr"/>
-      <c r="S149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -30520,8 +32552,6 @@
           <t>responses/20260703T125036Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R150" t="inlineStr"/>
-      <c r="S150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -30565,9 +32595,6 @@
       <c r="I151" t="n">
         <v>200</v>
       </c>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
       <c r="M151" t="n">
         <v>120347</v>
       </c>
@@ -30580,9 +32607,6 @@
       <c r="P151" t="n">
         <v>1</v>
       </c>
-      <c r="Q151" t="inlineStr"/>
-      <c r="R151" t="inlineStr"/>
-      <c r="S151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -30652,8 +32676,6 @@
           <t>responses/20260703T125036Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R152" t="inlineStr"/>
-      <c r="S152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -30697,9 +32719,6 @@
       <c r="I153" t="n">
         <v>200</v>
       </c>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
       <c r="M153" t="n">
         <v>300493</v>
       </c>
@@ -30712,9 +32731,1096 @@
       <c r="P153" t="n">
         <v>1</v>
       </c>
-      <c r="Q153" t="inlineStr"/>
-      <c r="R153" t="inlineStr"/>
-      <c r="S153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>11</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>429</v>
+      </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="n">
+        <v>1641</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" t="n">
+        <v>0</v>
+      </c>
+      <c r="P154" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>11</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>429</v>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="n">
+        <v>1019</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0</v>
+      </c>
+      <c r="P155" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q155" t="inlineStr"/>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>11</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>429</v>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="n">
+        <v>257</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0</v>
+      </c>
+      <c r="P156" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="inlineStr"/>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>11</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>429</v>
+      </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="n">
+        <v>295</v>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0</v>
+      </c>
+      <c r="P157" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q157" t="inlineStr"/>
+      <c r="R157" t="inlineStr"/>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>11</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>429</v>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="n">
+        <v>266</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0</v>
+      </c>
+      <c r="P158" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="inlineStr"/>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>11</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>200</v>
+      </c>
+      <c r="J159" t="n">
+        <v>650</v>
+      </c>
+      <c r="K159" t="n">
+        <v>968</v>
+      </c>
+      <c r="L159" t="n">
+        <v>1618</v>
+      </c>
+      <c r="M159" t="n">
+        <v>6812</v>
+      </c>
+      <c r="N159" t="n">
+        <v>3638</v>
+      </c>
+      <c r="O159" t="n">
+        <v>507</v>
+      </c>
+      <c r="P159" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr"/>
+      <c r="S159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>11</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>200</v>
+      </c>
+      <c r="J160" t="n">
+        <v>650</v>
+      </c>
+      <c r="K160" t="n">
+        <v>1611</v>
+      </c>
+      <c r="L160" t="n">
+        <v>2261</v>
+      </c>
+      <c r="M160" t="n">
+        <v>37343</v>
+      </c>
+      <c r="N160" t="n">
+        <v>5387</v>
+      </c>
+      <c r="O160" t="n">
+        <v>773</v>
+      </c>
+      <c r="P160" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr"/>
+      <c r="S160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>11</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>429</v>
+      </c>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="n">
+        <v>487</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0</v>
+      </c>
+      <c r="P161" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q161" t="inlineStr"/>
+      <c r="R161" t="inlineStr"/>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>11</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>200</v>
+      </c>
+      <c r="J162" t="n">
+        <v>662</v>
+      </c>
+      <c r="K162" t="n">
+        <v>686</v>
+      </c>
+      <c r="L162" t="n">
+        <v>1348</v>
+      </c>
+      <c r="M162" t="n">
+        <v>10212</v>
+      </c>
+      <c r="N162" t="n">
+        <v>2692</v>
+      </c>
+      <c r="O162" t="n">
+        <v>405</v>
+      </c>
+      <c r="P162" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr"/>
+      <c r="S162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>11</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>200</v>
+      </c>
+      <c r="J163" t="n">
+        <v>703</v>
+      </c>
+      <c r="K163" t="n">
+        <v>1010</v>
+      </c>
+      <c r="L163" t="n">
+        <v>1713</v>
+      </c>
+      <c r="M163" t="n">
+        <v>10669</v>
+      </c>
+      <c r="N163" t="n">
+        <v>3654</v>
+      </c>
+      <c r="O163" t="n">
+        <v>494</v>
+      </c>
+      <c r="P163" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr"/>
+      <c r="S163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>11</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>200</v>
+      </c>
+      <c r="J164" t="n">
+        <v>650</v>
+      </c>
+      <c r="K164" t="n">
+        <v>1019</v>
+      </c>
+      <c r="L164" t="n">
+        <v>1669</v>
+      </c>
+      <c r="M164" t="n">
+        <v>65550</v>
+      </c>
+      <c r="N164" t="n">
+        <v>3392</v>
+      </c>
+      <c r="O164" t="n">
+        <v>465</v>
+      </c>
+      <c r="P164" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr"/>
+      <c r="S164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>11</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>200</v>
+      </c>
+      <c r="J165" t="n">
+        <v>666</v>
+      </c>
+      <c r="K165" t="n">
+        <v>1271</v>
+      </c>
+      <c r="L165" t="n">
+        <v>1937</v>
+      </c>
+      <c r="M165" t="n">
+        <v>33385</v>
+      </c>
+      <c r="N165" t="n">
+        <v>2787</v>
+      </c>
+      <c r="O165" t="n">
+        <v>375</v>
+      </c>
+      <c r="P165" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr"/>
+      <c r="S165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>11</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>200</v>
+      </c>
+      <c r="J166" t="n">
+        <v>645</v>
+      </c>
+      <c r="K166" t="n">
+        <v>759</v>
+      </c>
+      <c r="L166" t="n">
+        <v>1404</v>
+      </c>
+      <c r="M166" t="n">
+        <v>17658</v>
+      </c>
+      <c r="N166" t="n">
+        <v>3452</v>
+      </c>
+      <c r="O166" t="n">
+        <v>467</v>
+      </c>
+      <c r="P166" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr"/>
+      <c r="S166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>11</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>200</v>
+      </c>
+      <c r="J167" t="n">
+        <v>578</v>
+      </c>
+      <c r="K167" t="n">
+        <v>1998</v>
+      </c>
+      <c r="L167" t="n">
+        <v>2576</v>
+      </c>
+      <c r="M167" t="n">
+        <v>45174</v>
+      </c>
+      <c r="N167" t="n">
+        <v>8326</v>
+      </c>
+      <c r="O167" t="n">
+        <v>1226</v>
+      </c>
+      <c r="P167" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr"/>
+      <c r="S167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>11</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>200</v>
+      </c>
+      <c r="J168" t="n">
+        <v>646</v>
+      </c>
+      <c r="K168" t="n">
+        <v>2277</v>
+      </c>
+      <c r="L168" t="n">
+        <v>2923</v>
+      </c>
+      <c r="M168" t="n">
+        <v>56894</v>
+      </c>
+      <c r="N168" t="n">
+        <v>5992</v>
+      </c>
+      <c r="O168" t="n">
+        <v>859</v>
+      </c>
+      <c r="P168" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>responses/20260704T180536Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr"/>
+      <c r="S168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>20260704T180536Z</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-07-04T18:05:36.272196+00:00</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>11</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Subject: Request for Mid‑Project Performance Metrics and Interim Reporting – Gra</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>200</v>
+      </c>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="n">
+        <v>120421</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q169" t="inlineStr"/>
+      <c r="R169" t="inlineStr"/>
+      <c r="S169" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-05 06:16 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S169"/>
+  <dimension ref="A1:S185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10523,8 +10523,6 @@
           <t>responses/20260704T180536Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R154" t="inlineStr"/>
-      <c r="S154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -10594,8 +10592,6 @@
           <t>responses/20260704T180536Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R155" t="inlineStr"/>
-      <c r="S155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -10639,9 +10635,6 @@
       <c r="I156" t="n">
         <v>200</v>
       </c>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
       <c r="M156" t="n">
         <v>10707</v>
       </c>
@@ -10654,9 +10647,6 @@
       <c r="P156" t="n">
         <v>1</v>
       </c>
-      <c r="Q156" t="inlineStr"/>
-      <c r="R156" t="inlineStr"/>
-      <c r="S156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10726,8 +10716,6 @@
           <t>responses/20260704T180536Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R157" t="inlineStr"/>
-      <c r="S157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10771,9 +10759,6 @@
       <c r="I158" t="n">
         <v>429</v>
       </c>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
       <c r="M158" t="n">
         <v>235</v>
       </c>
@@ -10786,8 +10771,6 @@
       <c r="P158" t="n">
         <v>3</v>
       </c>
-      <c r="Q158" t="inlineStr"/>
-      <c r="R158" t="inlineStr"/>
       <c r="S158" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -10836,9 +10819,6 @@
       <c r="I159" t="n">
         <v>429</v>
       </c>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
       <c r="M159" t="n">
         <v>240</v>
       </c>
@@ -10851,8 +10831,6 @@
       <c r="P159" t="n">
         <v>3</v>
       </c>
-      <c r="Q159" t="inlineStr"/>
-      <c r="R159" t="inlineStr"/>
       <c r="S159" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -10901,9 +10879,6 @@
       <c r="I160" t="n">
         <v>429</v>
       </c>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
       <c r="M160" t="n">
         <v>371</v>
       </c>
@@ -10916,8 +10891,6 @@
       <c r="P160" t="n">
         <v>3</v>
       </c>
-      <c r="Q160" t="inlineStr"/>
-      <c r="R160" t="inlineStr"/>
       <c r="S160" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -10966,9 +10939,6 @@
       <c r="I161" t="n">
         <v>429</v>
       </c>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
       <c r="M161" t="n">
         <v>221</v>
       </c>
@@ -10981,8 +10951,6 @@
       <c r="P161" t="n">
         <v>3</v>
       </c>
-      <c r="Q161" t="inlineStr"/>
-      <c r="R161" t="inlineStr"/>
       <c r="S161" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -11031,9 +10999,6 @@
       <c r="I162" t="n">
         <v>429</v>
       </c>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
       <c r="M162" t="n">
         <v>359</v>
       </c>
@@ -11046,8 +11011,6 @@
       <c r="P162" t="n">
         <v>3</v>
       </c>
-      <c r="Q162" t="inlineStr"/>
-      <c r="R162" t="inlineStr"/>
       <c r="S162" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -11096,9 +11059,6 @@
       <c r="I163" t="n">
         <v>429</v>
       </c>
-      <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
       <c r="M163" t="n">
         <v>223</v>
       </c>
@@ -11111,8 +11071,6 @@
       <c r="P163" t="n">
         <v>3</v>
       </c>
-      <c r="Q163" t="inlineStr"/>
-      <c r="R163" t="inlineStr"/>
       <c r="S163" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -11187,8 +11145,6 @@
           <t>responses/20260704T180536Z/code/poolside_laguna-m.1_free.java</t>
         </is>
       </c>
-      <c r="R164" t="inlineStr"/>
-      <c r="S164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11258,8 +11214,6 @@
           <t>responses/20260704T180536Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R165" t="inlineStr"/>
-      <c r="S165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11329,8 +11283,6 @@
           <t>responses/20260704T180536Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R166" t="inlineStr"/>
-      <c r="S166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11400,8 +11352,6 @@
           <t>responses/20260704T180536Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R167" t="inlineStr"/>
-      <c r="S167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11466,9 +11416,6 @@
       <c r="P168" t="n">
         <v>1</v>
       </c>
-      <c r="Q168" t="inlineStr"/>
-      <c r="R168" t="inlineStr"/>
-      <c r="S168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11512,9 +11459,6 @@
       <c r="I169" t="n">
         <v>200</v>
       </c>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
       <c r="M169" t="n">
         <v>120624</v>
       </c>
@@ -11527,9 +11471,1100 @@
       <c r="P169" t="n">
         <v>1</v>
       </c>
-      <c r="Q169" t="inlineStr"/>
-      <c r="R169" t="inlineStr"/>
-      <c r="S169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>12</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>429</v>
+      </c>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="n">
+        <v>146</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="inlineStr"/>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>12</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>429</v>
+      </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="n">
+        <v>187</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q171" t="inlineStr"/>
+      <c r="R171" t="inlineStr"/>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>12</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>429</v>
+      </c>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr"/>
+      <c r="M172" t="n">
+        <v>146</v>
+      </c>
+      <c r="N172" t="n">
+        <v>0</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0</v>
+      </c>
+      <c r="P172" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q172" t="inlineStr"/>
+      <c r="R172" t="inlineStr"/>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>12</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>429</v>
+      </c>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="n">
+        <v>164</v>
+      </c>
+      <c r="N173" t="n">
+        <v>0</v>
+      </c>
+      <c r="O173" t="n">
+        <v>0</v>
+      </c>
+      <c r="P173" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q173" t="inlineStr"/>
+      <c r="R173" t="inlineStr"/>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>12</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>429</v>
+      </c>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="n">
+        <v>199</v>
+      </c>
+      <c r="N174" t="n">
+        <v>0</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0</v>
+      </c>
+      <c r="P174" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q174" t="inlineStr"/>
+      <c r="R174" t="inlineStr"/>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>12</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>200</v>
+      </c>
+      <c r="J175" t="n">
+        <v>253</v>
+      </c>
+      <c r="K175" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L175" t="n">
+        <v>6253</v>
+      </c>
+      <c r="M175" t="n">
+        <v>25309</v>
+      </c>
+      <c r="N175" t="n">
+        <v>27366</v>
+      </c>
+      <c r="O175" t="n">
+        <v>4157</v>
+      </c>
+      <c r="P175" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr"/>
+      <c r="S175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>12</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>200</v>
+      </c>
+      <c r="J176" t="n">
+        <v>224</v>
+      </c>
+      <c r="K176" t="n">
+        <v>5999</v>
+      </c>
+      <c r="L176" t="n">
+        <v>6223</v>
+      </c>
+      <c r="M176" t="n">
+        <v>34794</v>
+      </c>
+      <c r="N176" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q176" t="inlineStr"/>
+      <c r="R176" t="inlineStr"/>
+      <c r="S176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>12</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>200</v>
+      </c>
+      <c r="J177" t="n">
+        <v>284</v>
+      </c>
+      <c r="K177" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L177" t="n">
+        <v>6284</v>
+      </c>
+      <c r="M177" t="n">
+        <v>62032</v>
+      </c>
+      <c r="N177" t="n">
+        <v>21820</v>
+      </c>
+      <c r="O177" t="n">
+        <v>2144</v>
+      </c>
+      <c r="P177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr"/>
+      <c r="S177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>12</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>200</v>
+      </c>
+      <c r="J178" t="n">
+        <v>249</v>
+      </c>
+      <c r="K178" t="n">
+        <v>2343</v>
+      </c>
+      <c r="L178" t="n">
+        <v>2592</v>
+      </c>
+      <c r="M178" t="n">
+        <v>65199</v>
+      </c>
+      <c r="N178" t="n">
+        <v>9991</v>
+      </c>
+      <c r="O178" t="n">
+        <v>921</v>
+      </c>
+      <c r="P178" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr"/>
+      <c r="S178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>12</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>200</v>
+      </c>
+      <c r="J179" t="n">
+        <v>253</v>
+      </c>
+      <c r="K179" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L179" t="n">
+        <v>6253</v>
+      </c>
+      <c r="M179" t="n">
+        <v>83620</v>
+      </c>
+      <c r="N179" t="n">
+        <v>9809</v>
+      </c>
+      <c r="O179" t="n">
+        <v>1170</v>
+      </c>
+      <c r="P179" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr"/>
+      <c r="S179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>12</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>200</v>
+      </c>
+      <c r="J180" t="n">
+        <v>253</v>
+      </c>
+      <c r="K180" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L180" t="n">
+        <v>6253</v>
+      </c>
+      <c r="M180" t="n">
+        <v>85846</v>
+      </c>
+      <c r="N180" t="n">
+        <v>9473</v>
+      </c>
+      <c r="O180" t="n">
+        <v>1119</v>
+      </c>
+      <c r="P180" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr"/>
+      <c r="S180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>12</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>200</v>
+      </c>
+      <c r="J181" t="n">
+        <v>295</v>
+      </c>
+      <c r="K181" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L181" t="n">
+        <v>6295</v>
+      </c>
+      <c r="M181" t="n">
+        <v>117561</v>
+      </c>
+      <c r="N181" t="n">
+        <v>4087</v>
+      </c>
+      <c r="O181" t="n">
+        <v>591</v>
+      </c>
+      <c r="P181" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr"/>
+      <c r="S181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>12</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>200</v>
+      </c>
+      <c r="J182" t="n">
+        <v>247</v>
+      </c>
+      <c r="K182" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L182" t="n">
+        <v>6247</v>
+      </c>
+      <c r="M182" t="n">
+        <v>141835</v>
+      </c>
+      <c r="N182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O182" t="n">
+        <v>0</v>
+      </c>
+      <c r="P182" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q182" t="inlineStr"/>
+      <c r="R182" t="inlineStr"/>
+      <c r="S182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>12</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>200</v>
+      </c>
+      <c r="J183" t="n">
+        <v>251</v>
+      </c>
+      <c r="K183" t="n">
+        <v>5632</v>
+      </c>
+      <c r="L183" t="n">
+        <v>5883</v>
+      </c>
+      <c r="M183" t="n">
+        <v>136023</v>
+      </c>
+      <c r="N183" t="n">
+        <v>25718</v>
+      </c>
+      <c r="O183" t="n">
+        <v>1357</v>
+      </c>
+      <c r="P183" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr"/>
+      <c r="S183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>12</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>200</v>
+      </c>
+      <c r="J184" t="n">
+        <v>293</v>
+      </c>
+      <c r="K184" t="n">
+        <v>4148</v>
+      </c>
+      <c r="L184" t="n">
+        <v>4441</v>
+      </c>
+      <c r="M184" t="n">
+        <v>170060</v>
+      </c>
+      <c r="N184" t="n">
+        <v>20080</v>
+      </c>
+      <c r="O184" t="n">
+        <v>2306</v>
+      </c>
+      <c r="P184" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr"/>
+      <c r="S184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>12</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Write a single, self‑contained Java program that defines a public class named `C</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>200</v>
+      </c>
+      <c r="J185" t="n">
+        <v>249</v>
+      </c>
+      <c r="K185" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L185" t="n">
+        <v>6249</v>
+      </c>
+      <c r="M185" t="n">
+        <v>145776</v>
+      </c>
+      <c r="N185" t="n">
+        <v>0</v>
+      </c>
+      <c r="O185" t="n">
+        <v>0</v>
+      </c>
+      <c r="P185" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q185" t="inlineStr"/>
+      <c r="R185" t="inlineStr"/>
+      <c r="S185" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11542,7 +12577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S169"/>
+  <dimension ref="A1:S185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21686,8 +22721,6 @@
           <t>responses/20260704T180536Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R154" t="inlineStr"/>
-      <c r="S154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -21731,9 +22764,6 @@
       <c r="I155" t="n">
         <v>429</v>
       </c>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
       <c r="M155" t="n">
         <v>226</v>
       </c>
@@ -21746,8 +22776,6 @@
       <c r="P155" t="n">
         <v>3</v>
       </c>
-      <c r="Q155" t="inlineStr"/>
-      <c r="R155" t="inlineStr"/>
       <c r="S155" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -21796,9 +22824,6 @@
       <c r="I156" t="n">
         <v>429</v>
       </c>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
       <c r="M156" t="n">
         <v>344</v>
       </c>
@@ -21811,8 +22836,6 @@
       <c r="P156" t="n">
         <v>3</v>
       </c>
-      <c r="Q156" t="inlineStr"/>
-      <c r="R156" t="inlineStr"/>
       <c r="S156" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -21861,9 +22884,6 @@
       <c r="I157" t="n">
         <v>429</v>
       </c>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
       <c r="M157" t="n">
         <v>363</v>
       </c>
@@ -21876,8 +22896,6 @@
       <c r="P157" t="n">
         <v>3</v>
       </c>
-      <c r="Q157" t="inlineStr"/>
-      <c r="R157" t="inlineStr"/>
       <c r="S157" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -21926,9 +22944,6 @@
       <c r="I158" t="n">
         <v>429</v>
       </c>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
       <c r="M158" t="n">
         <v>266</v>
       </c>
@@ -21941,8 +22956,6 @@
       <c r="P158" t="n">
         <v>3</v>
       </c>
-      <c r="Q158" t="inlineStr"/>
-      <c r="R158" t="inlineStr"/>
       <c r="S158" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -21991,9 +23004,6 @@
       <c r="I159" t="n">
         <v>429</v>
       </c>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
       <c r="M159" t="n">
         <v>215</v>
       </c>
@@ -22006,8 +23016,6 @@
       <c r="P159" t="n">
         <v>3</v>
       </c>
-      <c r="Q159" t="inlineStr"/>
-      <c r="R159" t="inlineStr"/>
       <c r="S159" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -22082,8 +23090,6 @@
           <t>responses/20260704T180536Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R160" t="inlineStr"/>
-      <c r="S160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -22153,8 +23159,6 @@
           <t>responses/20260704T180536Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R161" t="inlineStr"/>
-      <c r="S161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -22224,8 +23228,6 @@
           <t>responses/20260704T180536Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R162" t="inlineStr"/>
-      <c r="S162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -22295,8 +23297,6 @@
           <t>responses/20260704T180536Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R163" t="inlineStr"/>
-      <c r="S163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -22366,8 +23366,6 @@
           <t>responses/20260704T180536Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R164" t="inlineStr"/>
-      <c r="S164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -22437,8 +23435,6 @@
           <t>responses/20260704T180536Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R165" t="inlineStr"/>
-      <c r="S165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -22508,8 +23504,6 @@
           <t>responses/20260704T180536Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R166" t="inlineStr"/>
-      <c r="S166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -22579,8 +23573,6 @@
           <t>responses/20260704T180536Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R167" t="inlineStr"/>
-      <c r="S167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -22650,8 +23642,6 @@
           <t>responses/20260704T180536Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R168" t="inlineStr"/>
-      <c r="S168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -22721,8 +23711,1096 @@
           <t>responses/20260704T180536Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R169" t="inlineStr"/>
-      <c r="S169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>12</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>429</v>
+      </c>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="n">
+        <v>152</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="inlineStr"/>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>12</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>429</v>
+      </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="n">
+        <v>193</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q171" t="inlineStr"/>
+      <c r="R171" t="inlineStr"/>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>12</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>200</v>
+      </c>
+      <c r="J172" t="n">
+        <v>212</v>
+      </c>
+      <c r="K172" t="n">
+        <v>970</v>
+      </c>
+      <c r="L172" t="n">
+        <v>1182</v>
+      </c>
+      <c r="M172" t="n">
+        <v>20490</v>
+      </c>
+      <c r="N172" t="n">
+        <v>791</v>
+      </c>
+      <c r="O172" t="n">
+        <v>124</v>
+      </c>
+      <c r="P172" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr"/>
+      <c r="S172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>12</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>429</v>
+      </c>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="n">
+        <v>128</v>
+      </c>
+      <c r="N173" t="n">
+        <v>0</v>
+      </c>
+      <c r="O173" t="n">
+        <v>0</v>
+      </c>
+      <c r="P173" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q173" t="inlineStr"/>
+      <c r="R173" t="inlineStr"/>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>12</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>429</v>
+      </c>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="n">
+        <v>118</v>
+      </c>
+      <c r="N174" t="n">
+        <v>0</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0</v>
+      </c>
+      <c r="P174" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q174" t="inlineStr"/>
+      <c r="R174" t="inlineStr"/>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>12</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>429</v>
+      </c>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="n">
+        <v>331</v>
+      </c>
+      <c r="N175" t="n">
+        <v>0</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
+      <c r="P175" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q175" t="inlineStr"/>
+      <c r="R175" t="inlineStr"/>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>12</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>429</v>
+      </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="n">
+        <v>132</v>
+      </c>
+      <c r="N176" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q176" t="inlineStr"/>
+      <c r="R176" t="inlineStr"/>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>12</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>200</v>
+      </c>
+      <c r="J177" t="n">
+        <v>212</v>
+      </c>
+      <c r="K177" t="n">
+        <v>872</v>
+      </c>
+      <c r="L177" t="n">
+        <v>1084</v>
+      </c>
+      <c r="M177" t="n">
+        <v>7812</v>
+      </c>
+      <c r="N177" t="n">
+        <v>1993</v>
+      </c>
+      <c r="O177" t="n">
+        <v>299</v>
+      </c>
+      <c r="P177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr"/>
+      <c r="S177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>12</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>200</v>
+      </c>
+      <c r="J178" t="n">
+        <v>244</v>
+      </c>
+      <c r="K178" t="n">
+        <v>3104</v>
+      </c>
+      <c r="L178" t="n">
+        <v>3348</v>
+      </c>
+      <c r="M178" t="n">
+        <v>32917</v>
+      </c>
+      <c r="N178" t="n">
+        <v>14139</v>
+      </c>
+      <c r="O178" t="n">
+        <v>1854</v>
+      </c>
+      <c r="P178" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr"/>
+      <c r="S178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>12</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>200</v>
+      </c>
+      <c r="J179" t="n">
+        <v>254</v>
+      </c>
+      <c r="K179" t="n">
+        <v>3526</v>
+      </c>
+      <c r="L179" t="n">
+        <v>3780</v>
+      </c>
+      <c r="M179" t="n">
+        <v>45560</v>
+      </c>
+      <c r="N179" t="n">
+        <v>12869</v>
+      </c>
+      <c r="O179" t="n">
+        <v>1922</v>
+      </c>
+      <c r="P179" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr"/>
+      <c r="S179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>12</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>200</v>
+      </c>
+      <c r="J180" t="n">
+        <v>207</v>
+      </c>
+      <c r="K180" t="n">
+        <v>3620</v>
+      </c>
+      <c r="L180" t="n">
+        <v>3827</v>
+      </c>
+      <c r="M180" t="n">
+        <v>77370</v>
+      </c>
+      <c r="N180" t="n">
+        <v>11970</v>
+      </c>
+      <c r="O180" t="n">
+        <v>1532</v>
+      </c>
+      <c r="P180" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr"/>
+      <c r="S180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>12</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>200</v>
+      </c>
+      <c r="J181" t="n">
+        <v>176</v>
+      </c>
+      <c r="K181" t="n">
+        <v>7997</v>
+      </c>
+      <c r="L181" t="n">
+        <v>8173</v>
+      </c>
+      <c r="M181" t="n">
+        <v>103839</v>
+      </c>
+      <c r="N181" t="n">
+        <v>30637</v>
+      </c>
+      <c r="O181" t="n">
+        <v>4301</v>
+      </c>
+      <c r="P181" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr"/>
+      <c r="S181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>12</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>200</v>
+      </c>
+      <c r="J182" t="n">
+        <v>208</v>
+      </c>
+      <c r="K182" t="n">
+        <v>3039</v>
+      </c>
+      <c r="L182" t="n">
+        <v>3247</v>
+      </c>
+      <c r="M182" t="n">
+        <v>79893</v>
+      </c>
+      <c r="N182" t="n">
+        <v>7813</v>
+      </c>
+      <c r="O182" t="n">
+        <v>1030</v>
+      </c>
+      <c r="P182" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr"/>
+      <c r="S182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>12</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>200</v>
+      </c>
+      <c r="J183" t="n">
+        <v>212</v>
+      </c>
+      <c r="K183" t="n">
+        <v>7826</v>
+      </c>
+      <c r="L183" t="n">
+        <v>8038</v>
+      </c>
+      <c r="M183" t="n">
+        <v>198208</v>
+      </c>
+      <c r="N183" t="n">
+        <v>25183</v>
+      </c>
+      <c r="O183" t="n">
+        <v>3689</v>
+      </c>
+      <c r="P183" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr"/>
+      <c r="S183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>12</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>200</v>
+      </c>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="n">
+        <v>120274</v>
+      </c>
+      <c r="N184" t="n">
+        <v>0</v>
+      </c>
+      <c r="O184" t="n">
+        <v>0</v>
+      </c>
+      <c r="P184" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q184" t="inlineStr"/>
+      <c r="R184" t="inlineStr"/>
+      <c r="S184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>12</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>200</v>
+      </c>
+      <c r="J185" t="n">
+        <v>252</v>
+      </c>
+      <c r="K185" t="n">
+        <v>6495</v>
+      </c>
+      <c r="L185" t="n">
+        <v>6747</v>
+      </c>
+      <c r="M185" t="n">
+        <v>278857</v>
+      </c>
+      <c r="N185" t="n">
+        <v>25017</v>
+      </c>
+      <c r="O185" t="n">
+        <v>3713</v>
+      </c>
+      <c r="P185" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr"/>
+      <c r="S185" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22735,7 +24813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S169"/>
+  <dimension ref="A1:S185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32774,9 +34852,6 @@
       <c r="I154" t="n">
         <v>429</v>
       </c>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
       <c r="M154" t="n">
         <v>1641</v>
       </c>
@@ -32789,8 +34864,6 @@
       <c r="P154" t="n">
         <v>3</v>
       </c>
-      <c r="Q154" t="inlineStr"/>
-      <c r="R154" t="inlineStr"/>
       <c r="S154" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -32839,9 +34912,6 @@
       <c r="I155" t="n">
         <v>429</v>
       </c>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
       <c r="M155" t="n">
         <v>1019</v>
       </c>
@@ -32854,8 +34924,6 @@
       <c r="P155" t="n">
         <v>3</v>
       </c>
-      <c r="Q155" t="inlineStr"/>
-      <c r="R155" t="inlineStr"/>
       <c r="S155" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -32904,9 +34972,6 @@
       <c r="I156" t="n">
         <v>429</v>
       </c>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
       <c r="M156" t="n">
         <v>257</v>
       </c>
@@ -32919,8 +34984,6 @@
       <c r="P156" t="n">
         <v>3</v>
       </c>
-      <c r="Q156" t="inlineStr"/>
-      <c r="R156" t="inlineStr"/>
       <c r="S156" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -32969,9 +35032,6 @@
       <c r="I157" t="n">
         <v>429</v>
       </c>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
       <c r="M157" t="n">
         <v>295</v>
       </c>
@@ -32984,8 +35044,6 @@
       <c r="P157" t="n">
         <v>3</v>
       </c>
-      <c r="Q157" t="inlineStr"/>
-      <c r="R157" t="inlineStr"/>
       <c r="S157" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -33034,9 +35092,6 @@
       <c r="I158" t="n">
         <v>429</v>
       </c>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
       <c r="M158" t="n">
         <v>266</v>
       </c>
@@ -33049,8 +35104,6 @@
       <c r="P158" t="n">
         <v>3</v>
       </c>
-      <c r="Q158" t="inlineStr"/>
-      <c r="R158" t="inlineStr"/>
       <c r="S158" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -33125,8 +35178,6 @@
           <t>responses/20260704T180536Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R159" t="inlineStr"/>
-      <c r="S159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -33196,8 +35247,6 @@
           <t>responses/20260704T180536Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R160" t="inlineStr"/>
-      <c r="S160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -33241,9 +35290,6 @@
       <c r="I161" t="n">
         <v>429</v>
       </c>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
       <c r="M161" t="n">
         <v>487</v>
       </c>
@@ -33256,8 +35302,6 @@
       <c r="P161" t="n">
         <v>3</v>
       </c>
-      <c r="Q161" t="inlineStr"/>
-      <c r="R161" t="inlineStr"/>
       <c r="S161" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -33332,8 +35376,6 @@
           <t>responses/20260704T180536Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R162" t="inlineStr"/>
-      <c r="S162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -33403,8 +35445,6 @@
           <t>responses/20260704T180536Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R163" t="inlineStr"/>
-      <c r="S163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -33474,8 +35514,6 @@
           <t>responses/20260704T180536Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R164" t="inlineStr"/>
-      <c r="S164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -33545,8 +35583,6 @@
           <t>responses/20260704T180536Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R165" t="inlineStr"/>
-      <c r="S165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -33616,8 +35652,6 @@
           <t>responses/20260704T180536Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R166" t="inlineStr"/>
-      <c r="S166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -33687,8 +35721,6 @@
           <t>responses/20260704T180536Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R167" t="inlineStr"/>
-      <c r="S167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -33758,8 +35790,6 @@
           <t>responses/20260704T180536Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R168" t="inlineStr"/>
-      <c r="S168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -33803,9 +35833,6 @@
       <c r="I169" t="n">
         <v>200</v>
       </c>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
       <c r="M169" t="n">
         <v>120421</v>
       </c>
@@ -33818,9 +35845,1100 @@
       <c r="P169" t="n">
         <v>2</v>
       </c>
-      <c r="Q169" t="inlineStr"/>
-      <c r="R169" t="inlineStr"/>
-      <c r="S169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>12</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>429</v>
+      </c>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="n">
+        <v>137</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="inlineStr"/>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>12</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>429</v>
+      </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="n">
+        <v>279</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q171" t="inlineStr"/>
+      <c r="R171" t="inlineStr"/>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>12</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>200</v>
+      </c>
+      <c r="J172" t="n">
+        <v>461</v>
+      </c>
+      <c r="K172" t="n">
+        <v>841</v>
+      </c>
+      <c r="L172" t="n">
+        <v>1302</v>
+      </c>
+      <c r="M172" t="n">
+        <v>29705</v>
+      </c>
+      <c r="N172" t="n">
+        <v>2558</v>
+      </c>
+      <c r="O172" t="n">
+        <v>375</v>
+      </c>
+      <c r="P172" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr"/>
+      <c r="S172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>12</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>200</v>
+      </c>
+      <c r="J173" t="n">
+        <v>461</v>
+      </c>
+      <c r="K173" t="n">
+        <v>679</v>
+      </c>
+      <c r="L173" t="n">
+        <v>1140</v>
+      </c>
+      <c r="M173" t="n">
+        <v>12255</v>
+      </c>
+      <c r="N173" t="n">
+        <v>2576</v>
+      </c>
+      <c r="O173" t="n">
+        <v>373</v>
+      </c>
+      <c r="P173" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr"/>
+      <c r="S173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>12</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>429</v>
+      </c>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="n">
+        <v>179</v>
+      </c>
+      <c r="N174" t="n">
+        <v>0</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0</v>
+      </c>
+      <c r="P174" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q174" t="inlineStr"/>
+      <c r="R174" t="inlineStr"/>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>12</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>429</v>
+      </c>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="n">
+        <v>125</v>
+      </c>
+      <c r="N175" t="n">
+        <v>0</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
+      <c r="P175" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q175" t="inlineStr"/>
+      <c r="R175" t="inlineStr"/>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>12</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>429</v>
+      </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="n">
+        <v>142</v>
+      </c>
+      <c r="N176" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q176" t="inlineStr"/>
+      <c r="R176" t="inlineStr"/>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>12</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>200</v>
+      </c>
+      <c r="J177" t="n">
+        <v>461</v>
+      </c>
+      <c r="K177" t="n">
+        <v>841</v>
+      </c>
+      <c r="L177" t="n">
+        <v>1302</v>
+      </c>
+      <c r="M177" t="n">
+        <v>3796</v>
+      </c>
+      <c r="N177" t="n">
+        <v>3406</v>
+      </c>
+      <c r="O177" t="n">
+        <v>497</v>
+      </c>
+      <c r="P177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr"/>
+      <c r="S177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>12</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>429</v>
+      </c>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="n">
+        <v>306</v>
+      </c>
+      <c r="N178" t="n">
+        <v>0</v>
+      </c>
+      <c r="O178" t="n">
+        <v>0</v>
+      </c>
+      <c r="P178" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q178" t="inlineStr"/>
+      <c r="R178" t="inlineStr"/>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>12</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>429</v>
+      </c>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="n">
+        <v>121</v>
+      </c>
+      <c r="N179" t="n">
+        <v>0</v>
+      </c>
+      <c r="O179" t="n">
+        <v>0</v>
+      </c>
+      <c r="P179" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q179" t="inlineStr"/>
+      <c r="R179" t="inlineStr"/>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>12</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>200</v>
+      </c>
+      <c r="J180" t="n">
+        <v>497</v>
+      </c>
+      <c r="K180" t="n">
+        <v>553</v>
+      </c>
+      <c r="L180" t="n">
+        <v>1050</v>
+      </c>
+      <c r="M180" t="n">
+        <v>4266</v>
+      </c>
+      <c r="N180" t="n">
+        <v>1827</v>
+      </c>
+      <c r="O180" t="n">
+        <v>262</v>
+      </c>
+      <c r="P180" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr"/>
+      <c r="S180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>12</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>200</v>
+      </c>
+      <c r="J181" t="n">
+        <v>460</v>
+      </c>
+      <c r="K181" t="n">
+        <v>879</v>
+      </c>
+      <c r="L181" t="n">
+        <v>1339</v>
+      </c>
+      <c r="M181" t="n">
+        <v>18280</v>
+      </c>
+      <c r="N181" t="n">
+        <v>2597</v>
+      </c>
+      <c r="O181" t="n">
+        <v>376</v>
+      </c>
+      <c r="P181" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr"/>
+      <c r="S181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>12</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>200</v>
+      </c>
+      <c r="J182" t="n">
+        <v>402</v>
+      </c>
+      <c r="K182" t="n">
+        <v>825</v>
+      </c>
+      <c r="L182" t="n">
+        <v>1227</v>
+      </c>
+      <c r="M182" t="n">
+        <v>13988</v>
+      </c>
+      <c r="N182" t="n">
+        <v>3778</v>
+      </c>
+      <c r="O182" t="n">
+        <v>570</v>
+      </c>
+      <c r="P182" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr"/>
+      <c r="S182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>12</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>200</v>
+      </c>
+      <c r="J183" t="n">
+        <v>481</v>
+      </c>
+      <c r="K183" t="n">
+        <v>638</v>
+      </c>
+      <c r="L183" t="n">
+        <v>1119</v>
+      </c>
+      <c r="M183" t="n">
+        <v>16020</v>
+      </c>
+      <c r="N183" t="n">
+        <v>2585</v>
+      </c>
+      <c r="O183" t="n">
+        <v>383</v>
+      </c>
+      <c r="P183" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr"/>
+      <c r="S183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>12</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>200</v>
+      </c>
+      <c r="J184" t="n">
+        <v>452</v>
+      </c>
+      <c r="K184" t="n">
+        <v>597</v>
+      </c>
+      <c r="L184" t="n">
+        <v>1049</v>
+      </c>
+      <c r="M184" t="n">
+        <v>14053</v>
+      </c>
+      <c r="N184" t="n">
+        <v>2839</v>
+      </c>
+      <c r="O184" t="n">
+        <v>399</v>
+      </c>
+      <c r="P184" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr"/>
+      <c r="S184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>20260705T060937Z</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-07-05T06:09:37.602738+00:00</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>12</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Grant Application Deadline – "Heritage Art</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>200</v>
+      </c>
+      <c r="J185" t="n">
+        <v>457</v>
+      </c>
+      <c r="K185" t="n">
+        <v>1448</v>
+      </c>
+      <c r="L185" t="n">
+        <v>1905</v>
+      </c>
+      <c r="M185" t="n">
+        <v>48777</v>
+      </c>
+      <c r="N185" t="n">
+        <v>3680</v>
+      </c>
+      <c r="O185" t="n">
+        <v>530</v>
+      </c>
+      <c r="P185" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>responses/20260705T060937Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr"/>
+      <c r="S185" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-06 12:09 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S185"/>
+  <dimension ref="A1:S201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11514,9 +11514,6 @@
       <c r="I170" t="n">
         <v>429</v>
       </c>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
       <c r="M170" t="n">
         <v>146</v>
       </c>
@@ -11529,8 +11526,6 @@
       <c r="P170" t="n">
         <v>3</v>
       </c>
-      <c r="Q170" t="inlineStr"/>
-      <c r="R170" t="inlineStr"/>
       <c r="S170" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -11579,9 +11574,6 @@
       <c r="I171" t="n">
         <v>429</v>
       </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
       <c r="M171" t="n">
         <v>187</v>
       </c>
@@ -11594,8 +11586,6 @@
       <c r="P171" t="n">
         <v>3</v>
       </c>
-      <c r="Q171" t="inlineStr"/>
-      <c r="R171" t="inlineStr"/>
       <c r="S171" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -11644,9 +11634,6 @@
       <c r="I172" t="n">
         <v>429</v>
       </c>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
       <c r="M172" t="n">
         <v>146</v>
       </c>
@@ -11659,8 +11646,6 @@
       <c r="P172" t="n">
         <v>3</v>
       </c>
-      <c r="Q172" t="inlineStr"/>
-      <c r="R172" t="inlineStr"/>
       <c r="S172" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -11709,9 +11694,6 @@
       <c r="I173" t="n">
         <v>429</v>
       </c>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
       <c r="M173" t="n">
         <v>164</v>
       </c>
@@ -11724,8 +11706,6 @@
       <c r="P173" t="n">
         <v>3</v>
       </c>
-      <c r="Q173" t="inlineStr"/>
-      <c r="R173" t="inlineStr"/>
       <c r="S173" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -11774,9 +11754,6 @@
       <c r="I174" t="n">
         <v>429</v>
       </c>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
       <c r="M174" t="n">
         <v>199</v>
       </c>
@@ -11789,8 +11766,6 @@
       <c r="P174" t="n">
         <v>3</v>
       </c>
-      <c r="Q174" t="inlineStr"/>
-      <c r="R174" t="inlineStr"/>
       <c r="S174" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -11865,8 +11840,6 @@
           <t>responses/20260705T060937Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R175" t="inlineStr"/>
-      <c r="S175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -11931,9 +11904,6 @@
       <c r="P176" t="n">
         <v>1</v>
       </c>
-      <c r="Q176" t="inlineStr"/>
-      <c r="R176" t="inlineStr"/>
-      <c r="S176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12003,8 +11973,6 @@
           <t>responses/20260705T060937Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R177" t="inlineStr"/>
-      <c r="S177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12074,8 +12042,6 @@
           <t>responses/20260705T060937Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R178" t="inlineStr"/>
-      <c r="S178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12145,8 +12111,6 @@
           <t>responses/20260705T060937Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R179" t="inlineStr"/>
-      <c r="S179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12216,8 +12180,6 @@
           <t>responses/20260705T060937Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R180" t="inlineStr"/>
-      <c r="S180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12287,8 +12249,6 @@
           <t>responses/20260705T060937Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R181" t="inlineStr"/>
-      <c r="S181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12353,9 +12313,6 @@
       <c r="P182" t="n">
         <v>1</v>
       </c>
-      <c r="Q182" t="inlineStr"/>
-      <c r="R182" t="inlineStr"/>
-      <c r="S182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12425,8 +12382,6 @@
           <t>responses/20260705T060937Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R183" t="inlineStr"/>
-      <c r="S183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12496,8 +12451,6 @@
           <t>responses/20260705T060937Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R184" t="inlineStr"/>
-      <c r="S184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -12562,9 +12515,1084 @@
       <c r="P185" t="n">
         <v>1</v>
       </c>
-      <c r="Q185" t="inlineStr"/>
-      <c r="R185" t="inlineStr"/>
-      <c r="S185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>13</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>429</v>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="n">
+        <v>109</v>
+      </c>
+      <c r="N186" t="n">
+        <v>0</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q186" t="inlineStr"/>
+      <c r="R186" t="inlineStr"/>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>13</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>429</v>
+      </c>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="n">
+        <v>106</v>
+      </c>
+      <c r="N187" t="n">
+        <v>0</v>
+      </c>
+      <c r="O187" t="n">
+        <v>0</v>
+      </c>
+      <c r="P187" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q187" t="inlineStr"/>
+      <c r="R187" t="inlineStr"/>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>13</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>429</v>
+      </c>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="inlineStr"/>
+      <c r="M188" t="n">
+        <v>88</v>
+      </c>
+      <c r="N188" t="n">
+        <v>0</v>
+      </c>
+      <c r="O188" t="n">
+        <v>0</v>
+      </c>
+      <c r="P188" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q188" t="inlineStr"/>
+      <c r="R188" t="inlineStr"/>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>13</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>429</v>
+      </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="n">
+        <v>104</v>
+      </c>
+      <c r="N189" t="n">
+        <v>0</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0</v>
+      </c>
+      <c r="P189" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q189" t="inlineStr"/>
+      <c r="R189" t="inlineStr"/>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>13</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>429</v>
+      </c>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="n">
+        <v>281</v>
+      </c>
+      <c r="N190" t="n">
+        <v>0</v>
+      </c>
+      <c r="O190" t="n">
+        <v>0</v>
+      </c>
+      <c r="P190" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q190" t="inlineStr"/>
+      <c r="R190" t="inlineStr"/>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>13</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>429</v>
+      </c>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="n">
+        <v>204</v>
+      </c>
+      <c r="N191" t="n">
+        <v>0</v>
+      </c>
+      <c r="O191" t="n">
+        <v>0</v>
+      </c>
+      <c r="P191" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q191" t="inlineStr"/>
+      <c r="R191" t="inlineStr"/>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>13</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>200</v>
+      </c>
+      <c r="J192" t="n">
+        <v>247</v>
+      </c>
+      <c r="K192" t="n">
+        <v>5998</v>
+      </c>
+      <c r="L192" t="n">
+        <v>6245</v>
+      </c>
+      <c r="M192" t="n">
+        <v>34067</v>
+      </c>
+      <c r="N192" t="n">
+        <v>944</v>
+      </c>
+      <c r="O192" t="n">
+        <v>126</v>
+      </c>
+      <c r="P192" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr"/>
+      <c r="S192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>13</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>200</v>
+      </c>
+      <c r="J193" t="n">
+        <v>278</v>
+      </c>
+      <c r="K193" t="n">
+        <v>5709</v>
+      </c>
+      <c r="L193" t="n">
+        <v>5987</v>
+      </c>
+      <c r="M193" t="n">
+        <v>48647</v>
+      </c>
+      <c r="N193" t="n">
+        <v>16444</v>
+      </c>
+      <c r="O193" t="n">
+        <v>1618</v>
+      </c>
+      <c r="P193" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr"/>
+      <c r="S193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>13</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>200</v>
+      </c>
+      <c r="J194" t="n">
+        <v>278</v>
+      </c>
+      <c r="K194" t="n">
+        <v>5304</v>
+      </c>
+      <c r="L194" t="n">
+        <v>5582</v>
+      </c>
+      <c r="M194" t="n">
+        <v>79866</v>
+      </c>
+      <c r="N194" t="n">
+        <v>18383</v>
+      </c>
+      <c r="O194" t="n">
+        <v>1836</v>
+      </c>
+      <c r="P194" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr"/>
+      <c r="S194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>13</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>200</v>
+      </c>
+      <c r="J195" t="n">
+        <v>276</v>
+      </c>
+      <c r="K195" t="n">
+        <v>2059</v>
+      </c>
+      <c r="L195" t="n">
+        <v>2335</v>
+      </c>
+      <c r="M195" t="n">
+        <v>74493</v>
+      </c>
+      <c r="N195" t="n">
+        <v>9039</v>
+      </c>
+      <c r="O195" t="n">
+        <v>703</v>
+      </c>
+      <c r="P195" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr"/>
+      <c r="S195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>13</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>200</v>
+      </c>
+      <c r="J196" t="n">
+        <v>309</v>
+      </c>
+      <c r="K196" t="n">
+        <v>5558</v>
+      </c>
+      <c r="L196" t="n">
+        <v>5867</v>
+      </c>
+      <c r="M196" t="n">
+        <v>84040</v>
+      </c>
+      <c r="N196" t="n">
+        <v>18041</v>
+      </c>
+      <c r="O196" t="n">
+        <v>1545</v>
+      </c>
+      <c r="P196" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr"/>
+      <c r="S196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>13</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>200</v>
+      </c>
+      <c r="J197" t="n">
+        <v>335</v>
+      </c>
+      <c r="K197" t="n">
+        <v>3739</v>
+      </c>
+      <c r="L197" t="n">
+        <v>4074</v>
+      </c>
+      <c r="M197" t="n">
+        <v>125092</v>
+      </c>
+      <c r="N197" t="n">
+        <v>0</v>
+      </c>
+      <c r="O197" t="n">
+        <v>0</v>
+      </c>
+      <c r="P197" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q197" t="inlineStr"/>
+      <c r="R197" t="inlineStr"/>
+      <c r="S197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>13</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>200</v>
+      </c>
+      <c r="J198" t="n">
+        <v>272</v>
+      </c>
+      <c r="K198" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L198" t="n">
+        <v>6272</v>
+      </c>
+      <c r="M198" t="n">
+        <v>289273</v>
+      </c>
+      <c r="N198" t="n">
+        <v>0</v>
+      </c>
+      <c r="O198" t="n">
+        <v>0</v>
+      </c>
+      <c r="P198" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q198" t="inlineStr"/>
+      <c r="R198" t="inlineStr"/>
+      <c r="S198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>13</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>200</v>
+      </c>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
+      <c r="L199" t="inlineStr"/>
+      <c r="M199" t="n">
+        <v>300537</v>
+      </c>
+      <c r="N199" t="n">
+        <v>0</v>
+      </c>
+      <c r="O199" t="n">
+        <v>0</v>
+      </c>
+      <c r="P199" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q199" t="inlineStr"/>
+      <c r="R199" t="inlineStr"/>
+      <c r="S199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>13</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>200</v>
+      </c>
+      <c r="J200" t="n">
+        <v>274</v>
+      </c>
+      <c r="K200" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L200" t="n">
+        <v>6274</v>
+      </c>
+      <c r="M200" t="n">
+        <v>292685</v>
+      </c>
+      <c r="N200" t="n">
+        <v>0</v>
+      </c>
+      <c r="O200" t="n">
+        <v>0</v>
+      </c>
+      <c r="P200" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q200" t="inlineStr"/>
+      <c r="R200" t="inlineStr"/>
+      <c r="S200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>13</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `Concurren</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>200</v>
+      </c>
+      <c r="J201" t="n">
+        <v>278</v>
+      </c>
+      <c r="K201" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L201" t="n">
+        <v>6278</v>
+      </c>
+      <c r="M201" t="n">
+        <v>339465</v>
+      </c>
+      <c r="N201" t="n">
+        <v>6130</v>
+      </c>
+      <c r="O201" t="n">
+        <v>683</v>
+      </c>
+      <c r="P201" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr"/>
+      <c r="S201" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12577,7 +13605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S185"/>
+  <dimension ref="A1:S201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23754,9 +24782,6 @@
       <c r="I170" t="n">
         <v>429</v>
       </c>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
       <c r="M170" t="n">
         <v>152</v>
       </c>
@@ -23769,8 +24794,6 @@
       <c r="P170" t="n">
         <v>3</v>
       </c>
-      <c r="Q170" t="inlineStr"/>
-      <c r="R170" t="inlineStr"/>
       <c r="S170" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -23819,9 +24842,6 @@
       <c r="I171" t="n">
         <v>429</v>
       </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
       <c r="M171" t="n">
         <v>193</v>
       </c>
@@ -23834,8 +24854,6 @@
       <c r="P171" t="n">
         <v>3</v>
       </c>
-      <c r="Q171" t="inlineStr"/>
-      <c r="R171" t="inlineStr"/>
       <c r="S171" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -23910,8 +24928,6 @@
           <t>responses/20260705T060937Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R172" t="inlineStr"/>
-      <c r="S172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -23955,9 +24971,6 @@
       <c r="I173" t="n">
         <v>429</v>
       </c>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
       <c r="M173" t="n">
         <v>128</v>
       </c>
@@ -23970,8 +24983,6 @@
       <c r="P173" t="n">
         <v>3</v>
       </c>
-      <c r="Q173" t="inlineStr"/>
-      <c r="R173" t="inlineStr"/>
       <c r="S173" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -24020,9 +25031,6 @@
       <c r="I174" t="n">
         <v>429</v>
       </c>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
       <c r="M174" t="n">
         <v>118</v>
       </c>
@@ -24035,8 +25043,6 @@
       <c r="P174" t="n">
         <v>3</v>
       </c>
-      <c r="Q174" t="inlineStr"/>
-      <c r="R174" t="inlineStr"/>
       <c r="S174" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -24085,9 +25091,6 @@
       <c r="I175" t="n">
         <v>429</v>
       </c>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
       <c r="M175" t="n">
         <v>331</v>
       </c>
@@ -24100,8 +25103,6 @@
       <c r="P175" t="n">
         <v>3</v>
       </c>
-      <c r="Q175" t="inlineStr"/>
-      <c r="R175" t="inlineStr"/>
       <c r="S175" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -24150,9 +25151,6 @@
       <c r="I176" t="n">
         <v>429</v>
       </c>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
       <c r="M176" t="n">
         <v>132</v>
       </c>
@@ -24165,8 +25163,6 @@
       <c r="P176" t="n">
         <v>3</v>
       </c>
-      <c r="Q176" t="inlineStr"/>
-      <c r="R176" t="inlineStr"/>
       <c r="S176" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -24241,8 +25237,6 @@
           <t>responses/20260705T060937Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R177" t="inlineStr"/>
-      <c r="S177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -24312,8 +25306,6 @@
           <t>responses/20260705T060937Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R178" t="inlineStr"/>
-      <c r="S178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -24383,8 +25375,6 @@
           <t>responses/20260705T060937Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R179" t="inlineStr"/>
-      <c r="S179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -24454,8 +25444,6 @@
           <t>responses/20260705T060937Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R180" t="inlineStr"/>
-      <c r="S180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -24525,8 +25513,6 @@
           <t>responses/20260705T060937Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R181" t="inlineStr"/>
-      <c r="S181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -24596,8 +25582,6 @@
           <t>responses/20260705T060937Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R182" t="inlineStr"/>
-      <c r="S182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -24667,8 +25651,6 @@
           <t>responses/20260705T060937Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R183" t="inlineStr"/>
-      <c r="S183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -24712,9 +25694,6 @@
       <c r="I184" t="n">
         <v>200</v>
       </c>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
       <c r="M184" t="n">
         <v>120274</v>
       </c>
@@ -24727,9 +25706,6 @@
       <c r="P184" t="n">
         <v>1</v>
       </c>
-      <c r="Q184" t="inlineStr"/>
-      <c r="R184" t="inlineStr"/>
-      <c r="S184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -24799,8 +25775,1086 @@
           <t>responses/20260705T060937Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R185" t="inlineStr"/>
-      <c r="S185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>13</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>200</v>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="n">
+        <v>332</v>
+      </c>
+      <c r="N186" t="n">
+        <v>0</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q186" t="inlineStr"/>
+      <c r="R186" t="inlineStr"/>
+      <c r="S186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>13</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>429</v>
+      </c>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="n">
+        <v>119</v>
+      </c>
+      <c r="N187" t="n">
+        <v>0</v>
+      </c>
+      <c r="O187" t="n">
+        <v>0</v>
+      </c>
+      <c r="P187" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q187" t="inlineStr"/>
+      <c r="R187" t="inlineStr"/>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>13</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>200</v>
+      </c>
+      <c r="J188" t="n">
+        <v>201</v>
+      </c>
+      <c r="K188" t="n">
+        <v>885</v>
+      </c>
+      <c r="L188" t="n">
+        <v>1086</v>
+      </c>
+      <c r="M188" t="n">
+        <v>22414</v>
+      </c>
+      <c r="N188" t="n">
+        <v>610</v>
+      </c>
+      <c r="O188" t="n">
+        <v>99</v>
+      </c>
+      <c r="P188" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr"/>
+      <c r="S188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>13</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>429</v>
+      </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="n">
+        <v>141</v>
+      </c>
+      <c r="N189" t="n">
+        <v>0</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0</v>
+      </c>
+      <c r="P189" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q189" t="inlineStr"/>
+      <c r="R189" t="inlineStr"/>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>13</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>429</v>
+      </c>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="n">
+        <v>178</v>
+      </c>
+      <c r="N190" t="n">
+        <v>0</v>
+      </c>
+      <c r="O190" t="n">
+        <v>0</v>
+      </c>
+      <c r="P190" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q190" t="inlineStr"/>
+      <c r="R190" t="inlineStr"/>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>13</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>429</v>
+      </c>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="n">
+        <v>127</v>
+      </c>
+      <c r="N191" t="n">
+        <v>0</v>
+      </c>
+      <c r="O191" t="n">
+        <v>0</v>
+      </c>
+      <c r="P191" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q191" t="inlineStr"/>
+      <c r="R191" t="inlineStr"/>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>13</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>429</v>
+      </c>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="n">
+        <v>197</v>
+      </c>
+      <c r="N192" t="n">
+        <v>0</v>
+      </c>
+      <c r="O192" t="n">
+        <v>0</v>
+      </c>
+      <c r="P192" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q192" t="inlineStr"/>
+      <c r="R192" t="inlineStr"/>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>13</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>429</v>
+      </c>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="n">
+        <v>294</v>
+      </c>
+      <c r="N193" t="n">
+        <v>0</v>
+      </c>
+      <c r="O193" t="n">
+        <v>0</v>
+      </c>
+      <c r="P193" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q193" t="inlineStr"/>
+      <c r="R193" t="inlineStr"/>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>13</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>200</v>
+      </c>
+      <c r="J194" t="n">
+        <v>169</v>
+      </c>
+      <c r="K194" t="n">
+        <v>5714</v>
+      </c>
+      <c r="L194" t="n">
+        <v>5883</v>
+      </c>
+      <c r="M194" t="n">
+        <v>30645</v>
+      </c>
+      <c r="N194" t="n">
+        <v>20701</v>
+      </c>
+      <c r="O194" t="n">
+        <v>2918</v>
+      </c>
+      <c r="P194" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr"/>
+      <c r="S194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>13</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>200</v>
+      </c>
+      <c r="J195" t="n">
+        <v>201</v>
+      </c>
+      <c r="K195" t="n">
+        <v>7711</v>
+      </c>
+      <c r="L195" t="n">
+        <v>7912</v>
+      </c>
+      <c r="M195" t="n">
+        <v>57059</v>
+      </c>
+      <c r="N195" t="n">
+        <v>16033</v>
+      </c>
+      <c r="O195" t="n">
+        <v>2165</v>
+      </c>
+      <c r="P195" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr"/>
+      <c r="S195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>13</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>200</v>
+      </c>
+      <c r="J196" t="n">
+        <v>204</v>
+      </c>
+      <c r="K196" t="n">
+        <v>1805</v>
+      </c>
+      <c r="L196" t="n">
+        <v>2009</v>
+      </c>
+      <c r="M196" t="n">
+        <v>50899</v>
+      </c>
+      <c r="N196" t="n">
+        <v>8315</v>
+      </c>
+      <c r="O196" t="n">
+        <v>1034</v>
+      </c>
+      <c r="P196" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr"/>
+      <c r="S196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>13</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>200</v>
+      </c>
+      <c r="J197" t="n">
+        <v>240</v>
+      </c>
+      <c r="K197" t="n">
+        <v>4111</v>
+      </c>
+      <c r="L197" t="n">
+        <v>4351</v>
+      </c>
+      <c r="M197" t="n">
+        <v>104358</v>
+      </c>
+      <c r="N197" t="n">
+        <v>15907</v>
+      </c>
+      <c r="O197" t="n">
+        <v>2270</v>
+      </c>
+      <c r="P197" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr"/>
+      <c r="S197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>13</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>200</v>
+      </c>
+      <c r="J198" t="n">
+        <v>238</v>
+      </c>
+      <c r="K198" t="n">
+        <v>5066</v>
+      </c>
+      <c r="L198" t="n">
+        <v>5304</v>
+      </c>
+      <c r="M198" t="n">
+        <v>98542</v>
+      </c>
+      <c r="N198" t="n">
+        <v>23522</v>
+      </c>
+      <c r="O198" t="n">
+        <v>2690</v>
+      </c>
+      <c r="P198" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr"/>
+      <c r="S198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>13</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>200</v>
+      </c>
+      <c r="J199" t="n">
+        <v>238</v>
+      </c>
+      <c r="K199" t="n">
+        <v>4877</v>
+      </c>
+      <c r="L199" t="n">
+        <v>5115</v>
+      </c>
+      <c r="M199" t="n">
+        <v>193310</v>
+      </c>
+      <c r="N199" t="n">
+        <v>20616</v>
+      </c>
+      <c r="O199" t="n">
+        <v>2738</v>
+      </c>
+      <c r="P199" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr"/>
+      <c r="S199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>13</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>200</v>
+      </c>
+      <c r="J200" t="n">
+        <v>197</v>
+      </c>
+      <c r="K200" t="n">
+        <v>4279</v>
+      </c>
+      <c r="L200" t="n">
+        <v>4476</v>
+      </c>
+      <c r="M200" t="n">
+        <v>178527</v>
+      </c>
+      <c r="N200" t="n">
+        <v>12841</v>
+      </c>
+      <c r="O200" t="n">
+        <v>1622</v>
+      </c>
+      <c r="P200" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr"/>
+      <c r="S200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>13</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled “Leve</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>200</v>
+      </c>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="inlineStr"/>
+      <c r="M201" t="n">
+        <v>300724</v>
+      </c>
+      <c r="N201" t="n">
+        <v>0</v>
+      </c>
+      <c r="O201" t="n">
+        <v>0</v>
+      </c>
+      <c r="P201" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q201" t="inlineStr"/>
+      <c r="R201" t="inlineStr"/>
+      <c r="S201" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24813,7 +26867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S185"/>
+  <dimension ref="A1:S201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35888,9 +37942,6 @@
       <c r="I170" t="n">
         <v>429</v>
       </c>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
       <c r="M170" t="n">
         <v>137</v>
       </c>
@@ -35903,8 +37954,6 @@
       <c r="P170" t="n">
         <v>3</v>
       </c>
-      <c r="Q170" t="inlineStr"/>
-      <c r="R170" t="inlineStr"/>
       <c r="S170" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -35953,9 +38002,6 @@
       <c r="I171" t="n">
         <v>429</v>
       </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
       <c r="M171" t="n">
         <v>279</v>
       </c>
@@ -35968,8 +38014,6 @@
       <c r="P171" t="n">
         <v>3</v>
       </c>
-      <c r="Q171" t="inlineStr"/>
-      <c r="R171" t="inlineStr"/>
       <c r="S171" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -36044,8 +38088,6 @@
           <t>responses/20260705T060937Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R172" t="inlineStr"/>
-      <c r="S172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -36115,8 +38157,6 @@
           <t>responses/20260705T060937Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R173" t="inlineStr"/>
-      <c r="S173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -36160,9 +38200,6 @@
       <c r="I174" t="n">
         <v>429</v>
       </c>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
       <c r="M174" t="n">
         <v>179</v>
       </c>
@@ -36175,8 +38212,6 @@
       <c r="P174" t="n">
         <v>3</v>
       </c>
-      <c r="Q174" t="inlineStr"/>
-      <c r="R174" t="inlineStr"/>
       <c r="S174" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -36225,9 +38260,6 @@
       <c r="I175" t="n">
         <v>429</v>
       </c>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
       <c r="M175" t="n">
         <v>125</v>
       </c>
@@ -36240,8 +38272,6 @@
       <c r="P175" t="n">
         <v>3</v>
       </c>
-      <c r="Q175" t="inlineStr"/>
-      <c r="R175" t="inlineStr"/>
       <c r="S175" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -36290,9 +38320,6 @@
       <c r="I176" t="n">
         <v>429</v>
       </c>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
       <c r="M176" t="n">
         <v>142</v>
       </c>
@@ -36305,8 +38332,6 @@
       <c r="P176" t="n">
         <v>3</v>
       </c>
-      <c r="Q176" t="inlineStr"/>
-      <c r="R176" t="inlineStr"/>
       <c r="S176" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -36381,8 +38406,6 @@
           <t>responses/20260705T060937Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R177" t="inlineStr"/>
-      <c r="S177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -36426,9 +38449,6 @@
       <c r="I178" t="n">
         <v>429</v>
       </c>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
       <c r="M178" t="n">
         <v>306</v>
       </c>
@@ -36441,8 +38461,6 @@
       <c r="P178" t="n">
         <v>3</v>
       </c>
-      <c r="Q178" t="inlineStr"/>
-      <c r="R178" t="inlineStr"/>
       <c r="S178" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -36491,9 +38509,6 @@
       <c r="I179" t="n">
         <v>429</v>
       </c>
-      <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
       <c r="M179" t="n">
         <v>121</v>
       </c>
@@ -36506,8 +38521,6 @@
       <c r="P179" t="n">
         <v>3</v>
       </c>
-      <c r="Q179" t="inlineStr"/>
-      <c r="R179" t="inlineStr"/>
       <c r="S179" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -36582,8 +38595,6 @@
           <t>responses/20260705T060937Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R180" t="inlineStr"/>
-      <c r="S180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -36653,8 +38664,6 @@
           <t>responses/20260705T060937Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R181" t="inlineStr"/>
-      <c r="S181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -36724,8 +38733,6 @@
           <t>responses/20260705T060937Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R182" t="inlineStr"/>
-      <c r="S182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -36795,8 +38802,6 @@
           <t>responses/20260705T060937Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R183" t="inlineStr"/>
-      <c r="S183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -36866,8 +38871,6 @@
           <t>responses/20260705T060937Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R184" t="inlineStr"/>
-      <c r="S184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -36937,8 +38940,1090 @@
           <t>responses/20260705T060937Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R185" t="inlineStr"/>
-      <c r="S185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>13</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>429</v>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="n">
+        <v>143</v>
+      </c>
+      <c r="N186" t="n">
+        <v>0</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q186" t="inlineStr"/>
+      <c r="R186" t="inlineStr"/>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>13</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>429</v>
+      </c>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="n">
+        <v>234</v>
+      </c>
+      <c r="N187" t="n">
+        <v>0</v>
+      </c>
+      <c r="O187" t="n">
+        <v>0</v>
+      </c>
+      <c r="P187" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q187" t="inlineStr"/>
+      <c r="R187" t="inlineStr"/>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>13</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>200</v>
+      </c>
+      <c r="J188" t="n">
+        <v>453</v>
+      </c>
+      <c r="K188" t="n">
+        <v>773</v>
+      </c>
+      <c r="L188" t="n">
+        <v>1226</v>
+      </c>
+      <c r="M188" t="n">
+        <v>13452</v>
+      </c>
+      <c r="N188" t="n">
+        <v>3081</v>
+      </c>
+      <c r="O188" t="n">
+        <v>428</v>
+      </c>
+      <c r="P188" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr"/>
+      <c r="S188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>13</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>429</v>
+      </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="n">
+        <v>164</v>
+      </c>
+      <c r="N189" t="n">
+        <v>0</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0</v>
+      </c>
+      <c r="P189" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q189" t="inlineStr"/>
+      <c r="R189" t="inlineStr"/>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>13</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>429</v>
+      </c>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="n">
+        <v>105</v>
+      </c>
+      <c r="N190" t="n">
+        <v>0</v>
+      </c>
+      <c r="O190" t="n">
+        <v>0</v>
+      </c>
+      <c r="P190" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q190" t="inlineStr"/>
+      <c r="R190" t="inlineStr"/>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>13</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>429</v>
+      </c>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="n">
+        <v>95</v>
+      </c>
+      <c r="N191" t="n">
+        <v>0</v>
+      </c>
+      <c r="O191" t="n">
+        <v>0</v>
+      </c>
+      <c r="P191" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q191" t="inlineStr"/>
+      <c r="R191" t="inlineStr"/>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>13</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>200</v>
+      </c>
+      <c r="J192" t="n">
+        <v>453</v>
+      </c>
+      <c r="K192" t="n">
+        <v>736</v>
+      </c>
+      <c r="L192" t="n">
+        <v>1189</v>
+      </c>
+      <c r="M192" t="n">
+        <v>79843</v>
+      </c>
+      <c r="N192" t="n">
+        <v>2962</v>
+      </c>
+      <c r="O192" t="n">
+        <v>412</v>
+      </c>
+      <c r="P192" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr"/>
+      <c r="S192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>13</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>200</v>
+      </c>
+      <c r="J193" t="n">
+        <v>453</v>
+      </c>
+      <c r="K193" t="n">
+        <v>602</v>
+      </c>
+      <c r="L193" t="n">
+        <v>1055</v>
+      </c>
+      <c r="M193" t="n">
+        <v>4508</v>
+      </c>
+      <c r="N193" t="n">
+        <v>2841</v>
+      </c>
+      <c r="O193" t="n">
+        <v>400</v>
+      </c>
+      <c r="P193" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr"/>
+      <c r="S193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>13</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>429</v>
+      </c>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="n">
+        <v>109</v>
+      </c>
+      <c r="N194" t="n">
+        <v>0</v>
+      </c>
+      <c r="O194" t="n">
+        <v>0</v>
+      </c>
+      <c r="P194" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q194" t="inlineStr"/>
+      <c r="R194" t="inlineStr"/>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>13</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>429</v>
+      </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="n">
+        <v>314</v>
+      </c>
+      <c r="N195" t="n">
+        <v>0</v>
+      </c>
+      <c r="O195" t="n">
+        <v>0</v>
+      </c>
+      <c r="P195" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q195" t="inlineStr"/>
+      <c r="R195" t="inlineStr"/>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>13</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>200</v>
+      </c>
+      <c r="J196" t="n">
+        <v>401</v>
+      </c>
+      <c r="K196" t="n">
+        <v>651</v>
+      </c>
+      <c r="L196" t="n">
+        <v>1052</v>
+      </c>
+      <c r="M196" t="n">
+        <v>5701</v>
+      </c>
+      <c r="N196" t="n">
+        <v>2715</v>
+      </c>
+      <c r="O196" t="n">
+        <v>405</v>
+      </c>
+      <c r="P196" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr"/>
+      <c r="S196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>13</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>200</v>
+      </c>
+      <c r="J197" t="n">
+        <v>496</v>
+      </c>
+      <c r="K197" t="n">
+        <v>708</v>
+      </c>
+      <c r="L197" t="n">
+        <v>1204</v>
+      </c>
+      <c r="M197" t="n">
+        <v>8105</v>
+      </c>
+      <c r="N197" t="n">
+        <v>2234</v>
+      </c>
+      <c r="O197" t="n">
+        <v>323</v>
+      </c>
+      <c r="P197" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr"/>
+      <c r="S197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>13</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>200</v>
+      </c>
+      <c r="J198" t="n">
+        <v>472</v>
+      </c>
+      <c r="K198" t="n">
+        <v>772</v>
+      </c>
+      <c r="L198" t="n">
+        <v>1244</v>
+      </c>
+      <c r="M198" t="n">
+        <v>11898</v>
+      </c>
+      <c r="N198" t="n">
+        <v>3358</v>
+      </c>
+      <c r="O198" t="n">
+        <v>482</v>
+      </c>
+      <c r="P198" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr"/>
+      <c r="S198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>13</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>200</v>
+      </c>
+      <c r="J199" t="n">
+        <v>446</v>
+      </c>
+      <c r="K199" t="n">
+        <v>536</v>
+      </c>
+      <c r="L199" t="n">
+        <v>982</v>
+      </c>
+      <c r="M199" t="n">
+        <v>18865</v>
+      </c>
+      <c r="N199" t="n">
+        <v>2751</v>
+      </c>
+      <c r="O199" t="n">
+        <v>372</v>
+      </c>
+      <c r="P199" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr"/>
+      <c r="S199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>13</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>200</v>
+      </c>
+      <c r="J200" t="n">
+        <v>449</v>
+      </c>
+      <c r="K200" t="n">
+        <v>1920</v>
+      </c>
+      <c r="L200" t="n">
+        <v>2369</v>
+      </c>
+      <c r="M200" t="n">
+        <v>82445</v>
+      </c>
+      <c r="N200" t="n">
+        <v>4619</v>
+      </c>
+      <c r="O200" t="n">
+        <v>680</v>
+      </c>
+      <c r="P200" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>responses/20260706T115904Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr"/>
+      <c r="S200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>20260706T115904Z</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-07-06T11:59:04.544928+00:00</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>13</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Northern Rur</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>200</v>
+      </c>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="inlineStr"/>
+      <c r="M201" t="n">
+        <v>300679</v>
+      </c>
+      <c r="N201" t="n">
+        <v>0</v>
+      </c>
+      <c r="O201" t="n">
+        <v>0</v>
+      </c>
+      <c r="P201" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q201" t="inlineStr"/>
+      <c r="R201" t="inlineStr"/>
+      <c r="S201" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-07 16:35 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S201"/>
+  <dimension ref="A1:S217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12558,9 +12558,6 @@
       <c r="I186" t="n">
         <v>429</v>
       </c>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr"/>
       <c r="M186" t="n">
         <v>109</v>
       </c>
@@ -12573,8 +12570,6 @@
       <c r="P186" t="n">
         <v>3</v>
       </c>
-      <c r="Q186" t="inlineStr"/>
-      <c r="R186" t="inlineStr"/>
       <c r="S186" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -12623,9 +12618,6 @@
       <c r="I187" t="n">
         <v>429</v>
       </c>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
       <c r="M187" t="n">
         <v>106</v>
       </c>
@@ -12638,8 +12630,6 @@
       <c r="P187" t="n">
         <v>3</v>
       </c>
-      <c r="Q187" t="inlineStr"/>
-      <c r="R187" t="inlineStr"/>
       <c r="S187" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -12688,9 +12678,6 @@
       <c r="I188" t="n">
         <v>429</v>
       </c>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
       <c r="M188" t="n">
         <v>88</v>
       </c>
@@ -12703,8 +12690,6 @@
       <c r="P188" t="n">
         <v>3</v>
       </c>
-      <c r="Q188" t="inlineStr"/>
-      <c r="R188" t="inlineStr"/>
       <c r="S188" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -12753,9 +12738,6 @@
       <c r="I189" t="n">
         <v>429</v>
       </c>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
       <c r="M189" t="n">
         <v>104</v>
       </c>
@@ -12768,8 +12750,6 @@
       <c r="P189" t="n">
         <v>3</v>
       </c>
-      <c r="Q189" t="inlineStr"/>
-      <c r="R189" t="inlineStr"/>
       <c r="S189" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -12818,9 +12798,6 @@
       <c r="I190" t="n">
         <v>429</v>
       </c>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
       <c r="M190" t="n">
         <v>281</v>
       </c>
@@ -12833,8 +12810,6 @@
       <c r="P190" t="n">
         <v>3</v>
       </c>
-      <c r="Q190" t="inlineStr"/>
-      <c r="R190" t="inlineStr"/>
       <c r="S190" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -12883,9 +12858,6 @@
       <c r="I191" t="n">
         <v>429</v>
       </c>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
       <c r="M191" t="n">
         <v>204</v>
       </c>
@@ -12898,8 +12870,6 @@
       <c r="P191" t="n">
         <v>3</v>
       </c>
-      <c r="Q191" t="inlineStr"/>
-      <c r="R191" t="inlineStr"/>
       <c r="S191" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -12974,8 +12944,6 @@
           <t>responses/20260706T115904Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R192" t="inlineStr"/>
-      <c r="S192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13045,8 +13013,6 @@
           <t>responses/20260706T115904Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R193" t="inlineStr"/>
-      <c r="S193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13116,8 +13082,6 @@
           <t>responses/20260706T115904Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R194" t="inlineStr"/>
-      <c r="S194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -13187,8 +13151,6 @@
           <t>responses/20260706T115904Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R195" t="inlineStr"/>
-      <c r="S195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -13258,8 +13220,6 @@
           <t>responses/20260706T115904Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R196" t="inlineStr"/>
-      <c r="S196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13324,9 +13284,6 @@
       <c r="P197" t="n">
         <v>1</v>
       </c>
-      <c r="Q197" t="inlineStr"/>
-      <c r="R197" t="inlineStr"/>
-      <c r="S197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -13391,9 +13348,6 @@
       <c r="P198" t="n">
         <v>2</v>
       </c>
-      <c r="Q198" t="inlineStr"/>
-      <c r="R198" t="inlineStr"/>
-      <c r="S198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -13437,9 +13391,6 @@
       <c r="I199" t="n">
         <v>200</v>
       </c>
-      <c r="J199" t="inlineStr"/>
-      <c r="K199" t="inlineStr"/>
-      <c r="L199" t="inlineStr"/>
       <c r="M199" t="n">
         <v>300537</v>
       </c>
@@ -13452,9 +13403,6 @@
       <c r="P199" t="n">
         <v>1</v>
       </c>
-      <c r="Q199" t="inlineStr"/>
-      <c r="R199" t="inlineStr"/>
-      <c r="S199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13519,9 +13467,6 @@
       <c r="P200" t="n">
         <v>1</v>
       </c>
-      <c r="Q200" t="inlineStr"/>
-      <c r="R200" t="inlineStr"/>
-      <c r="S200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13591,8 +13536,1088 @@
           <t>responses/20260706T115904Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R201" t="inlineStr"/>
-      <c r="S201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>14</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>429</v>
+      </c>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="n">
+        <v>208</v>
+      </c>
+      <c r="N202" t="n">
+        <v>0</v>
+      </c>
+      <c r="O202" t="n">
+        <v>0</v>
+      </c>
+      <c r="P202" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q202" t="inlineStr"/>
+      <c r="R202" t="inlineStr"/>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>14</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>429</v>
+      </c>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr"/>
+      <c r="L203" t="inlineStr"/>
+      <c r="M203" t="n">
+        <v>237</v>
+      </c>
+      <c r="N203" t="n">
+        <v>0</v>
+      </c>
+      <c r="O203" t="n">
+        <v>0</v>
+      </c>
+      <c r="P203" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q203" t="inlineStr"/>
+      <c r="R203" t="inlineStr"/>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>14</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>429</v>
+      </c>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr"/>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="n">
+        <v>235</v>
+      </c>
+      <c r="N204" t="n">
+        <v>0</v>
+      </c>
+      <c r="O204" t="n">
+        <v>0</v>
+      </c>
+      <c r="P204" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q204" t="inlineStr"/>
+      <c r="R204" t="inlineStr"/>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>14</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>429</v>
+      </c>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr"/>
+      <c r="L205" t="inlineStr"/>
+      <c r="M205" t="n">
+        <v>423</v>
+      </c>
+      <c r="N205" t="n">
+        <v>0</v>
+      </c>
+      <c r="O205" t="n">
+        <v>0</v>
+      </c>
+      <c r="P205" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q205" t="inlineStr"/>
+      <c r="R205" t="inlineStr"/>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>14</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>429</v>
+      </c>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr"/>
+      <c r="L206" t="inlineStr"/>
+      <c r="M206" t="n">
+        <v>257</v>
+      </c>
+      <c r="N206" t="n">
+        <v>0</v>
+      </c>
+      <c r="O206" t="n">
+        <v>0</v>
+      </c>
+      <c r="P206" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q206" t="inlineStr"/>
+      <c r="R206" t="inlineStr"/>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>14</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>429</v>
+      </c>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr"/>
+      <c r="L207" t="inlineStr"/>
+      <c r="M207" t="n">
+        <v>437</v>
+      </c>
+      <c r="N207" t="n">
+        <v>0</v>
+      </c>
+      <c r="O207" t="n">
+        <v>0</v>
+      </c>
+      <c r="P207" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q207" t="inlineStr"/>
+      <c r="R207" t="inlineStr"/>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>14</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>429</v>
+      </c>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr"/>
+      <c r="L208" t="inlineStr"/>
+      <c r="M208" t="n">
+        <v>407</v>
+      </c>
+      <c r="N208" t="n">
+        <v>0</v>
+      </c>
+      <c r="O208" t="n">
+        <v>0</v>
+      </c>
+      <c r="P208" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q208" t="inlineStr"/>
+      <c r="R208" t="inlineStr"/>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>14</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>200</v>
+      </c>
+      <c r="J209" t="n">
+        <v>63</v>
+      </c>
+      <c r="K209" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L209" t="n">
+        <v>6063</v>
+      </c>
+      <c r="M209" t="n">
+        <v>17439</v>
+      </c>
+      <c r="N209" t="n">
+        <v>0</v>
+      </c>
+      <c r="O209" t="n">
+        <v>0</v>
+      </c>
+      <c r="P209" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q209" t="inlineStr"/>
+      <c r="R209" t="inlineStr"/>
+      <c r="S209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>14</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>200</v>
+      </c>
+      <c r="J210" t="n">
+        <v>86</v>
+      </c>
+      <c r="K210" t="n">
+        <v>5047</v>
+      </c>
+      <c r="L210" t="n">
+        <v>5133</v>
+      </c>
+      <c r="M210" t="n">
+        <v>27358</v>
+      </c>
+      <c r="N210" t="n">
+        <v>19474</v>
+      </c>
+      <c r="O210" t="n">
+        <v>2358</v>
+      </c>
+      <c r="P210" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr"/>
+      <c r="S210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>14</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>200</v>
+      </c>
+      <c r="J211" t="n">
+        <v>84</v>
+      </c>
+      <c r="K211" t="n">
+        <v>1196</v>
+      </c>
+      <c r="L211" t="n">
+        <v>1280</v>
+      </c>
+      <c r="M211" t="n">
+        <v>28791</v>
+      </c>
+      <c r="N211" t="n">
+        <v>5416</v>
+      </c>
+      <c r="O211" t="n">
+        <v>552</v>
+      </c>
+      <c r="P211" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr"/>
+      <c r="S211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>14</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>200</v>
+      </c>
+      <c r="J212" t="n">
+        <v>86</v>
+      </c>
+      <c r="K212" t="n">
+        <v>4775</v>
+      </c>
+      <c r="L212" t="n">
+        <v>4861</v>
+      </c>
+      <c r="M212" t="n">
+        <v>57362</v>
+      </c>
+      <c r="N212" t="n">
+        <v>16999</v>
+      </c>
+      <c r="O212" t="n">
+        <v>1994</v>
+      </c>
+      <c r="P212" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr"/>
+      <c r="S212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>14</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>200</v>
+      </c>
+      <c r="J213" t="n">
+        <v>114</v>
+      </c>
+      <c r="K213" t="n">
+        <v>5183</v>
+      </c>
+      <c r="L213" t="n">
+        <v>5297</v>
+      </c>
+      <c r="M213" t="n">
+        <v>44615</v>
+      </c>
+      <c r="N213" t="n">
+        <v>21150</v>
+      </c>
+      <c r="O213" t="n">
+        <v>1872</v>
+      </c>
+      <c r="P213" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr"/>
+      <c r="S213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>14</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>200</v>
+      </c>
+      <c r="J214" t="n">
+        <v>135</v>
+      </c>
+      <c r="K214" t="n">
+        <v>3506</v>
+      </c>
+      <c r="L214" t="n">
+        <v>3641</v>
+      </c>
+      <c r="M214" t="n">
+        <v>97500</v>
+      </c>
+      <c r="N214" t="n">
+        <v>12763</v>
+      </c>
+      <c r="O214" t="n">
+        <v>1436</v>
+      </c>
+      <c r="P214" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr"/>
+      <c r="S214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>14</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>200</v>
+      </c>
+      <c r="J215" t="n">
+        <v>82</v>
+      </c>
+      <c r="K215" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L215" t="n">
+        <v>6082</v>
+      </c>
+      <c r="M215" t="n">
+        <v>123047</v>
+      </c>
+      <c r="N215" t="n">
+        <v>0</v>
+      </c>
+      <c r="O215" t="n">
+        <v>0</v>
+      </c>
+      <c r="P215" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q215" t="inlineStr"/>
+      <c r="R215" t="inlineStr"/>
+      <c r="S215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>14</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>200</v>
+      </c>
+      <c r="J216" t="n">
+        <v>77</v>
+      </c>
+      <c r="K216" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L216" t="n">
+        <v>6077</v>
+      </c>
+      <c r="M216" t="n">
+        <v>141054</v>
+      </c>
+      <c r="N216" t="n">
+        <v>0</v>
+      </c>
+      <c r="O216" t="n">
+        <v>0</v>
+      </c>
+      <c r="P216" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q216" t="inlineStr"/>
+      <c r="R216" t="inlineStr"/>
+      <c r="S216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>14</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>200</v>
+      </c>
+      <c r="J217" t="n">
+        <v>86</v>
+      </c>
+      <c r="K217" t="n">
+        <v>5174</v>
+      </c>
+      <c r="L217" t="n">
+        <v>5260</v>
+      </c>
+      <c r="M217" t="n">
+        <v>313273</v>
+      </c>
+      <c r="N217" t="n">
+        <v>19218</v>
+      </c>
+      <c r="O217" t="n">
+        <v>1970</v>
+      </c>
+      <c r="P217" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr"/>
+      <c r="S217" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13605,7 +14630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S201"/>
+  <dimension ref="A1:S217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25818,9 +26843,6 @@
       <c r="I186" t="n">
         <v>200</v>
       </c>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr"/>
       <c r="M186" t="n">
         <v>332</v>
       </c>
@@ -25833,9 +26855,6 @@
       <c r="P186" t="n">
         <v>1</v>
       </c>
-      <c r="Q186" t="inlineStr"/>
-      <c r="R186" t="inlineStr"/>
-      <c r="S186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -25879,9 +26898,6 @@
       <c r="I187" t="n">
         <v>429</v>
       </c>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
       <c r="M187" t="n">
         <v>119</v>
       </c>
@@ -25894,8 +26910,6 @@
       <c r="P187" t="n">
         <v>3</v>
       </c>
-      <c r="Q187" t="inlineStr"/>
-      <c r="R187" t="inlineStr"/>
       <c r="S187" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -25970,8 +26984,6 @@
           <t>responses/20260706T115904Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R188" t="inlineStr"/>
-      <c r="S188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -26015,9 +27027,6 @@
       <c r="I189" t="n">
         <v>429</v>
       </c>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
       <c r="M189" t="n">
         <v>141</v>
       </c>
@@ -26030,8 +27039,6 @@
       <c r="P189" t="n">
         <v>3</v>
       </c>
-      <c r="Q189" t="inlineStr"/>
-      <c r="R189" t="inlineStr"/>
       <c r="S189" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -26080,9 +27087,6 @@
       <c r="I190" t="n">
         <v>429</v>
       </c>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
       <c r="M190" t="n">
         <v>178</v>
       </c>
@@ -26095,8 +27099,6 @@
       <c r="P190" t="n">
         <v>3</v>
       </c>
-      <c r="Q190" t="inlineStr"/>
-      <c r="R190" t="inlineStr"/>
       <c r="S190" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -26145,9 +27147,6 @@
       <c r="I191" t="n">
         <v>429</v>
       </c>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
       <c r="M191" t="n">
         <v>127</v>
       </c>
@@ -26160,8 +27159,6 @@
       <c r="P191" t="n">
         <v>3</v>
       </c>
-      <c r="Q191" t="inlineStr"/>
-      <c r="R191" t="inlineStr"/>
       <c r="S191" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -26210,9 +27207,6 @@
       <c r="I192" t="n">
         <v>429</v>
       </c>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
       <c r="M192" t="n">
         <v>197</v>
       </c>
@@ -26225,8 +27219,6 @@
       <c r="P192" t="n">
         <v>3</v>
       </c>
-      <c r="Q192" t="inlineStr"/>
-      <c r="R192" t="inlineStr"/>
       <c r="S192" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
@@ -26275,9 +27267,6 @@
       <c r="I193" t="n">
         <v>429</v>
       </c>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
       <c r="M193" t="n">
         <v>294</v>
       </c>
@@ -26290,8 +27279,6 @@
       <c r="P193" t="n">
         <v>3</v>
       </c>
-      <c r="Q193" t="inlineStr"/>
-      <c r="R193" t="inlineStr"/>
       <c r="S193" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -26366,8 +27353,6 @@
           <t>responses/20260706T115904Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R194" t="inlineStr"/>
-      <c r="S194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -26437,8 +27422,6 @@
           <t>responses/20260706T115904Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R195" t="inlineStr"/>
-      <c r="S195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -26508,8 +27491,6 @@
           <t>responses/20260706T115904Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R196" t="inlineStr"/>
-      <c r="S196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -26579,8 +27560,6 @@
           <t>responses/20260706T115904Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R197" t="inlineStr"/>
-      <c r="S197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -26650,8 +27629,6 @@
           <t>responses/20260706T115904Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R198" t="inlineStr"/>
-      <c r="S198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -26721,8 +27698,6 @@
           <t>responses/20260706T115904Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R199" t="inlineStr"/>
-      <c r="S199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -26792,8 +27767,6 @@
           <t>responses/20260706T115904Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R200" t="inlineStr"/>
-      <c r="S200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -26837,9 +27810,6 @@
       <c r="I201" t="n">
         <v>200</v>
       </c>
-      <c r="J201" t="inlineStr"/>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr"/>
       <c r="M201" t="n">
         <v>300724</v>
       </c>
@@ -26852,9 +27822,1080 @@
       <c r="P201" t="n">
         <v>1</v>
       </c>
-      <c r="Q201" t="inlineStr"/>
-      <c r="R201" t="inlineStr"/>
-      <c r="S201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>14</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>200</v>
+      </c>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="n">
+        <v>510</v>
+      </c>
+      <c r="N202" t="n">
+        <v>0</v>
+      </c>
+      <c r="O202" t="n">
+        <v>0</v>
+      </c>
+      <c r="P202" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q202" t="inlineStr"/>
+      <c r="R202" t="inlineStr"/>
+      <c r="S202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>14</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>429</v>
+      </c>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr"/>
+      <c r="L203" t="inlineStr"/>
+      <c r="M203" t="n">
+        <v>245</v>
+      </c>
+      <c r="N203" t="n">
+        <v>0</v>
+      </c>
+      <c r="O203" t="n">
+        <v>0</v>
+      </c>
+      <c r="P203" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q203" t="inlineStr"/>
+      <c r="R203" t="inlineStr"/>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>14</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>429</v>
+      </c>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr"/>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="n">
+        <v>519</v>
+      </c>
+      <c r="N204" t="n">
+        <v>0</v>
+      </c>
+      <c r="O204" t="n">
+        <v>0</v>
+      </c>
+      <c r="P204" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q204" t="inlineStr"/>
+      <c r="R204" t="inlineStr"/>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>14</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>429</v>
+      </c>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr"/>
+      <c r="L205" t="inlineStr"/>
+      <c r="M205" t="n">
+        <v>240</v>
+      </c>
+      <c r="N205" t="n">
+        <v>0</v>
+      </c>
+      <c r="O205" t="n">
+        <v>0</v>
+      </c>
+      <c r="P205" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q205" t="inlineStr"/>
+      <c r="R205" t="inlineStr"/>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>14</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>429</v>
+      </c>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr"/>
+      <c r="L206" t="inlineStr"/>
+      <c r="M206" t="n">
+        <v>233</v>
+      </c>
+      <c r="N206" t="n">
+        <v>0</v>
+      </c>
+      <c r="O206" t="n">
+        <v>0</v>
+      </c>
+      <c r="P206" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q206" t="inlineStr"/>
+      <c r="R206" t="inlineStr"/>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>14</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>429</v>
+      </c>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr"/>
+      <c r="L207" t="inlineStr"/>
+      <c r="M207" t="n">
+        <v>271</v>
+      </c>
+      <c r="N207" t="n">
+        <v>0</v>
+      </c>
+      <c r="O207" t="n">
+        <v>0</v>
+      </c>
+      <c r="P207" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q207" t="inlineStr"/>
+      <c r="R207" t="inlineStr"/>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>14</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>429</v>
+      </c>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr"/>
+      <c r="L208" t="inlineStr"/>
+      <c r="M208" t="n">
+        <v>637</v>
+      </c>
+      <c r="N208" t="n">
+        <v>0</v>
+      </c>
+      <c r="O208" t="n">
+        <v>0</v>
+      </c>
+      <c r="P208" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q208" t="inlineStr"/>
+      <c r="R208" t="inlineStr"/>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>14</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>429</v>
+      </c>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="n">
+        <v>222</v>
+      </c>
+      <c r="N209" t="n">
+        <v>0</v>
+      </c>
+      <c r="O209" t="n">
+        <v>0</v>
+      </c>
+      <c r="P209" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q209" t="inlineStr"/>
+      <c r="R209" t="inlineStr"/>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>14</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>200</v>
+      </c>
+      <c r="J210" t="n">
+        <v>50</v>
+      </c>
+      <c r="K210" t="n">
+        <v>4384</v>
+      </c>
+      <c r="L210" t="n">
+        <v>4434</v>
+      </c>
+      <c r="M210" t="n">
+        <v>22586</v>
+      </c>
+      <c r="N210" t="n">
+        <v>18317</v>
+      </c>
+      <c r="O210" t="n">
+        <v>2406</v>
+      </c>
+      <c r="P210" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr"/>
+      <c r="S210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>14</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>200</v>
+      </c>
+      <c r="J211" t="n">
+        <v>75</v>
+      </c>
+      <c r="K211" t="n">
+        <v>6114</v>
+      </c>
+      <c r="L211" t="n">
+        <v>6189</v>
+      </c>
+      <c r="M211" t="n">
+        <v>29644</v>
+      </c>
+      <c r="N211" t="n">
+        <v>21723</v>
+      </c>
+      <c r="O211" t="n">
+        <v>2784</v>
+      </c>
+      <c r="P211" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr"/>
+      <c r="S211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>14</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>200</v>
+      </c>
+      <c r="J212" t="n">
+        <v>108</v>
+      </c>
+      <c r="K212" t="n">
+        <v>3936</v>
+      </c>
+      <c r="L212" t="n">
+        <v>4044</v>
+      </c>
+      <c r="M212" t="n">
+        <v>27979</v>
+      </c>
+      <c r="N212" t="n">
+        <v>24279</v>
+      </c>
+      <c r="O212" t="n">
+        <v>2978</v>
+      </c>
+      <c r="P212" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr"/>
+      <c r="S212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>14</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>200</v>
+      </c>
+      <c r="J213" t="n">
+        <v>71</v>
+      </c>
+      <c r="K213" t="n">
+        <v>2736</v>
+      </c>
+      <c r="L213" t="n">
+        <v>2807</v>
+      </c>
+      <c r="M213" t="n">
+        <v>44812</v>
+      </c>
+      <c r="N213" t="n">
+        <v>12229</v>
+      </c>
+      <c r="O213" t="n">
+        <v>1527</v>
+      </c>
+      <c r="P213" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr"/>
+      <c r="S213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>14</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr"/>
+      <c r="K214" t="inlineStr"/>
+      <c r="L214" t="inlineStr"/>
+      <c r="M214" t="inlineStr"/>
+      <c r="N214" t="n">
+        <v>0</v>
+      </c>
+      <c r="O214" t="n">
+        <v>0</v>
+      </c>
+      <c r="P214" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q214" t="inlineStr"/>
+      <c r="R214" t="inlineStr"/>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>JSONDecodeError: Expecting value: line 123 column 1 (char 671)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>14</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>200</v>
+      </c>
+      <c r="J215" t="n">
+        <v>75</v>
+      </c>
+      <c r="K215" t="n">
+        <v>5292</v>
+      </c>
+      <c r="L215" t="n">
+        <v>5367</v>
+      </c>
+      <c r="M215" t="n">
+        <v>89249</v>
+      </c>
+      <c r="N215" t="n">
+        <v>23186</v>
+      </c>
+      <c r="O215" t="n">
+        <v>2979</v>
+      </c>
+      <c r="P215" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr"/>
+      <c r="S215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>14</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>200</v>
+      </c>
+      <c r="J216" t="n">
+        <v>71</v>
+      </c>
+      <c r="K216" t="n">
+        <v>4492</v>
+      </c>
+      <c r="L216" t="n">
+        <v>4563</v>
+      </c>
+      <c r="M216" t="n">
+        <v>77133</v>
+      </c>
+      <c r="N216" t="n">
+        <v>16248</v>
+      </c>
+      <c r="O216" t="n">
+        <v>2033</v>
+      </c>
+      <c r="P216" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr"/>
+      <c r="S216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>14</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>200</v>
+      </c>
+      <c r="J217" t="n">
+        <v>125</v>
+      </c>
+      <c r="K217" t="n">
+        <v>4337</v>
+      </c>
+      <c r="L217" t="n">
+        <v>4462</v>
+      </c>
+      <c r="M217" t="n">
+        <v>101672</v>
+      </c>
+      <c r="N217" t="n">
+        <v>16005</v>
+      </c>
+      <c r="O217" t="n">
+        <v>2445</v>
+      </c>
+      <c r="P217" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr"/>
+      <c r="S217" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26867,7 +28908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S201"/>
+  <dimension ref="A1:S217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38983,9 +41024,6 @@
       <c r="I186" t="n">
         <v>429</v>
       </c>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr"/>
       <c r="M186" t="n">
         <v>143</v>
       </c>
@@ -38998,8 +41036,6 @@
       <c r="P186" t="n">
         <v>3</v>
       </c>
-      <c r="Q186" t="inlineStr"/>
-      <c r="R186" t="inlineStr"/>
       <c r="S186" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -39048,9 +41084,6 @@
       <c r="I187" t="n">
         <v>429</v>
       </c>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
       <c r="M187" t="n">
         <v>234</v>
       </c>
@@ -39063,8 +41096,6 @@
       <c r="P187" t="n">
         <v>3</v>
       </c>
-      <c r="Q187" t="inlineStr"/>
-      <c r="R187" t="inlineStr"/>
       <c r="S187" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -39139,8 +41170,6 @@
           <t>responses/20260706T115904Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R188" t="inlineStr"/>
-      <c r="S188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -39184,9 +41213,6 @@
       <c r="I189" t="n">
         <v>429</v>
       </c>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
       <c r="M189" t="n">
         <v>164</v>
       </c>
@@ -39199,8 +41225,6 @@
       <c r="P189" t="n">
         <v>3</v>
       </c>
-      <c r="Q189" t="inlineStr"/>
-      <c r="R189" t="inlineStr"/>
       <c r="S189" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -39249,9 +41273,6 @@
       <c r="I190" t="n">
         <v>429</v>
       </c>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
       <c r="M190" t="n">
         <v>105</v>
       </c>
@@ -39264,8 +41285,6 @@
       <c r="P190" t="n">
         <v>3</v>
       </c>
-      <c r="Q190" t="inlineStr"/>
-      <c r="R190" t="inlineStr"/>
       <c r="S190" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -39314,9 +41333,6 @@
       <c r="I191" t="n">
         <v>429</v>
       </c>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
       <c r="M191" t="n">
         <v>95</v>
       </c>
@@ -39329,8 +41345,6 @@
       <c r="P191" t="n">
         <v>3</v>
       </c>
-      <c r="Q191" t="inlineStr"/>
-      <c r="R191" t="inlineStr"/>
       <c r="S191" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -39405,8 +41419,6 @@
           <t>responses/20260706T115904Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R192" t="inlineStr"/>
-      <c r="S192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -39476,8 +41488,6 @@
           <t>responses/20260706T115904Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R193" t="inlineStr"/>
-      <c r="S193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -39521,9 +41531,6 @@
       <c r="I194" t="n">
         <v>429</v>
       </c>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
       <c r="M194" t="n">
         <v>109</v>
       </c>
@@ -39536,8 +41543,6 @@
       <c r="P194" t="n">
         <v>3</v>
       </c>
-      <c r="Q194" t="inlineStr"/>
-      <c r="R194" t="inlineStr"/>
       <c r="S194" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"poolside/laguna-m.1:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Poolside","is_byok":false</t>
@@ -39586,9 +41591,6 @@
       <c r="I195" t="n">
         <v>429</v>
       </c>
-      <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr"/>
       <c r="M195" t="n">
         <v>314</v>
       </c>
@@ -39601,8 +41603,6 @@
       <c r="P195" t="n">
         <v>3</v>
       </c>
-      <c r="Q195" t="inlineStr"/>
-      <c r="R195" t="inlineStr"/>
       <c r="S195" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -39677,8 +41677,6 @@
           <t>responses/20260706T115904Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R196" t="inlineStr"/>
-      <c r="S196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -39748,8 +41746,6 @@
           <t>responses/20260706T115904Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R197" t="inlineStr"/>
-      <c r="S197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -39819,8 +41815,6 @@
           <t>responses/20260706T115904Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R198" t="inlineStr"/>
-      <c r="S198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -39890,8 +41884,6 @@
           <t>responses/20260706T115904Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R199" t="inlineStr"/>
-      <c r="S199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -39961,8 +41953,6 @@
           <t>responses/20260706T115904Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R200" t="inlineStr"/>
-      <c r="S200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -40006,9 +41996,6 @@
       <c r="I201" t="n">
         <v>200</v>
       </c>
-      <c r="J201" t="inlineStr"/>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr"/>
       <c r="M201" t="n">
         <v>300679</v>
       </c>
@@ -40021,9 +42008,1102 @@
       <c r="P201" t="n">
         <v>1</v>
       </c>
-      <c r="Q201" t="inlineStr"/>
-      <c r="R201" t="inlineStr"/>
-      <c r="S201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>14</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>429</v>
+      </c>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="n">
+        <v>257</v>
+      </c>
+      <c r="N202" t="n">
+        <v>0</v>
+      </c>
+      <c r="O202" t="n">
+        <v>0</v>
+      </c>
+      <c r="P202" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q202" t="inlineStr"/>
+      <c r="R202" t="inlineStr"/>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>14</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>200</v>
+      </c>
+      <c r="J203" t="n">
+        <v>292</v>
+      </c>
+      <c r="K203" t="n">
+        <v>926</v>
+      </c>
+      <c r="L203" t="n">
+        <v>1218</v>
+      </c>
+      <c r="M203" t="n">
+        <v>14893</v>
+      </c>
+      <c r="N203" t="n">
+        <v>3653</v>
+      </c>
+      <c r="O203" t="n">
+        <v>512</v>
+      </c>
+      <c r="P203" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr"/>
+      <c r="S203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>14</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>429</v>
+      </c>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr"/>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="n">
+        <v>228</v>
+      </c>
+      <c r="N204" t="n">
+        <v>0</v>
+      </c>
+      <c r="O204" t="n">
+        <v>0</v>
+      </c>
+      <c r="P204" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q204" t="inlineStr"/>
+      <c r="R204" t="inlineStr"/>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>14</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>429</v>
+      </c>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr"/>
+      <c r="L205" t="inlineStr"/>
+      <c r="M205" t="n">
+        <v>276</v>
+      </c>
+      <c r="N205" t="n">
+        <v>0</v>
+      </c>
+      <c r="O205" t="n">
+        <v>0</v>
+      </c>
+      <c r="P205" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q205" t="inlineStr"/>
+      <c r="R205" t="inlineStr"/>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>14</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>200</v>
+      </c>
+      <c r="J206" t="n">
+        <v>292</v>
+      </c>
+      <c r="K206" t="n">
+        <v>612</v>
+      </c>
+      <c r="L206" t="n">
+        <v>904</v>
+      </c>
+      <c r="M206" t="n">
+        <v>37843</v>
+      </c>
+      <c r="N206" t="n">
+        <v>2750</v>
+      </c>
+      <c r="O206" t="n">
+        <v>396</v>
+      </c>
+      <c r="P206" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr"/>
+      <c r="S206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>14</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>200</v>
+      </c>
+      <c r="J207" t="n">
+        <v>292</v>
+      </c>
+      <c r="K207" t="n">
+        <v>841</v>
+      </c>
+      <c r="L207" t="n">
+        <v>1133</v>
+      </c>
+      <c r="M207" t="n">
+        <v>7214</v>
+      </c>
+      <c r="N207" t="n">
+        <v>3760</v>
+      </c>
+      <c r="O207" t="n">
+        <v>506</v>
+      </c>
+      <c r="P207" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr"/>
+      <c r="S207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>14</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>200</v>
+      </c>
+      <c r="J208" t="n">
+        <v>256</v>
+      </c>
+      <c r="K208" t="n">
+        <v>1034</v>
+      </c>
+      <c r="L208" t="n">
+        <v>1290</v>
+      </c>
+      <c r="M208" t="n">
+        <v>7413</v>
+      </c>
+      <c r="N208" t="n">
+        <v>5228</v>
+      </c>
+      <c r="O208" t="n">
+        <v>735</v>
+      </c>
+      <c r="P208" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr"/>
+      <c r="S208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>14</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>429</v>
+      </c>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="n">
+        <v>259</v>
+      </c>
+      <c r="N209" t="n">
+        <v>0</v>
+      </c>
+      <c r="O209" t="n">
+        <v>0</v>
+      </c>
+      <c r="P209" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q209" t="inlineStr"/>
+      <c r="R209" t="inlineStr"/>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>14</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>429</v>
+      </c>
+      <c r="J210" t="inlineStr"/>
+      <c r="K210" t="inlineStr"/>
+      <c r="L210" t="inlineStr"/>
+      <c r="M210" t="n">
+        <v>362</v>
+      </c>
+      <c r="N210" t="n">
+        <v>0</v>
+      </c>
+      <c r="O210" t="n">
+        <v>0</v>
+      </c>
+      <c r="P210" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q210" t="inlineStr"/>
+      <c r="R210" t="inlineStr"/>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>14</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>200</v>
+      </c>
+      <c r="J211" t="n">
+        <v>330</v>
+      </c>
+      <c r="K211" t="n">
+        <v>1013</v>
+      </c>
+      <c r="L211" t="n">
+        <v>1343</v>
+      </c>
+      <c r="M211" t="n">
+        <v>35513</v>
+      </c>
+      <c r="N211" t="n">
+        <v>5001</v>
+      </c>
+      <c r="O211" t="n">
+        <v>723</v>
+      </c>
+      <c r="P211" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr"/>
+      <c r="S211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>14</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>200</v>
+      </c>
+      <c r="J212" t="n">
+        <v>277</v>
+      </c>
+      <c r="K212" t="n">
+        <v>449</v>
+      </c>
+      <c r="L212" t="n">
+        <v>726</v>
+      </c>
+      <c r="M212" t="n">
+        <v>15863</v>
+      </c>
+      <c r="N212" t="n">
+        <v>2353</v>
+      </c>
+      <c r="O212" t="n">
+        <v>361</v>
+      </c>
+      <c r="P212" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr"/>
+      <c r="S212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>14</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>200</v>
+      </c>
+      <c r="J213" t="n">
+        <v>332</v>
+      </c>
+      <c r="K213" t="n">
+        <v>578</v>
+      </c>
+      <c r="L213" t="n">
+        <v>910</v>
+      </c>
+      <c r="M213" t="n">
+        <v>11916</v>
+      </c>
+      <c r="N213" t="n">
+        <v>2162</v>
+      </c>
+      <c r="O213" t="n">
+        <v>298</v>
+      </c>
+      <c r="P213" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr"/>
+      <c r="S213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>14</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>200</v>
+      </c>
+      <c r="J214" t="n">
+        <v>295</v>
+      </c>
+      <c r="K214" t="n">
+        <v>927</v>
+      </c>
+      <c r="L214" t="n">
+        <v>1222</v>
+      </c>
+      <c r="M214" t="n">
+        <v>22826</v>
+      </c>
+      <c r="N214" t="n">
+        <v>2875</v>
+      </c>
+      <c r="O214" t="n">
+        <v>406</v>
+      </c>
+      <c r="P214" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr"/>
+      <c r="S214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>14</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>200</v>
+      </c>
+      <c r="J215" t="n">
+        <v>332</v>
+      </c>
+      <c r="K215" t="n">
+        <v>742</v>
+      </c>
+      <c r="L215" t="n">
+        <v>1074</v>
+      </c>
+      <c r="M215" t="n">
+        <v>20197</v>
+      </c>
+      <c r="N215" t="n">
+        <v>3089</v>
+      </c>
+      <c r="O215" t="n">
+        <v>478</v>
+      </c>
+      <c r="P215" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr"/>
+      <c r="S215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>14</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>200</v>
+      </c>
+      <c r="J216" t="n">
+        <v>288</v>
+      </c>
+      <c r="K216" t="n">
+        <v>1610</v>
+      </c>
+      <c r="L216" t="n">
+        <v>1898</v>
+      </c>
+      <c r="M216" t="n">
+        <v>32122</v>
+      </c>
+      <c r="N216" t="n">
+        <v>5154</v>
+      </c>
+      <c r="O216" t="n">
+        <v>728</v>
+      </c>
+      <c r="P216" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>responses/20260707T162941Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr"/>
+      <c r="S216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>20260707T162941Z</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:29:41.328113+00:00</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>14</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>200</v>
+      </c>
+      <c r="J217" t="inlineStr"/>
+      <c r="K217" t="inlineStr"/>
+      <c r="L217" t="inlineStr"/>
+      <c r="M217" t="n">
+        <v>120537</v>
+      </c>
+      <c r="N217" t="n">
+        <v>0</v>
+      </c>
+      <c r="O217" t="n">
+        <v>0</v>
+      </c>
+      <c r="P217" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q217" t="inlineStr"/>
+      <c r="R217" t="inlineStr"/>
+      <c r="S217" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-08 21:11 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S217"/>
+  <dimension ref="A1:S233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13579,9 +13579,6 @@
       <c r="I202" t="n">
         <v>429</v>
       </c>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr"/>
       <c r="M202" t="n">
         <v>208</v>
       </c>
@@ -13594,8 +13591,6 @@
       <c r="P202" t="n">
         <v>3</v>
       </c>
-      <c r="Q202" t="inlineStr"/>
-      <c r="R202" t="inlineStr"/>
       <c r="S202" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -13644,9 +13639,6 @@
       <c r="I203" t="n">
         <v>429</v>
       </c>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr"/>
       <c r="M203" t="n">
         <v>237</v>
       </c>
@@ -13659,8 +13651,6 @@
       <c r="P203" t="n">
         <v>3</v>
       </c>
-      <c r="Q203" t="inlineStr"/>
-      <c r="R203" t="inlineStr"/>
       <c r="S203" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -13709,9 +13699,6 @@
       <c r="I204" t="n">
         <v>429</v>
       </c>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
       <c r="M204" t="n">
         <v>235</v>
       </c>
@@ -13724,8 +13711,6 @@
       <c r="P204" t="n">
         <v>3</v>
       </c>
-      <c r="Q204" t="inlineStr"/>
-      <c r="R204" t="inlineStr"/>
       <c r="S204" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -13774,9 +13759,6 @@
       <c r="I205" t="n">
         <v>429</v>
       </c>
-      <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr"/>
       <c r="M205" t="n">
         <v>423</v>
       </c>
@@ -13789,8 +13771,6 @@
       <c r="P205" t="n">
         <v>3</v>
       </c>
-      <c r="Q205" t="inlineStr"/>
-      <c r="R205" t="inlineStr"/>
       <c r="S205" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -13839,9 +13819,6 @@
       <c r="I206" t="n">
         <v>429</v>
       </c>
-      <c r="J206" t="inlineStr"/>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
       <c r="M206" t="n">
         <v>257</v>
       </c>
@@ -13854,8 +13831,6 @@
       <c r="P206" t="n">
         <v>3</v>
       </c>
-      <c r="Q206" t="inlineStr"/>
-      <c r="R206" t="inlineStr"/>
       <c r="S206" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -13904,9 +13879,6 @@
       <c r="I207" t="n">
         <v>429</v>
       </c>
-      <c r="J207" t="inlineStr"/>
-      <c r="K207" t="inlineStr"/>
-      <c r="L207" t="inlineStr"/>
       <c r="M207" t="n">
         <v>437</v>
       </c>
@@ -13919,8 +13891,6 @@
       <c r="P207" t="n">
         <v>3</v>
       </c>
-      <c r="Q207" t="inlineStr"/>
-      <c r="R207" t="inlineStr"/>
       <c r="S207" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -13969,9 +13939,6 @@
       <c r="I208" t="n">
         <v>429</v>
       </c>
-      <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="inlineStr"/>
       <c r="M208" t="n">
         <v>407</v>
       </c>
@@ -13984,8 +13951,6 @@
       <c r="P208" t="n">
         <v>3</v>
       </c>
-      <c r="Q208" t="inlineStr"/>
-      <c r="R208" t="inlineStr"/>
       <c r="S208" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -14055,9 +14020,6 @@
       <c r="P209" t="n">
         <v>1</v>
       </c>
-      <c r="Q209" t="inlineStr"/>
-      <c r="R209" t="inlineStr"/>
-      <c r="S209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -14127,8 +14089,6 @@
           <t>responses/20260707T162941Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R210" t="inlineStr"/>
-      <c r="S210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -14198,8 +14158,6 @@
           <t>responses/20260707T162941Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R211" t="inlineStr"/>
-      <c r="S211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -14269,8 +14227,6 @@
           <t>responses/20260707T162941Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R212" t="inlineStr"/>
-      <c r="S212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -14340,8 +14296,6 @@
           <t>responses/20260707T162941Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R213" t="inlineStr"/>
-      <c r="S213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -14411,8 +14365,6 @@
           <t>responses/20260707T162941Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R214" t="inlineStr"/>
-      <c r="S214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -14477,9 +14429,6 @@
       <c r="P215" t="n">
         <v>1</v>
       </c>
-      <c r="Q215" t="inlineStr"/>
-      <c r="R215" t="inlineStr"/>
-      <c r="S215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -14544,9 +14493,6 @@
       <c r="P216" t="n">
         <v>1</v>
       </c>
-      <c r="Q216" t="inlineStr"/>
-      <c r="R216" t="inlineStr"/>
-      <c r="S216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -14616,8 +14562,1092 @@
           <t>responses/20260707T162941Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R217" t="inlineStr"/>
-      <c r="S217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>15</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>429</v>
+      </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="inlineStr"/>
+      <c r="M218" t="n">
+        <v>282</v>
+      </c>
+      <c r="N218" t="n">
+        <v>0</v>
+      </c>
+      <c r="O218" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q218" t="inlineStr"/>
+      <c r="R218" t="inlineStr"/>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>15</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>429</v>
+      </c>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr"/>
+      <c r="L219" t="inlineStr"/>
+      <c r="M219" t="n">
+        <v>275</v>
+      </c>
+      <c r="N219" t="n">
+        <v>0</v>
+      </c>
+      <c r="O219" t="n">
+        <v>0</v>
+      </c>
+      <c r="P219" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q219" t="inlineStr"/>
+      <c r="R219" t="inlineStr"/>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>15</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>429</v>
+      </c>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr"/>
+      <c r="L220" t="inlineStr"/>
+      <c r="M220" t="n">
+        <v>255</v>
+      </c>
+      <c r="N220" t="n">
+        <v>0</v>
+      </c>
+      <c r="O220" t="n">
+        <v>0</v>
+      </c>
+      <c r="P220" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q220" t="inlineStr"/>
+      <c r="R220" t="inlineStr"/>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>15</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>429</v>
+      </c>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="inlineStr"/>
+      <c r="M221" t="n">
+        <v>359</v>
+      </c>
+      <c r="N221" t="n">
+        <v>0</v>
+      </c>
+      <c r="O221" t="n">
+        <v>0</v>
+      </c>
+      <c r="P221" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q221" t="inlineStr"/>
+      <c r="R221" t="inlineStr"/>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>15</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>429</v>
+      </c>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr"/>
+      <c r="L222" t="inlineStr"/>
+      <c r="M222" t="n">
+        <v>276</v>
+      </c>
+      <c r="N222" t="n">
+        <v>0</v>
+      </c>
+      <c r="O222" t="n">
+        <v>0</v>
+      </c>
+      <c r="P222" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q222" t="inlineStr"/>
+      <c r="R222" t="inlineStr"/>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>15</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>429</v>
+      </c>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="inlineStr"/>
+      <c r="M223" t="n">
+        <v>458</v>
+      </c>
+      <c r="N223" t="n">
+        <v>0</v>
+      </c>
+      <c r="O223" t="n">
+        <v>0</v>
+      </c>
+      <c r="P223" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q223" t="inlineStr"/>
+      <c r="R223" t="inlineStr"/>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>15</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>429</v>
+      </c>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr"/>
+      <c r="L224" t="inlineStr"/>
+      <c r="M224" t="n">
+        <v>799</v>
+      </c>
+      <c r="N224" t="n">
+        <v>0</v>
+      </c>
+      <c r="O224" t="n">
+        <v>0</v>
+      </c>
+      <c r="P224" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q224" t="inlineStr"/>
+      <c r="R224" t="inlineStr"/>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>15</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>200</v>
+      </c>
+      <c r="J225" t="n">
+        <v>66</v>
+      </c>
+      <c r="K225" t="n">
+        <v>5992</v>
+      </c>
+      <c r="L225" t="n">
+        <v>6058</v>
+      </c>
+      <c r="M225" t="n">
+        <v>23371</v>
+      </c>
+      <c r="N225" t="n">
+        <v>28131</v>
+      </c>
+      <c r="O225" t="n">
+        <v>3121</v>
+      </c>
+      <c r="P225" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr"/>
+      <c r="S225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>15</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>200</v>
+      </c>
+      <c r="J226" t="n">
+        <v>88</v>
+      </c>
+      <c r="K226" t="n">
+        <v>4622</v>
+      </c>
+      <c r="L226" t="n">
+        <v>4710</v>
+      </c>
+      <c r="M226" t="n">
+        <v>26669</v>
+      </c>
+      <c r="N226" t="n">
+        <v>19539</v>
+      </c>
+      <c r="O226" t="n">
+        <v>2277</v>
+      </c>
+      <c r="P226" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr"/>
+      <c r="S226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>15</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>200</v>
+      </c>
+      <c r="J227" t="n">
+        <v>88</v>
+      </c>
+      <c r="K227" t="n">
+        <v>4950</v>
+      </c>
+      <c r="L227" t="n">
+        <v>5038</v>
+      </c>
+      <c r="M227" t="n">
+        <v>44433</v>
+      </c>
+      <c r="N227" t="n">
+        <v>17566</v>
+      </c>
+      <c r="O227" t="n">
+        <v>2011</v>
+      </c>
+      <c r="P227" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr"/>
+      <c r="S227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>15</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>200</v>
+      </c>
+      <c r="J228" t="n">
+        <v>118</v>
+      </c>
+      <c r="K228" t="n">
+        <v>5106</v>
+      </c>
+      <c r="L228" t="n">
+        <v>5224</v>
+      </c>
+      <c r="M228" t="n">
+        <v>39263</v>
+      </c>
+      <c r="N228" t="n">
+        <v>21243</v>
+      </c>
+      <c r="O228" t="n">
+        <v>1942</v>
+      </c>
+      <c r="P228" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr"/>
+      <c r="S228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>15</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I229" t="n">
+        <v>200</v>
+      </c>
+      <c r="J229" t="n">
+        <v>86</v>
+      </c>
+      <c r="K229" t="n">
+        <v>1555</v>
+      </c>
+      <c r="L229" t="n">
+        <v>1641</v>
+      </c>
+      <c r="M229" t="n">
+        <v>52748</v>
+      </c>
+      <c r="N229" t="n">
+        <v>7055</v>
+      </c>
+      <c r="O229" t="n">
+        <v>667</v>
+      </c>
+      <c r="P229" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr"/>
+      <c r="S229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>15</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I230" t="n">
+        <v>200</v>
+      </c>
+      <c r="J230" t="n">
+        <v>139</v>
+      </c>
+      <c r="K230" t="n">
+        <v>4241</v>
+      </c>
+      <c r="L230" t="n">
+        <v>4380</v>
+      </c>
+      <c r="M230" t="n">
+        <v>65977</v>
+      </c>
+      <c r="N230" t="n">
+        <v>17118</v>
+      </c>
+      <c r="O230" t="n">
+        <v>1817</v>
+      </c>
+      <c r="P230" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr"/>
+      <c r="S230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>15</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I231" t="n">
+        <v>200</v>
+      </c>
+      <c r="J231" t="n">
+        <v>81</v>
+      </c>
+      <c r="K231" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L231" t="n">
+        <v>6081</v>
+      </c>
+      <c r="M231" t="n">
+        <v>120442</v>
+      </c>
+      <c r="N231" t="n">
+        <v>0</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0</v>
+      </c>
+      <c r="P231" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q231" t="inlineStr"/>
+      <c r="R231" t="inlineStr"/>
+      <c r="S231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>15</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I232" t="n">
+        <v>200</v>
+      </c>
+      <c r="J232" t="n">
+        <v>84</v>
+      </c>
+      <c r="K232" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L232" t="n">
+        <v>6084</v>
+      </c>
+      <c r="M232" t="n">
+        <v>151179</v>
+      </c>
+      <c r="N232" t="n">
+        <v>0</v>
+      </c>
+      <c r="O232" t="n">
+        <v>0</v>
+      </c>
+      <c r="P232" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q232" t="inlineStr"/>
+      <c r="R232" t="inlineStr"/>
+      <c r="S232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>15</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I233" t="n">
+        <v>200</v>
+      </c>
+      <c r="J233" t="n">
+        <v>88</v>
+      </c>
+      <c r="K233" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L233" t="n">
+        <v>6088</v>
+      </c>
+      <c r="M233" t="n">
+        <v>338723</v>
+      </c>
+      <c r="N233" t="n">
+        <v>24776</v>
+      </c>
+      <c r="O233" t="n">
+        <v>2502</v>
+      </c>
+      <c r="P233" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr"/>
+      <c r="S233" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14630,7 +15660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S217"/>
+  <dimension ref="A1:S233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27865,9 +28895,6 @@
       <c r="I202" t="n">
         <v>200</v>
       </c>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr"/>
       <c r="M202" t="n">
         <v>510</v>
       </c>
@@ -27880,9 +28907,6 @@
       <c r="P202" t="n">
         <v>1</v>
       </c>
-      <c r="Q202" t="inlineStr"/>
-      <c r="R202" t="inlineStr"/>
-      <c r="S202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -27926,9 +28950,6 @@
       <c r="I203" t="n">
         <v>429</v>
       </c>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr"/>
       <c r="M203" t="n">
         <v>245</v>
       </c>
@@ -27941,8 +28962,6 @@
       <c r="P203" t="n">
         <v>3</v>
       </c>
-      <c r="Q203" t="inlineStr"/>
-      <c r="R203" t="inlineStr"/>
       <c r="S203" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -27991,9 +29010,6 @@
       <c r="I204" t="n">
         <v>429</v>
       </c>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
       <c r="M204" t="n">
         <v>519</v>
       </c>
@@ -28006,8 +29022,6 @@
       <c r="P204" t="n">
         <v>3</v>
       </c>
-      <c r="Q204" t="inlineStr"/>
-      <c r="R204" t="inlineStr"/>
       <c r="S204" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -28056,9 +29070,6 @@
       <c r="I205" t="n">
         <v>429</v>
       </c>
-      <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr"/>
       <c r="M205" t="n">
         <v>240</v>
       </c>
@@ -28071,8 +29082,6 @@
       <c r="P205" t="n">
         <v>3</v>
       </c>
-      <c r="Q205" t="inlineStr"/>
-      <c r="R205" t="inlineStr"/>
       <c r="S205" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -28121,9 +29130,6 @@
       <c r="I206" t="n">
         <v>429</v>
       </c>
-      <c r="J206" t="inlineStr"/>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
       <c r="M206" t="n">
         <v>233</v>
       </c>
@@ -28136,8 +29142,6 @@
       <c r="P206" t="n">
         <v>3</v>
       </c>
-      <c r="Q206" t="inlineStr"/>
-      <c r="R206" t="inlineStr"/>
       <c r="S206" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -28186,9 +29190,6 @@
       <c r="I207" t="n">
         <v>429</v>
       </c>
-      <c r="J207" t="inlineStr"/>
-      <c r="K207" t="inlineStr"/>
-      <c r="L207" t="inlineStr"/>
       <c r="M207" t="n">
         <v>271</v>
       </c>
@@ -28201,8 +29202,6 @@
       <c r="P207" t="n">
         <v>3</v>
       </c>
-      <c r="Q207" t="inlineStr"/>
-      <c r="R207" t="inlineStr"/>
       <c r="S207" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -28251,9 +29250,6 @@
       <c r="I208" t="n">
         <v>429</v>
       </c>
-      <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="inlineStr"/>
       <c r="M208" t="n">
         <v>637</v>
       </c>
@@ -28266,8 +29262,6 @@
       <c r="P208" t="n">
         <v>3</v>
       </c>
-      <c r="Q208" t="inlineStr"/>
-      <c r="R208" t="inlineStr"/>
       <c r="S208" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -28316,9 +29310,6 @@
       <c r="I209" t="n">
         <v>429</v>
       </c>
-      <c r="J209" t="inlineStr"/>
-      <c r="K209" t="inlineStr"/>
-      <c r="L209" t="inlineStr"/>
       <c r="M209" t="n">
         <v>222</v>
       </c>
@@ -28331,8 +29322,6 @@
       <c r="P209" t="n">
         <v>3</v>
       </c>
-      <c r="Q209" t="inlineStr"/>
-      <c r="R209" t="inlineStr"/>
       <c r="S209" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -28407,8 +29396,6 @@
           <t>responses/20260707T162941Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R210" t="inlineStr"/>
-      <c r="S210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -28478,8 +29465,6 @@
           <t>responses/20260707T162941Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R211" t="inlineStr"/>
-      <c r="S211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -28549,8 +29534,6 @@
           <t>responses/20260707T162941Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R212" t="inlineStr"/>
-      <c r="S212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -28620,8 +29603,6 @@
           <t>responses/20260707T162941Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R213" t="inlineStr"/>
-      <c r="S213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -28662,11 +29643,6 @@
           <t>error</t>
         </is>
       </c>
-      <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr"/>
-      <c r="K214" t="inlineStr"/>
-      <c r="L214" t="inlineStr"/>
-      <c r="M214" t="inlineStr"/>
       <c r="N214" t="n">
         <v>0</v>
       </c>
@@ -28676,8 +29652,6 @@
       <c r="P214" t="n">
         <v>3</v>
       </c>
-      <c r="Q214" t="inlineStr"/>
-      <c r="R214" t="inlineStr"/>
       <c r="S214" t="inlineStr">
         <is>
           <t>JSONDecodeError: Expecting value: line 123 column 1 (char 671)</t>
@@ -28752,8 +29726,6 @@
           <t>responses/20260707T162941Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R215" t="inlineStr"/>
-      <c r="S215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -28823,8 +29795,6 @@
           <t>responses/20260707T162941Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R216" t="inlineStr"/>
-      <c r="S216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -28894,8 +29864,1090 @@
           <t>responses/20260707T162941Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R217" t="inlineStr"/>
-      <c r="S217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>15</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>429</v>
+      </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="inlineStr"/>
+      <c r="M218" t="n">
+        <v>345</v>
+      </c>
+      <c r="N218" t="n">
+        <v>0</v>
+      </c>
+      <c r="O218" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q218" t="inlineStr"/>
+      <c r="R218" t="inlineStr"/>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>15</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>429</v>
+      </c>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr"/>
+      <c r="L219" t="inlineStr"/>
+      <c r="M219" t="n">
+        <v>1255</v>
+      </c>
+      <c r="N219" t="n">
+        <v>0</v>
+      </c>
+      <c r="O219" t="n">
+        <v>0</v>
+      </c>
+      <c r="P219" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q219" t="inlineStr"/>
+      <c r="R219" t="inlineStr"/>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>15</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>429</v>
+      </c>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr"/>
+      <c r="L220" t="inlineStr"/>
+      <c r="M220" t="n">
+        <v>369</v>
+      </c>
+      <c r="N220" t="n">
+        <v>0</v>
+      </c>
+      <c r="O220" t="n">
+        <v>0</v>
+      </c>
+      <c r="P220" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q220" t="inlineStr"/>
+      <c r="R220" t="inlineStr"/>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>15</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>429</v>
+      </c>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="inlineStr"/>
+      <c r="M221" t="n">
+        <v>345</v>
+      </c>
+      <c r="N221" t="n">
+        <v>0</v>
+      </c>
+      <c r="O221" t="n">
+        <v>0</v>
+      </c>
+      <c r="P221" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q221" t="inlineStr"/>
+      <c r="R221" t="inlineStr"/>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>15</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>429</v>
+      </c>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr"/>
+      <c r="L222" t="inlineStr"/>
+      <c r="M222" t="n">
+        <v>245</v>
+      </c>
+      <c r="N222" t="n">
+        <v>0</v>
+      </c>
+      <c r="O222" t="n">
+        <v>0</v>
+      </c>
+      <c r="P222" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q222" t="inlineStr"/>
+      <c r="R222" t="inlineStr"/>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>15</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>429</v>
+      </c>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="inlineStr"/>
+      <c r="M223" t="n">
+        <v>462</v>
+      </c>
+      <c r="N223" t="n">
+        <v>0</v>
+      </c>
+      <c r="O223" t="n">
+        <v>0</v>
+      </c>
+      <c r="P223" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q223" t="inlineStr"/>
+      <c r="R223" t="inlineStr"/>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>15</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>429</v>
+      </c>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr"/>
+      <c r="L224" t="inlineStr"/>
+      <c r="M224" t="n">
+        <v>576</v>
+      </c>
+      <c r="N224" t="n">
+        <v>0</v>
+      </c>
+      <c r="O224" t="n">
+        <v>0</v>
+      </c>
+      <c r="P224" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q224" t="inlineStr"/>
+      <c r="R224" t="inlineStr"/>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>15</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>200</v>
+      </c>
+      <c r="J225" t="n">
+        <v>51</v>
+      </c>
+      <c r="K225" t="n">
+        <v>3914</v>
+      </c>
+      <c r="L225" t="n">
+        <v>3965</v>
+      </c>
+      <c r="M225" t="n">
+        <v>21874</v>
+      </c>
+      <c r="N225" t="n">
+        <v>13166</v>
+      </c>
+      <c r="O225" t="n">
+        <v>1874</v>
+      </c>
+      <c r="P225" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr"/>
+      <c r="S225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>15</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>200</v>
+      </c>
+      <c r="J226" t="n">
+        <v>73</v>
+      </c>
+      <c r="K226" t="n">
+        <v>6938</v>
+      </c>
+      <c r="L226" t="n">
+        <v>7011</v>
+      </c>
+      <c r="M226" t="n">
+        <v>29331</v>
+      </c>
+      <c r="N226" t="n">
+        <v>17282</v>
+      </c>
+      <c r="O226" t="n">
+        <v>2354</v>
+      </c>
+      <c r="P226" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr"/>
+      <c r="S226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>15</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>200</v>
+      </c>
+      <c r="J227" t="n">
+        <v>69</v>
+      </c>
+      <c r="K227" t="n">
+        <v>2846</v>
+      </c>
+      <c r="L227" t="n">
+        <v>2915</v>
+      </c>
+      <c r="M227" t="n">
+        <v>58645</v>
+      </c>
+      <c r="N227" t="n">
+        <v>9682</v>
+      </c>
+      <c r="O227" t="n">
+        <v>1306</v>
+      </c>
+      <c r="P227" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr"/>
+      <c r="S227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>15</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>200</v>
+      </c>
+      <c r="J228" t="n">
+        <v>106</v>
+      </c>
+      <c r="K228" t="n">
+        <v>3926</v>
+      </c>
+      <c r="L228" t="n">
+        <v>4032</v>
+      </c>
+      <c r="M228" t="n">
+        <v>52200</v>
+      </c>
+      <c r="N228" t="n">
+        <v>20050</v>
+      </c>
+      <c r="O228" t="n">
+        <v>2662</v>
+      </c>
+      <c r="P228" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr"/>
+      <c r="S228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>15</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I229" t="n">
+        <v>200</v>
+      </c>
+      <c r="J229" t="n">
+        <v>73</v>
+      </c>
+      <c r="K229" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L229" t="n">
+        <v>8073</v>
+      </c>
+      <c r="M229" t="n">
+        <v>99058</v>
+      </c>
+      <c r="N229" t="n">
+        <v>31339</v>
+      </c>
+      <c r="O229" t="n">
+        <v>4325</v>
+      </c>
+      <c r="P229" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr"/>
+      <c r="S229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>15</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I230" t="n">
+        <v>200</v>
+      </c>
+      <c r="J230" t="n">
+        <v>122</v>
+      </c>
+      <c r="K230" t="n">
+        <v>4217</v>
+      </c>
+      <c r="L230" t="n">
+        <v>4339</v>
+      </c>
+      <c r="M230" t="n">
+        <v>62143</v>
+      </c>
+      <c r="N230" t="n">
+        <v>16651</v>
+      </c>
+      <c r="O230" t="n">
+        <v>2508</v>
+      </c>
+      <c r="P230" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr"/>
+      <c r="S230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>15</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I231" t="n">
+        <v>200</v>
+      </c>
+      <c r="J231" t="n">
+        <v>71</v>
+      </c>
+      <c r="K231" t="n">
+        <v>2273</v>
+      </c>
+      <c r="L231" t="n">
+        <v>2344</v>
+      </c>
+      <c r="M231" t="n">
+        <v>50343</v>
+      </c>
+      <c r="N231" t="n">
+        <v>9347</v>
+      </c>
+      <c r="O231" t="n">
+        <v>1339</v>
+      </c>
+      <c r="P231" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr"/>
+      <c r="S231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>15</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr"/>
+      <c r="J232" t="inlineStr"/>
+      <c r="K232" t="inlineStr"/>
+      <c r="L232" t="inlineStr"/>
+      <c r="M232" t="inlineStr"/>
+      <c r="N232" t="n">
+        <v>0</v>
+      </c>
+      <c r="O232" t="n">
+        <v>0</v>
+      </c>
+      <c r="P232" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q232" t="inlineStr"/>
+      <c r="R232" t="inlineStr"/>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>ChunkedEncodingError: Response ended prematurely</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>15</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I233" t="n">
+        <v>200</v>
+      </c>
+      <c r="J233" t="n">
+        <v>69</v>
+      </c>
+      <c r="K233" t="n">
+        <v>4876</v>
+      </c>
+      <c r="L233" t="n">
+        <v>4945</v>
+      </c>
+      <c r="M233" t="n">
+        <v>96698</v>
+      </c>
+      <c r="N233" t="n">
+        <v>15840</v>
+      </c>
+      <c r="O233" t="n">
+        <v>2451</v>
+      </c>
+      <c r="P233" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr"/>
+      <c r="S233" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28908,7 +30960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S217"/>
+  <dimension ref="A1:S233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42051,9 +44103,6 @@
       <c r="I202" t="n">
         <v>429</v>
       </c>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr"/>
       <c r="M202" t="n">
         <v>257</v>
       </c>
@@ -42066,8 +44115,6 @@
       <c r="P202" t="n">
         <v>3</v>
       </c>
-      <c r="Q202" t="inlineStr"/>
-      <c r="R202" t="inlineStr"/>
       <c r="S202" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -42142,8 +44189,6 @@
           <t>responses/20260707T162941Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R203" t="inlineStr"/>
-      <c r="S203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -42187,9 +44232,6 @@
       <c r="I204" t="n">
         <v>429</v>
       </c>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
       <c r="M204" t="n">
         <v>228</v>
       </c>
@@ -42202,8 +44244,6 @@
       <c r="P204" t="n">
         <v>3</v>
       </c>
-      <c r="Q204" t="inlineStr"/>
-      <c r="R204" t="inlineStr"/>
       <c r="S204" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -42252,9 +44292,6 @@
       <c r="I205" t="n">
         <v>429</v>
       </c>
-      <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr"/>
       <c r="M205" t="n">
         <v>276</v>
       </c>
@@ -42267,8 +44304,6 @@
       <c r="P205" t="n">
         <v>3</v>
       </c>
-      <c r="Q205" t="inlineStr"/>
-      <c r="R205" t="inlineStr"/>
       <c r="S205" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -42343,8 +44378,6 @@
           <t>responses/20260707T162941Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R206" t="inlineStr"/>
-      <c r="S206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -42414,8 +44447,6 @@
           <t>responses/20260707T162941Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R207" t="inlineStr"/>
-      <c r="S207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -42485,8 +44516,6 @@
           <t>responses/20260707T162941Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R208" t="inlineStr"/>
-      <c r="S208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -42530,9 +44559,6 @@
       <c r="I209" t="n">
         <v>429</v>
       </c>
-      <c r="J209" t="inlineStr"/>
-      <c r="K209" t="inlineStr"/>
-      <c r="L209" t="inlineStr"/>
       <c r="M209" t="n">
         <v>259</v>
       </c>
@@ -42545,8 +44571,6 @@
       <c r="P209" t="n">
         <v>3</v>
       </c>
-      <c r="Q209" t="inlineStr"/>
-      <c r="R209" t="inlineStr"/>
       <c r="S209" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -42595,9 +44619,6 @@
       <c r="I210" t="n">
         <v>429</v>
       </c>
-      <c r="J210" t="inlineStr"/>
-      <c r="K210" t="inlineStr"/>
-      <c r="L210" t="inlineStr"/>
       <c r="M210" t="n">
         <v>362</v>
       </c>
@@ -42610,8 +44631,6 @@
       <c r="P210" t="n">
         <v>3</v>
       </c>
-      <c r="Q210" t="inlineStr"/>
-      <c r="R210" t="inlineStr"/>
       <c r="S210" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -42686,8 +44705,6 @@
           <t>responses/20260707T162941Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R211" t="inlineStr"/>
-      <c r="S211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -42757,8 +44774,6 @@
           <t>responses/20260707T162941Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R212" t="inlineStr"/>
-      <c r="S212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -42828,8 +44843,6 @@
           <t>responses/20260707T162941Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R213" t="inlineStr"/>
-      <c r="S213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -42899,8 +44912,6 @@
           <t>responses/20260707T162941Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R214" t="inlineStr"/>
-      <c r="S214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -42970,8 +44981,6 @@
           <t>responses/20260707T162941Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R215" t="inlineStr"/>
-      <c r="S215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -43041,8 +45050,6 @@
           <t>responses/20260707T162941Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R216" t="inlineStr"/>
-      <c r="S216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -43086,9 +45093,6 @@
       <c r="I217" t="n">
         <v>200</v>
       </c>
-      <c r="J217" t="inlineStr"/>
-      <c r="K217" t="inlineStr"/>
-      <c r="L217" t="inlineStr"/>
       <c r="M217" t="n">
         <v>120537</v>
       </c>
@@ -43101,9 +45105,1086 @@
       <c r="P217" t="n">
         <v>1</v>
       </c>
-      <c r="Q217" t="inlineStr"/>
-      <c r="R217" t="inlineStr"/>
-      <c r="S217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>15</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>200</v>
+      </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="inlineStr"/>
+      <c r="M218" t="n">
+        <v>277</v>
+      </c>
+      <c r="N218" t="n">
+        <v>0</v>
+      </c>
+      <c r="O218" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q218" t="inlineStr"/>
+      <c r="R218" t="inlineStr"/>
+      <c r="S218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>15</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>429</v>
+      </c>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr"/>
+      <c r="L219" t="inlineStr"/>
+      <c r="M219" t="n">
+        <v>257</v>
+      </c>
+      <c r="N219" t="n">
+        <v>0</v>
+      </c>
+      <c r="O219" t="n">
+        <v>0</v>
+      </c>
+      <c r="P219" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q219" t="inlineStr"/>
+      <c r="R219" t="inlineStr"/>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>15</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>429</v>
+      </c>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr"/>
+      <c r="L220" t="inlineStr"/>
+      <c r="M220" t="n">
+        <v>267</v>
+      </c>
+      <c r="N220" t="n">
+        <v>0</v>
+      </c>
+      <c r="O220" t="n">
+        <v>0</v>
+      </c>
+      <c r="P220" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q220" t="inlineStr"/>
+      <c r="R220" t="inlineStr"/>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>15</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>429</v>
+      </c>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="inlineStr"/>
+      <c r="M221" t="n">
+        <v>388</v>
+      </c>
+      <c r="N221" t="n">
+        <v>0</v>
+      </c>
+      <c r="O221" t="n">
+        <v>0</v>
+      </c>
+      <c r="P221" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q221" t="inlineStr"/>
+      <c r="R221" t="inlineStr"/>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>15</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>429</v>
+      </c>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr"/>
+      <c r="L222" t="inlineStr"/>
+      <c r="M222" t="n">
+        <v>229</v>
+      </c>
+      <c r="N222" t="n">
+        <v>0</v>
+      </c>
+      <c r="O222" t="n">
+        <v>0</v>
+      </c>
+      <c r="P222" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q222" t="inlineStr"/>
+      <c r="R222" t="inlineStr"/>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>15</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>429</v>
+      </c>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="inlineStr"/>
+      <c r="M223" t="n">
+        <v>476</v>
+      </c>
+      <c r="N223" t="n">
+        <v>0</v>
+      </c>
+      <c r="O223" t="n">
+        <v>0</v>
+      </c>
+      <c r="P223" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q223" t="inlineStr"/>
+      <c r="R223" t="inlineStr"/>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>15</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>200</v>
+      </c>
+      <c r="J224" t="n">
+        <v>292</v>
+      </c>
+      <c r="K224" t="n">
+        <v>700</v>
+      </c>
+      <c r="L224" t="n">
+        <v>992</v>
+      </c>
+      <c r="M224" t="n">
+        <v>8648</v>
+      </c>
+      <c r="N224" t="n">
+        <v>3037</v>
+      </c>
+      <c r="O224" t="n">
+        <v>419</v>
+      </c>
+      <c r="P224" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr"/>
+      <c r="S224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>15</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>200</v>
+      </c>
+      <c r="J225" t="n">
+        <v>292</v>
+      </c>
+      <c r="K225" t="n">
+        <v>741</v>
+      </c>
+      <c r="L225" t="n">
+        <v>1033</v>
+      </c>
+      <c r="M225" t="n">
+        <v>51559</v>
+      </c>
+      <c r="N225" t="n">
+        <v>2663</v>
+      </c>
+      <c r="O225" t="n">
+        <v>394</v>
+      </c>
+      <c r="P225" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr"/>
+      <c r="S225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>15</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>200</v>
+      </c>
+      <c r="J226" t="n">
+        <v>256</v>
+      </c>
+      <c r="K226" t="n">
+        <v>873</v>
+      </c>
+      <c r="L226" t="n">
+        <v>1129</v>
+      </c>
+      <c r="M226" t="n">
+        <v>12158</v>
+      </c>
+      <c r="N226" t="n">
+        <v>4411</v>
+      </c>
+      <c r="O226" t="n">
+        <v>629</v>
+      </c>
+      <c r="P226" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr"/>
+      <c r="S226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>15</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>429</v>
+      </c>
+      <c r="J227" t="inlineStr"/>
+      <c r="K227" t="inlineStr"/>
+      <c r="L227" t="inlineStr"/>
+      <c r="M227" t="n">
+        <v>280</v>
+      </c>
+      <c r="N227" t="n">
+        <v>0</v>
+      </c>
+      <c r="O227" t="n">
+        <v>0</v>
+      </c>
+      <c r="P227" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q227" t="inlineStr"/>
+      <c r="R227" t="inlineStr"/>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>15</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>200</v>
+      </c>
+      <c r="J228" t="n">
+        <v>332</v>
+      </c>
+      <c r="K228" t="n">
+        <v>689</v>
+      </c>
+      <c r="L228" t="n">
+        <v>1021</v>
+      </c>
+      <c r="M228" t="n">
+        <v>5215</v>
+      </c>
+      <c r="N228" t="n">
+        <v>2321</v>
+      </c>
+      <c r="O228" t="n">
+        <v>319</v>
+      </c>
+      <c r="P228" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr"/>
+      <c r="S228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>15</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I229" t="n">
+        <v>200</v>
+      </c>
+      <c r="J229" t="n">
+        <v>330</v>
+      </c>
+      <c r="K229" t="n">
+        <v>1015</v>
+      </c>
+      <c r="L229" t="n">
+        <v>1345</v>
+      </c>
+      <c r="M229" t="n">
+        <v>41592</v>
+      </c>
+      <c r="N229" t="n">
+        <v>4924</v>
+      </c>
+      <c r="O229" t="n">
+        <v>729</v>
+      </c>
+      <c r="P229" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr"/>
+      <c r="S229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>15</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I230" t="n">
+        <v>200</v>
+      </c>
+      <c r="J230" t="n">
+        <v>332</v>
+      </c>
+      <c r="K230" t="n">
+        <v>968</v>
+      </c>
+      <c r="L230" t="n">
+        <v>1300</v>
+      </c>
+      <c r="M230" t="n">
+        <v>16935</v>
+      </c>
+      <c r="N230" t="n">
+        <v>4380</v>
+      </c>
+      <c r="O230" t="n">
+        <v>632</v>
+      </c>
+      <c r="P230" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr"/>
+      <c r="S230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>15</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I231" t="n">
+        <v>200</v>
+      </c>
+      <c r="J231" t="n">
+        <v>295</v>
+      </c>
+      <c r="K231" t="n">
+        <v>952</v>
+      </c>
+      <c r="L231" t="n">
+        <v>1247</v>
+      </c>
+      <c r="M231" t="n">
+        <v>26407</v>
+      </c>
+      <c r="N231" t="n">
+        <v>2768</v>
+      </c>
+      <c r="O231" t="n">
+        <v>390</v>
+      </c>
+      <c r="P231" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr"/>
+      <c r="S231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>15</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I232" t="n">
+        <v>200</v>
+      </c>
+      <c r="J232" t="n">
+        <v>288</v>
+      </c>
+      <c r="K232" t="n">
+        <v>1375</v>
+      </c>
+      <c r="L232" t="n">
+        <v>1663</v>
+      </c>
+      <c r="M232" t="n">
+        <v>22071</v>
+      </c>
+      <c r="N232" t="n">
+        <v>4845</v>
+      </c>
+      <c r="O232" t="n">
+        <v>679</v>
+      </c>
+      <c r="P232" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>responses/20260708T210536Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr"/>
+      <c r="S232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>20260708T210536Z</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-07-08T21:05:36.433685+00:00</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>15</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I233" t="n">
+        <v>200</v>
+      </c>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="inlineStr"/>
+      <c r="L233" t="inlineStr"/>
+      <c r="M233" t="n">
+        <v>120550</v>
+      </c>
+      <c r="N233" t="n">
+        <v>0</v>
+      </c>
+      <c r="O233" t="n">
+        <v>0</v>
+      </c>
+      <c r="P233" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q233" t="inlineStr"/>
+      <c r="R233" t="inlineStr"/>
+      <c r="S233" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-09 08:32 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S233"/>
+  <dimension ref="A1:S249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14605,9 +14605,6 @@
       <c r="I218" t="n">
         <v>429</v>
       </c>
-      <c r="J218" t="inlineStr"/>
-      <c r="K218" t="inlineStr"/>
-      <c r="L218" t="inlineStr"/>
       <c r="M218" t="n">
         <v>282</v>
       </c>
@@ -14620,8 +14617,6 @@
       <c r="P218" t="n">
         <v>3</v>
       </c>
-      <c r="Q218" t="inlineStr"/>
-      <c r="R218" t="inlineStr"/>
       <c r="S218" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -14670,9 +14665,6 @@
       <c r="I219" t="n">
         <v>429</v>
       </c>
-      <c r="J219" t="inlineStr"/>
-      <c r="K219" t="inlineStr"/>
-      <c r="L219" t="inlineStr"/>
       <c r="M219" t="n">
         <v>275</v>
       </c>
@@ -14685,8 +14677,6 @@
       <c r="P219" t="n">
         <v>3</v>
       </c>
-      <c r="Q219" t="inlineStr"/>
-      <c r="R219" t="inlineStr"/>
       <c r="S219" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -14735,9 +14725,6 @@
       <c r="I220" t="n">
         <v>429</v>
       </c>
-      <c r="J220" t="inlineStr"/>
-      <c r="K220" t="inlineStr"/>
-      <c r="L220" t="inlineStr"/>
       <c r="M220" t="n">
         <v>255</v>
       </c>
@@ -14750,8 +14737,6 @@
       <c r="P220" t="n">
         <v>3</v>
       </c>
-      <c r="Q220" t="inlineStr"/>
-      <c r="R220" t="inlineStr"/>
       <c r="S220" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -14800,9 +14785,6 @@
       <c r="I221" t="n">
         <v>429</v>
       </c>
-      <c r="J221" t="inlineStr"/>
-      <c r="K221" t="inlineStr"/>
-      <c r="L221" t="inlineStr"/>
       <c r="M221" t="n">
         <v>359</v>
       </c>
@@ -14815,8 +14797,6 @@
       <c r="P221" t="n">
         <v>3</v>
       </c>
-      <c r="Q221" t="inlineStr"/>
-      <c r="R221" t="inlineStr"/>
       <c r="S221" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -14865,9 +14845,6 @@
       <c r="I222" t="n">
         <v>429</v>
       </c>
-      <c r="J222" t="inlineStr"/>
-      <c r="K222" t="inlineStr"/>
-      <c r="L222" t="inlineStr"/>
       <c r="M222" t="n">
         <v>276</v>
       </c>
@@ -14880,8 +14857,6 @@
       <c r="P222" t="n">
         <v>3</v>
       </c>
-      <c r="Q222" t="inlineStr"/>
-      <c r="R222" t="inlineStr"/>
       <c r="S222" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -14930,9 +14905,6 @@
       <c r="I223" t="n">
         <v>429</v>
       </c>
-      <c r="J223" t="inlineStr"/>
-      <c r="K223" t="inlineStr"/>
-      <c r="L223" t="inlineStr"/>
       <c r="M223" t="n">
         <v>458</v>
       </c>
@@ -14945,8 +14917,6 @@
       <c r="P223" t="n">
         <v>3</v>
       </c>
-      <c r="Q223" t="inlineStr"/>
-      <c r="R223" t="inlineStr"/>
       <c r="S223" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -14995,9 +14965,6 @@
       <c r="I224" t="n">
         <v>429</v>
       </c>
-      <c r="J224" t="inlineStr"/>
-      <c r="K224" t="inlineStr"/>
-      <c r="L224" t="inlineStr"/>
       <c r="M224" t="n">
         <v>799</v>
       </c>
@@ -15010,8 +14977,6 @@
       <c r="P224" t="n">
         <v>3</v>
       </c>
-      <c r="Q224" t="inlineStr"/>
-      <c r="R224" t="inlineStr"/>
       <c r="S224" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -15086,8 +15051,6 @@
           <t>responses/20260708T210536Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R225" t="inlineStr"/>
-      <c r="S225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -15157,8 +15120,6 @@
           <t>responses/20260708T210536Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R226" t="inlineStr"/>
-      <c r="S226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -15228,8 +15189,6 @@
           <t>responses/20260708T210536Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R227" t="inlineStr"/>
-      <c r="S227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -15299,8 +15258,6 @@
           <t>responses/20260708T210536Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R228" t="inlineStr"/>
-      <c r="S228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -15370,8 +15327,6 @@
           <t>responses/20260708T210536Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R229" t="inlineStr"/>
-      <c r="S229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -15441,8 +15396,6 @@
           <t>responses/20260708T210536Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R230" t="inlineStr"/>
-      <c r="S230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -15507,9 +15460,6 @@
       <c r="P231" t="n">
         <v>1</v>
       </c>
-      <c r="Q231" t="inlineStr"/>
-      <c r="R231" t="inlineStr"/>
-      <c r="S231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -15574,9 +15524,6 @@
       <c r="P232" t="n">
         <v>1</v>
       </c>
-      <c r="Q232" t="inlineStr"/>
-      <c r="R232" t="inlineStr"/>
-      <c r="S232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -15646,8 +15593,1102 @@
           <t>responses/20260708T210536Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R233" t="inlineStr"/>
-      <c r="S233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>16</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I234" t="n">
+        <v>400</v>
+      </c>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr"/>
+      <c r="L234" t="inlineStr"/>
+      <c r="M234" t="n">
+        <v>177</v>
+      </c>
+      <c r="N234" t="n">
+        <v>0</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0</v>
+      </c>
+      <c r="P234" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q234" t="inlineStr"/>
+      <c r="R234" t="inlineStr"/>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>16</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I235" t="n">
+        <v>429</v>
+      </c>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="inlineStr"/>
+      <c r="M235" t="n">
+        <v>225</v>
+      </c>
+      <c r="N235" t="n">
+        <v>0</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q235" t="inlineStr"/>
+      <c r="R235" t="inlineStr"/>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>16</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I236" t="n">
+        <v>429</v>
+      </c>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="inlineStr"/>
+      <c r="M236" t="n">
+        <v>217</v>
+      </c>
+      <c r="N236" t="n">
+        <v>0</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q236" t="inlineStr"/>
+      <c r="R236" t="inlineStr"/>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>16</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>429</v>
+      </c>
+      <c r="J237" t="inlineStr"/>
+      <c r="K237" t="inlineStr"/>
+      <c r="L237" t="inlineStr"/>
+      <c r="M237" t="n">
+        <v>233</v>
+      </c>
+      <c r="N237" t="n">
+        <v>0</v>
+      </c>
+      <c r="O237" t="n">
+        <v>0</v>
+      </c>
+      <c r="P237" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q237" t="inlineStr"/>
+      <c r="R237" t="inlineStr"/>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>16</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>429</v>
+      </c>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="inlineStr"/>
+      <c r="M238" t="n">
+        <v>231</v>
+      </c>
+      <c r="N238" t="n">
+        <v>0</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q238" t="inlineStr"/>
+      <c r="R238" t="inlineStr"/>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>16</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>429</v>
+      </c>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="inlineStr"/>
+      <c r="M239" t="n">
+        <v>393</v>
+      </c>
+      <c r="N239" t="n">
+        <v>0</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q239" t="inlineStr"/>
+      <c r="R239" t="inlineStr"/>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>16</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>200</v>
+      </c>
+      <c r="J240" t="n">
+        <v>81</v>
+      </c>
+      <c r="K240" t="n">
+        <v>4920</v>
+      </c>
+      <c r="L240" t="n">
+        <v>5001</v>
+      </c>
+      <c r="M240" t="n">
+        <v>27376</v>
+      </c>
+      <c r="N240" t="n">
+        <v>18654</v>
+      </c>
+      <c r="O240" t="n">
+        <v>2377</v>
+      </c>
+      <c r="P240" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr"/>
+      <c r="S240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>16</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>200</v>
+      </c>
+      <c r="J241" t="n">
+        <v>110</v>
+      </c>
+      <c r="K241" t="n">
+        <v>1975</v>
+      </c>
+      <c r="L241" t="n">
+        <v>2085</v>
+      </c>
+      <c r="M241" t="n">
+        <v>20011</v>
+      </c>
+      <c r="N241" t="n">
+        <v>6704</v>
+      </c>
+      <c r="O241" t="n">
+        <v>678</v>
+      </c>
+      <c r="P241" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/poolside_laguna-xs.2_free.java</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr"/>
+      <c r="S241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>16</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I242" t="n">
+        <v>200</v>
+      </c>
+      <c r="J242" t="n">
+        <v>62</v>
+      </c>
+      <c r="K242" t="n">
+        <v>1978</v>
+      </c>
+      <c r="L242" t="n">
+        <v>2040</v>
+      </c>
+      <c r="M242" t="n">
+        <v>42255</v>
+      </c>
+      <c r="N242" t="n">
+        <v>7750</v>
+      </c>
+      <c r="O242" t="n">
+        <v>851</v>
+      </c>
+      <c r="P242" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr"/>
+      <c r="S242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>16</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>200</v>
+      </c>
+      <c r="J243" t="n">
+        <v>79</v>
+      </c>
+      <c r="K243" t="n">
+        <v>1784</v>
+      </c>
+      <c r="L243" t="n">
+        <v>1863</v>
+      </c>
+      <c r="M243" t="n">
+        <v>49338</v>
+      </c>
+      <c r="N243" t="n">
+        <v>7506</v>
+      </c>
+      <c r="O243" t="n">
+        <v>779</v>
+      </c>
+      <c r="P243" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr"/>
+      <c r="S243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>16</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I244" t="n">
+        <v>200</v>
+      </c>
+      <c r="J244" t="n">
+        <v>58</v>
+      </c>
+      <c r="K244" t="n">
+        <v>5997</v>
+      </c>
+      <c r="L244" t="n">
+        <v>6055</v>
+      </c>
+      <c r="M244" t="n">
+        <v>73155</v>
+      </c>
+      <c r="N244" t="n">
+        <v>12787</v>
+      </c>
+      <c r="O244" t="n">
+        <v>1211</v>
+      </c>
+      <c r="P244" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr"/>
+      <c r="S244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>16</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>200</v>
+      </c>
+      <c r="J245" t="n">
+        <v>129</v>
+      </c>
+      <c r="K245" t="n">
+        <v>3009</v>
+      </c>
+      <c r="L245" t="n">
+        <v>3138</v>
+      </c>
+      <c r="M245" t="n">
+        <v>97462</v>
+      </c>
+      <c r="N245" t="n">
+        <v>12785</v>
+      </c>
+      <c r="O245" t="n">
+        <v>1532</v>
+      </c>
+      <c r="P245" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr"/>
+      <c r="S245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>16</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I246" t="n">
+        <v>200</v>
+      </c>
+      <c r="J246" t="n">
+        <v>73</v>
+      </c>
+      <c r="K246" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L246" t="n">
+        <v>6073</v>
+      </c>
+      <c r="M246" t="n">
+        <v>171639</v>
+      </c>
+      <c r="N246" t="n">
+        <v>0</v>
+      </c>
+      <c r="O246" t="n">
+        <v>0</v>
+      </c>
+      <c r="P246" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q246" t="inlineStr"/>
+      <c r="R246" t="inlineStr"/>
+      <c r="S246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>16</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I247" t="n">
+        <v>200</v>
+      </c>
+      <c r="J247" t="n">
+        <v>77</v>
+      </c>
+      <c r="K247" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L247" t="n">
+        <v>6077</v>
+      </c>
+      <c r="M247" t="n">
+        <v>175315</v>
+      </c>
+      <c r="N247" t="n">
+        <v>3645</v>
+      </c>
+      <c r="O247" t="n">
+        <v>394</v>
+      </c>
+      <c r="P247" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr"/>
+      <c r="S247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>16</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I248" t="n">
+        <v>200</v>
+      </c>
+      <c r="J248" t="n">
+        <v>129</v>
+      </c>
+      <c r="K248" t="n">
+        <v>4461</v>
+      </c>
+      <c r="L248" t="n">
+        <v>4590</v>
+      </c>
+      <c r="M248" t="n">
+        <v>212503</v>
+      </c>
+      <c r="N248" t="n">
+        <v>19256</v>
+      </c>
+      <c r="O248" t="n">
+        <v>2387</v>
+      </c>
+      <c r="P248" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr"/>
+      <c r="S248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>16</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Implement a thread-safe concurrent LRU cache in Java with a configurable capacit</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I249" t="n">
+        <v>200</v>
+      </c>
+      <c r="J249" t="n">
+        <v>81</v>
+      </c>
+      <c r="K249" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L249" t="n">
+        <v>6081</v>
+      </c>
+      <c r="M249" t="n">
+        <v>371190</v>
+      </c>
+      <c r="N249" t="n">
+        <v>26958</v>
+      </c>
+      <c r="O249" t="n">
+        <v>1861</v>
+      </c>
+      <c r="P249" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr"/>
+      <c r="S249" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15660,7 +16701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S233"/>
+  <dimension ref="A1:S249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29907,9 +30948,6 @@
       <c r="I218" t="n">
         <v>429</v>
       </c>
-      <c r="J218" t="inlineStr"/>
-      <c r="K218" t="inlineStr"/>
-      <c r="L218" t="inlineStr"/>
       <c r="M218" t="n">
         <v>345</v>
       </c>
@@ -29922,8 +30960,6 @@
       <c r="P218" t="n">
         <v>3</v>
       </c>
-      <c r="Q218" t="inlineStr"/>
-      <c r="R218" t="inlineStr"/>
       <c r="S218" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -29972,9 +31008,6 @@
       <c r="I219" t="n">
         <v>429</v>
       </c>
-      <c r="J219" t="inlineStr"/>
-      <c r="K219" t="inlineStr"/>
-      <c r="L219" t="inlineStr"/>
       <c r="M219" t="n">
         <v>1255</v>
       </c>
@@ -29987,8 +31020,6 @@
       <c r="P219" t="n">
         <v>3</v>
       </c>
-      <c r="Q219" t="inlineStr"/>
-      <c r="R219" t="inlineStr"/>
       <c r="S219" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -30037,9 +31068,6 @@
       <c r="I220" t="n">
         <v>429</v>
       </c>
-      <c r="J220" t="inlineStr"/>
-      <c r="K220" t="inlineStr"/>
-      <c r="L220" t="inlineStr"/>
       <c r="M220" t="n">
         <v>369</v>
       </c>
@@ -30052,8 +31080,6 @@
       <c r="P220" t="n">
         <v>3</v>
       </c>
-      <c r="Q220" t="inlineStr"/>
-      <c r="R220" t="inlineStr"/>
       <c r="S220" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -30102,9 +31128,6 @@
       <c r="I221" t="n">
         <v>429</v>
       </c>
-      <c r="J221" t="inlineStr"/>
-      <c r="K221" t="inlineStr"/>
-      <c r="L221" t="inlineStr"/>
       <c r="M221" t="n">
         <v>345</v>
       </c>
@@ -30117,8 +31140,6 @@
       <c r="P221" t="n">
         <v>3</v>
       </c>
-      <c r="Q221" t="inlineStr"/>
-      <c r="R221" t="inlineStr"/>
       <c r="S221" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -30167,9 +31188,6 @@
       <c r="I222" t="n">
         <v>429</v>
       </c>
-      <c r="J222" t="inlineStr"/>
-      <c r="K222" t="inlineStr"/>
-      <c r="L222" t="inlineStr"/>
       <c r="M222" t="n">
         <v>245</v>
       </c>
@@ -30182,8 +31200,6 @@
       <c r="P222" t="n">
         <v>3</v>
       </c>
-      <c r="Q222" t="inlineStr"/>
-      <c r="R222" t="inlineStr"/>
       <c r="S222" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -30232,9 +31248,6 @@
       <c r="I223" t="n">
         <v>429</v>
       </c>
-      <c r="J223" t="inlineStr"/>
-      <c r="K223" t="inlineStr"/>
-      <c r="L223" t="inlineStr"/>
       <c r="M223" t="n">
         <v>462</v>
       </c>
@@ -30247,8 +31260,6 @@
       <c r="P223" t="n">
         <v>3</v>
       </c>
-      <c r="Q223" t="inlineStr"/>
-      <c r="R223" t="inlineStr"/>
       <c r="S223" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -30297,9 +31308,6 @@
       <c r="I224" t="n">
         <v>429</v>
       </c>
-      <c r="J224" t="inlineStr"/>
-      <c r="K224" t="inlineStr"/>
-      <c r="L224" t="inlineStr"/>
       <c r="M224" t="n">
         <v>576</v>
       </c>
@@ -30312,8 +31320,6 @@
       <c r="P224" t="n">
         <v>3</v>
       </c>
-      <c r="Q224" t="inlineStr"/>
-      <c r="R224" t="inlineStr"/>
       <c r="S224" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -30388,8 +31394,6 @@
           <t>responses/20260708T210536Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R225" t="inlineStr"/>
-      <c r="S225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -30459,8 +31463,6 @@
           <t>responses/20260708T210536Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R226" t="inlineStr"/>
-      <c r="S226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -30530,8 +31532,6 @@
           <t>responses/20260708T210536Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R227" t="inlineStr"/>
-      <c r="S227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -30601,8 +31601,6 @@
           <t>responses/20260708T210536Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R228" t="inlineStr"/>
-      <c r="S228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -30672,8 +31670,6 @@
           <t>responses/20260708T210536Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R229" t="inlineStr"/>
-      <c r="S229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -30743,8 +31739,6 @@
           <t>responses/20260708T210536Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R230" t="inlineStr"/>
-      <c r="S230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -30814,8 +31808,6 @@
           <t>responses/20260708T210536Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R231" t="inlineStr"/>
-      <c r="S231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -30856,11 +31848,6 @@
           <t>error</t>
         </is>
       </c>
-      <c r="I232" t="inlineStr"/>
-      <c r="J232" t="inlineStr"/>
-      <c r="K232" t="inlineStr"/>
-      <c r="L232" t="inlineStr"/>
-      <c r="M232" t="inlineStr"/>
       <c r="N232" t="n">
         <v>0</v>
       </c>
@@ -30870,8 +31857,6 @@
       <c r="P232" t="n">
         <v>3</v>
       </c>
-      <c r="Q232" t="inlineStr"/>
-      <c r="R232" t="inlineStr"/>
       <c r="S232" t="inlineStr">
         <is>
           <t>ChunkedEncodingError: Response ended prematurely</t>
@@ -30946,8 +31931,1100 @@
           <t>responses/20260708T210536Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R233" t="inlineStr"/>
-      <c r="S233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>16</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I234" t="n">
+        <v>400</v>
+      </c>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr"/>
+      <c r="L234" t="inlineStr"/>
+      <c r="M234" t="n">
+        <v>123</v>
+      </c>
+      <c r="N234" t="n">
+        <v>0</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0</v>
+      </c>
+      <c r="P234" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q234" t="inlineStr"/>
+      <c r="R234" t="inlineStr"/>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>16</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I235" t="n">
+        <v>429</v>
+      </c>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="inlineStr"/>
+      <c r="M235" t="n">
+        <v>226</v>
+      </c>
+      <c r="N235" t="n">
+        <v>0</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q235" t="inlineStr"/>
+      <c r="R235" t="inlineStr"/>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>16</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I236" t="n">
+        <v>429</v>
+      </c>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="inlineStr"/>
+      <c r="M236" t="n">
+        <v>429</v>
+      </c>
+      <c r="N236" t="n">
+        <v>0</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q236" t="inlineStr"/>
+      <c r="R236" t="inlineStr"/>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>16</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>200</v>
+      </c>
+      <c r="J237" t="n">
+        <v>78</v>
+      </c>
+      <c r="K237" t="n">
+        <v>481</v>
+      </c>
+      <c r="L237" t="n">
+        <v>559</v>
+      </c>
+      <c r="M237" t="n">
+        <v>10978</v>
+      </c>
+      <c r="N237" t="n">
+        <v>1187</v>
+      </c>
+      <c r="O237" t="n">
+        <v>185</v>
+      </c>
+      <c r="P237" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr"/>
+      <c r="S237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>16</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>429</v>
+      </c>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="inlineStr"/>
+      <c r="M238" t="n">
+        <v>215</v>
+      </c>
+      <c r="N238" t="n">
+        <v>0</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q238" t="inlineStr"/>
+      <c r="R238" t="inlineStr"/>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>16</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>429</v>
+      </c>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="inlineStr"/>
+      <c r="M239" t="n">
+        <v>215</v>
+      </c>
+      <c r="N239" t="n">
+        <v>0</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q239" t="inlineStr"/>
+      <c r="R239" t="inlineStr"/>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>16</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>429</v>
+      </c>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="inlineStr"/>
+      <c r="L240" t="inlineStr"/>
+      <c r="M240" t="n">
+        <v>407</v>
+      </c>
+      <c r="N240" t="n">
+        <v>0</v>
+      </c>
+      <c r="O240" t="n">
+        <v>0</v>
+      </c>
+      <c r="P240" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q240" t="inlineStr"/>
+      <c r="R240" t="inlineStr"/>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>16</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>429</v>
+      </c>
+      <c r="J241" t="inlineStr"/>
+      <c r="K241" t="inlineStr"/>
+      <c r="L241" t="inlineStr"/>
+      <c r="M241" t="n">
+        <v>266</v>
+      </c>
+      <c r="N241" t="n">
+        <v>0</v>
+      </c>
+      <c r="O241" t="n">
+        <v>0</v>
+      </c>
+      <c r="P241" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q241" t="inlineStr"/>
+      <c r="R241" t="inlineStr"/>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>16</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I242" t="n">
+        <v>200</v>
+      </c>
+      <c r="J242" t="n">
+        <v>78</v>
+      </c>
+      <c r="K242" t="n">
+        <v>5730</v>
+      </c>
+      <c r="L242" t="n">
+        <v>5808</v>
+      </c>
+      <c r="M242" t="n">
+        <v>36810</v>
+      </c>
+      <c r="N242" t="n">
+        <v>18061</v>
+      </c>
+      <c r="O242" t="n">
+        <v>2485</v>
+      </c>
+      <c r="P242" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr"/>
+      <c r="S242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>16</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>200</v>
+      </c>
+      <c r="J243" t="n">
+        <v>54</v>
+      </c>
+      <c r="K243" t="n">
+        <v>2932</v>
+      </c>
+      <c r="L243" t="n">
+        <v>2986</v>
+      </c>
+      <c r="M243" t="n">
+        <v>41139</v>
+      </c>
+      <c r="N243" t="n">
+        <v>898</v>
+      </c>
+      <c r="O243" t="n">
+        <v>138</v>
+      </c>
+      <c r="P243" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr"/>
+      <c r="S243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>16</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I244" t="n">
+        <v>200</v>
+      </c>
+      <c r="J244" t="n">
+        <v>73</v>
+      </c>
+      <c r="K244" t="n">
+        <v>2710</v>
+      </c>
+      <c r="L244" t="n">
+        <v>2783</v>
+      </c>
+      <c r="M244" t="n">
+        <v>63581</v>
+      </c>
+      <c r="N244" t="n">
+        <v>12219</v>
+      </c>
+      <c r="O244" t="n">
+        <v>1854</v>
+      </c>
+      <c r="P244" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr"/>
+      <c r="S244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>16</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>200</v>
+      </c>
+      <c r="J245" t="n">
+        <v>112</v>
+      </c>
+      <c r="K245" t="n">
+        <v>4010</v>
+      </c>
+      <c r="L245" t="n">
+        <v>4122</v>
+      </c>
+      <c r="M245" t="n">
+        <v>53840</v>
+      </c>
+      <c r="N245" t="n">
+        <v>23484</v>
+      </c>
+      <c r="O245" t="n">
+        <v>2804</v>
+      </c>
+      <c r="P245" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr"/>
+      <c r="S245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>16</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I246" t="n">
+        <v>200</v>
+      </c>
+      <c r="J246" t="n">
+        <v>75</v>
+      </c>
+      <c r="K246" t="n">
+        <v>3842</v>
+      </c>
+      <c r="L246" t="n">
+        <v>3917</v>
+      </c>
+      <c r="M246" t="n">
+        <v>96261</v>
+      </c>
+      <c r="N246" t="n">
+        <v>11719</v>
+      </c>
+      <c r="O246" t="n">
+        <v>1511</v>
+      </c>
+      <c r="P246" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr"/>
+      <c r="S246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>16</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I247" t="n">
+        <v>200</v>
+      </c>
+      <c r="J247" t="n">
+        <v>127</v>
+      </c>
+      <c r="K247" t="n">
+        <v>5349</v>
+      </c>
+      <c r="L247" t="n">
+        <v>5476</v>
+      </c>
+      <c r="M247" t="n">
+        <v>100609</v>
+      </c>
+      <c r="N247" t="n">
+        <v>19746</v>
+      </c>
+      <c r="O247" t="n">
+        <v>2743</v>
+      </c>
+      <c r="P247" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr"/>
+      <c r="S247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>16</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I248" t="n">
+        <v>200</v>
+      </c>
+      <c r="J248" t="n">
+        <v>74</v>
+      </c>
+      <c r="K248" t="n">
+        <v>3702</v>
+      </c>
+      <c r="L248" t="n">
+        <v>3776</v>
+      </c>
+      <c r="M248" t="n">
+        <v>72377</v>
+      </c>
+      <c r="N248" t="n">
+        <v>11345</v>
+      </c>
+      <c r="O248" t="n">
+        <v>1502</v>
+      </c>
+      <c r="P248" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr"/>
+      <c r="S248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>16</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on grant compliance and acqui</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I249" t="n">
+        <v>200</v>
+      </c>
+      <c r="J249" t="n">
+        <v>76</v>
+      </c>
+      <c r="K249" t="n">
+        <v>2054</v>
+      </c>
+      <c r="L249" t="n">
+        <v>2130</v>
+      </c>
+      <c r="M249" t="n">
+        <v>123119</v>
+      </c>
+      <c r="N249" t="n">
+        <v>9912</v>
+      </c>
+      <c r="O249" t="n">
+        <v>1313</v>
+      </c>
+      <c r="P249" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr"/>
+      <c r="S249" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -30960,7 +33037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S233"/>
+  <dimension ref="A1:S249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45148,9 +47225,6 @@
       <c r="I218" t="n">
         <v>200</v>
       </c>
-      <c r="J218" t="inlineStr"/>
-      <c r="K218" t="inlineStr"/>
-      <c r="L218" t="inlineStr"/>
       <c r="M218" t="n">
         <v>277</v>
       </c>
@@ -45163,9 +47237,6 @@
       <c r="P218" t="n">
         <v>1</v>
       </c>
-      <c r="Q218" t="inlineStr"/>
-      <c r="R218" t="inlineStr"/>
-      <c r="S218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -45209,9 +47280,6 @@
       <c r="I219" t="n">
         <v>429</v>
       </c>
-      <c r="J219" t="inlineStr"/>
-      <c r="K219" t="inlineStr"/>
-      <c r="L219" t="inlineStr"/>
       <c r="M219" t="n">
         <v>257</v>
       </c>
@@ -45224,8 +47292,6 @@
       <c r="P219" t="n">
         <v>3</v>
       </c>
-      <c r="Q219" t="inlineStr"/>
-      <c r="R219" t="inlineStr"/>
       <c r="S219" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -45274,9 +47340,6 @@
       <c r="I220" t="n">
         <v>429</v>
       </c>
-      <c r="J220" t="inlineStr"/>
-      <c r="K220" t="inlineStr"/>
-      <c r="L220" t="inlineStr"/>
       <c r="M220" t="n">
         <v>267</v>
       </c>
@@ -45289,8 +47352,6 @@
       <c r="P220" t="n">
         <v>3</v>
       </c>
-      <c r="Q220" t="inlineStr"/>
-      <c r="R220" t="inlineStr"/>
       <c r="S220" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -45339,9 +47400,6 @@
       <c r="I221" t="n">
         <v>429</v>
       </c>
-      <c r="J221" t="inlineStr"/>
-      <c r="K221" t="inlineStr"/>
-      <c r="L221" t="inlineStr"/>
       <c r="M221" t="n">
         <v>388</v>
       </c>
@@ -45354,8 +47412,6 @@
       <c r="P221" t="n">
         <v>3</v>
       </c>
-      <c r="Q221" t="inlineStr"/>
-      <c r="R221" t="inlineStr"/>
       <c r="S221" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -45404,9 +47460,6 @@
       <c r="I222" t="n">
         <v>429</v>
       </c>
-      <c r="J222" t="inlineStr"/>
-      <c r="K222" t="inlineStr"/>
-      <c r="L222" t="inlineStr"/>
       <c r="M222" t="n">
         <v>229</v>
       </c>
@@ -45419,8 +47472,6 @@
       <c r="P222" t="n">
         <v>3</v>
       </c>
-      <c r="Q222" t="inlineStr"/>
-      <c r="R222" t="inlineStr"/>
       <c r="S222" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -45469,9 +47520,6 @@
       <c r="I223" t="n">
         <v>429</v>
       </c>
-      <c r="J223" t="inlineStr"/>
-      <c r="K223" t="inlineStr"/>
-      <c r="L223" t="inlineStr"/>
       <c r="M223" t="n">
         <v>476</v>
       </c>
@@ -45484,8 +47532,6 @@
       <c r="P223" t="n">
         <v>3</v>
       </c>
-      <c r="Q223" t="inlineStr"/>
-      <c r="R223" t="inlineStr"/>
       <c r="S223" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -45560,8 +47606,6 @@
           <t>responses/20260708T210536Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R224" t="inlineStr"/>
-      <c r="S224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -45631,8 +47675,6 @@
           <t>responses/20260708T210536Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R225" t="inlineStr"/>
-      <c r="S225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -45702,8 +47744,6 @@
           <t>responses/20260708T210536Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R226" t="inlineStr"/>
-      <c r="S226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -45747,9 +47787,6 @@
       <c r="I227" t="n">
         <v>429</v>
       </c>
-      <c r="J227" t="inlineStr"/>
-      <c r="K227" t="inlineStr"/>
-      <c r="L227" t="inlineStr"/>
       <c r="M227" t="n">
         <v>280</v>
       </c>
@@ -45762,8 +47799,6 @@
       <c r="P227" t="n">
         <v>3</v>
       </c>
-      <c r="Q227" t="inlineStr"/>
-      <c r="R227" t="inlineStr"/>
       <c r="S227" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -45838,8 +47873,6 @@
           <t>responses/20260708T210536Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R228" t="inlineStr"/>
-      <c r="S228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -45909,8 +47942,6 @@
           <t>responses/20260708T210536Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R229" t="inlineStr"/>
-      <c r="S229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -45980,8 +48011,6 @@
           <t>responses/20260708T210536Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R230" t="inlineStr"/>
-      <c r="S230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -46051,8 +48080,6 @@
           <t>responses/20260708T210536Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R231" t="inlineStr"/>
-      <c r="S231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -46122,8 +48149,6 @@
           <t>responses/20260708T210536Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R232" t="inlineStr"/>
-      <c r="S232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -46167,9 +48192,6 @@
       <c r="I233" t="n">
         <v>200</v>
       </c>
-      <c r="J233" t="inlineStr"/>
-      <c r="K233" t="inlineStr"/>
-      <c r="L233" t="inlineStr"/>
       <c r="M233" t="n">
         <v>120550</v>
       </c>
@@ -46182,9 +48204,1094 @@
       <c r="P233" t="n">
         <v>1</v>
       </c>
-      <c r="Q233" t="inlineStr"/>
-      <c r="R233" t="inlineStr"/>
-      <c r="S233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>16</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I234" t="n">
+        <v>400</v>
+      </c>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr"/>
+      <c r="L234" t="inlineStr"/>
+      <c r="M234" t="n">
+        <v>89</v>
+      </c>
+      <c r="N234" t="n">
+        <v>0</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0</v>
+      </c>
+      <c r="P234" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q234" t="inlineStr"/>
+      <c r="R234" t="inlineStr"/>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>16</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I235" t="n">
+        <v>429</v>
+      </c>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="inlineStr"/>
+      <c r="M235" t="n">
+        <v>265</v>
+      </c>
+      <c r="N235" t="n">
+        <v>0</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q235" t="inlineStr"/>
+      <c r="R235" t="inlineStr"/>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>16</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I236" t="n">
+        <v>429</v>
+      </c>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="inlineStr"/>
+      <c r="M236" t="n">
+        <v>409</v>
+      </c>
+      <c r="N236" t="n">
+        <v>0</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q236" t="inlineStr"/>
+      <c r="R236" t="inlineStr"/>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>16</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>200</v>
+      </c>
+      <c r="J237" t="n">
+        <v>292</v>
+      </c>
+      <c r="K237" t="n">
+        <v>838</v>
+      </c>
+      <c r="L237" t="n">
+        <v>1130</v>
+      </c>
+      <c r="M237" t="n">
+        <v>12363</v>
+      </c>
+      <c r="N237" t="n">
+        <v>3660</v>
+      </c>
+      <c r="O237" t="n">
+        <v>518</v>
+      </c>
+      <c r="P237" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr"/>
+      <c r="S237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>16</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>429</v>
+      </c>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="inlineStr"/>
+      <c r="M238" t="n">
+        <v>242</v>
+      </c>
+      <c r="N238" t="n">
+        <v>0</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q238" t="inlineStr"/>
+      <c r="R238" t="inlineStr"/>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>16</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>429</v>
+      </c>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="inlineStr"/>
+      <c r="M239" t="n">
+        <v>313</v>
+      </c>
+      <c r="N239" t="n">
+        <v>0</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q239" t="inlineStr"/>
+      <c r="R239" t="inlineStr"/>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>16</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>429</v>
+      </c>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="inlineStr"/>
+      <c r="L240" t="inlineStr"/>
+      <c r="M240" t="n">
+        <v>250</v>
+      </c>
+      <c r="N240" t="n">
+        <v>0</v>
+      </c>
+      <c r="O240" t="n">
+        <v>0</v>
+      </c>
+      <c r="P240" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q240" t="inlineStr"/>
+      <c r="R240" t="inlineStr"/>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>16</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>429</v>
+      </c>
+      <c r="J241" t="inlineStr"/>
+      <c r="K241" t="inlineStr"/>
+      <c r="L241" t="inlineStr"/>
+      <c r="M241" t="n">
+        <v>457</v>
+      </c>
+      <c r="N241" t="n">
+        <v>0</v>
+      </c>
+      <c r="O241" t="n">
+        <v>0</v>
+      </c>
+      <c r="P241" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q241" t="inlineStr"/>
+      <c r="R241" t="inlineStr"/>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>16</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I242" t="n">
+        <v>429</v>
+      </c>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="inlineStr"/>
+      <c r="L242" t="inlineStr"/>
+      <c r="M242" t="n">
+        <v>708</v>
+      </c>
+      <c r="N242" t="n">
+        <v>0</v>
+      </c>
+      <c r="O242" t="n">
+        <v>0</v>
+      </c>
+      <c r="P242" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q242" t="inlineStr"/>
+      <c r="R242" t="inlineStr"/>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>16</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>200</v>
+      </c>
+      <c r="J243" t="n">
+        <v>292</v>
+      </c>
+      <c r="K243" t="n">
+        <v>981</v>
+      </c>
+      <c r="L243" t="n">
+        <v>1273</v>
+      </c>
+      <c r="M243" t="n">
+        <v>11397</v>
+      </c>
+      <c r="N243" t="n">
+        <v>4227</v>
+      </c>
+      <c r="O243" t="n">
+        <v>595</v>
+      </c>
+      <c r="P243" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr"/>
+      <c r="S243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>16</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I244" t="n">
+        <v>200</v>
+      </c>
+      <c r="J244" t="n">
+        <v>332</v>
+      </c>
+      <c r="K244" t="n">
+        <v>600</v>
+      </c>
+      <c r="L244" t="n">
+        <v>932</v>
+      </c>
+      <c r="M244" t="n">
+        <v>9565</v>
+      </c>
+      <c r="N244" t="n">
+        <v>2138</v>
+      </c>
+      <c r="O244" t="n">
+        <v>303</v>
+      </c>
+      <c r="P244" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/poolside_laguna-xs.2_free.md</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr"/>
+      <c r="S244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>16</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>200</v>
+      </c>
+      <c r="J245" t="n">
+        <v>256</v>
+      </c>
+      <c r="K245" t="n">
+        <v>1274</v>
+      </c>
+      <c r="L245" t="n">
+        <v>1530</v>
+      </c>
+      <c r="M245" t="n">
+        <v>17563</v>
+      </c>
+      <c r="N245" t="n">
+        <v>4796</v>
+      </c>
+      <c r="O245" t="n">
+        <v>700</v>
+      </c>
+      <c r="P245" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr"/>
+      <c r="S245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>16</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I246" t="n">
+        <v>200</v>
+      </c>
+      <c r="J246" t="n">
+        <v>287</v>
+      </c>
+      <c r="K246" t="n">
+        <v>519</v>
+      </c>
+      <c r="L246" t="n">
+        <v>806</v>
+      </c>
+      <c r="M246" t="n">
+        <v>15279</v>
+      </c>
+      <c r="N246" t="n">
+        <v>2742</v>
+      </c>
+      <c r="O246" t="n">
+        <v>380</v>
+      </c>
+      <c r="P246" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr"/>
+      <c r="S246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>16</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I247" t="n">
+        <v>200</v>
+      </c>
+      <c r="J247" t="n">
+        <v>295</v>
+      </c>
+      <c r="K247" t="n">
+        <v>1076</v>
+      </c>
+      <c r="L247" t="n">
+        <v>1371</v>
+      </c>
+      <c r="M247" t="n">
+        <v>38572</v>
+      </c>
+      <c r="N247" t="n">
+        <v>3113</v>
+      </c>
+      <c r="O247" t="n">
+        <v>433</v>
+      </c>
+      <c r="P247" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr"/>
+      <c r="S247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>16</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I248" t="n">
+        <v>200</v>
+      </c>
+      <c r="J248" t="n">
+        <v>332</v>
+      </c>
+      <c r="K248" t="n">
+        <v>903</v>
+      </c>
+      <c r="L248" t="n">
+        <v>1235</v>
+      </c>
+      <c r="M248" t="n">
+        <v>59063</v>
+      </c>
+      <c r="N248" t="n">
+        <v>3528</v>
+      </c>
+      <c r="O248" t="n">
+        <v>503</v>
+      </c>
+      <c r="P248" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr"/>
+      <c r="S248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>20260709T082632Z</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-07-09T08:26:32.010844+00:00</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>16</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I249" t="n">
+        <v>200</v>
+      </c>
+      <c r="J249" t="n">
+        <v>288</v>
+      </c>
+      <c r="K249" t="n">
+        <v>1340</v>
+      </c>
+      <c r="L249" t="n">
+        <v>1628</v>
+      </c>
+      <c r="M249" t="n">
+        <v>62897</v>
+      </c>
+      <c r="N249" t="n">
+        <v>5417</v>
+      </c>
+      <c r="O249" t="n">
+        <v>771</v>
+      </c>
+      <c r="P249" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>responses/20260709T082632Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr"/>
+      <c r="S249" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-10 13:08 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S249"/>
+  <dimension ref="A1:S265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15636,9 +15636,6 @@
       <c r="I234" t="n">
         <v>400</v>
       </c>
-      <c r="J234" t="inlineStr"/>
-      <c r="K234" t="inlineStr"/>
-      <c r="L234" t="inlineStr"/>
       <c r="M234" t="n">
         <v>177</v>
       </c>
@@ -15651,8 +15648,6 @@
       <c r="P234" t="n">
         <v>1</v>
       </c>
-      <c r="Q234" t="inlineStr"/>
-      <c r="R234" t="inlineStr"/>
       <c r="S234" t="inlineStr">
         <is>
           <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
@@ -15701,9 +15696,6 @@
       <c r="I235" t="n">
         <v>429</v>
       </c>
-      <c r="J235" t="inlineStr"/>
-      <c r="K235" t="inlineStr"/>
-      <c r="L235" t="inlineStr"/>
       <c r="M235" t="n">
         <v>225</v>
       </c>
@@ -15716,8 +15708,6 @@
       <c r="P235" t="n">
         <v>3</v>
       </c>
-      <c r="Q235" t="inlineStr"/>
-      <c r="R235" t="inlineStr"/>
       <c r="S235" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -15766,9 +15756,6 @@
       <c r="I236" t="n">
         <v>429</v>
       </c>
-      <c r="J236" t="inlineStr"/>
-      <c r="K236" t="inlineStr"/>
-      <c r="L236" t="inlineStr"/>
       <c r="M236" t="n">
         <v>217</v>
       </c>
@@ -15781,8 +15768,6 @@
       <c r="P236" t="n">
         <v>3</v>
       </c>
-      <c r="Q236" t="inlineStr"/>
-      <c r="R236" t="inlineStr"/>
       <c r="S236" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -15831,9 +15816,6 @@
       <c r="I237" t="n">
         <v>429</v>
       </c>
-      <c r="J237" t="inlineStr"/>
-      <c r="K237" t="inlineStr"/>
-      <c r="L237" t="inlineStr"/>
       <c r="M237" t="n">
         <v>233</v>
       </c>
@@ -15846,8 +15828,6 @@
       <c r="P237" t="n">
         <v>3</v>
       </c>
-      <c r="Q237" t="inlineStr"/>
-      <c r="R237" t="inlineStr"/>
       <c r="S237" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -15896,9 +15876,6 @@
       <c r="I238" t="n">
         <v>429</v>
       </c>
-      <c r="J238" t="inlineStr"/>
-      <c r="K238" t="inlineStr"/>
-      <c r="L238" t="inlineStr"/>
       <c r="M238" t="n">
         <v>231</v>
       </c>
@@ -15911,8 +15888,6 @@
       <c r="P238" t="n">
         <v>3</v>
       </c>
-      <c r="Q238" t="inlineStr"/>
-      <c r="R238" t="inlineStr"/>
       <c r="S238" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -15961,9 +15936,6 @@
       <c r="I239" t="n">
         <v>429</v>
       </c>
-      <c r="J239" t="inlineStr"/>
-      <c r="K239" t="inlineStr"/>
-      <c r="L239" t="inlineStr"/>
       <c r="M239" t="n">
         <v>393</v>
       </c>
@@ -15976,8 +15948,6 @@
       <c r="P239" t="n">
         <v>3</v>
       </c>
-      <c r="Q239" t="inlineStr"/>
-      <c r="R239" t="inlineStr"/>
       <c r="S239" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -16052,8 +16022,6 @@
           <t>responses/20260709T082632Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R240" t="inlineStr"/>
-      <c r="S240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -16123,8 +16091,6 @@
           <t>responses/20260709T082632Z/code/poolside_laguna-xs.2_free.java</t>
         </is>
       </c>
-      <c r="R241" t="inlineStr"/>
-      <c r="S241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -16194,8 +16160,6 @@
           <t>responses/20260709T082632Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R242" t="inlineStr"/>
-      <c r="S242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -16265,8 +16229,6 @@
           <t>responses/20260709T082632Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R243" t="inlineStr"/>
-      <c r="S243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -16336,8 +16298,6 @@
           <t>responses/20260709T082632Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R244" t="inlineStr"/>
-      <c r="S244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -16407,8 +16367,6 @@
           <t>responses/20260709T082632Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R245" t="inlineStr"/>
-      <c r="S245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -16473,9 +16431,6 @@
       <c r="P246" t="n">
         <v>1</v>
       </c>
-      <c r="Q246" t="inlineStr"/>
-      <c r="R246" t="inlineStr"/>
-      <c r="S246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -16545,8 +16500,6 @@
           <t>responses/20260709T082632Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
         </is>
       </c>
-      <c r="R247" t="inlineStr"/>
-      <c r="S247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -16616,8 +16569,6 @@
           <t>responses/20260709T082632Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R248" t="inlineStr"/>
-      <c r="S248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -16687,8 +16638,1082 @@
           <t>responses/20260709T082632Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R249" t="inlineStr"/>
-      <c r="S249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>17</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I250" t="n">
+        <v>429</v>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr"/>
+      <c r="L250" t="inlineStr"/>
+      <c r="M250" t="n">
+        <v>171</v>
+      </c>
+      <c r="N250" t="n">
+        <v>0</v>
+      </c>
+      <c r="O250" t="n">
+        <v>0</v>
+      </c>
+      <c r="P250" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q250" t="inlineStr"/>
+      <c r="R250" t="inlineStr"/>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>17</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I251" t="n">
+        <v>429</v>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr"/>
+      <c r="L251" t="inlineStr"/>
+      <c r="M251" t="n">
+        <v>461</v>
+      </c>
+      <c r="N251" t="n">
+        <v>0</v>
+      </c>
+      <c r="O251" t="n">
+        <v>0</v>
+      </c>
+      <c r="P251" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q251" t="inlineStr"/>
+      <c r="R251" t="inlineStr"/>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>17</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I252" t="n">
+        <v>429</v>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr"/>
+      <c r="L252" t="inlineStr"/>
+      <c r="M252" t="n">
+        <v>483</v>
+      </c>
+      <c r="N252" t="n">
+        <v>0</v>
+      </c>
+      <c r="O252" t="n">
+        <v>0</v>
+      </c>
+      <c r="P252" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q252" t="inlineStr"/>
+      <c r="R252" t="inlineStr"/>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>17</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I253" t="n">
+        <v>429</v>
+      </c>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr"/>
+      <c r="L253" t="inlineStr"/>
+      <c r="M253" t="n">
+        <v>509</v>
+      </c>
+      <c r="N253" t="n">
+        <v>0</v>
+      </c>
+      <c r="O253" t="n">
+        <v>0</v>
+      </c>
+      <c r="P253" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q253" t="inlineStr"/>
+      <c r="R253" t="inlineStr"/>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>17</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I254" t="n">
+        <v>404</v>
+      </c>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr"/>
+      <c r="L254" t="inlineStr"/>
+      <c r="M254" t="n">
+        <v>178</v>
+      </c>
+      <c r="N254" t="n">
+        <v>0</v>
+      </c>
+      <c r="O254" t="n">
+        <v>0</v>
+      </c>
+      <c r="P254" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q254" t="inlineStr"/>
+      <c r="R254" t="inlineStr"/>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>17</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I255" t="n">
+        <v>429</v>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="inlineStr"/>
+      <c r="M255" t="n">
+        <v>728</v>
+      </c>
+      <c r="N255" t="n">
+        <v>0</v>
+      </c>
+      <c r="O255" t="n">
+        <v>0</v>
+      </c>
+      <c r="P255" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q255" t="inlineStr"/>
+      <c r="R255" t="inlineStr"/>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>17</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I256" t="n">
+        <v>429</v>
+      </c>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr"/>
+      <c r="L256" t="inlineStr"/>
+      <c r="M256" t="n">
+        <v>437</v>
+      </c>
+      <c r="N256" t="n">
+        <v>0</v>
+      </c>
+      <c r="O256" t="n">
+        <v>0</v>
+      </c>
+      <c r="P256" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q256" t="inlineStr"/>
+      <c r="R256" t="inlineStr"/>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>17</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I257" t="n">
+        <v>200</v>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr"/>
+      <c r="L257" t="inlineStr"/>
+      <c r="M257" t="n">
+        <v>12504</v>
+      </c>
+      <c r="N257" t="n">
+        <v>0</v>
+      </c>
+      <c r="O257" t="n">
+        <v>0</v>
+      </c>
+      <c r="P257" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q257" t="inlineStr"/>
+      <c r="R257" t="inlineStr"/>
+      <c r="S257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>17</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I258" t="n">
+        <v>200</v>
+      </c>
+      <c r="J258" t="n">
+        <v>86</v>
+      </c>
+      <c r="K258" t="n">
+        <v>4077</v>
+      </c>
+      <c r="L258" t="n">
+        <v>4163</v>
+      </c>
+      <c r="M258" t="n">
+        <v>38142</v>
+      </c>
+      <c r="N258" t="n">
+        <v>15368</v>
+      </c>
+      <c r="O258" t="n">
+        <v>1863</v>
+      </c>
+      <c r="P258" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr"/>
+      <c r="S258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>17</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I259" t="n">
+        <v>200</v>
+      </c>
+      <c r="J259" t="n">
+        <v>84</v>
+      </c>
+      <c r="K259" t="n">
+        <v>1185</v>
+      </c>
+      <c r="L259" t="n">
+        <v>1269</v>
+      </c>
+      <c r="M259" t="n">
+        <v>42458</v>
+      </c>
+      <c r="N259" t="n">
+        <v>5338</v>
+      </c>
+      <c r="O259" t="n">
+        <v>498</v>
+      </c>
+      <c r="P259" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R259" t="inlineStr"/>
+      <c r="S259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>17</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I260" t="n">
+        <v>200</v>
+      </c>
+      <c r="J260" t="n">
+        <v>63</v>
+      </c>
+      <c r="K260" t="n">
+        <v>3467</v>
+      </c>
+      <c r="L260" t="n">
+        <v>3530</v>
+      </c>
+      <c r="M260" t="n">
+        <v>43392</v>
+      </c>
+      <c r="N260" t="n">
+        <v>16872</v>
+      </c>
+      <c r="O260" t="n">
+        <v>1764</v>
+      </c>
+      <c r="P260" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr"/>
+      <c r="S260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>17</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I261" t="n">
+        <v>200</v>
+      </c>
+      <c r="J261" t="n">
+        <v>86</v>
+      </c>
+      <c r="K261" t="n">
+        <v>5929</v>
+      </c>
+      <c r="L261" t="n">
+        <v>6015</v>
+      </c>
+      <c r="M261" t="n">
+        <v>61781</v>
+      </c>
+      <c r="N261" t="n">
+        <v>23369</v>
+      </c>
+      <c r="O261" t="n">
+        <v>2416</v>
+      </c>
+      <c r="P261" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr"/>
+      <c r="S261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>17</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I262" t="n">
+        <v>200</v>
+      </c>
+      <c r="J262" t="n">
+        <v>86</v>
+      </c>
+      <c r="K262" t="n">
+        <v>3891</v>
+      </c>
+      <c r="L262" t="n">
+        <v>3977</v>
+      </c>
+      <c r="M262" t="n">
+        <v>73193</v>
+      </c>
+      <c r="N262" t="n">
+        <v>14042</v>
+      </c>
+      <c r="O262" t="n">
+        <v>1741</v>
+      </c>
+      <c r="P262" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr"/>
+      <c r="S262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>17</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I263" t="n">
+        <v>200</v>
+      </c>
+      <c r="J263" t="n">
+        <v>135</v>
+      </c>
+      <c r="K263" t="n">
+        <v>3690</v>
+      </c>
+      <c r="L263" t="n">
+        <v>3825</v>
+      </c>
+      <c r="M263" t="n">
+        <v>73839</v>
+      </c>
+      <c r="N263" t="n">
+        <v>11835</v>
+      </c>
+      <c r="O263" t="n">
+        <v>1396</v>
+      </c>
+      <c r="P263" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr"/>
+      <c r="S263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>17</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I264" t="n">
+        <v>200</v>
+      </c>
+      <c r="J264" t="n">
+        <v>77</v>
+      </c>
+      <c r="K264" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L264" t="n">
+        <v>6077</v>
+      </c>
+      <c r="M264" t="n">
+        <v>176734</v>
+      </c>
+      <c r="N264" t="n">
+        <v>0</v>
+      </c>
+      <c r="O264" t="n">
+        <v>0</v>
+      </c>
+      <c r="P264" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q264" t="inlineStr"/>
+      <c r="R264" t="inlineStr"/>
+      <c r="S264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>17</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Implement a token-bucket rate limiter in Java that is safe for use by many threa</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I265" t="n">
+        <v>200</v>
+      </c>
+      <c r="J265" t="n">
+        <v>82</v>
+      </c>
+      <c r="K265" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L265" t="n">
+        <v>6082</v>
+      </c>
+      <c r="M265" t="n">
+        <v>189475</v>
+      </c>
+      <c r="N265" t="n">
+        <v>0</v>
+      </c>
+      <c r="O265" t="n">
+        <v>0</v>
+      </c>
+      <c r="P265" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q265" t="inlineStr"/>
+      <c r="R265" t="inlineStr"/>
+      <c r="S265" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16701,7 +17726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S249"/>
+  <dimension ref="A1:S265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31974,9 +32999,6 @@
       <c r="I234" t="n">
         <v>400</v>
       </c>
-      <c r="J234" t="inlineStr"/>
-      <c r="K234" t="inlineStr"/>
-      <c r="L234" t="inlineStr"/>
       <c r="M234" t="n">
         <v>123</v>
       </c>
@@ -31989,8 +33011,6 @@
       <c r="P234" t="n">
         <v>1</v>
       </c>
-      <c r="Q234" t="inlineStr"/>
-      <c r="R234" t="inlineStr"/>
       <c r="S234" t="inlineStr">
         <is>
           <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
@@ -32039,9 +33059,6 @@
       <c r="I235" t="n">
         <v>429</v>
       </c>
-      <c r="J235" t="inlineStr"/>
-      <c r="K235" t="inlineStr"/>
-      <c r="L235" t="inlineStr"/>
       <c r="M235" t="n">
         <v>226</v>
       </c>
@@ -32054,8 +33071,6 @@
       <c r="P235" t="n">
         <v>3</v>
       </c>
-      <c r="Q235" t="inlineStr"/>
-      <c r="R235" t="inlineStr"/>
       <c r="S235" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -32104,9 +33119,6 @@
       <c r="I236" t="n">
         <v>429</v>
       </c>
-      <c r="J236" t="inlineStr"/>
-      <c r="K236" t="inlineStr"/>
-      <c r="L236" t="inlineStr"/>
       <c r="M236" t="n">
         <v>429</v>
       </c>
@@ -32119,8 +33131,6 @@
       <c r="P236" t="n">
         <v>3</v>
       </c>
-      <c r="Q236" t="inlineStr"/>
-      <c r="R236" t="inlineStr"/>
       <c r="S236" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -32195,8 +33205,6 @@
           <t>responses/20260709T082632Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R237" t="inlineStr"/>
-      <c r="S237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -32240,9 +33248,6 @@
       <c r="I238" t="n">
         <v>429</v>
       </c>
-      <c r="J238" t="inlineStr"/>
-      <c r="K238" t="inlineStr"/>
-      <c r="L238" t="inlineStr"/>
       <c r="M238" t="n">
         <v>215</v>
       </c>
@@ -32255,8 +33260,6 @@
       <c r="P238" t="n">
         <v>3</v>
       </c>
-      <c r="Q238" t="inlineStr"/>
-      <c r="R238" t="inlineStr"/>
       <c r="S238" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -32305,9 +33308,6 @@
       <c r="I239" t="n">
         <v>429</v>
       </c>
-      <c r="J239" t="inlineStr"/>
-      <c r="K239" t="inlineStr"/>
-      <c r="L239" t="inlineStr"/>
       <c r="M239" t="n">
         <v>215</v>
       </c>
@@ -32320,8 +33320,6 @@
       <c r="P239" t="n">
         <v>3</v>
       </c>
-      <c r="Q239" t="inlineStr"/>
-      <c r="R239" t="inlineStr"/>
       <c r="S239" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -32370,9 +33368,6 @@
       <c r="I240" t="n">
         <v>429</v>
       </c>
-      <c r="J240" t="inlineStr"/>
-      <c r="K240" t="inlineStr"/>
-      <c r="L240" t="inlineStr"/>
       <c r="M240" t="n">
         <v>407</v>
       </c>
@@ -32385,8 +33380,6 @@
       <c r="P240" t="n">
         <v>3</v>
       </c>
-      <c r="Q240" t="inlineStr"/>
-      <c r="R240" t="inlineStr"/>
       <c r="S240" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -32435,9 +33428,6 @@
       <c r="I241" t="n">
         <v>429</v>
       </c>
-      <c r="J241" t="inlineStr"/>
-      <c r="K241" t="inlineStr"/>
-      <c r="L241" t="inlineStr"/>
       <c r="M241" t="n">
         <v>266</v>
       </c>
@@ -32450,8 +33440,6 @@
       <c r="P241" t="n">
         <v>3</v>
       </c>
-      <c r="Q241" t="inlineStr"/>
-      <c r="R241" t="inlineStr"/>
       <c r="S241" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -32526,8 +33514,6 @@
           <t>responses/20260709T082632Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R242" t="inlineStr"/>
-      <c r="S242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -32597,8 +33583,6 @@
           <t>responses/20260709T082632Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R243" t="inlineStr"/>
-      <c r="S243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -32668,8 +33652,6 @@
           <t>responses/20260709T082632Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R244" t="inlineStr"/>
-      <c r="S244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -32739,8 +33721,6 @@
           <t>responses/20260709T082632Z/text/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R245" t="inlineStr"/>
-      <c r="S245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -32810,8 +33790,6 @@
           <t>responses/20260709T082632Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R246" t="inlineStr"/>
-      <c r="S246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -32881,8 +33859,6 @@
           <t>responses/20260709T082632Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R247" t="inlineStr"/>
-      <c r="S247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -32952,8 +33928,6 @@
           <t>responses/20260709T082632Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R248" t="inlineStr"/>
-      <c r="S248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -33023,8 +33997,1084 @@
           <t>responses/20260709T082632Z/text/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R249" t="inlineStr"/>
-      <c r="S249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>17</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I250" t="n">
+        <v>429</v>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr"/>
+      <c r="L250" t="inlineStr"/>
+      <c r="M250" t="n">
+        <v>177</v>
+      </c>
+      <c r="N250" t="n">
+        <v>0</v>
+      </c>
+      <c r="O250" t="n">
+        <v>0</v>
+      </c>
+      <c r="P250" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q250" t="inlineStr"/>
+      <c r="R250" t="inlineStr"/>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>17</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I251" t="n">
+        <v>429</v>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr"/>
+      <c r="L251" t="inlineStr"/>
+      <c r="M251" t="n">
+        <v>691</v>
+      </c>
+      <c r="N251" t="n">
+        <v>0</v>
+      </c>
+      <c r="O251" t="n">
+        <v>0</v>
+      </c>
+      <c r="P251" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q251" t="inlineStr"/>
+      <c r="R251" t="inlineStr"/>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>17</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I252" t="n">
+        <v>429</v>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr"/>
+      <c r="L252" t="inlineStr"/>
+      <c r="M252" t="n">
+        <v>212</v>
+      </c>
+      <c r="N252" t="n">
+        <v>0</v>
+      </c>
+      <c r="O252" t="n">
+        <v>0</v>
+      </c>
+      <c r="P252" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q252" t="inlineStr"/>
+      <c r="R252" t="inlineStr"/>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>17</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I253" t="n">
+        <v>429</v>
+      </c>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr"/>
+      <c r="L253" t="inlineStr"/>
+      <c r="M253" t="n">
+        <v>234</v>
+      </c>
+      <c r="N253" t="n">
+        <v>0</v>
+      </c>
+      <c r="O253" t="n">
+        <v>0</v>
+      </c>
+      <c r="P253" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q253" t="inlineStr"/>
+      <c r="R253" t="inlineStr"/>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>17</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I254" t="n">
+        <v>429</v>
+      </c>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr"/>
+      <c r="L254" t="inlineStr"/>
+      <c r="M254" t="n">
+        <v>160</v>
+      </c>
+      <c r="N254" t="n">
+        <v>0</v>
+      </c>
+      <c r="O254" t="n">
+        <v>0</v>
+      </c>
+      <c r="P254" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q254" t="inlineStr"/>
+      <c r="R254" t="inlineStr"/>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>17</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I255" t="n">
+        <v>429</v>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="inlineStr"/>
+      <c r="M255" t="n">
+        <v>920</v>
+      </c>
+      <c r="N255" t="n">
+        <v>0</v>
+      </c>
+      <c r="O255" t="n">
+        <v>0</v>
+      </c>
+      <c r="P255" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q255" t="inlineStr"/>
+      <c r="R255" t="inlineStr"/>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>17</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I256" t="n">
+        <v>429</v>
+      </c>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr"/>
+      <c r="L256" t="inlineStr"/>
+      <c r="M256" t="n">
+        <v>245</v>
+      </c>
+      <c r="N256" t="n">
+        <v>0</v>
+      </c>
+      <c r="O256" t="n">
+        <v>0</v>
+      </c>
+      <c r="P256" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q256" t="inlineStr"/>
+      <c r="R256" t="inlineStr"/>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>17</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I257" t="n">
+        <v>404</v>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr"/>
+      <c r="L257" t="inlineStr"/>
+      <c r="M257" t="n">
+        <v>103</v>
+      </c>
+      <c r="N257" t="n">
+        <v>0</v>
+      </c>
+      <c r="O257" t="n">
+        <v>0</v>
+      </c>
+      <c r="P257" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q257" t="inlineStr"/>
+      <c r="R257" t="inlineStr"/>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>17</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I258" t="n">
+        <v>200</v>
+      </c>
+      <c r="J258" t="n">
+        <v>125</v>
+      </c>
+      <c r="K258" t="n">
+        <v>4222</v>
+      </c>
+      <c r="L258" t="n">
+        <v>4347</v>
+      </c>
+      <c r="M258" t="n">
+        <v>50093</v>
+      </c>
+      <c r="N258" t="n">
+        <v>16194</v>
+      </c>
+      <c r="O258" t="n">
+        <v>2267</v>
+      </c>
+      <c r="P258" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr"/>
+      <c r="S258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>17</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I259" t="n">
+        <v>200</v>
+      </c>
+      <c r="J259" t="n">
+        <v>75</v>
+      </c>
+      <c r="K259" t="n">
+        <v>6894</v>
+      </c>
+      <c r="L259" t="n">
+        <v>6969</v>
+      </c>
+      <c r="M259" t="n">
+        <v>76461</v>
+      </c>
+      <c r="N259" t="n">
+        <v>31760</v>
+      </c>
+      <c r="O259" t="n">
+        <v>4175</v>
+      </c>
+      <c r="P259" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R259" t="inlineStr"/>
+      <c r="S259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>17</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I260" t="n">
+        <v>200</v>
+      </c>
+      <c r="J260" t="n">
+        <v>75</v>
+      </c>
+      <c r="K260" t="n">
+        <v>7313</v>
+      </c>
+      <c r="L260" t="n">
+        <v>7388</v>
+      </c>
+      <c r="M260" t="n">
+        <v>108978</v>
+      </c>
+      <c r="N260" t="n">
+        <v>25812</v>
+      </c>
+      <c r="O260" t="n">
+        <v>3587</v>
+      </c>
+      <c r="P260" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr"/>
+      <c r="S260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>17</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I261" t="n">
+        <v>200</v>
+      </c>
+      <c r="J261" t="n">
+        <v>50</v>
+      </c>
+      <c r="K261" t="n">
+        <v>4777</v>
+      </c>
+      <c r="L261" t="n">
+        <v>4827</v>
+      </c>
+      <c r="M261" t="n">
+        <v>78582</v>
+      </c>
+      <c r="N261" t="n">
+        <v>19894</v>
+      </c>
+      <c r="O261" t="n">
+        <v>2624</v>
+      </c>
+      <c r="P261" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr"/>
+      <c r="S261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>17</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I262" t="n">
+        <v>200</v>
+      </c>
+      <c r="J262" t="n">
+        <v>71</v>
+      </c>
+      <c r="K262" t="n">
+        <v>3172</v>
+      </c>
+      <c r="L262" t="n">
+        <v>3243</v>
+      </c>
+      <c r="M262" t="n">
+        <v>81714</v>
+      </c>
+      <c r="N262" t="n">
+        <v>12414</v>
+      </c>
+      <c r="O262" t="n">
+        <v>1505</v>
+      </c>
+      <c r="P262" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr"/>
+      <c r="S262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>17</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I263" t="n">
+        <v>200</v>
+      </c>
+      <c r="J263" t="n">
+        <v>75</v>
+      </c>
+      <c r="K263" t="n">
+        <v>6722</v>
+      </c>
+      <c r="L263" t="n">
+        <v>6797</v>
+      </c>
+      <c r="M263" t="n">
+        <v>83566</v>
+      </c>
+      <c r="N263" t="n">
+        <v>18690</v>
+      </c>
+      <c r="O263" t="n">
+        <v>2576</v>
+      </c>
+      <c r="P263" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr"/>
+      <c r="S263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>17</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I264" t="n">
+        <v>200</v>
+      </c>
+      <c r="J264" t="inlineStr"/>
+      <c r="K264" t="inlineStr"/>
+      <c r="L264" t="inlineStr"/>
+      <c r="M264" t="n">
+        <v>120250</v>
+      </c>
+      <c r="N264" t="n">
+        <v>0</v>
+      </c>
+      <c r="O264" t="n">
+        <v>0</v>
+      </c>
+      <c r="P264" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q264" t="inlineStr"/>
+      <c r="R264" t="inlineStr"/>
+      <c r="S264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>17</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on how grant management softw</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I265" t="n">
+        <v>200</v>
+      </c>
+      <c r="J265" t="n">
+        <v>71</v>
+      </c>
+      <c r="K265" t="n">
+        <v>4494</v>
+      </c>
+      <c r="L265" t="n">
+        <v>4565</v>
+      </c>
+      <c r="M265" t="n">
+        <v>150012</v>
+      </c>
+      <c r="N265" t="n">
+        <v>15512</v>
+      </c>
+      <c r="O265" t="n">
+        <v>1990</v>
+      </c>
+      <c r="P265" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R265" t="inlineStr"/>
+      <c r="S265" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -33037,7 +35087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S249"/>
+  <dimension ref="A1:S265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48247,9 +50297,6 @@
       <c r="I234" t="n">
         <v>400</v>
       </c>
-      <c r="J234" t="inlineStr"/>
-      <c r="K234" t="inlineStr"/>
-      <c r="L234" t="inlineStr"/>
       <c r="M234" t="n">
         <v>89</v>
       </c>
@@ -48262,8 +50309,6 @@
       <c r="P234" t="n">
         <v>1</v>
       </c>
-      <c r="Q234" t="inlineStr"/>
-      <c r="R234" t="inlineStr"/>
       <c r="S234" t="inlineStr">
         <is>
           <t>HTTP 400: {"error":{"message":"Provider returned error","code":400,"metadata":{"raw":"{\"status\":400,\"title\":\"Bad Request\",\"detail\":\"Function id '948fe171-ce7a-4332-8bc0-5e14e90259f9': DEGRADED function cannot be invoked\"}","provider_name":"Nvidia","is_byok":false}},"user_id":"user_3FWWx2cLEsPQ6tm6LV</t>
@@ -48312,9 +50357,6 @@
       <c r="I235" t="n">
         <v>429</v>
       </c>
-      <c r="J235" t="inlineStr"/>
-      <c r="K235" t="inlineStr"/>
-      <c r="L235" t="inlineStr"/>
       <c r="M235" t="n">
         <v>265</v>
       </c>
@@ -48327,8 +50369,6 @@
       <c r="P235" t="n">
         <v>3</v>
       </c>
-      <c r="Q235" t="inlineStr"/>
-      <c r="R235" t="inlineStr"/>
       <c r="S235" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -48377,9 +50417,6 @@
       <c r="I236" t="n">
         <v>429</v>
       </c>
-      <c r="J236" t="inlineStr"/>
-      <c r="K236" t="inlineStr"/>
-      <c r="L236" t="inlineStr"/>
       <c r="M236" t="n">
         <v>409</v>
       </c>
@@ -48392,8 +50429,6 @@
       <c r="P236" t="n">
         <v>3</v>
       </c>
-      <c r="Q236" t="inlineStr"/>
-      <c r="R236" t="inlineStr"/>
       <c r="S236" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -48468,8 +50503,6 @@
           <t>responses/20260709T082632Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R237" t="inlineStr"/>
-      <c r="S237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -48513,9 +50546,6 @@
       <c r="I238" t="n">
         <v>429</v>
       </c>
-      <c r="J238" t="inlineStr"/>
-      <c r="K238" t="inlineStr"/>
-      <c r="L238" t="inlineStr"/>
       <c r="M238" t="n">
         <v>242</v>
       </c>
@@ -48528,8 +50558,6 @@
       <c r="P238" t="n">
         <v>3</v>
       </c>
-      <c r="Q238" t="inlineStr"/>
-      <c r="R238" t="inlineStr"/>
       <c r="S238" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -48578,9 +50606,6 @@
       <c r="I239" t="n">
         <v>429</v>
       </c>
-      <c r="J239" t="inlineStr"/>
-      <c r="K239" t="inlineStr"/>
-      <c r="L239" t="inlineStr"/>
       <c r="M239" t="n">
         <v>313</v>
       </c>
@@ -48593,8 +50618,6 @@
       <c r="P239" t="n">
         <v>3</v>
       </c>
-      <c r="Q239" t="inlineStr"/>
-      <c r="R239" t="inlineStr"/>
       <c r="S239" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -48643,9 +50666,6 @@
       <c r="I240" t="n">
         <v>429</v>
       </c>
-      <c r="J240" t="inlineStr"/>
-      <c r="K240" t="inlineStr"/>
-      <c r="L240" t="inlineStr"/>
       <c r="M240" t="n">
         <v>250</v>
       </c>
@@ -48658,8 +50678,6 @@
       <c r="P240" t="n">
         <v>3</v>
       </c>
-      <c r="Q240" t="inlineStr"/>
-      <c r="R240" t="inlineStr"/>
       <c r="S240" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -48708,9 +50726,6 @@
       <c r="I241" t="n">
         <v>429</v>
       </c>
-      <c r="J241" t="inlineStr"/>
-      <c r="K241" t="inlineStr"/>
-      <c r="L241" t="inlineStr"/>
       <c r="M241" t="n">
         <v>457</v>
       </c>
@@ -48723,8 +50738,6 @@
       <c r="P241" t="n">
         <v>3</v>
       </c>
-      <c r="Q241" t="inlineStr"/>
-      <c r="R241" t="inlineStr"/>
       <c r="S241" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -48773,9 +50786,6 @@
       <c r="I242" t="n">
         <v>429</v>
       </c>
-      <c r="J242" t="inlineStr"/>
-      <c r="K242" t="inlineStr"/>
-      <c r="L242" t="inlineStr"/>
       <c r="M242" t="n">
         <v>708</v>
       </c>
@@ -48788,8 +50798,6 @@
       <c r="P242" t="n">
         <v>3</v>
       </c>
-      <c r="Q242" t="inlineStr"/>
-      <c r="R242" t="inlineStr"/>
       <c r="S242" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -48864,8 +50872,6 @@
           <t>responses/20260709T082632Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R243" t="inlineStr"/>
-      <c r="S243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -48935,8 +50941,6 @@
           <t>responses/20260709T082632Z/email/poolside_laguna-xs.2_free.md</t>
         </is>
       </c>
-      <c r="R244" t="inlineStr"/>
-      <c r="S244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -49006,8 +51010,6 @@
           <t>responses/20260709T082632Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R245" t="inlineStr"/>
-      <c r="S245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -49077,8 +51079,6 @@
           <t>responses/20260709T082632Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R246" t="inlineStr"/>
-      <c r="S246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -49148,8 +51148,6 @@
           <t>responses/20260709T082632Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R247" t="inlineStr"/>
-      <c r="S247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -49219,8 +51217,6 @@
           <t>responses/20260709T082632Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R248" t="inlineStr"/>
-      <c r="S248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -49290,8 +51286,1090 @@
           <t>responses/20260709T082632Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R249" t="inlineStr"/>
-      <c r="S249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>17</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I250" t="n">
+        <v>200</v>
+      </c>
+      <c r="J250" t="n">
+        <v>292</v>
+      </c>
+      <c r="K250" t="n">
+        <v>809</v>
+      </c>
+      <c r="L250" t="n">
+        <v>1101</v>
+      </c>
+      <c r="M250" t="n">
+        <v>9216</v>
+      </c>
+      <c r="N250" t="n">
+        <v>2923</v>
+      </c>
+      <c r="O250" t="n">
+        <v>403</v>
+      </c>
+      <c r="P250" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr"/>
+      <c r="S250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>17</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I251" t="n">
+        <v>429</v>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr"/>
+      <c r="L251" t="inlineStr"/>
+      <c r="M251" t="n">
+        <v>188</v>
+      </c>
+      <c r="N251" t="n">
+        <v>0</v>
+      </c>
+      <c r="O251" t="n">
+        <v>0</v>
+      </c>
+      <c r="P251" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q251" t="inlineStr"/>
+      <c r="R251" t="inlineStr"/>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>17</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I252" t="n">
+        <v>429</v>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr"/>
+      <c r="L252" t="inlineStr"/>
+      <c r="M252" t="n">
+        <v>339</v>
+      </c>
+      <c r="N252" t="n">
+        <v>0</v>
+      </c>
+      <c r="O252" t="n">
+        <v>0</v>
+      </c>
+      <c r="P252" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q252" t="inlineStr"/>
+      <c r="R252" t="inlineStr"/>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>17</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I253" t="n">
+        <v>200</v>
+      </c>
+      <c r="J253" t="n">
+        <v>292</v>
+      </c>
+      <c r="K253" t="n">
+        <v>982</v>
+      </c>
+      <c r="L253" t="n">
+        <v>1274</v>
+      </c>
+      <c r="M253" t="n">
+        <v>18258</v>
+      </c>
+      <c r="N253" t="n">
+        <v>4381</v>
+      </c>
+      <c r="O253" t="n">
+        <v>609</v>
+      </c>
+      <c r="P253" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr"/>
+      <c r="S253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>17</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I254" t="n">
+        <v>429</v>
+      </c>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr"/>
+      <c r="L254" t="inlineStr"/>
+      <c r="M254" t="n">
+        <v>264</v>
+      </c>
+      <c r="N254" t="n">
+        <v>0</v>
+      </c>
+      <c r="O254" t="n">
+        <v>0</v>
+      </c>
+      <c r="P254" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q254" t="inlineStr"/>
+      <c r="R254" t="inlineStr"/>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>17</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I255" t="n">
+        <v>429</v>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="inlineStr"/>
+      <c r="M255" t="n">
+        <v>705</v>
+      </c>
+      <c r="N255" t="n">
+        <v>0</v>
+      </c>
+      <c r="O255" t="n">
+        <v>0</v>
+      </c>
+      <c r="P255" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q255" t="inlineStr"/>
+      <c r="R255" t="inlineStr"/>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>17</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I256" t="n">
+        <v>200</v>
+      </c>
+      <c r="J256" t="n">
+        <v>292</v>
+      </c>
+      <c r="K256" t="n">
+        <v>618</v>
+      </c>
+      <c r="L256" t="n">
+        <v>910</v>
+      </c>
+      <c r="M256" t="n">
+        <v>6695</v>
+      </c>
+      <c r="N256" t="n">
+        <v>2821</v>
+      </c>
+      <c r="O256" t="n">
+        <v>413</v>
+      </c>
+      <c r="P256" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr"/>
+      <c r="S256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>17</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I257" t="n">
+        <v>429</v>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr"/>
+      <c r="L257" t="inlineStr"/>
+      <c r="M257" t="n">
+        <v>453</v>
+      </c>
+      <c r="N257" t="n">
+        <v>0</v>
+      </c>
+      <c r="O257" t="n">
+        <v>0</v>
+      </c>
+      <c r="P257" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q257" t="inlineStr"/>
+      <c r="R257" t="inlineStr"/>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>17</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I258" t="n">
+        <v>404</v>
+      </c>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="inlineStr"/>
+      <c r="L258" t="inlineStr"/>
+      <c r="M258" t="n">
+        <v>92</v>
+      </c>
+      <c r="N258" t="n">
+        <v>0</v>
+      </c>
+      <c r="O258" t="n">
+        <v>0</v>
+      </c>
+      <c r="P258" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q258" t="inlineStr"/>
+      <c r="R258" t="inlineStr"/>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>17</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I259" t="n">
+        <v>429</v>
+      </c>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="inlineStr"/>
+      <c r="L259" t="inlineStr"/>
+      <c r="M259" t="n">
+        <v>459</v>
+      </c>
+      <c r="N259" t="n">
+        <v>0</v>
+      </c>
+      <c r="O259" t="n">
+        <v>0</v>
+      </c>
+      <c r="P259" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q259" t="inlineStr"/>
+      <c r="R259" t="inlineStr"/>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>17</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I260" t="n">
+        <v>200</v>
+      </c>
+      <c r="J260" t="n">
+        <v>277</v>
+      </c>
+      <c r="K260" t="n">
+        <v>411</v>
+      </c>
+      <c r="L260" t="n">
+        <v>688</v>
+      </c>
+      <c r="M260" t="n">
+        <v>11977</v>
+      </c>
+      <c r="N260" t="n">
+        <v>2170</v>
+      </c>
+      <c r="O260" t="n">
+        <v>327</v>
+      </c>
+      <c r="P260" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr"/>
+      <c r="S260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>17</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I261" t="n">
+        <v>200</v>
+      </c>
+      <c r="J261" t="n">
+        <v>256</v>
+      </c>
+      <c r="K261" t="n">
+        <v>1007</v>
+      </c>
+      <c r="L261" t="n">
+        <v>1263</v>
+      </c>
+      <c r="M261" t="n">
+        <v>16346</v>
+      </c>
+      <c r="N261" t="n">
+        <v>5086</v>
+      </c>
+      <c r="O261" t="n">
+        <v>709</v>
+      </c>
+      <c r="P261" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr"/>
+      <c r="S261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>17</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I262" t="n">
+        <v>200</v>
+      </c>
+      <c r="J262" t="n">
+        <v>295</v>
+      </c>
+      <c r="K262" t="n">
+        <v>938</v>
+      </c>
+      <c r="L262" t="n">
+        <v>1233</v>
+      </c>
+      <c r="M262" t="n">
+        <v>27919</v>
+      </c>
+      <c r="N262" t="n">
+        <v>2715</v>
+      </c>
+      <c r="O262" t="n">
+        <v>378</v>
+      </c>
+      <c r="P262" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr"/>
+      <c r="S262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>17</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I263" t="n">
+        <v>200</v>
+      </c>
+      <c r="J263" t="n">
+        <v>332</v>
+      </c>
+      <c r="K263" t="n">
+        <v>1112</v>
+      </c>
+      <c r="L263" t="n">
+        <v>1444</v>
+      </c>
+      <c r="M263" t="n">
+        <v>25692</v>
+      </c>
+      <c r="N263" t="n">
+        <v>4473</v>
+      </c>
+      <c r="O263" t="n">
+        <v>676</v>
+      </c>
+      <c r="P263" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr"/>
+      <c r="S263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>17</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I264" t="n">
+        <v>200</v>
+      </c>
+      <c r="J264" t="n">
+        <v>288</v>
+      </c>
+      <c r="K264" t="n">
+        <v>1685</v>
+      </c>
+      <c r="L264" t="n">
+        <v>1973</v>
+      </c>
+      <c r="M264" t="n">
+        <v>64515</v>
+      </c>
+      <c r="N264" t="n">
+        <v>5062</v>
+      </c>
+      <c r="O264" t="n">
+        <v>711</v>
+      </c>
+      <c r="P264" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>responses/20260710T130300Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R264" t="inlineStr"/>
+      <c r="S264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>20260710T130300Z</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2026-07-10T13:03:00.336106+00:00</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>17</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I265" t="n">
+        <v>200</v>
+      </c>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="inlineStr"/>
+      <c r="L265" t="inlineStr"/>
+      <c r="M265" t="n">
+        <v>120397</v>
+      </c>
+      <c r="N265" t="n">
+        <v>0</v>
+      </c>
+      <c r="O265" t="n">
+        <v>0</v>
+      </c>
+      <c r="P265" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q265" t="inlineStr"/>
+      <c r="R265" t="inlineStr"/>
+      <c r="S265" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-11 18:02 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S265"/>
+  <dimension ref="A1:S281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16681,9 +16681,6 @@
       <c r="I250" t="n">
         <v>429</v>
       </c>
-      <c r="J250" t="inlineStr"/>
-      <c r="K250" t="inlineStr"/>
-      <c r="L250" t="inlineStr"/>
       <c r="M250" t="n">
         <v>171</v>
       </c>
@@ -16696,8 +16693,6 @@
       <c r="P250" t="n">
         <v>3</v>
       </c>
-      <c r="Q250" t="inlineStr"/>
-      <c r="R250" t="inlineStr"/>
       <c r="S250" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -16746,9 +16741,6 @@
       <c r="I251" t="n">
         <v>429</v>
       </c>
-      <c r="J251" t="inlineStr"/>
-      <c r="K251" t="inlineStr"/>
-      <c r="L251" t="inlineStr"/>
       <c r="M251" t="n">
         <v>461</v>
       </c>
@@ -16761,8 +16753,6 @@
       <c r="P251" t="n">
         <v>3</v>
       </c>
-      <c r="Q251" t="inlineStr"/>
-      <c r="R251" t="inlineStr"/>
       <c r="S251" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -16811,9 +16801,6 @@
       <c r="I252" t="n">
         <v>429</v>
       </c>
-      <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr"/>
-      <c r="L252" t="inlineStr"/>
       <c r="M252" t="n">
         <v>483</v>
       </c>
@@ -16826,8 +16813,6 @@
       <c r="P252" t="n">
         <v>3</v>
       </c>
-      <c r="Q252" t="inlineStr"/>
-      <c r="R252" t="inlineStr"/>
       <c r="S252" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -16876,9 +16861,6 @@
       <c r="I253" t="n">
         <v>429</v>
       </c>
-      <c r="J253" t="inlineStr"/>
-      <c r="K253" t="inlineStr"/>
-      <c r="L253" t="inlineStr"/>
       <c r="M253" t="n">
         <v>509</v>
       </c>
@@ -16891,8 +16873,6 @@
       <c r="P253" t="n">
         <v>3</v>
       </c>
-      <c r="Q253" t="inlineStr"/>
-      <c r="R253" t="inlineStr"/>
       <c r="S253" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -16941,9 +16921,6 @@
       <c r="I254" t="n">
         <v>404</v>
       </c>
-      <c r="J254" t="inlineStr"/>
-      <c r="K254" t="inlineStr"/>
-      <c r="L254" t="inlineStr"/>
       <c r="M254" t="n">
         <v>178</v>
       </c>
@@ -16956,8 +16933,6 @@
       <c r="P254" t="n">
         <v>1</v>
       </c>
-      <c r="Q254" t="inlineStr"/>
-      <c r="R254" t="inlineStr"/>
       <c r="S254" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -17006,9 +16981,6 @@
       <c r="I255" t="n">
         <v>429</v>
       </c>
-      <c r="J255" t="inlineStr"/>
-      <c r="K255" t="inlineStr"/>
-      <c r="L255" t="inlineStr"/>
       <c r="M255" t="n">
         <v>728</v>
       </c>
@@ -17021,8 +16993,6 @@
       <c r="P255" t="n">
         <v>3</v>
       </c>
-      <c r="Q255" t="inlineStr"/>
-      <c r="R255" t="inlineStr"/>
       <c r="S255" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -17071,9 +17041,6 @@
       <c r="I256" t="n">
         <v>429</v>
       </c>
-      <c r="J256" t="inlineStr"/>
-      <c r="K256" t="inlineStr"/>
-      <c r="L256" t="inlineStr"/>
       <c r="M256" t="n">
         <v>437</v>
       </c>
@@ -17086,8 +17053,6 @@
       <c r="P256" t="n">
         <v>3</v>
       </c>
-      <c r="Q256" t="inlineStr"/>
-      <c r="R256" t="inlineStr"/>
       <c r="S256" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -17136,9 +17101,6 @@
       <c r="I257" t="n">
         <v>200</v>
       </c>
-      <c r="J257" t="inlineStr"/>
-      <c r="K257" t="inlineStr"/>
-      <c r="L257" t="inlineStr"/>
       <c r="M257" t="n">
         <v>12504</v>
       </c>
@@ -17151,9 +17113,6 @@
       <c r="P257" t="n">
         <v>3</v>
       </c>
-      <c r="Q257" t="inlineStr"/>
-      <c r="R257" t="inlineStr"/>
-      <c r="S257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -17223,8 +17182,6 @@
           <t>responses/20260710T130300Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R258" t="inlineStr"/>
-      <c r="S258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -17294,8 +17251,6 @@
           <t>responses/20260710T130300Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R259" t="inlineStr"/>
-      <c r="S259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -17365,8 +17320,6 @@
           <t>responses/20260710T130300Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R260" t="inlineStr"/>
-      <c r="S260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -17436,8 +17389,6 @@
           <t>responses/20260710T130300Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R261" t="inlineStr"/>
-      <c r="S261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -17507,8 +17458,6 @@
           <t>responses/20260710T130300Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R262" t="inlineStr"/>
-      <c r="S262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -17578,8 +17527,6 @@
           <t>responses/20260710T130300Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R263" t="inlineStr"/>
-      <c r="S263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -17644,9 +17591,6 @@
       <c r="P264" t="n">
         <v>1</v>
       </c>
-      <c r="Q264" t="inlineStr"/>
-      <c r="R264" t="inlineStr"/>
-      <c r="S264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -17711,9 +17655,1092 @@
       <c r="P265" t="n">
         <v>1</v>
       </c>
-      <c r="Q265" t="inlineStr"/>
-      <c r="R265" t="inlineStr"/>
-      <c r="S265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>18</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I266" t="n">
+        <v>402</v>
+      </c>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="inlineStr"/>
+      <c r="L266" t="inlineStr"/>
+      <c r="M266" t="n">
+        <v>251</v>
+      </c>
+      <c r="N266" t="n">
+        <v>0</v>
+      </c>
+      <c r="O266" t="n">
+        <v>0</v>
+      </c>
+      <c r="P266" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q266" t="inlineStr"/>
+      <c r="R266" t="inlineStr"/>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>HTTP 402: {"error":{"message":"Provider returned error","code":402,"metadata":{"raw":"{\"error\":\"API key USD spend limit exceeded. Your account may still have USD balance, but this API key has reached its configured USD spending limit.\"}","provider_name":"Venice","is_byok":false,"retry_after_seconds":30,"r</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>18</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>429</v>
+      </c>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="inlineStr"/>
+      <c r="M267" t="n">
+        <v>221</v>
+      </c>
+      <c r="N267" t="n">
+        <v>0</v>
+      </c>
+      <c r="O267" t="n">
+        <v>0</v>
+      </c>
+      <c r="P267" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q267" t="inlineStr"/>
+      <c r="R267" t="inlineStr"/>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>18</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I268" t="n">
+        <v>429</v>
+      </c>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr"/>
+      <c r="L268" t="inlineStr"/>
+      <c r="M268" t="n">
+        <v>292</v>
+      </c>
+      <c r="N268" t="n">
+        <v>0</v>
+      </c>
+      <c r="O268" t="n">
+        <v>0</v>
+      </c>
+      <c r="P268" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q268" t="inlineStr"/>
+      <c r="R268" t="inlineStr"/>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>18</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>429</v>
+      </c>
+      <c r="J269" t="inlineStr"/>
+      <c r="K269" t="inlineStr"/>
+      <c r="L269" t="inlineStr"/>
+      <c r="M269" t="n">
+        <v>258</v>
+      </c>
+      <c r="N269" t="n">
+        <v>0</v>
+      </c>
+      <c r="O269" t="n">
+        <v>0</v>
+      </c>
+      <c r="P269" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q269" t="inlineStr"/>
+      <c r="R269" t="inlineStr"/>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>18</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>404</v>
+      </c>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr"/>
+      <c r="L270" t="inlineStr"/>
+      <c r="M270" t="n">
+        <v>75</v>
+      </c>
+      <c r="N270" t="n">
+        <v>0</v>
+      </c>
+      <c r="O270" t="n">
+        <v>0</v>
+      </c>
+      <c r="P270" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q270" t="inlineStr"/>
+      <c r="R270" t="inlineStr"/>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>18</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I271" t="n">
+        <v>429</v>
+      </c>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="inlineStr"/>
+      <c r="L271" t="inlineStr"/>
+      <c r="M271" t="n">
+        <v>548</v>
+      </c>
+      <c r="N271" t="n">
+        <v>0</v>
+      </c>
+      <c r="O271" t="n">
+        <v>0</v>
+      </c>
+      <c r="P271" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q271" t="inlineStr"/>
+      <c r="R271" t="inlineStr"/>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>18</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I272" t="n">
+        <v>429</v>
+      </c>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="inlineStr"/>
+      <c r="L272" t="inlineStr"/>
+      <c r="M272" t="n">
+        <v>369</v>
+      </c>
+      <c r="N272" t="n">
+        <v>0</v>
+      </c>
+      <c r="O272" t="n">
+        <v>0</v>
+      </c>
+      <c r="P272" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q272" t="inlineStr"/>
+      <c r="R272" t="inlineStr"/>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>18</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I273" t="n">
+        <v>200</v>
+      </c>
+      <c r="J273" t="n">
+        <v>88</v>
+      </c>
+      <c r="K273" t="n">
+        <v>4680</v>
+      </c>
+      <c r="L273" t="n">
+        <v>4768</v>
+      </c>
+      <c r="M273" t="n">
+        <v>17585</v>
+      </c>
+      <c r="N273" t="n">
+        <v>17651</v>
+      </c>
+      <c r="O273" t="n">
+        <v>1997</v>
+      </c>
+      <c r="P273" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr"/>
+      <c r="S273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>18</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I274" t="n">
+        <v>200</v>
+      </c>
+      <c r="J274" t="n">
+        <v>88</v>
+      </c>
+      <c r="K274" t="n">
+        <v>4413</v>
+      </c>
+      <c r="L274" t="n">
+        <v>4501</v>
+      </c>
+      <c r="M274" t="n">
+        <v>33366</v>
+      </c>
+      <c r="N274" t="n">
+        <v>17834</v>
+      </c>
+      <c r="O274" t="n">
+        <v>1949</v>
+      </c>
+      <c r="P274" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr"/>
+      <c r="S274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>18</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I275" t="n">
+        <v>200</v>
+      </c>
+      <c r="J275" t="n">
+        <v>86</v>
+      </c>
+      <c r="K275" t="n">
+        <v>2242</v>
+      </c>
+      <c r="L275" t="n">
+        <v>2328</v>
+      </c>
+      <c r="M275" t="n">
+        <v>58727</v>
+      </c>
+      <c r="N275" t="n">
+        <v>10512</v>
+      </c>
+      <c r="O275" t="n">
+        <v>991</v>
+      </c>
+      <c r="P275" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr"/>
+      <c r="S275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>18</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I276" t="n">
+        <v>200</v>
+      </c>
+      <c r="J276" t="n">
+        <v>73</v>
+      </c>
+      <c r="K276" t="n">
+        <v>2772</v>
+      </c>
+      <c r="L276" t="n">
+        <v>2845</v>
+      </c>
+      <c r="M276" t="n">
+        <v>62042</v>
+      </c>
+      <c r="N276" t="n">
+        <v>11590</v>
+      </c>
+      <c r="O276" t="n">
+        <v>1174</v>
+      </c>
+      <c r="P276" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R276" t="inlineStr"/>
+      <c r="S276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>18</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>200</v>
+      </c>
+      <c r="J277" t="n">
+        <v>139</v>
+      </c>
+      <c r="K277" t="n">
+        <v>5419</v>
+      </c>
+      <c r="L277" t="n">
+        <v>5558</v>
+      </c>
+      <c r="M277" t="n">
+        <v>82905</v>
+      </c>
+      <c r="N277" t="n">
+        <v>18697</v>
+      </c>
+      <c r="O277" t="n">
+        <v>2104</v>
+      </c>
+      <c r="P277" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr"/>
+      <c r="S277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>18</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>200</v>
+      </c>
+      <c r="J278" t="n">
+        <v>66</v>
+      </c>
+      <c r="K278" t="n">
+        <v>5995</v>
+      </c>
+      <c r="L278" t="n">
+        <v>6061</v>
+      </c>
+      <c r="M278" t="n">
+        <v>86168</v>
+      </c>
+      <c r="N278" t="n">
+        <v>28681</v>
+      </c>
+      <c r="O278" t="n">
+        <v>2510</v>
+      </c>
+      <c r="P278" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R278" t="inlineStr"/>
+      <c r="S278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>18</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>200</v>
+      </c>
+      <c r="J279" t="n">
+        <v>84</v>
+      </c>
+      <c r="K279" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L279" t="n">
+        <v>6084</v>
+      </c>
+      <c r="M279" t="n">
+        <v>125476</v>
+      </c>
+      <c r="N279" t="n">
+        <v>0</v>
+      </c>
+      <c r="O279" t="n">
+        <v>0</v>
+      </c>
+      <c r="P279" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q279" t="inlineStr"/>
+      <c r="R279" t="inlineStr"/>
+      <c r="S279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>18</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>200</v>
+      </c>
+      <c r="J280" t="n">
+        <v>88</v>
+      </c>
+      <c r="K280" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L280" t="n">
+        <v>6088</v>
+      </c>
+      <c r="M280" t="n">
+        <v>149721</v>
+      </c>
+      <c r="N280" t="n">
+        <v>26605</v>
+      </c>
+      <c r="O280" t="n">
+        <v>2655</v>
+      </c>
+      <c r="P280" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr"/>
+      <c r="S280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>18</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>200</v>
+      </c>
+      <c r="J281" t="n">
+        <v>81</v>
+      </c>
+      <c r="K281" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L281" t="n">
+        <v>6081</v>
+      </c>
+      <c r="M281" t="n">
+        <v>159654</v>
+      </c>
+      <c r="N281" t="n">
+        <v>0</v>
+      </c>
+      <c r="O281" t="n">
+        <v>0</v>
+      </c>
+      <c r="P281" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q281" t="inlineStr"/>
+      <c r="R281" t="inlineStr"/>
+      <c r="S281" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17726,7 +18753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S265"/>
+  <dimension ref="A1:S281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34040,9 +35067,6 @@
       <c r="I250" t="n">
         <v>429</v>
       </c>
-      <c r="J250" t="inlineStr"/>
-      <c r="K250" t="inlineStr"/>
-      <c r="L250" t="inlineStr"/>
       <c r="M250" t="n">
         <v>177</v>
       </c>
@@ -34055,8 +35079,6 @@
       <c r="P250" t="n">
         <v>3</v>
       </c>
-      <c r="Q250" t="inlineStr"/>
-      <c r="R250" t="inlineStr"/>
       <c r="S250" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -34105,9 +35127,6 @@
       <c r="I251" t="n">
         <v>429</v>
       </c>
-      <c r="J251" t="inlineStr"/>
-      <c r="K251" t="inlineStr"/>
-      <c r="L251" t="inlineStr"/>
       <c r="M251" t="n">
         <v>691</v>
       </c>
@@ -34120,8 +35139,6 @@
       <c r="P251" t="n">
         <v>3</v>
       </c>
-      <c r="Q251" t="inlineStr"/>
-      <c r="R251" t="inlineStr"/>
       <c r="S251" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -34170,9 +35187,6 @@
       <c r="I252" t="n">
         <v>429</v>
       </c>
-      <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr"/>
-      <c r="L252" t="inlineStr"/>
       <c r="M252" t="n">
         <v>212</v>
       </c>
@@ -34185,8 +35199,6 @@
       <c r="P252" t="n">
         <v>3</v>
       </c>
-      <c r="Q252" t="inlineStr"/>
-      <c r="R252" t="inlineStr"/>
       <c r="S252" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -34235,9 +35247,6 @@
       <c r="I253" t="n">
         <v>429</v>
       </c>
-      <c r="J253" t="inlineStr"/>
-      <c r="K253" t="inlineStr"/>
-      <c r="L253" t="inlineStr"/>
       <c r="M253" t="n">
         <v>234</v>
       </c>
@@ -34250,8 +35259,6 @@
       <c r="P253" t="n">
         <v>3</v>
       </c>
-      <c r="Q253" t="inlineStr"/>
-      <c r="R253" t="inlineStr"/>
       <c r="S253" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -34300,9 +35307,6 @@
       <c r="I254" t="n">
         <v>429</v>
       </c>
-      <c r="J254" t="inlineStr"/>
-      <c r="K254" t="inlineStr"/>
-      <c r="L254" t="inlineStr"/>
       <c r="M254" t="n">
         <v>160</v>
       </c>
@@ -34315,8 +35319,6 @@
       <c r="P254" t="n">
         <v>3</v>
       </c>
-      <c r="Q254" t="inlineStr"/>
-      <c r="R254" t="inlineStr"/>
       <c r="S254" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -34365,9 +35367,6 @@
       <c r="I255" t="n">
         <v>429</v>
       </c>
-      <c r="J255" t="inlineStr"/>
-      <c r="K255" t="inlineStr"/>
-      <c r="L255" t="inlineStr"/>
       <c r="M255" t="n">
         <v>920</v>
       </c>
@@ -34380,8 +35379,6 @@
       <c r="P255" t="n">
         <v>3</v>
       </c>
-      <c r="Q255" t="inlineStr"/>
-      <c r="R255" t="inlineStr"/>
       <c r="S255" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -34430,9 +35427,6 @@
       <c r="I256" t="n">
         <v>429</v>
       </c>
-      <c r="J256" t="inlineStr"/>
-      <c r="K256" t="inlineStr"/>
-      <c r="L256" t="inlineStr"/>
       <c r="M256" t="n">
         <v>245</v>
       </c>
@@ -34445,8 +35439,6 @@
       <c r="P256" t="n">
         <v>3</v>
       </c>
-      <c r="Q256" t="inlineStr"/>
-      <c r="R256" t="inlineStr"/>
       <c r="S256" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","</t>
@@ -34495,9 +35487,6 @@
       <c r="I257" t="n">
         <v>404</v>
       </c>
-      <c r="J257" t="inlineStr"/>
-      <c r="K257" t="inlineStr"/>
-      <c r="L257" t="inlineStr"/>
       <c r="M257" t="n">
         <v>103</v>
       </c>
@@ -34510,8 +35499,6 @@
       <c r="P257" t="n">
         <v>1</v>
       </c>
-      <c r="Q257" t="inlineStr"/>
-      <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -34586,8 +35573,6 @@
           <t>responses/20260710T130300Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R258" t="inlineStr"/>
-      <c r="S258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -34657,8 +35642,6 @@
           <t>responses/20260710T130300Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R259" t="inlineStr"/>
-      <c r="S259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -34728,8 +35711,6 @@
           <t>responses/20260710T130300Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R260" t="inlineStr"/>
-      <c r="S260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -34799,8 +35780,6 @@
           <t>responses/20260710T130300Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R261" t="inlineStr"/>
-      <c r="S261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -34870,8 +35849,6 @@
           <t>responses/20260710T130300Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R262" t="inlineStr"/>
-      <c r="S262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -34941,8 +35918,6 @@
           <t>responses/20260710T130300Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R263" t="inlineStr"/>
-      <c r="S263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -34986,9 +35961,6 @@
       <c r="I264" t="n">
         <v>200</v>
       </c>
-      <c r="J264" t="inlineStr"/>
-      <c r="K264" t="inlineStr"/>
-      <c r="L264" t="inlineStr"/>
       <c r="M264" t="n">
         <v>120250</v>
       </c>
@@ -35001,9 +35973,6 @@
       <c r="P264" t="n">
         <v>1</v>
       </c>
-      <c r="Q264" t="inlineStr"/>
-      <c r="R264" t="inlineStr"/>
-      <c r="S264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -35073,8 +36042,1096 @@
           <t>responses/20260710T130300Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R265" t="inlineStr"/>
-      <c r="S265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>18</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I266" t="n">
+        <v>429</v>
+      </c>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="inlineStr"/>
+      <c r="L266" t="inlineStr"/>
+      <c r="M266" t="n">
+        <v>282</v>
+      </c>
+      <c r="N266" t="n">
+        <v>0</v>
+      </c>
+      <c r="O266" t="n">
+        <v>0</v>
+      </c>
+      <c r="P266" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q266" t="inlineStr"/>
+      <c r="R266" t="inlineStr"/>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>18</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>429</v>
+      </c>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="inlineStr"/>
+      <c r="M267" t="n">
+        <v>374</v>
+      </c>
+      <c r="N267" t="n">
+        <v>0</v>
+      </c>
+      <c r="O267" t="n">
+        <v>0</v>
+      </c>
+      <c r="P267" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q267" t="inlineStr"/>
+      <c r="R267" t="inlineStr"/>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>18</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I268" t="n">
+        <v>402</v>
+      </c>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr"/>
+      <c r="L268" t="inlineStr"/>
+      <c r="M268" t="n">
+        <v>521</v>
+      </c>
+      <c r="N268" t="n">
+        <v>0</v>
+      </c>
+      <c r="O268" t="n">
+        <v>0</v>
+      </c>
+      <c r="P268" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q268" t="inlineStr"/>
+      <c r="R268" t="inlineStr"/>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>HTTP 402: {"error":{"message":"Provider returned error","code":402,"metadata":{"raw":"{\"error\":\"API key USD spend limit exceeded. Your account may still have USD balance, but this API key has reached its configured USD spending limit.\"}","provider_name":"Venice","is_byok":false,"retry_after_seconds":30,"r</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>18</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>200</v>
+      </c>
+      <c r="J269" t="n">
+        <v>73</v>
+      </c>
+      <c r="K269" t="n">
+        <v>5078</v>
+      </c>
+      <c r="L269" t="n">
+        <v>5151</v>
+      </c>
+      <c r="M269" t="n">
+        <v>49413</v>
+      </c>
+      <c r="N269" t="n">
+        <v>16430</v>
+      </c>
+      <c r="O269" t="n">
+        <v>2288</v>
+      </c>
+      <c r="P269" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr"/>
+      <c r="S269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>18</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>429</v>
+      </c>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr"/>
+      <c r="L270" t="inlineStr"/>
+      <c r="M270" t="n">
+        <v>253</v>
+      </c>
+      <c r="N270" t="n">
+        <v>0</v>
+      </c>
+      <c r="O270" t="n">
+        <v>0</v>
+      </c>
+      <c r="P270" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q270" t="inlineStr"/>
+      <c r="R270" t="inlineStr"/>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>18</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I271" t="n">
+        <v>429</v>
+      </c>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="inlineStr"/>
+      <c r="L271" t="inlineStr"/>
+      <c r="M271" t="n">
+        <v>202</v>
+      </c>
+      <c r="N271" t="n">
+        <v>0</v>
+      </c>
+      <c r="O271" t="n">
+        <v>0</v>
+      </c>
+      <c r="P271" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q271" t="inlineStr"/>
+      <c r="R271" t="inlineStr"/>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>18</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I272" t="n">
+        <v>200</v>
+      </c>
+      <c r="J272" t="n">
+        <v>73</v>
+      </c>
+      <c r="K272" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L272" t="n">
+        <v>8073</v>
+      </c>
+      <c r="M272" t="n">
+        <v>38095</v>
+      </c>
+      <c r="N272" t="n">
+        <v>22696</v>
+      </c>
+      <c r="O272" t="n">
+        <v>4072</v>
+      </c>
+      <c r="P272" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr"/>
+      <c r="S272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>18</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I273" t="n">
+        <v>200</v>
+      </c>
+      <c r="J273" t="n">
+        <v>56</v>
+      </c>
+      <c r="K273" t="n">
+        <v>1986</v>
+      </c>
+      <c r="L273" t="n">
+        <v>2042</v>
+      </c>
+      <c r="M273" t="n">
+        <v>42657</v>
+      </c>
+      <c r="N273" t="n">
+        <v>8092</v>
+      </c>
+      <c r="O273" t="n">
+        <v>1276</v>
+      </c>
+      <c r="P273" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr"/>
+      <c r="S273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>18</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I274" t="n">
+        <v>404</v>
+      </c>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="inlineStr"/>
+      <c r="L274" t="inlineStr"/>
+      <c r="M274" t="n">
+        <v>105</v>
+      </c>
+      <c r="N274" t="n">
+        <v>0</v>
+      </c>
+      <c r="O274" t="n">
+        <v>0</v>
+      </c>
+      <c r="P274" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q274" t="inlineStr"/>
+      <c r="R274" t="inlineStr"/>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>18</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I275" t="n">
+        <v>200</v>
+      </c>
+      <c r="J275" t="n">
+        <v>73</v>
+      </c>
+      <c r="K275" t="n">
+        <v>7665</v>
+      </c>
+      <c r="L275" t="n">
+        <v>7738</v>
+      </c>
+      <c r="M275" t="n">
+        <v>82245</v>
+      </c>
+      <c r="N275" t="n">
+        <v>28264</v>
+      </c>
+      <c r="O275" t="n">
+        <v>3884</v>
+      </c>
+      <c r="P275" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr"/>
+      <c r="S275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>18</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I276" t="n">
+        <v>200</v>
+      </c>
+      <c r="J276" t="n">
+        <v>56</v>
+      </c>
+      <c r="K276" t="n">
+        <v>2352</v>
+      </c>
+      <c r="L276" t="n">
+        <v>2408</v>
+      </c>
+      <c r="M276" t="n">
+        <v>67314</v>
+      </c>
+      <c r="N276" t="n">
+        <v>9738</v>
+      </c>
+      <c r="O276" t="n">
+        <v>1493</v>
+      </c>
+      <c r="P276" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R276" t="inlineStr"/>
+      <c r="S276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>18</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>200</v>
+      </c>
+      <c r="J277" t="n">
+        <v>69</v>
+      </c>
+      <c r="K277" t="n">
+        <v>3166</v>
+      </c>
+      <c r="L277" t="n">
+        <v>3235</v>
+      </c>
+      <c r="M277" t="n">
+        <v>96156</v>
+      </c>
+      <c r="N277" t="n">
+        <v>11012</v>
+      </c>
+      <c r="O277" t="n">
+        <v>1542</v>
+      </c>
+      <c r="P277" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr"/>
+      <c r="S277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>18</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>200</v>
+      </c>
+      <c r="J278" t="n">
+        <v>51</v>
+      </c>
+      <c r="K278" t="n">
+        <v>7998</v>
+      </c>
+      <c r="L278" t="n">
+        <v>8049</v>
+      </c>
+      <c r="M278" t="n">
+        <v>97361</v>
+      </c>
+      <c r="N278" t="n">
+        <v>32443</v>
+      </c>
+      <c r="O278" t="n">
+        <v>4528</v>
+      </c>
+      <c r="P278" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R278" t="inlineStr"/>
+      <c r="S278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>18</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>200</v>
+      </c>
+      <c r="J279" t="n">
+        <v>69</v>
+      </c>
+      <c r="K279" t="n">
+        <v>4715</v>
+      </c>
+      <c r="L279" t="n">
+        <v>4784</v>
+      </c>
+      <c r="M279" t="n">
+        <v>88200</v>
+      </c>
+      <c r="N279" t="n">
+        <v>12370</v>
+      </c>
+      <c r="O279" t="n">
+        <v>1772</v>
+      </c>
+      <c r="P279" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr"/>
+      <c r="S279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>18</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>200</v>
+      </c>
+      <c r="J280" t="n">
+        <v>70</v>
+      </c>
+      <c r="K280" t="n">
+        <v>2819</v>
+      </c>
+      <c r="L280" t="n">
+        <v>2889</v>
+      </c>
+      <c r="M280" t="n">
+        <v>120546</v>
+      </c>
+      <c r="N280" t="n">
+        <v>9661</v>
+      </c>
+      <c r="O280" t="n">
+        <v>1603</v>
+      </c>
+      <c r="P280" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr"/>
+      <c r="S280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>18</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>200</v>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="inlineStr"/>
+      <c r="L281" t="inlineStr"/>
+      <c r="M281" t="n">
+        <v>120355</v>
+      </c>
+      <c r="N281" t="n">
+        <v>0</v>
+      </c>
+      <c r="O281" t="n">
+        <v>0</v>
+      </c>
+      <c r="P281" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q281" t="inlineStr"/>
+      <c r="R281" t="inlineStr"/>
+      <c r="S281" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -35087,7 +37144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S265"/>
+  <dimension ref="A1:S281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51355,8 +53412,6 @@
           <t>responses/20260710T130300Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R250" t="inlineStr"/>
-      <c r="S250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -51400,9 +53455,6 @@
       <c r="I251" t="n">
         <v>429</v>
       </c>
-      <c r="J251" t="inlineStr"/>
-      <c r="K251" t="inlineStr"/>
-      <c r="L251" t="inlineStr"/>
       <c r="M251" t="n">
         <v>188</v>
       </c>
@@ -51415,8 +53467,6 @@
       <c r="P251" t="n">
         <v>3</v>
       </c>
-      <c r="Q251" t="inlineStr"/>
-      <c r="R251" t="inlineStr"/>
       <c r="S251" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -51465,9 +53515,6 @@
       <c r="I252" t="n">
         <v>429</v>
       </c>
-      <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr"/>
-      <c r="L252" t="inlineStr"/>
       <c r="M252" t="n">
         <v>339</v>
       </c>
@@ -51480,8 +53527,6 @@
       <c r="P252" t="n">
         <v>3</v>
       </c>
-      <c r="Q252" t="inlineStr"/>
-      <c r="R252" t="inlineStr"/>
       <c r="S252" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -51556,8 +53601,6 @@
           <t>responses/20260710T130300Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R253" t="inlineStr"/>
-      <c r="S253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -51601,9 +53644,6 @@
       <c r="I254" t="n">
         <v>429</v>
       </c>
-      <c r="J254" t="inlineStr"/>
-      <c r="K254" t="inlineStr"/>
-      <c r="L254" t="inlineStr"/>
       <c r="M254" t="n">
         <v>264</v>
       </c>
@@ -51616,8 +53656,6 @@
       <c r="P254" t="n">
         <v>3</v>
       </c>
-      <c r="Q254" t="inlineStr"/>
-      <c r="R254" t="inlineStr"/>
       <c r="S254" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -51666,9 +53704,6 @@
       <c r="I255" t="n">
         <v>429</v>
       </c>
-      <c r="J255" t="inlineStr"/>
-      <c r="K255" t="inlineStr"/>
-      <c r="L255" t="inlineStr"/>
       <c r="M255" t="n">
         <v>705</v>
       </c>
@@ -51681,8 +53716,6 @@
       <c r="P255" t="n">
         <v>3</v>
       </c>
-      <c r="Q255" t="inlineStr"/>
-      <c r="R255" t="inlineStr"/>
       <c r="S255" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -51757,8 +53790,6 @@
           <t>responses/20260710T130300Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R256" t="inlineStr"/>
-      <c r="S256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -51802,9 +53833,6 @@
       <c r="I257" t="n">
         <v>429</v>
       </c>
-      <c r="J257" t="inlineStr"/>
-      <c r="K257" t="inlineStr"/>
-      <c r="L257" t="inlineStr"/>
       <c r="M257" t="n">
         <v>453</v>
       </c>
@@ -51817,8 +53845,6 @@
       <c r="P257" t="n">
         <v>3</v>
       </c>
-      <c r="Q257" t="inlineStr"/>
-      <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -51867,9 +53893,6 @@
       <c r="I258" t="n">
         <v>404</v>
       </c>
-      <c r="J258" t="inlineStr"/>
-      <c r="K258" t="inlineStr"/>
-      <c r="L258" t="inlineStr"/>
       <c r="M258" t="n">
         <v>92</v>
       </c>
@@ -51882,8 +53905,6 @@
       <c r="P258" t="n">
         <v>1</v>
       </c>
-      <c r="Q258" t="inlineStr"/>
-      <c r="R258" t="inlineStr"/>
       <c r="S258" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -51932,9 +53953,6 @@
       <c r="I259" t="n">
         <v>429</v>
       </c>
-      <c r="J259" t="inlineStr"/>
-      <c r="K259" t="inlineStr"/>
-      <c r="L259" t="inlineStr"/>
       <c r="M259" t="n">
         <v>459</v>
       </c>
@@ -51947,8 +53965,6 @@
       <c r="P259" t="n">
         <v>3</v>
       </c>
-      <c r="Q259" t="inlineStr"/>
-      <c r="R259" t="inlineStr"/>
       <c r="S259" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -52023,8 +54039,6 @@
           <t>responses/20260710T130300Z/email/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R260" t="inlineStr"/>
-      <c r="S260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -52094,8 +54108,6 @@
           <t>responses/20260710T130300Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R261" t="inlineStr"/>
-      <c r="S261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -52165,8 +54177,6 @@
           <t>responses/20260710T130300Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R262" t="inlineStr"/>
-      <c r="S262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -52236,8 +54246,6 @@
           <t>responses/20260710T130300Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R263" t="inlineStr"/>
-      <c r="S263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -52307,8 +54315,6 @@
           <t>responses/20260710T130300Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R264" t="inlineStr"/>
-      <c r="S264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -52352,9 +54358,6 @@
       <c r="I265" t="n">
         <v>200</v>
       </c>
-      <c r="J265" t="inlineStr"/>
-      <c r="K265" t="inlineStr"/>
-      <c r="L265" t="inlineStr"/>
       <c r="M265" t="n">
         <v>120397</v>
       </c>
@@ -52367,9 +54370,1084 @@
       <c r="P265" t="n">
         <v>1</v>
       </c>
-      <c r="Q265" t="inlineStr"/>
-      <c r="R265" t="inlineStr"/>
-      <c r="S265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>18</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I266" t="n">
+        <v>200</v>
+      </c>
+      <c r="J266" t="n">
+        <v>292</v>
+      </c>
+      <c r="K266" t="n">
+        <v>809</v>
+      </c>
+      <c r="L266" t="n">
+        <v>1101</v>
+      </c>
+      <c r="M266" t="n">
+        <v>31352</v>
+      </c>
+      <c r="N266" t="n">
+        <v>2923</v>
+      </c>
+      <c r="O266" t="n">
+        <v>442</v>
+      </c>
+      <c r="P266" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R266" t="inlineStr"/>
+      <c r="S266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>18</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>429</v>
+      </c>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="inlineStr"/>
+      <c r="M267" t="n">
+        <v>233</v>
+      </c>
+      <c r="N267" t="n">
+        <v>0</v>
+      </c>
+      <c r="O267" t="n">
+        <v>0</v>
+      </c>
+      <c r="P267" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q267" t="inlineStr"/>
+      <c r="R267" t="inlineStr"/>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>18</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I268" t="n">
+        <v>429</v>
+      </c>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr"/>
+      <c r="L268" t="inlineStr"/>
+      <c r="M268" t="n">
+        <v>573</v>
+      </c>
+      <c r="N268" t="n">
+        <v>0</v>
+      </c>
+      <c r="O268" t="n">
+        <v>0</v>
+      </c>
+      <c r="P268" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q268" t="inlineStr"/>
+      <c r="R268" t="inlineStr"/>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>18</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>200</v>
+      </c>
+      <c r="J269" t="n">
+        <v>292</v>
+      </c>
+      <c r="K269" t="n">
+        <v>859</v>
+      </c>
+      <c r="L269" t="n">
+        <v>1151</v>
+      </c>
+      <c r="M269" t="n">
+        <v>11452</v>
+      </c>
+      <c r="N269" t="n">
+        <v>3679</v>
+      </c>
+      <c r="O269" t="n">
+        <v>531</v>
+      </c>
+      <c r="P269" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr"/>
+      <c r="S269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>18</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>429</v>
+      </c>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr"/>
+      <c r="L270" t="inlineStr"/>
+      <c r="M270" t="n">
+        <v>292</v>
+      </c>
+      <c r="N270" t="n">
+        <v>0</v>
+      </c>
+      <c r="O270" t="n">
+        <v>0</v>
+      </c>
+      <c r="P270" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q270" t="inlineStr"/>
+      <c r="R270" t="inlineStr"/>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>18</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I271" t="n">
+        <v>429</v>
+      </c>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="inlineStr"/>
+      <c r="L271" t="inlineStr"/>
+      <c r="M271" t="n">
+        <v>258</v>
+      </c>
+      <c r="N271" t="n">
+        <v>0</v>
+      </c>
+      <c r="O271" t="n">
+        <v>0</v>
+      </c>
+      <c r="P271" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q271" t="inlineStr"/>
+      <c r="R271" t="inlineStr"/>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>18</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I272" t="n">
+        <v>429</v>
+      </c>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="inlineStr"/>
+      <c r="L272" t="inlineStr"/>
+      <c r="M272" t="n">
+        <v>406</v>
+      </c>
+      <c r="N272" t="n">
+        <v>0</v>
+      </c>
+      <c r="O272" t="n">
+        <v>0</v>
+      </c>
+      <c r="P272" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q272" t="inlineStr"/>
+      <c r="R272" t="inlineStr"/>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>18</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I273" t="n">
+        <v>429</v>
+      </c>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="inlineStr"/>
+      <c r="L273" t="inlineStr"/>
+      <c r="M273" t="n">
+        <v>224</v>
+      </c>
+      <c r="N273" t="n">
+        <v>0</v>
+      </c>
+      <c r="O273" t="n">
+        <v>0</v>
+      </c>
+      <c r="P273" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q273" t="inlineStr"/>
+      <c r="R273" t="inlineStr"/>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>18</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I274" t="n">
+        <v>404</v>
+      </c>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="inlineStr"/>
+      <c r="L274" t="inlineStr"/>
+      <c r="M274" t="n">
+        <v>52</v>
+      </c>
+      <c r="N274" t="n">
+        <v>0</v>
+      </c>
+      <c r="O274" t="n">
+        <v>0</v>
+      </c>
+      <c r="P274" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q274" t="inlineStr"/>
+      <c r="R274" t="inlineStr"/>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>18</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I275" t="n">
+        <v>200</v>
+      </c>
+      <c r="J275" t="n">
+        <v>292</v>
+      </c>
+      <c r="K275" t="n">
+        <v>701</v>
+      </c>
+      <c r="L275" t="n">
+        <v>993</v>
+      </c>
+      <c r="M275" t="n">
+        <v>4655</v>
+      </c>
+      <c r="N275" t="n">
+        <v>3164</v>
+      </c>
+      <c r="O275" t="n">
+        <v>439</v>
+      </c>
+      <c r="P275" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr"/>
+      <c r="S275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>18</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I276" t="n">
+        <v>429</v>
+      </c>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="inlineStr"/>
+      <c r="L276" t="inlineStr"/>
+      <c r="M276" t="n">
+        <v>1800</v>
+      </c>
+      <c r="N276" t="n">
+        <v>0</v>
+      </c>
+      <c r="O276" t="n">
+        <v>0</v>
+      </c>
+      <c r="P276" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q276" t="inlineStr"/>
+      <c r="R276" t="inlineStr"/>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>18</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>200</v>
+      </c>
+      <c r="J277" t="n">
+        <v>256</v>
+      </c>
+      <c r="K277" t="n">
+        <v>1117</v>
+      </c>
+      <c r="L277" t="n">
+        <v>1373</v>
+      </c>
+      <c r="M277" t="n">
+        <v>12822</v>
+      </c>
+      <c r="N277" t="n">
+        <v>5202</v>
+      </c>
+      <c r="O277" t="n">
+        <v>744</v>
+      </c>
+      <c r="P277" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr"/>
+      <c r="S277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>18</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>200</v>
+      </c>
+      <c r="J278" t="n">
+        <v>295</v>
+      </c>
+      <c r="K278" t="n">
+        <v>944</v>
+      </c>
+      <c r="L278" t="n">
+        <v>1239</v>
+      </c>
+      <c r="M278" t="n">
+        <v>24175</v>
+      </c>
+      <c r="N278" t="n">
+        <v>2945</v>
+      </c>
+      <c r="O278" t="n">
+        <v>420</v>
+      </c>
+      <c r="P278" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R278" t="inlineStr"/>
+      <c r="S278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>18</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>200</v>
+      </c>
+      <c r="J279" t="n">
+        <v>332</v>
+      </c>
+      <c r="K279" t="n">
+        <v>830</v>
+      </c>
+      <c r="L279" t="n">
+        <v>1162</v>
+      </c>
+      <c r="M279" t="n">
+        <v>26929</v>
+      </c>
+      <c r="N279" t="n">
+        <v>3860</v>
+      </c>
+      <c r="O279" t="n">
+        <v>583</v>
+      </c>
+      <c r="P279" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr"/>
+      <c r="S279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>18</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>200</v>
+      </c>
+      <c r="J280" t="n">
+        <v>288</v>
+      </c>
+      <c r="K280" t="n">
+        <v>1588</v>
+      </c>
+      <c r="L280" t="n">
+        <v>1876</v>
+      </c>
+      <c r="M280" t="n">
+        <v>48690</v>
+      </c>
+      <c r="N280" t="n">
+        <v>4849</v>
+      </c>
+      <c r="O280" t="n">
+        <v>675</v>
+      </c>
+      <c r="P280" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>responses/20260711T175732Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr"/>
+      <c r="S280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>20260711T175732Z</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-07-11T17:57:32.338560+00:00</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>18</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Reply professionally to this email in at least 200 words: Subject: Question abou</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>200</v>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="inlineStr"/>
+      <c r="L281" t="inlineStr"/>
+      <c r="M281" t="n">
+        <v>120499</v>
+      </c>
+      <c r="N281" t="n">
+        <v>0</v>
+      </c>
+      <c r="O281" t="n">
+        <v>0</v>
+      </c>
+      <c r="P281" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q281" t="inlineStr"/>
+      <c r="R281" t="inlineStr"/>
+      <c r="S281" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-12 05:37 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S281"/>
+  <dimension ref="A1:S297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17698,9 +17698,6 @@
       <c r="I266" t="n">
         <v>402</v>
       </c>
-      <c r="J266" t="inlineStr"/>
-      <c r="K266" t="inlineStr"/>
-      <c r="L266" t="inlineStr"/>
       <c r="M266" t="n">
         <v>251</v>
       </c>
@@ -17713,8 +17710,6 @@
       <c r="P266" t="n">
         <v>2</v>
       </c>
-      <c r="Q266" t="inlineStr"/>
-      <c r="R266" t="inlineStr"/>
       <c r="S266" t="inlineStr">
         <is>
           <t>HTTP 402: {"error":{"message":"Provider returned error","code":402,"metadata":{"raw":"{\"error\":\"API key USD spend limit exceeded. Your account may still have USD balance, but this API key has reached its configured USD spending limit.\"}","provider_name":"Venice","is_byok":false,"retry_after_seconds":30,"r</t>
@@ -17763,9 +17758,6 @@
       <c r="I267" t="n">
         <v>429</v>
       </c>
-      <c r="J267" t="inlineStr"/>
-      <c r="K267" t="inlineStr"/>
-      <c r="L267" t="inlineStr"/>
       <c r="M267" t="n">
         <v>221</v>
       </c>
@@ -17778,8 +17770,6 @@
       <c r="P267" t="n">
         <v>3</v>
       </c>
-      <c r="Q267" t="inlineStr"/>
-      <c r="R267" t="inlineStr"/>
       <c r="S267" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -17828,9 +17818,6 @@
       <c r="I268" t="n">
         <v>429</v>
       </c>
-      <c r="J268" t="inlineStr"/>
-      <c r="K268" t="inlineStr"/>
-      <c r="L268" t="inlineStr"/>
       <c r="M268" t="n">
         <v>292</v>
       </c>
@@ -17843,8 +17830,6 @@
       <c r="P268" t="n">
         <v>3</v>
       </c>
-      <c r="Q268" t="inlineStr"/>
-      <c r="R268" t="inlineStr"/>
       <c r="S268" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -17893,9 +17878,6 @@
       <c r="I269" t="n">
         <v>429</v>
       </c>
-      <c r="J269" t="inlineStr"/>
-      <c r="K269" t="inlineStr"/>
-      <c r="L269" t="inlineStr"/>
       <c r="M269" t="n">
         <v>258</v>
       </c>
@@ -17908,8 +17890,6 @@
       <c r="P269" t="n">
         <v>3</v>
       </c>
-      <c r="Q269" t="inlineStr"/>
-      <c r="R269" t="inlineStr"/>
       <c r="S269" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -17958,9 +17938,6 @@
       <c r="I270" t="n">
         <v>404</v>
       </c>
-      <c r="J270" t="inlineStr"/>
-      <c r="K270" t="inlineStr"/>
-      <c r="L270" t="inlineStr"/>
       <c r="M270" t="n">
         <v>75</v>
       </c>
@@ -17973,8 +17950,6 @@
       <c r="P270" t="n">
         <v>1</v>
       </c>
-      <c r="Q270" t="inlineStr"/>
-      <c r="R270" t="inlineStr"/>
       <c r="S270" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -18023,9 +17998,6 @@
       <c r="I271" t="n">
         <v>429</v>
       </c>
-      <c r="J271" t="inlineStr"/>
-      <c r="K271" t="inlineStr"/>
-      <c r="L271" t="inlineStr"/>
       <c r="M271" t="n">
         <v>548</v>
       </c>
@@ -18038,8 +18010,6 @@
       <c r="P271" t="n">
         <v>3</v>
       </c>
-      <c r="Q271" t="inlineStr"/>
-      <c r="R271" t="inlineStr"/>
       <c r="S271" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -18088,9 +18058,6 @@
       <c r="I272" t="n">
         <v>429</v>
       </c>
-      <c r="J272" t="inlineStr"/>
-      <c r="K272" t="inlineStr"/>
-      <c r="L272" t="inlineStr"/>
       <c r="M272" t="n">
         <v>369</v>
       </c>
@@ -18103,8 +18070,6 @@
       <c r="P272" t="n">
         <v>3</v>
       </c>
-      <c r="Q272" t="inlineStr"/>
-      <c r="R272" t="inlineStr"/>
       <c r="S272" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -18179,8 +18144,6 @@
           <t>responses/20260711T175732Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R273" t="inlineStr"/>
-      <c r="S273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -18250,8 +18213,6 @@
           <t>responses/20260711T175732Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R274" t="inlineStr"/>
-      <c r="S274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -18321,8 +18282,6 @@
           <t>responses/20260711T175732Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
         </is>
       </c>
-      <c r="R275" t="inlineStr"/>
-      <c r="S275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -18392,8 +18351,6 @@
           <t>responses/20260711T175732Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R276" t="inlineStr"/>
-      <c r="S276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -18463,8 +18420,6 @@
           <t>responses/20260711T175732Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R277" t="inlineStr"/>
-      <c r="S277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -18534,8 +18489,6 @@
           <t>responses/20260711T175732Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R278" t="inlineStr"/>
-      <c r="S278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -18600,9 +18553,6 @@
       <c r="P279" t="n">
         <v>1</v>
       </c>
-      <c r="Q279" t="inlineStr"/>
-      <c r="R279" t="inlineStr"/>
-      <c r="S279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -18672,8 +18622,6 @@
           <t>responses/20260711T175732Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R280" t="inlineStr"/>
-      <c r="S280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -18738,9 +18686,1084 @@
       <c r="P281" t="n">
         <v>1</v>
       </c>
-      <c r="Q281" t="inlineStr"/>
-      <c r="R281" t="inlineStr"/>
-      <c r="S281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>19</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>200</v>
+      </c>
+      <c r="J282" t="n">
+        <v>348</v>
+      </c>
+      <c r="K282" t="n">
+        <v>59</v>
+      </c>
+      <c r="L282" t="n">
+        <v>407</v>
+      </c>
+      <c r="M282" t="n">
+        <v>4778</v>
+      </c>
+      <c r="N282" t="n">
+        <v>44</v>
+      </c>
+      <c r="O282" t="n">
+        <v>8</v>
+      </c>
+      <c r="P282" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr"/>
+      <c r="S282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>19</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>200</v>
+      </c>
+      <c r="J283" t="n">
+        <v>299</v>
+      </c>
+      <c r="K283" t="n">
+        <v>825</v>
+      </c>
+      <c r="L283" t="n">
+        <v>1124</v>
+      </c>
+      <c r="M283" t="n">
+        <v>9216</v>
+      </c>
+      <c r="N283" t="n">
+        <v>3188</v>
+      </c>
+      <c r="O283" t="n">
+        <v>457</v>
+      </c>
+      <c r="P283" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr"/>
+      <c r="S283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>19</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>429</v>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr"/>
+      <c r="L284" t="inlineStr"/>
+      <c r="M284" t="n">
+        <v>98</v>
+      </c>
+      <c r="N284" t="n">
+        <v>0</v>
+      </c>
+      <c r="O284" t="n">
+        <v>0</v>
+      </c>
+      <c r="P284" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q284" t="inlineStr"/>
+      <c r="R284" t="inlineStr"/>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>19</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>429</v>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr"/>
+      <c r="L285" t="inlineStr"/>
+      <c r="M285" t="n">
+        <v>170</v>
+      </c>
+      <c r="N285" t="n">
+        <v>0</v>
+      </c>
+      <c r="O285" t="n">
+        <v>0</v>
+      </c>
+      <c r="P285" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q285" t="inlineStr"/>
+      <c r="R285" t="inlineStr"/>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>19</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>429</v>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr"/>
+      <c r="L286" t="inlineStr"/>
+      <c r="M286" t="n">
+        <v>92</v>
+      </c>
+      <c r="N286" t="n">
+        <v>0</v>
+      </c>
+      <c r="O286" t="n">
+        <v>0</v>
+      </c>
+      <c r="P286" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q286" t="inlineStr"/>
+      <c r="R286" t="inlineStr"/>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>19</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>404</v>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr"/>
+      <c r="L287" t="inlineStr"/>
+      <c r="M287" t="n">
+        <v>38</v>
+      </c>
+      <c r="N287" t="n">
+        <v>0</v>
+      </c>
+      <c r="O287" t="n">
+        <v>0</v>
+      </c>
+      <c r="P287" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q287" t="inlineStr"/>
+      <c r="R287" t="inlineStr"/>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>19</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>429</v>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr"/>
+      <c r="L288" t="inlineStr"/>
+      <c r="M288" t="n">
+        <v>113</v>
+      </c>
+      <c r="N288" t="n">
+        <v>0</v>
+      </c>
+      <c r="O288" t="n">
+        <v>0</v>
+      </c>
+      <c r="P288" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q288" t="inlineStr"/>
+      <c r="R288" t="inlineStr"/>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>19</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>200</v>
+      </c>
+      <c r="J289" t="n">
+        <v>299</v>
+      </c>
+      <c r="K289" t="n">
+        <v>2067</v>
+      </c>
+      <c r="L289" t="n">
+        <v>2366</v>
+      </c>
+      <c r="M289" t="n">
+        <v>11873</v>
+      </c>
+      <c r="N289" t="n">
+        <v>4731</v>
+      </c>
+      <c r="O289" t="n">
+        <v>687</v>
+      </c>
+      <c r="P289" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr"/>
+      <c r="S289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>19</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>429</v>
+      </c>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr"/>
+      <c r="L290" t="inlineStr"/>
+      <c r="M290" t="n">
+        <v>269</v>
+      </c>
+      <c r="N290" t="n">
+        <v>0</v>
+      </c>
+      <c r="O290" t="n">
+        <v>0</v>
+      </c>
+      <c r="P290" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q290" t="inlineStr"/>
+      <c r="R290" t="inlineStr"/>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>19</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>200</v>
+      </c>
+      <c r="J291" t="n">
+        <v>350</v>
+      </c>
+      <c r="K291" t="n">
+        <v>991</v>
+      </c>
+      <c r="L291" t="n">
+        <v>1341</v>
+      </c>
+      <c r="M291" t="n">
+        <v>10181</v>
+      </c>
+      <c r="N291" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O291" t="n">
+        <v>326</v>
+      </c>
+      <c r="P291" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr"/>
+      <c r="S291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>19</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>200</v>
+      </c>
+      <c r="J292" t="n">
+        <v>305</v>
+      </c>
+      <c r="K292" t="n">
+        <v>2284</v>
+      </c>
+      <c r="L292" t="n">
+        <v>2589</v>
+      </c>
+      <c r="M292" t="n">
+        <v>29940</v>
+      </c>
+      <c r="N292" t="n">
+        <v>9156</v>
+      </c>
+      <c r="O292" t="n">
+        <v>995</v>
+      </c>
+      <c r="P292" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr"/>
+      <c r="S292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>19</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>200</v>
+      </c>
+      <c r="J293" t="n">
+        <v>299</v>
+      </c>
+      <c r="K293" t="n">
+        <v>1777</v>
+      </c>
+      <c r="L293" t="n">
+        <v>2076</v>
+      </c>
+      <c r="M293" t="n">
+        <v>38110</v>
+      </c>
+      <c r="N293" t="n">
+        <v>5086</v>
+      </c>
+      <c r="O293" t="n">
+        <v>735</v>
+      </c>
+      <c r="P293" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr"/>
+      <c r="S293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>19</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>200</v>
+      </c>
+      <c r="J294" t="n">
+        <v>274</v>
+      </c>
+      <c r="K294" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L294" t="n">
+        <v>6274</v>
+      </c>
+      <c r="M294" t="n">
+        <v>40662</v>
+      </c>
+      <c r="N294" t="n">
+        <v>0</v>
+      </c>
+      <c r="O294" t="n">
+        <v>0</v>
+      </c>
+      <c r="P294" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q294" t="inlineStr"/>
+      <c r="R294" t="inlineStr"/>
+      <c r="S294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>19</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>200</v>
+      </c>
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="inlineStr"/>
+      <c r="L295" t="inlineStr"/>
+      <c r="M295" t="n">
+        <v>57582</v>
+      </c>
+      <c r="N295" t="n">
+        <v>0</v>
+      </c>
+      <c r="O295" t="n">
+        <v>0</v>
+      </c>
+      <c r="P295" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q295" t="inlineStr"/>
+      <c r="R295" t="inlineStr"/>
+      <c r="S295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>19</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>200</v>
+      </c>
+      <c r="J296" t="n">
+        <v>299</v>
+      </c>
+      <c r="K296" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L296" t="n">
+        <v>6299</v>
+      </c>
+      <c r="M296" t="n">
+        <v>111417</v>
+      </c>
+      <c r="N296" t="n">
+        <v>0</v>
+      </c>
+      <c r="O296" t="n">
+        <v>0</v>
+      </c>
+      <c r="P296" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q296" t="inlineStr"/>
+      <c r="R296" t="inlineStr"/>
+      <c r="S296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>19</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write a single, self‑contained Java program that implements a highly concurrent </t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>200</v>
+      </c>
+      <c r="J297" t="n">
+        <v>295</v>
+      </c>
+      <c r="K297" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L297" t="n">
+        <v>6295</v>
+      </c>
+      <c r="M297" t="n">
+        <v>113794</v>
+      </c>
+      <c r="N297" t="n">
+        <v>0</v>
+      </c>
+      <c r="O297" t="n">
+        <v>0</v>
+      </c>
+      <c r="P297" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q297" t="inlineStr"/>
+      <c r="R297" t="inlineStr"/>
+      <c r="S297" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18753,7 +19776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S281"/>
+  <dimension ref="A1:S297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36085,9 +37108,6 @@
       <c r="I266" t="n">
         <v>429</v>
       </c>
-      <c r="J266" t="inlineStr"/>
-      <c r="K266" t="inlineStr"/>
-      <c r="L266" t="inlineStr"/>
       <c r="M266" t="n">
         <v>282</v>
       </c>
@@ -36100,8 +37120,6 @@
       <c r="P266" t="n">
         <v>3</v>
       </c>
-      <c r="Q266" t="inlineStr"/>
-      <c r="R266" t="inlineStr"/>
       <c r="S266" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -36150,9 +37168,6 @@
       <c r="I267" t="n">
         <v>429</v>
       </c>
-      <c r="J267" t="inlineStr"/>
-      <c r="K267" t="inlineStr"/>
-      <c r="L267" t="inlineStr"/>
       <c r="M267" t="n">
         <v>374</v>
       </c>
@@ -36165,8 +37180,6 @@
       <c r="P267" t="n">
         <v>3</v>
       </c>
-      <c r="Q267" t="inlineStr"/>
-      <c r="R267" t="inlineStr"/>
       <c r="S267" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -36215,9 +37228,6 @@
       <c r="I268" t="n">
         <v>402</v>
       </c>
-      <c r="J268" t="inlineStr"/>
-      <c r="K268" t="inlineStr"/>
-      <c r="L268" t="inlineStr"/>
       <c r="M268" t="n">
         <v>521</v>
       </c>
@@ -36230,8 +37240,6 @@
       <c r="P268" t="n">
         <v>3</v>
       </c>
-      <c r="Q268" t="inlineStr"/>
-      <c r="R268" t="inlineStr"/>
       <c r="S268" t="inlineStr">
         <is>
           <t>HTTP 402: {"error":{"message":"Provider returned error","code":402,"metadata":{"raw":"{\"error\":\"API key USD spend limit exceeded. Your account may still have USD balance, but this API key has reached its configured USD spending limit.\"}","provider_name":"Venice","is_byok":false,"retry_after_seconds":30,"r</t>
@@ -36306,8 +37314,6 @@
           <t>responses/20260711T175732Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R269" t="inlineStr"/>
-      <c r="S269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -36351,9 +37357,6 @@
       <c r="I270" t="n">
         <v>429</v>
       </c>
-      <c r="J270" t="inlineStr"/>
-      <c r="K270" t="inlineStr"/>
-      <c r="L270" t="inlineStr"/>
       <c r="M270" t="n">
         <v>253</v>
       </c>
@@ -36366,8 +37369,6 @@
       <c r="P270" t="n">
         <v>3</v>
       </c>
-      <c r="Q270" t="inlineStr"/>
-      <c r="R270" t="inlineStr"/>
       <c r="S270" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -36416,9 +37417,6 @@
       <c r="I271" t="n">
         <v>429</v>
       </c>
-      <c r="J271" t="inlineStr"/>
-      <c r="K271" t="inlineStr"/>
-      <c r="L271" t="inlineStr"/>
       <c r="M271" t="n">
         <v>202</v>
       </c>
@@ -36431,8 +37429,6 @@
       <c r="P271" t="n">
         <v>3</v>
       </c>
-      <c r="Q271" t="inlineStr"/>
-      <c r="R271" t="inlineStr"/>
       <c r="S271" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -36507,8 +37503,6 @@
           <t>responses/20260711T175732Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R272" t="inlineStr"/>
-      <c r="S272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -36578,8 +37572,6 @@
           <t>responses/20260711T175732Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R273" t="inlineStr"/>
-      <c r="S273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -36623,9 +37615,6 @@
       <c r="I274" t="n">
         <v>404</v>
       </c>
-      <c r="J274" t="inlineStr"/>
-      <c r="K274" t="inlineStr"/>
-      <c r="L274" t="inlineStr"/>
       <c r="M274" t="n">
         <v>105</v>
       </c>
@@ -36638,8 +37627,6 @@
       <c r="P274" t="n">
         <v>1</v>
       </c>
-      <c r="Q274" t="inlineStr"/>
-      <c r="R274" t="inlineStr"/>
       <c r="S274" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -36714,8 +37701,6 @@
           <t>responses/20260711T175732Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R275" t="inlineStr"/>
-      <c r="S275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -36785,8 +37770,6 @@
           <t>responses/20260711T175732Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R276" t="inlineStr"/>
-      <c r="S276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -36856,8 +37839,6 @@
           <t>responses/20260711T175732Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R277" t="inlineStr"/>
-      <c r="S277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -36927,8 +37908,6 @@
           <t>responses/20260711T175732Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R278" t="inlineStr"/>
-      <c r="S278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -36998,8 +37977,6 @@
           <t>responses/20260711T175732Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R279" t="inlineStr"/>
-      <c r="S279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -37069,8 +38046,6 @@
           <t>responses/20260711T175732Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R280" t="inlineStr"/>
-      <c r="S280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -37114,9 +38089,6 @@
       <c r="I281" t="n">
         <v>200</v>
       </c>
-      <c r="J281" t="inlineStr"/>
-      <c r="K281" t="inlineStr"/>
-      <c r="L281" t="inlineStr"/>
       <c r="M281" t="n">
         <v>120355</v>
       </c>
@@ -37129,9 +38101,1096 @@
       <c r="P281" t="n">
         <v>1</v>
       </c>
-      <c r="Q281" t="inlineStr"/>
-      <c r="R281" t="inlineStr"/>
-      <c r="S281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>19</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>429</v>
+      </c>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="inlineStr"/>
+      <c r="L282" t="inlineStr"/>
+      <c r="M282" t="n">
+        <v>87</v>
+      </c>
+      <c r="N282" t="n">
+        <v>0</v>
+      </c>
+      <c r="O282" t="n">
+        <v>0</v>
+      </c>
+      <c r="P282" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q282" t="inlineStr"/>
+      <c r="R282" t="inlineStr"/>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>19</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>200</v>
+      </c>
+      <c r="J283" t="n">
+        <v>287</v>
+      </c>
+      <c r="K283" t="n">
+        <v>1568</v>
+      </c>
+      <c r="L283" t="n">
+        <v>1855</v>
+      </c>
+      <c r="M283" t="n">
+        <v>17141</v>
+      </c>
+      <c r="N283" t="n">
+        <v>5820</v>
+      </c>
+      <c r="O283" t="n">
+        <v>732</v>
+      </c>
+      <c r="P283" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr"/>
+      <c r="S283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>19</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>429</v>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr"/>
+      <c r="L284" t="inlineStr"/>
+      <c r="M284" t="n">
+        <v>93</v>
+      </c>
+      <c r="N284" t="n">
+        <v>0</v>
+      </c>
+      <c r="O284" t="n">
+        <v>0</v>
+      </c>
+      <c r="P284" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q284" t="inlineStr"/>
+      <c r="R284" t="inlineStr"/>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>19</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>429</v>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr"/>
+      <c r="L285" t="inlineStr"/>
+      <c r="M285" t="n">
+        <v>150</v>
+      </c>
+      <c r="N285" t="n">
+        <v>0</v>
+      </c>
+      <c r="O285" t="n">
+        <v>0</v>
+      </c>
+      <c r="P285" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q285" t="inlineStr"/>
+      <c r="R285" t="inlineStr"/>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>19</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>200</v>
+      </c>
+      <c r="J286" t="n">
+        <v>287</v>
+      </c>
+      <c r="K286" t="n">
+        <v>2382</v>
+      </c>
+      <c r="L286" t="n">
+        <v>2669</v>
+      </c>
+      <c r="M286" t="n">
+        <v>22089</v>
+      </c>
+      <c r="N286" t="n">
+        <v>9462</v>
+      </c>
+      <c r="O286" t="n">
+        <v>1206</v>
+      </c>
+      <c r="P286" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr"/>
+      <c r="S286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>19</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>429</v>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr"/>
+      <c r="L287" t="inlineStr"/>
+      <c r="M287" t="n">
+        <v>135</v>
+      </c>
+      <c r="N287" t="n">
+        <v>0</v>
+      </c>
+      <c r="O287" t="n">
+        <v>0</v>
+      </c>
+      <c r="P287" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q287" t="inlineStr"/>
+      <c r="R287" t="inlineStr"/>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>19</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>429</v>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr"/>
+      <c r="L288" t="inlineStr"/>
+      <c r="M288" t="n">
+        <v>316</v>
+      </c>
+      <c r="N288" t="n">
+        <v>0</v>
+      </c>
+      <c r="O288" t="n">
+        <v>0</v>
+      </c>
+      <c r="P288" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q288" t="inlineStr"/>
+      <c r="R288" t="inlineStr"/>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>19</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>404</v>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr"/>
+      <c r="L289" t="inlineStr"/>
+      <c r="M289" t="n">
+        <v>39</v>
+      </c>
+      <c r="N289" t="n">
+        <v>0</v>
+      </c>
+      <c r="O289" t="n">
+        <v>0</v>
+      </c>
+      <c r="P289" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q289" t="inlineStr"/>
+      <c r="R289" t="inlineStr"/>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>19</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>200</v>
+      </c>
+      <c r="J290" t="n">
+        <v>287</v>
+      </c>
+      <c r="K290" t="n">
+        <v>1934</v>
+      </c>
+      <c r="L290" t="n">
+        <v>2221</v>
+      </c>
+      <c r="M290" t="n">
+        <v>10403</v>
+      </c>
+      <c r="N290" t="n">
+        <v>6125</v>
+      </c>
+      <c r="O290" t="n">
+        <v>814</v>
+      </c>
+      <c r="P290" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr"/>
+      <c r="S290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>19</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>200</v>
+      </c>
+      <c r="J291" t="n">
+        <v>323</v>
+      </c>
+      <c r="K291" t="n">
+        <v>964</v>
+      </c>
+      <c r="L291" t="n">
+        <v>1287</v>
+      </c>
+      <c r="M291" t="n">
+        <v>11394</v>
+      </c>
+      <c r="N291" t="n">
+        <v>3563</v>
+      </c>
+      <c r="O291" t="n">
+        <v>434</v>
+      </c>
+      <c r="P291" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr"/>
+      <c r="S291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>19</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>200</v>
+      </c>
+      <c r="J292" t="n">
+        <v>278</v>
+      </c>
+      <c r="K292" t="n">
+        <v>1356</v>
+      </c>
+      <c r="L292" t="n">
+        <v>1634</v>
+      </c>
+      <c r="M292" t="n">
+        <v>20377</v>
+      </c>
+      <c r="N292" t="n">
+        <v>5798</v>
+      </c>
+      <c r="O292" t="n">
+        <v>848</v>
+      </c>
+      <c r="P292" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr"/>
+      <c r="S292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>19</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>200</v>
+      </c>
+      <c r="J293" t="n">
+        <v>247</v>
+      </c>
+      <c r="K293" t="n">
+        <v>2144</v>
+      </c>
+      <c r="L293" t="n">
+        <v>2391</v>
+      </c>
+      <c r="M293" t="n">
+        <v>18597</v>
+      </c>
+      <c r="N293" t="n">
+        <v>8163</v>
+      </c>
+      <c r="O293" t="n">
+        <v>1030</v>
+      </c>
+      <c r="P293" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr"/>
+      <c r="S293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>19</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>200</v>
+      </c>
+      <c r="J294" t="n">
+        <v>292</v>
+      </c>
+      <c r="K294" t="n">
+        <v>1976</v>
+      </c>
+      <c r="L294" t="n">
+        <v>2268</v>
+      </c>
+      <c r="M294" t="n">
+        <v>39246</v>
+      </c>
+      <c r="N294" t="n">
+        <v>6087</v>
+      </c>
+      <c r="O294" t="n">
+        <v>737</v>
+      </c>
+      <c r="P294" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr"/>
+      <c r="S294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>19</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>200</v>
+      </c>
+      <c r="J295" t="n">
+        <v>283</v>
+      </c>
+      <c r="K295" t="n">
+        <v>3550</v>
+      </c>
+      <c r="L295" t="n">
+        <v>3833</v>
+      </c>
+      <c r="M295" t="n">
+        <v>56191</v>
+      </c>
+      <c r="N295" t="n">
+        <v>8235</v>
+      </c>
+      <c r="O295" t="n">
+        <v>1042</v>
+      </c>
+      <c r="P295" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr"/>
+      <c r="S295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>19</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>200</v>
+      </c>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="inlineStr"/>
+      <c r="L296" t="inlineStr"/>
+      <c r="M296" t="n">
+        <v>120280</v>
+      </c>
+      <c r="N296" t="n">
+        <v>0</v>
+      </c>
+      <c r="O296" t="n">
+        <v>0</v>
+      </c>
+      <c r="P296" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q296" t="inlineStr"/>
+      <c r="R296" t="inlineStr"/>
+      <c r="S296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>19</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line, in‑depth, well‑structured article titled **“St</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>200</v>
+      </c>
+      <c r="J297" t="n">
+        <v>321</v>
+      </c>
+      <c r="K297" t="n">
+        <v>2799</v>
+      </c>
+      <c r="L297" t="n">
+        <v>3120</v>
+      </c>
+      <c r="M297" t="n">
+        <v>160553</v>
+      </c>
+      <c r="N297" t="n">
+        <v>10986</v>
+      </c>
+      <c r="O297" t="n">
+        <v>1448</v>
+      </c>
+      <c r="P297" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr"/>
+      <c r="S297" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -37144,7 +39203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S281"/>
+  <dimension ref="A1:S297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54439,8 +56498,6 @@
           <t>responses/20260711T175732Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R266" t="inlineStr"/>
-      <c r="S266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -54484,9 +56541,6 @@
       <c r="I267" t="n">
         <v>429</v>
       </c>
-      <c r="J267" t="inlineStr"/>
-      <c r="K267" t="inlineStr"/>
-      <c r="L267" t="inlineStr"/>
       <c r="M267" t="n">
         <v>233</v>
       </c>
@@ -54499,8 +56553,6 @@
       <c r="P267" t="n">
         <v>3</v>
       </c>
-      <c r="Q267" t="inlineStr"/>
-      <c r="R267" t="inlineStr"/>
       <c r="S267" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -54549,9 +56601,6 @@
       <c r="I268" t="n">
         <v>429</v>
       </c>
-      <c r="J268" t="inlineStr"/>
-      <c r="K268" t="inlineStr"/>
-      <c r="L268" t="inlineStr"/>
       <c r="M268" t="n">
         <v>573</v>
       </c>
@@ -54564,8 +56613,6 @@
       <c r="P268" t="n">
         <v>3</v>
       </c>
-      <c r="Q268" t="inlineStr"/>
-      <c r="R268" t="inlineStr"/>
       <c r="S268" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"openai/gpt-oss-120b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok":</t>
@@ -54640,8 +56687,6 @@
           <t>responses/20260711T175732Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R269" t="inlineStr"/>
-      <c r="S269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -54685,9 +56730,6 @@
       <c r="I270" t="n">
         <v>429</v>
       </c>
-      <c r="J270" t="inlineStr"/>
-      <c r="K270" t="inlineStr"/>
-      <c r="L270" t="inlineStr"/>
       <c r="M270" t="n">
         <v>292</v>
       </c>
@@ -54700,8 +56742,6 @@
       <c r="P270" t="n">
         <v>3</v>
       </c>
-      <c r="Q270" t="inlineStr"/>
-      <c r="R270" t="inlineStr"/>
       <c r="S270" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -54750,9 +56790,6 @@
       <c r="I271" t="n">
         <v>429</v>
       </c>
-      <c r="J271" t="inlineStr"/>
-      <c r="K271" t="inlineStr"/>
-      <c r="L271" t="inlineStr"/>
       <c r="M271" t="n">
         <v>258</v>
       </c>
@@ -54765,8 +56802,6 @@
       <c r="P271" t="n">
         <v>3</v>
       </c>
-      <c r="Q271" t="inlineStr"/>
-      <c r="R271" t="inlineStr"/>
       <c r="S271" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -54815,9 +56850,6 @@
       <c r="I272" t="n">
         <v>429</v>
       </c>
-      <c r="J272" t="inlineStr"/>
-      <c r="K272" t="inlineStr"/>
-      <c r="L272" t="inlineStr"/>
       <c r="M272" t="n">
         <v>406</v>
       </c>
@@ -54830,8 +56862,6 @@
       <c r="P272" t="n">
         <v>3</v>
       </c>
-      <c r="Q272" t="inlineStr"/>
-      <c r="R272" t="inlineStr"/>
       <c r="S272" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
@@ -54880,9 +56910,6 @@
       <c r="I273" t="n">
         <v>429</v>
       </c>
-      <c r="J273" t="inlineStr"/>
-      <c r="K273" t="inlineStr"/>
-      <c r="L273" t="inlineStr"/>
       <c r="M273" t="n">
         <v>224</v>
       </c>
@@ -54895,8 +56922,6 @@
       <c r="P273" t="n">
         <v>3</v>
       </c>
-      <c r="Q273" t="inlineStr"/>
-      <c r="R273" t="inlineStr"/>
       <c r="S273" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -54945,9 +56970,6 @@
       <c r="I274" t="n">
         <v>404</v>
       </c>
-      <c r="J274" t="inlineStr"/>
-      <c r="K274" t="inlineStr"/>
-      <c r="L274" t="inlineStr"/>
       <c r="M274" t="n">
         <v>52</v>
       </c>
@@ -54960,8 +56982,6 @@
       <c r="P274" t="n">
         <v>1</v>
       </c>
-      <c r="Q274" t="inlineStr"/>
-      <c r="R274" t="inlineStr"/>
       <c r="S274" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -55036,8 +57056,6 @@
           <t>responses/20260711T175732Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R275" t="inlineStr"/>
-      <c r="S275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -55081,9 +57099,6 @@
       <c r="I276" t="n">
         <v>429</v>
       </c>
-      <c r="J276" t="inlineStr"/>
-      <c r="K276" t="inlineStr"/>
-      <c r="L276" t="inlineStr"/>
       <c r="M276" t="n">
         <v>1800</v>
       </c>
@@ -55096,8 +57111,6 @@
       <c r="P276" t="n">
         <v>3</v>
       </c>
-      <c r="Q276" t="inlineStr"/>
-      <c r="R276" t="inlineStr"/>
       <c r="S276" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-26b-a4b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Darkbloom","is_byok</t>
@@ -55172,8 +57185,6 @@
           <t>responses/20260711T175732Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R277" t="inlineStr"/>
-      <c r="S277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -55243,8 +57254,6 @@
           <t>responses/20260711T175732Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R278" t="inlineStr"/>
-      <c r="S278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -55314,8 +57323,6 @@
           <t>responses/20260711T175732Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R279" t="inlineStr"/>
-      <c r="S279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -55385,8 +57392,6 @@
           <t>responses/20260711T175732Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R280" t="inlineStr"/>
-      <c r="S280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -55430,9 +57435,6 @@
       <c r="I281" t="n">
         <v>200</v>
       </c>
-      <c r="J281" t="inlineStr"/>
-      <c r="K281" t="inlineStr"/>
-      <c r="L281" t="inlineStr"/>
       <c r="M281" t="n">
         <v>120499</v>
       </c>
@@ -55445,9 +57447,1106 @@
       <c r="P281" t="n">
         <v>1</v>
       </c>
-      <c r="Q281" t="inlineStr"/>
-      <c r="R281" t="inlineStr"/>
-      <c r="S281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>19</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>200</v>
+      </c>
+      <c r="J282" t="n">
+        <v>476</v>
+      </c>
+      <c r="K282" t="n">
+        <v>884</v>
+      </c>
+      <c r="L282" t="n">
+        <v>1360</v>
+      </c>
+      <c r="M282" t="n">
+        <v>7046</v>
+      </c>
+      <c r="N282" t="n">
+        <v>2646</v>
+      </c>
+      <c r="O282" t="n">
+        <v>370</v>
+      </c>
+      <c r="P282" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr"/>
+      <c r="S282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>19</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>200</v>
+      </c>
+      <c r="J283" t="n">
+        <v>476</v>
+      </c>
+      <c r="K283" t="n">
+        <v>761</v>
+      </c>
+      <c r="L283" t="n">
+        <v>1237</v>
+      </c>
+      <c r="M283" t="n">
+        <v>12441</v>
+      </c>
+      <c r="N283" t="n">
+        <v>3039</v>
+      </c>
+      <c r="O283" t="n">
+        <v>436</v>
+      </c>
+      <c r="P283" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr"/>
+      <c r="S283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>19</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>429</v>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr"/>
+      <c r="L284" t="inlineStr"/>
+      <c r="M284" t="n">
+        <v>147</v>
+      </c>
+      <c r="N284" t="n">
+        <v>0</v>
+      </c>
+      <c r="O284" t="n">
+        <v>0</v>
+      </c>
+      <c r="P284" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q284" t="inlineStr"/>
+      <c r="R284" t="inlineStr"/>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>19</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>429</v>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr"/>
+      <c r="L285" t="inlineStr"/>
+      <c r="M285" t="n">
+        <v>135</v>
+      </c>
+      <c r="N285" t="n">
+        <v>0</v>
+      </c>
+      <c r="O285" t="n">
+        <v>0</v>
+      </c>
+      <c r="P285" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q285" t="inlineStr"/>
+      <c r="R285" t="inlineStr"/>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>19</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>429</v>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr"/>
+      <c r="L286" t="inlineStr"/>
+      <c r="M286" t="n">
+        <v>120</v>
+      </c>
+      <c r="N286" t="n">
+        <v>0</v>
+      </c>
+      <c r="O286" t="n">
+        <v>0</v>
+      </c>
+      <c r="P286" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q286" t="inlineStr"/>
+      <c r="R286" t="inlineStr"/>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>19</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>429</v>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr"/>
+      <c r="L287" t="inlineStr"/>
+      <c r="M287" t="n">
+        <v>102</v>
+      </c>
+      <c r="N287" t="n">
+        <v>0</v>
+      </c>
+      <c r="O287" t="n">
+        <v>0</v>
+      </c>
+      <c r="P287" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q287" t="inlineStr"/>
+      <c r="R287" t="inlineStr"/>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>19</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>200</v>
+      </c>
+      <c r="J288" t="n">
+        <v>465</v>
+      </c>
+      <c r="K288" t="n">
+        <v>472</v>
+      </c>
+      <c r="L288" t="n">
+        <v>937</v>
+      </c>
+      <c r="M288" t="n">
+        <v>8189</v>
+      </c>
+      <c r="N288" t="n">
+        <v>2312</v>
+      </c>
+      <c r="O288" t="n">
+        <v>328</v>
+      </c>
+      <c r="P288" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr"/>
+      <c r="S288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>19</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>200</v>
+      </c>
+      <c r="J289" t="n">
+        <v>476</v>
+      </c>
+      <c r="K289" t="n">
+        <v>706</v>
+      </c>
+      <c r="L289" t="n">
+        <v>1182</v>
+      </c>
+      <c r="M289" t="n">
+        <v>3231</v>
+      </c>
+      <c r="N289" t="n">
+        <v>2899</v>
+      </c>
+      <c r="O289" t="n">
+        <v>415</v>
+      </c>
+      <c r="P289" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr"/>
+      <c r="S289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>19</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>200</v>
+      </c>
+      <c r="J290" t="n">
+        <v>417</v>
+      </c>
+      <c r="K290" t="n">
+        <v>620</v>
+      </c>
+      <c r="L290" t="n">
+        <v>1037</v>
+      </c>
+      <c r="M290" t="n">
+        <v>4476</v>
+      </c>
+      <c r="N290" t="n">
+        <v>2927</v>
+      </c>
+      <c r="O290" t="n">
+        <v>437</v>
+      </c>
+      <c r="P290" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr"/>
+      <c r="S290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>19</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>404</v>
+      </c>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr"/>
+      <c r="L291" t="inlineStr"/>
+      <c r="M291" t="n">
+        <v>61</v>
+      </c>
+      <c r="N291" t="n">
+        <v>0</v>
+      </c>
+      <c r="O291" t="n">
+        <v>0</v>
+      </c>
+      <c r="P291" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q291" t="inlineStr"/>
+      <c r="R291" t="inlineStr"/>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>19</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>429</v>
+      </c>
+      <c r="J292" t="inlineStr"/>
+      <c r="K292" t="inlineStr"/>
+      <c r="L292" t="inlineStr"/>
+      <c r="M292" t="n">
+        <v>302</v>
+      </c>
+      <c r="N292" t="n">
+        <v>0</v>
+      </c>
+      <c r="O292" t="n">
+        <v>0</v>
+      </c>
+      <c r="P292" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q292" t="inlineStr"/>
+      <c r="R292" t="inlineStr"/>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>19</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>200</v>
+      </c>
+      <c r="J293" t="n">
+        <v>491</v>
+      </c>
+      <c r="K293" t="n">
+        <v>784</v>
+      </c>
+      <c r="L293" t="n">
+        <v>1275</v>
+      </c>
+      <c r="M293" t="n">
+        <v>7989</v>
+      </c>
+      <c r="N293" t="n">
+        <v>2671</v>
+      </c>
+      <c r="O293" t="n">
+        <v>390</v>
+      </c>
+      <c r="P293" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr"/>
+      <c r="S293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>19</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>200</v>
+      </c>
+      <c r="J294" t="n">
+        <v>475</v>
+      </c>
+      <c r="K294" t="n">
+        <v>800</v>
+      </c>
+      <c r="L294" t="n">
+        <v>1275</v>
+      </c>
+      <c r="M294" t="n">
+        <v>17547</v>
+      </c>
+      <c r="N294" t="n">
+        <v>2187</v>
+      </c>
+      <c r="O294" t="n">
+        <v>310</v>
+      </c>
+      <c r="P294" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr"/>
+      <c r="S294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>19</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>200</v>
+      </c>
+      <c r="J295" t="n">
+        <v>466</v>
+      </c>
+      <c r="K295" t="n">
+        <v>603</v>
+      </c>
+      <c r="L295" t="n">
+        <v>1069</v>
+      </c>
+      <c r="M295" t="n">
+        <v>26320</v>
+      </c>
+      <c r="N295" t="n">
+        <v>3033</v>
+      </c>
+      <c r="O295" t="n">
+        <v>437</v>
+      </c>
+      <c r="P295" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr"/>
+      <c r="S295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>19</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>200</v>
+      </c>
+      <c r="J296" t="n">
+        <v>472</v>
+      </c>
+      <c r="K296" t="n">
+        <v>1518</v>
+      </c>
+      <c r="L296" t="n">
+        <v>1990</v>
+      </c>
+      <c r="M296" t="n">
+        <v>28447</v>
+      </c>
+      <c r="N296" t="n">
+        <v>3769</v>
+      </c>
+      <c r="O296" t="n">
+        <v>534</v>
+      </c>
+      <c r="P296" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr"/>
+      <c r="S296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20260712T053238Z</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-07-12T05:32:38.711713+00:00</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>19</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Subject: Request for Extension of the Application Deadline for the "Midwest Rura</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>200</v>
+      </c>
+      <c r="J297" t="n">
+        <v>489</v>
+      </c>
+      <c r="K297" t="n">
+        <v>750</v>
+      </c>
+      <c r="L297" t="n">
+        <v>1239</v>
+      </c>
+      <c r="M297" t="n">
+        <v>64296</v>
+      </c>
+      <c r="N297" t="n">
+        <v>3586</v>
+      </c>
+      <c r="O297" t="n">
+        <v>522</v>
+      </c>
+      <c r="P297" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>responses/20260712T053238Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr"/>
+      <c r="S297" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-13 10:59 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S297"/>
+  <dimension ref="A1:S313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18755,8 +18755,6 @@
           <t>responses/20260712T053238Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R282" t="inlineStr"/>
-      <c r="S282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -18826,8 +18824,6 @@
           <t>responses/20260712T053238Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R283" t="inlineStr"/>
-      <c r="S283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -18871,9 +18867,6 @@
       <c r="I284" t="n">
         <v>429</v>
       </c>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
-      <c r="L284" t="inlineStr"/>
       <c r="M284" t="n">
         <v>98</v>
       </c>
@@ -18886,8 +18879,6 @@
       <c r="P284" t="n">
         <v>3</v>
       </c>
-      <c r="Q284" t="inlineStr"/>
-      <c r="R284" t="inlineStr"/>
       <c r="S284" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -18936,9 +18927,6 @@
       <c r="I285" t="n">
         <v>429</v>
       </c>
-      <c r="J285" t="inlineStr"/>
-      <c r="K285" t="inlineStr"/>
-      <c r="L285" t="inlineStr"/>
       <c r="M285" t="n">
         <v>170</v>
       </c>
@@ -18951,8 +18939,6 @@
       <c r="P285" t="n">
         <v>3</v>
       </c>
-      <c r="Q285" t="inlineStr"/>
-      <c r="R285" t="inlineStr"/>
       <c r="S285" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -19001,9 +18987,6 @@
       <c r="I286" t="n">
         <v>429</v>
       </c>
-      <c r="J286" t="inlineStr"/>
-      <c r="K286" t="inlineStr"/>
-      <c r="L286" t="inlineStr"/>
       <c r="M286" t="n">
         <v>92</v>
       </c>
@@ -19016,8 +18999,6 @@
       <c r="P286" t="n">
         <v>3</v>
       </c>
-      <c r="Q286" t="inlineStr"/>
-      <c r="R286" t="inlineStr"/>
       <c r="S286" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -19066,9 +19047,6 @@
       <c r="I287" t="n">
         <v>404</v>
       </c>
-      <c r="J287" t="inlineStr"/>
-      <c r="K287" t="inlineStr"/>
-      <c r="L287" t="inlineStr"/>
       <c r="M287" t="n">
         <v>38</v>
       </c>
@@ -19081,8 +19059,6 @@
       <c r="P287" t="n">
         <v>1</v>
       </c>
-      <c r="Q287" t="inlineStr"/>
-      <c r="R287" t="inlineStr"/>
       <c r="S287" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -19131,9 +19107,6 @@
       <c r="I288" t="n">
         <v>429</v>
       </c>
-      <c r="J288" t="inlineStr"/>
-      <c r="K288" t="inlineStr"/>
-      <c r="L288" t="inlineStr"/>
       <c r="M288" t="n">
         <v>113</v>
       </c>
@@ -19146,8 +19119,6 @@
       <c r="P288" t="n">
         <v>3</v>
       </c>
-      <c r="Q288" t="inlineStr"/>
-      <c r="R288" t="inlineStr"/>
       <c r="S288" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -19222,8 +19193,6 @@
           <t>responses/20260712T053238Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R289" t="inlineStr"/>
-      <c r="S289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -19267,9 +19236,6 @@
       <c r="I290" t="n">
         <v>429</v>
       </c>
-      <c r="J290" t="inlineStr"/>
-      <c r="K290" t="inlineStr"/>
-      <c r="L290" t="inlineStr"/>
       <c r="M290" t="n">
         <v>269</v>
       </c>
@@ -19282,8 +19248,6 @@
       <c r="P290" t="n">
         <v>3</v>
       </c>
-      <c r="Q290" t="inlineStr"/>
-      <c r="R290" t="inlineStr"/>
       <c r="S290" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -19358,8 +19322,6 @@
           <t>responses/20260712T053238Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R291" t="inlineStr"/>
-      <c r="S291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -19429,8 +19391,6 @@
           <t>responses/20260712T053238Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R292" t="inlineStr"/>
-      <c r="S292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -19500,8 +19460,6 @@
           <t>responses/20260712T053238Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R293" t="inlineStr"/>
-      <c r="S293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -19566,9 +19524,6 @@
       <c r="P294" t="n">
         <v>1</v>
       </c>
-      <c r="Q294" t="inlineStr"/>
-      <c r="R294" t="inlineStr"/>
-      <c r="S294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -19612,9 +19567,6 @@
       <c r="I295" t="n">
         <v>200</v>
       </c>
-      <c r="J295" t="inlineStr"/>
-      <c r="K295" t="inlineStr"/>
-      <c r="L295" t="inlineStr"/>
       <c r="M295" t="n">
         <v>57582</v>
       </c>
@@ -19627,9 +19579,6 @@
       <c r="P295" t="n">
         <v>1</v>
       </c>
-      <c r="Q295" t="inlineStr"/>
-      <c r="R295" t="inlineStr"/>
-      <c r="S295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -19694,9 +19643,6 @@
       <c r="P296" t="n">
         <v>1</v>
       </c>
-      <c r="Q296" t="inlineStr"/>
-      <c r="R296" t="inlineStr"/>
-      <c r="S296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -19761,9 +19707,1102 @@
       <c r="P297" t="n">
         <v>1</v>
       </c>
-      <c r="Q297" t="inlineStr"/>
-      <c r="R297" t="inlineStr"/>
-      <c r="S297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>20</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>200</v>
+      </c>
+      <c r="J298" t="n">
+        <v>256</v>
+      </c>
+      <c r="K298" t="n">
+        <v>357</v>
+      </c>
+      <c r="L298" t="n">
+        <v>613</v>
+      </c>
+      <c r="M298" t="n">
+        <v>3920</v>
+      </c>
+      <c r="N298" t="n">
+        <v>1228</v>
+      </c>
+      <c r="O298" t="n">
+        <v>182</v>
+      </c>
+      <c r="P298" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr"/>
+      <c r="S298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>20</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>200</v>
+      </c>
+      <c r="J299" t="n">
+        <v>256</v>
+      </c>
+      <c r="K299" t="n">
+        <v>469</v>
+      </c>
+      <c r="L299" t="n">
+        <v>725</v>
+      </c>
+      <c r="M299" t="n">
+        <v>4021</v>
+      </c>
+      <c r="N299" t="n">
+        <v>1228</v>
+      </c>
+      <c r="O299" t="n">
+        <v>182</v>
+      </c>
+      <c r="P299" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr"/>
+      <c r="S299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>20</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>200</v>
+      </c>
+      <c r="J300" t="n">
+        <v>255</v>
+      </c>
+      <c r="K300" t="n">
+        <v>241</v>
+      </c>
+      <c r="L300" t="n">
+        <v>496</v>
+      </c>
+      <c r="M300" t="n">
+        <v>8718</v>
+      </c>
+      <c r="N300" t="n">
+        <v>1228</v>
+      </c>
+      <c r="O300" t="n">
+        <v>182</v>
+      </c>
+      <c r="P300" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/google_gemma-4-31b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr"/>
+      <c r="S300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>20</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>429</v>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr"/>
+      <c r="L301" t="inlineStr"/>
+      <c r="M301" t="n">
+        <v>271</v>
+      </c>
+      <c r="N301" t="n">
+        <v>0</v>
+      </c>
+      <c r="O301" t="n">
+        <v>0</v>
+      </c>
+      <c r="P301" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q301" t="inlineStr"/>
+      <c r="R301" t="inlineStr"/>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>20</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>429</v>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="inlineStr"/>
+      <c r="L302" t="inlineStr"/>
+      <c r="M302" t="n">
+        <v>334</v>
+      </c>
+      <c r="N302" t="n">
+        <v>0</v>
+      </c>
+      <c r="O302" t="n">
+        <v>0</v>
+      </c>
+      <c r="P302" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q302" t="inlineStr"/>
+      <c r="R302" t="inlineStr"/>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>20</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>429</v>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="inlineStr"/>
+      <c r="L303" t="inlineStr"/>
+      <c r="M303" t="n">
+        <v>243</v>
+      </c>
+      <c r="N303" t="n">
+        <v>0</v>
+      </c>
+      <c r="O303" t="n">
+        <v>0</v>
+      </c>
+      <c r="P303" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q303" t="inlineStr"/>
+      <c r="R303" t="inlineStr"/>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>20</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>404</v>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="inlineStr"/>
+      <c r="L304" t="inlineStr"/>
+      <c r="M304" t="n">
+        <v>113</v>
+      </c>
+      <c r="N304" t="n">
+        <v>0</v>
+      </c>
+      <c r="O304" t="n">
+        <v>0</v>
+      </c>
+      <c r="P304" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q304" t="inlineStr"/>
+      <c r="R304" t="inlineStr"/>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>20</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>200</v>
+      </c>
+      <c r="J305" t="n">
+        <v>256</v>
+      </c>
+      <c r="K305" t="n">
+        <v>1214</v>
+      </c>
+      <c r="L305" t="n">
+        <v>1470</v>
+      </c>
+      <c r="M305" t="n">
+        <v>14706</v>
+      </c>
+      <c r="N305" t="n">
+        <v>3726</v>
+      </c>
+      <c r="O305" t="n">
+        <v>529</v>
+      </c>
+      <c r="P305" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr"/>
+      <c r="S305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>20</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>200</v>
+      </c>
+      <c r="J306" t="n">
+        <v>301</v>
+      </c>
+      <c r="K306" t="n">
+        <v>301</v>
+      </c>
+      <c r="L306" t="n">
+        <v>602</v>
+      </c>
+      <c r="M306" t="n">
+        <v>18787</v>
+      </c>
+      <c r="N306" t="n">
+        <v>1228</v>
+      </c>
+      <c r="O306" t="n">
+        <v>182</v>
+      </c>
+      <c r="P306" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/openai_gpt-oss-120b_free.java</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr"/>
+      <c r="S306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>20</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>429</v>
+      </c>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="inlineStr"/>
+      <c r="L307" t="inlineStr"/>
+      <c r="M307" t="n">
+        <v>271</v>
+      </c>
+      <c r="N307" t="n">
+        <v>0</v>
+      </c>
+      <c r="O307" t="n">
+        <v>0</v>
+      </c>
+      <c r="P307" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q307" t="inlineStr"/>
+      <c r="R307" t="inlineStr"/>
+      <c r="S307" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>20</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>200</v>
+      </c>
+      <c r="J308" t="n">
+        <v>256</v>
+      </c>
+      <c r="K308" t="n">
+        <v>320</v>
+      </c>
+      <c r="L308" t="n">
+        <v>576</v>
+      </c>
+      <c r="M308" t="n">
+        <v>28441</v>
+      </c>
+      <c r="N308" t="n">
+        <v>1551</v>
+      </c>
+      <c r="O308" t="n">
+        <v>218</v>
+      </c>
+      <c r="P308" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr"/>
+      <c r="S308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>20</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>200</v>
+      </c>
+      <c r="J309" t="n">
+        <v>232</v>
+      </c>
+      <c r="K309" t="n">
+        <v>3714</v>
+      </c>
+      <c r="L309" t="n">
+        <v>3946</v>
+      </c>
+      <c r="M309" t="n">
+        <v>31869</v>
+      </c>
+      <c r="N309" t="n">
+        <v>6376</v>
+      </c>
+      <c r="O309" t="n">
+        <v>892</v>
+      </c>
+      <c r="P309" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr"/>
+      <c r="S309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>20</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>200</v>
+      </c>
+      <c r="J310" t="n">
+        <v>252</v>
+      </c>
+      <c r="K310" t="n">
+        <v>1505</v>
+      </c>
+      <c r="L310" t="n">
+        <v>1757</v>
+      </c>
+      <c r="M310" t="n">
+        <v>35127</v>
+      </c>
+      <c r="N310" t="n">
+        <v>937</v>
+      </c>
+      <c r="O310" t="n">
+        <v>121</v>
+      </c>
+      <c r="P310" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr"/>
+      <c r="S310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>20</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>200</v>
+      </c>
+      <c r="J311" t="n">
+        <v>303</v>
+      </c>
+      <c r="K311" t="n">
+        <v>1136</v>
+      </c>
+      <c r="L311" t="n">
+        <v>1439</v>
+      </c>
+      <c r="M311" t="n">
+        <v>57901</v>
+      </c>
+      <c r="N311" t="n">
+        <v>3938</v>
+      </c>
+      <c r="O311" t="n">
+        <v>615</v>
+      </c>
+      <c r="P311" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr"/>
+      <c r="S311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>20</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>200</v>
+      </c>
+      <c r="J312" t="n">
+        <v>250</v>
+      </c>
+      <c r="K312" t="n">
+        <v>4448</v>
+      </c>
+      <c r="L312" t="n">
+        <v>4698</v>
+      </c>
+      <c r="M312" t="n">
+        <v>121739</v>
+      </c>
+      <c r="N312" t="n">
+        <v>2974</v>
+      </c>
+      <c r="O312" t="n">
+        <v>432</v>
+      </c>
+      <c r="P312" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/code/poolside_laguna-m.1_free.java</t>
+        </is>
+      </c>
+      <c r="R312" t="inlineStr"/>
+      <c r="S312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>20</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Write a self‑contained Java program that defines a public class named `CyclicBar</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>200</v>
+      </c>
+      <c r="J313" t="inlineStr"/>
+      <c r="K313" t="inlineStr"/>
+      <c r="L313" t="inlineStr"/>
+      <c r="M313" t="n">
+        <v>120394</v>
+      </c>
+      <c r="N313" t="n">
+        <v>0</v>
+      </c>
+      <c r="O313" t="n">
+        <v>0</v>
+      </c>
+      <c r="P313" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q313" t="inlineStr"/>
+      <c r="R313" t="inlineStr"/>
+      <c r="S313" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19776,7 +20815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S297"/>
+  <dimension ref="A1:S313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38144,9 +39183,6 @@
       <c r="I282" t="n">
         <v>429</v>
       </c>
-      <c r="J282" t="inlineStr"/>
-      <c r="K282" t="inlineStr"/>
-      <c r="L282" t="inlineStr"/>
       <c r="M282" t="n">
         <v>87</v>
       </c>
@@ -38159,8 +39195,6 @@
       <c r="P282" t="n">
         <v>3</v>
       </c>
-      <c r="Q282" t="inlineStr"/>
-      <c r="R282" t="inlineStr"/>
       <c r="S282" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -38235,8 +39269,6 @@
           <t>responses/20260712T053238Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R283" t="inlineStr"/>
-      <c r="S283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -38280,9 +39312,6 @@
       <c r="I284" t="n">
         <v>429</v>
       </c>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
-      <c r="L284" t="inlineStr"/>
       <c r="M284" t="n">
         <v>93</v>
       </c>
@@ -38295,8 +39324,6 @@
       <c r="P284" t="n">
         <v>3</v>
       </c>
-      <c r="Q284" t="inlineStr"/>
-      <c r="R284" t="inlineStr"/>
       <c r="S284" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -38345,9 +39372,6 @@
       <c r="I285" t="n">
         <v>429</v>
       </c>
-      <c r="J285" t="inlineStr"/>
-      <c r="K285" t="inlineStr"/>
-      <c r="L285" t="inlineStr"/>
       <c r="M285" t="n">
         <v>150</v>
       </c>
@@ -38360,8 +39384,6 @@
       <c r="P285" t="n">
         <v>3</v>
       </c>
-      <c r="Q285" t="inlineStr"/>
-      <c r="R285" t="inlineStr"/>
       <c r="S285" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -38436,8 +39458,6 @@
           <t>responses/20260712T053238Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R286" t="inlineStr"/>
-      <c r="S286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -38481,9 +39501,6 @@
       <c r="I287" t="n">
         <v>429</v>
       </c>
-      <c r="J287" t="inlineStr"/>
-      <c r="K287" t="inlineStr"/>
-      <c r="L287" t="inlineStr"/>
       <c r="M287" t="n">
         <v>135</v>
       </c>
@@ -38496,8 +39513,6 @@
       <c r="P287" t="n">
         <v>3</v>
       </c>
-      <c r="Q287" t="inlineStr"/>
-      <c r="R287" t="inlineStr"/>
       <c r="S287" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -38546,9 +39561,6 @@
       <c r="I288" t="n">
         <v>429</v>
       </c>
-      <c r="J288" t="inlineStr"/>
-      <c r="K288" t="inlineStr"/>
-      <c r="L288" t="inlineStr"/>
       <c r="M288" t="n">
         <v>316</v>
       </c>
@@ -38561,8 +39573,6 @@
       <c r="P288" t="n">
         <v>3</v>
       </c>
-      <c r="Q288" t="inlineStr"/>
-      <c r="R288" t="inlineStr"/>
       <c r="S288" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -38611,9 +39621,6 @@
       <c r="I289" t="n">
         <v>404</v>
       </c>
-      <c r="J289" t="inlineStr"/>
-      <c r="K289" t="inlineStr"/>
-      <c r="L289" t="inlineStr"/>
       <c r="M289" t="n">
         <v>39</v>
       </c>
@@ -38626,8 +39633,6 @@
       <c r="P289" t="n">
         <v>1</v>
       </c>
-      <c r="Q289" t="inlineStr"/>
-      <c r="R289" t="inlineStr"/>
       <c r="S289" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -38702,8 +39707,6 @@
           <t>responses/20260712T053238Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R290" t="inlineStr"/>
-      <c r="S290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -38773,8 +39776,6 @@
           <t>responses/20260712T053238Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R291" t="inlineStr"/>
-      <c r="S291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -38844,8 +39845,6 @@
           <t>responses/20260712T053238Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R292" t="inlineStr"/>
-      <c r="S292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -38915,8 +39914,6 @@
           <t>responses/20260712T053238Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R293" t="inlineStr"/>
-      <c r="S293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -38986,8 +39983,6 @@
           <t>responses/20260712T053238Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R294" t="inlineStr"/>
-      <c r="S294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -39057,8 +40052,6 @@
           <t>responses/20260712T053238Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R295" t="inlineStr"/>
-      <c r="S295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -39102,9 +40095,6 @@
       <c r="I296" t="n">
         <v>200</v>
       </c>
-      <c r="J296" t="inlineStr"/>
-      <c r="K296" t="inlineStr"/>
-      <c r="L296" t="inlineStr"/>
       <c r="M296" t="n">
         <v>120280</v>
       </c>
@@ -39117,9 +40107,6 @@
       <c r="P296" t="n">
         <v>1</v>
       </c>
-      <c r="Q296" t="inlineStr"/>
-      <c r="R296" t="inlineStr"/>
-      <c r="S296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -39189,8 +40176,1102 @@
           <t>responses/20260712T053238Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R297" t="inlineStr"/>
-      <c r="S297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>20</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>200</v>
+      </c>
+      <c r="J298" t="n">
+        <v>299</v>
+      </c>
+      <c r="K298" t="n">
+        <v>232</v>
+      </c>
+      <c r="L298" t="n">
+        <v>531</v>
+      </c>
+      <c r="M298" t="n">
+        <v>2337</v>
+      </c>
+      <c r="N298" t="n">
+        <v>281</v>
+      </c>
+      <c r="O298" t="n">
+        <v>44</v>
+      </c>
+      <c r="P298" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr"/>
+      <c r="S298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>20</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>200</v>
+      </c>
+      <c r="J299" t="n">
+        <v>299</v>
+      </c>
+      <c r="K299" t="n">
+        <v>275</v>
+      </c>
+      <c r="L299" t="n">
+        <v>574</v>
+      </c>
+      <c r="M299" t="n">
+        <v>4044</v>
+      </c>
+      <c r="N299" t="n">
+        <v>65</v>
+      </c>
+      <c r="O299" t="n">
+        <v>13</v>
+      </c>
+      <c r="P299" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr"/>
+      <c r="S299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>20</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>429</v>
+      </c>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr"/>
+      <c r="L300" t="inlineStr"/>
+      <c r="M300" t="n">
+        <v>221</v>
+      </c>
+      <c r="N300" t="n">
+        <v>0</v>
+      </c>
+      <c r="O300" t="n">
+        <v>0</v>
+      </c>
+      <c r="P300" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q300" t="inlineStr"/>
+      <c r="R300" t="inlineStr"/>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>20</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>429</v>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr"/>
+      <c r="L301" t="inlineStr"/>
+      <c r="M301" t="n">
+        <v>236</v>
+      </c>
+      <c r="N301" t="n">
+        <v>0</v>
+      </c>
+      <c r="O301" t="n">
+        <v>0</v>
+      </c>
+      <c r="P301" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q301" t="inlineStr"/>
+      <c r="R301" t="inlineStr"/>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>20</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>429</v>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="inlineStr"/>
+      <c r="L302" t="inlineStr"/>
+      <c r="M302" t="n">
+        <v>199</v>
+      </c>
+      <c r="N302" t="n">
+        <v>0</v>
+      </c>
+      <c r="O302" t="n">
+        <v>0</v>
+      </c>
+      <c r="P302" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q302" t="inlineStr"/>
+      <c r="R302" t="inlineStr"/>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>20</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>429</v>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="inlineStr"/>
+      <c r="L303" t="inlineStr"/>
+      <c r="M303" t="n">
+        <v>188</v>
+      </c>
+      <c r="N303" t="n">
+        <v>0</v>
+      </c>
+      <c r="O303" t="n">
+        <v>0</v>
+      </c>
+      <c r="P303" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q303" t="inlineStr"/>
+      <c r="R303" t="inlineStr"/>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>20</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>200</v>
+      </c>
+      <c r="J304" t="n">
+        <v>305</v>
+      </c>
+      <c r="K304" t="n">
+        <v>351</v>
+      </c>
+      <c r="L304" t="n">
+        <v>656</v>
+      </c>
+      <c r="M304" t="n">
+        <v>13152</v>
+      </c>
+      <c r="N304" t="n">
+        <v>289</v>
+      </c>
+      <c r="O304" t="n">
+        <v>48</v>
+      </c>
+      <c r="P304" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr"/>
+      <c r="S304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>20</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>404</v>
+      </c>
+      <c r="J305" t="inlineStr"/>
+      <c r="K305" t="inlineStr"/>
+      <c r="L305" t="inlineStr"/>
+      <c r="M305" t="n">
+        <v>82</v>
+      </c>
+      <c r="N305" t="n">
+        <v>0</v>
+      </c>
+      <c r="O305" t="n">
+        <v>0</v>
+      </c>
+      <c r="P305" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q305" t="inlineStr"/>
+      <c r="R305" t="inlineStr"/>
+      <c r="S305" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>20</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>200</v>
+      </c>
+      <c r="J306" t="n">
+        <v>292</v>
+      </c>
+      <c r="K306" t="n">
+        <v>1687</v>
+      </c>
+      <c r="L306" t="n">
+        <v>1979</v>
+      </c>
+      <c r="M306" t="n">
+        <v>39975</v>
+      </c>
+      <c r="N306" t="n">
+        <v>7088</v>
+      </c>
+      <c r="O306" t="n">
+        <v>967</v>
+      </c>
+      <c r="P306" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr"/>
+      <c r="S306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>20</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>200</v>
+      </c>
+      <c r="J307" t="n">
+        <v>291</v>
+      </c>
+      <c r="K307" t="n">
+        <v>1729</v>
+      </c>
+      <c r="L307" t="n">
+        <v>2020</v>
+      </c>
+      <c r="M307" t="n">
+        <v>34166</v>
+      </c>
+      <c r="N307" t="n">
+        <v>7131</v>
+      </c>
+      <c r="O307" t="n">
+        <v>1027</v>
+      </c>
+      <c r="P307" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr"/>
+      <c r="S307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>20</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>200</v>
+      </c>
+      <c r="J308" t="n">
+        <v>261</v>
+      </c>
+      <c r="K308" t="n">
+        <v>5049</v>
+      </c>
+      <c r="L308" t="n">
+        <v>5310</v>
+      </c>
+      <c r="M308" t="n">
+        <v>69475</v>
+      </c>
+      <c r="N308" t="n">
+        <v>20249</v>
+      </c>
+      <c r="O308" t="n">
+        <v>2798</v>
+      </c>
+      <c r="P308" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr"/>
+      <c r="S308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>20</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>200</v>
+      </c>
+      <c r="J309" t="n">
+        <v>331</v>
+      </c>
+      <c r="K309" t="n">
+        <v>2190</v>
+      </c>
+      <c r="L309" t="n">
+        <v>2521</v>
+      </c>
+      <c r="M309" t="n">
+        <v>65266</v>
+      </c>
+      <c r="N309" t="n">
+        <v>9015</v>
+      </c>
+      <c r="O309" t="n">
+        <v>1280</v>
+      </c>
+      <c r="P309" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr"/>
+      <c r="S309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>20</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>200</v>
+      </c>
+      <c r="J310" t="n">
+        <v>295</v>
+      </c>
+      <c r="K310" t="n">
+        <v>3766</v>
+      </c>
+      <c r="L310" t="n">
+        <v>4061</v>
+      </c>
+      <c r="M310" t="n">
+        <v>58353</v>
+      </c>
+      <c r="N310" t="n">
+        <v>12077</v>
+      </c>
+      <c r="O310" t="n">
+        <v>1616</v>
+      </c>
+      <c r="P310" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr"/>
+      <c r="S310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>20</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>200</v>
+      </c>
+      <c r="J311" t="n">
+        <v>299</v>
+      </c>
+      <c r="K311" t="n">
+        <v>4411</v>
+      </c>
+      <c r="L311" t="n">
+        <v>4710</v>
+      </c>
+      <c r="M311" t="n">
+        <v>91559</v>
+      </c>
+      <c r="N311" t="n">
+        <v>14689</v>
+      </c>
+      <c r="O311" t="n">
+        <v>2059</v>
+      </c>
+      <c r="P311" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr"/>
+      <c r="S311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>20</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>200</v>
+      </c>
+      <c r="J312" t="inlineStr"/>
+      <c r="K312" t="inlineStr"/>
+      <c r="L312" t="inlineStr"/>
+      <c r="M312" t="n">
+        <v>120424</v>
+      </c>
+      <c r="N312" t="n">
+        <v>0</v>
+      </c>
+      <c r="O312" t="n">
+        <v>0</v>
+      </c>
+      <c r="P312" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q312" t="inlineStr"/>
+      <c r="R312" t="inlineStr"/>
+      <c r="S312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>20</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Write an approximately 1000‑line (around 12,000‑15,000 words) in‑depth, well‑str</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>200</v>
+      </c>
+      <c r="J313" t="n">
+        <v>331</v>
+      </c>
+      <c r="K313" t="n">
+        <v>4142</v>
+      </c>
+      <c r="L313" t="n">
+        <v>4473</v>
+      </c>
+      <c r="M313" t="n">
+        <v>166253</v>
+      </c>
+      <c r="N313" t="n">
+        <v>16365</v>
+      </c>
+      <c r="O313" t="n">
+        <v>2475</v>
+      </c>
+      <c r="P313" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/text/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr"/>
+      <c r="S313" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -39203,7 +41284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S297"/>
+  <dimension ref="A1:S313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57516,8 +59597,6 @@
           <t>responses/20260712T053238Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R282" t="inlineStr"/>
-      <c r="S282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -57587,8 +59666,6 @@
           <t>responses/20260712T053238Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R283" t="inlineStr"/>
-      <c r="S283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -57632,9 +59709,6 @@
       <c r="I284" t="n">
         <v>429</v>
       </c>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
-      <c r="L284" t="inlineStr"/>
       <c r="M284" t="n">
         <v>147</v>
       </c>
@@ -57647,8 +59721,6 @@
       <c r="P284" t="n">
         <v>3</v>
       </c>
-      <c r="Q284" t="inlineStr"/>
-      <c r="R284" t="inlineStr"/>
       <c r="S284" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -57697,9 +59769,6 @@
       <c r="I285" t="n">
         <v>429</v>
       </c>
-      <c r="J285" t="inlineStr"/>
-      <c r="K285" t="inlineStr"/>
-      <c r="L285" t="inlineStr"/>
       <c r="M285" t="n">
         <v>135</v>
       </c>
@@ -57712,8 +59781,6 @@
       <c r="P285" t="n">
         <v>3</v>
       </c>
-      <c r="Q285" t="inlineStr"/>
-      <c r="R285" t="inlineStr"/>
       <c r="S285" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -57762,9 +59829,6 @@
       <c r="I286" t="n">
         <v>429</v>
       </c>
-      <c r="J286" t="inlineStr"/>
-      <c r="K286" t="inlineStr"/>
-      <c r="L286" t="inlineStr"/>
       <c r="M286" t="n">
         <v>120</v>
       </c>
@@ -57777,8 +59841,6 @@
       <c r="P286" t="n">
         <v>3</v>
       </c>
-      <c r="Q286" t="inlineStr"/>
-      <c r="R286" t="inlineStr"/>
       <c r="S286" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -57827,9 +59889,6 @@
       <c r="I287" t="n">
         <v>429</v>
       </c>
-      <c r="J287" t="inlineStr"/>
-      <c r="K287" t="inlineStr"/>
-      <c r="L287" t="inlineStr"/>
       <c r="M287" t="n">
         <v>102</v>
       </c>
@@ -57842,8 +59901,6 @@
       <c r="P287" t="n">
         <v>3</v>
       </c>
-      <c r="Q287" t="inlineStr"/>
-      <c r="R287" t="inlineStr"/>
       <c r="S287" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -57918,8 +59975,6 @@
           <t>responses/20260712T053238Z/email/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R288" t="inlineStr"/>
-      <c r="S288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -57989,8 +60044,6 @@
           <t>responses/20260712T053238Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R289" t="inlineStr"/>
-      <c r="S289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -58060,8 +60113,6 @@
           <t>responses/20260712T053238Z/email/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R290" t="inlineStr"/>
-      <c r="S290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -58105,9 +60156,6 @@
       <c r="I291" t="n">
         <v>404</v>
       </c>
-      <c r="J291" t="inlineStr"/>
-      <c r="K291" t="inlineStr"/>
-      <c r="L291" t="inlineStr"/>
       <c r="M291" t="n">
         <v>61</v>
       </c>
@@ -58120,8 +60168,6 @@
       <c r="P291" t="n">
         <v>1</v>
       </c>
-      <c r="Q291" t="inlineStr"/>
-      <c r="R291" t="inlineStr"/>
       <c r="S291" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -58170,9 +60216,6 @@
       <c r="I292" t="n">
         <v>429</v>
       </c>
-      <c r="J292" t="inlineStr"/>
-      <c r="K292" t="inlineStr"/>
-      <c r="L292" t="inlineStr"/>
       <c r="M292" t="n">
         <v>302</v>
       </c>
@@ -58185,8 +60228,6 @@
       <c r="P292" t="n">
         <v>3</v>
       </c>
-      <c r="Q292" t="inlineStr"/>
-      <c r="R292" t="inlineStr"/>
       <c r="S292" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"OpenInference","is_byok</t>
@@ -58261,8 +60302,6 @@
           <t>responses/20260712T053238Z/email/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R293" t="inlineStr"/>
-      <c r="S293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -58332,8 +60371,6 @@
           <t>responses/20260712T053238Z/email/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R294" t="inlineStr"/>
-      <c r="S294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -58403,8 +60440,6 @@
           <t>responses/20260712T053238Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
         </is>
       </c>
-      <c r="R295" t="inlineStr"/>
-      <c r="S295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -58474,8 +60509,6 @@
           <t>responses/20260712T053238Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R296" t="inlineStr"/>
-      <c r="S296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -58545,8 +60578,1112 @@
           <t>responses/20260712T053238Z/email/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R297" t="inlineStr"/>
-      <c r="S297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>20</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>200</v>
+      </c>
+      <c r="J298" t="n">
+        <v>621</v>
+      </c>
+      <c r="K298" t="n">
+        <v>661</v>
+      </c>
+      <c r="L298" t="n">
+        <v>1282</v>
+      </c>
+      <c r="M298" t="n">
+        <v>5390</v>
+      </c>
+      <c r="N298" t="n">
+        <v>2845</v>
+      </c>
+      <c r="O298" t="n">
+        <v>426</v>
+      </c>
+      <c r="P298" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr"/>
+      <c r="S298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>20</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>429</v>
+      </c>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr"/>
+      <c r="L299" t="inlineStr"/>
+      <c r="M299" t="n">
+        <v>231</v>
+      </c>
+      <c r="N299" t="n">
+        <v>0</v>
+      </c>
+      <c r="O299" t="n">
+        <v>0</v>
+      </c>
+      <c r="P299" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q299" t="inlineStr"/>
+      <c r="R299" t="inlineStr"/>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>20</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>429</v>
+      </c>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr"/>
+      <c r="L300" t="inlineStr"/>
+      <c r="M300" t="n">
+        <v>216</v>
+      </c>
+      <c r="N300" t="n">
+        <v>0</v>
+      </c>
+      <c r="O300" t="n">
+        <v>0</v>
+      </c>
+      <c r="P300" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q300" t="inlineStr"/>
+      <c r="R300" t="inlineStr"/>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>20</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>429</v>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr"/>
+      <c r="L301" t="inlineStr"/>
+      <c r="M301" t="n">
+        <v>250</v>
+      </c>
+      <c r="N301" t="n">
+        <v>0</v>
+      </c>
+      <c r="O301" t="n">
+        <v>0</v>
+      </c>
+      <c r="P301" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q301" t="inlineStr"/>
+      <c r="R301" t="inlineStr"/>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>20</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>429</v>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="inlineStr"/>
+      <c r="L302" t="inlineStr"/>
+      <c r="M302" t="n">
+        <v>278</v>
+      </c>
+      <c r="N302" t="n">
+        <v>0</v>
+      </c>
+      <c r="O302" t="n">
+        <v>0</v>
+      </c>
+      <c r="P302" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q302" t="inlineStr"/>
+      <c r="R302" t="inlineStr"/>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>20</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>200</v>
+      </c>
+      <c r="J303" t="n">
+        <v>621</v>
+      </c>
+      <c r="K303" t="n">
+        <v>982</v>
+      </c>
+      <c r="L303" t="n">
+        <v>1603</v>
+      </c>
+      <c r="M303" t="n">
+        <v>11215</v>
+      </c>
+      <c r="N303" t="n">
+        <v>4623</v>
+      </c>
+      <c r="O303" t="n">
+        <v>692</v>
+      </c>
+      <c r="P303" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr"/>
+      <c r="S303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>20</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>404</v>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="inlineStr"/>
+      <c r="L304" t="inlineStr"/>
+      <c r="M304" t="n">
+        <v>89</v>
+      </c>
+      <c r="N304" t="n">
+        <v>0</v>
+      </c>
+      <c r="O304" t="n">
+        <v>0</v>
+      </c>
+      <c r="P304" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q304" t="inlineStr"/>
+      <c r="R304" t="inlineStr"/>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>20</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>200</v>
+      </c>
+      <c r="J305" t="n">
+        <v>605</v>
+      </c>
+      <c r="K305" t="n">
+        <v>693</v>
+      </c>
+      <c r="L305" t="n">
+        <v>1298</v>
+      </c>
+      <c r="M305" t="n">
+        <v>13672</v>
+      </c>
+      <c r="N305" t="n">
+        <v>3648</v>
+      </c>
+      <c r="O305" t="n">
+        <v>542</v>
+      </c>
+      <c r="P305" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr"/>
+      <c r="S305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>20</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>200</v>
+      </c>
+      <c r="J306" t="n">
+        <v>604</v>
+      </c>
+      <c r="K306" t="n">
+        <v>573</v>
+      </c>
+      <c r="L306" t="n">
+        <v>1177</v>
+      </c>
+      <c r="M306" t="n">
+        <v>20998</v>
+      </c>
+      <c r="N306" t="n">
+        <v>3011</v>
+      </c>
+      <c r="O306" t="n">
+        <v>446</v>
+      </c>
+      <c r="P306" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/google_gemma-4-31b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr"/>
+      <c r="S306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>20</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>200</v>
+      </c>
+      <c r="J307" t="n">
+        <v>556</v>
+      </c>
+      <c r="K307" t="n">
+        <v>793</v>
+      </c>
+      <c r="L307" t="n">
+        <v>1349</v>
+      </c>
+      <c r="M307" t="n">
+        <v>11067</v>
+      </c>
+      <c r="N307" t="n">
+        <v>3922</v>
+      </c>
+      <c r="O307" t="n">
+        <v>569</v>
+      </c>
+      <c r="P307" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/cohere_north-mini-code_free.md</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr"/>
+      <c r="S307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>20</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>200</v>
+      </c>
+      <c r="J308" t="n">
+        <v>629</v>
+      </c>
+      <c r="K308" t="n">
+        <v>996</v>
+      </c>
+      <c r="L308" t="n">
+        <v>1625</v>
+      </c>
+      <c r="M308" t="n">
+        <v>67584</v>
+      </c>
+      <c r="N308" t="n">
+        <v>5041</v>
+      </c>
+      <c r="O308" t="n">
+        <v>749</v>
+      </c>
+      <c r="P308" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/openai_gpt-oss-120b_free.md</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr"/>
+      <c r="S308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>20</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>200</v>
+      </c>
+      <c r="J309" t="n">
+        <v>620</v>
+      </c>
+      <c r="K309" t="n">
+        <v>685</v>
+      </c>
+      <c r="L309" t="n">
+        <v>1305</v>
+      </c>
+      <c r="M309" t="n">
+        <v>15790</v>
+      </c>
+      <c r="N309" t="n">
+        <v>3438</v>
+      </c>
+      <c r="O309" t="n">
+        <v>476</v>
+      </c>
+      <c r="P309" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/nvidia_nemotron-nano-12b-v2-vl_free.md</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr"/>
+      <c r="S309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>20</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>200</v>
+      </c>
+      <c r="J310" t="n">
+        <v>626</v>
+      </c>
+      <c r="K310" t="n">
+        <v>1037</v>
+      </c>
+      <c r="L310" t="n">
+        <v>1663</v>
+      </c>
+      <c r="M310" t="n">
+        <v>32438</v>
+      </c>
+      <c r="N310" t="n">
+        <v>2821</v>
+      </c>
+      <c r="O310" t="n">
+        <v>392</v>
+      </c>
+      <c r="P310" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/poolside_laguna-m.1_free.md</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr"/>
+      <c r="S310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>20</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>200</v>
+      </c>
+      <c r="J311" t="n">
+        <v>617</v>
+      </c>
+      <c r="K311" t="n">
+        <v>1705</v>
+      </c>
+      <c r="L311" t="n">
+        <v>2322</v>
+      </c>
+      <c r="M311" t="n">
+        <v>31974</v>
+      </c>
+      <c r="N311" t="n">
+        <v>5515</v>
+      </c>
+      <c r="O311" t="n">
+        <v>801</v>
+      </c>
+      <c r="P311" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/nvidia_nemotron-nano-9b-v2_free.md</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr"/>
+      <c r="S311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>20</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>200</v>
+      </c>
+      <c r="J312" t="n">
+        <v>631</v>
+      </c>
+      <c r="K312" t="n">
+        <v>968</v>
+      </c>
+      <c r="L312" t="n">
+        <v>1599</v>
+      </c>
+      <c r="M312" t="n">
+        <v>42061</v>
+      </c>
+      <c r="N312" t="n">
+        <v>4349</v>
+      </c>
+      <c r="O312" t="n">
+        <v>640</v>
+      </c>
+      <c r="P312" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R312" t="inlineStr"/>
+      <c r="S312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>20260713T105517Z</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-07-13T10:55:17.511895+00:00</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>20</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>generate</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Subject: Request for Clarification on Post‑Award Audit Requirements for the Comm</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>200</v>
+      </c>
+      <c r="J313" t="n">
+        <v>621</v>
+      </c>
+      <c r="K313" t="n">
+        <v>4096</v>
+      </c>
+      <c r="L313" t="n">
+        <v>4717</v>
+      </c>
+      <c r="M313" t="n">
+        <v>128167</v>
+      </c>
+      <c r="N313" t="n">
+        <v>17665</v>
+      </c>
+      <c r="O313" t="n">
+        <v>1069</v>
+      </c>
+      <c r="P313" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>responses/20260713T105517Z/email/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr"/>
+      <c r="S313" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bench: run 2026-07-14 15:27 UTC
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S313"/>
+  <dimension ref="A1:S329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19776,8 +19776,6 @@
           <t>responses/20260713T105517Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
         </is>
       </c>
-      <c r="R298" t="inlineStr"/>
-      <c r="S298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -19847,8 +19845,6 @@
           <t>responses/20260713T105517Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
         </is>
       </c>
-      <c r="R299" t="inlineStr"/>
-      <c r="S299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -19918,8 +19914,6 @@
           <t>responses/20260713T105517Z/code/google_gemma-4-31b-it_free.java</t>
         </is>
       </c>
-      <c r="R300" t="inlineStr"/>
-      <c r="S300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -19963,9 +19957,6 @@
       <c r="I301" t="n">
         <v>429</v>
       </c>
-      <c r="J301" t="inlineStr"/>
-      <c r="K301" t="inlineStr"/>
-      <c r="L301" t="inlineStr"/>
       <c r="M301" t="n">
         <v>271</v>
       </c>
@@ -19978,8 +19969,6 @@
       <c r="P301" t="n">
         <v>3</v>
       </c>
-      <c r="Q301" t="inlineStr"/>
-      <c r="R301" t="inlineStr"/>
       <c r="S301" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -20028,9 +20017,6 @@
       <c r="I302" t="n">
         <v>429</v>
       </c>
-      <c r="J302" t="inlineStr"/>
-      <c r="K302" t="inlineStr"/>
-      <c r="L302" t="inlineStr"/>
       <c r="M302" t="n">
         <v>334</v>
       </c>
@@ -20043,8 +20029,6 @@
       <c r="P302" t="n">
         <v>3</v>
       </c>
-      <c r="Q302" t="inlineStr"/>
-      <c r="R302" t="inlineStr"/>
       <c r="S302" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -20093,9 +20077,6 @@
       <c r="I303" t="n">
         <v>429</v>
       </c>
-      <c r="J303" t="inlineStr"/>
-      <c r="K303" t="inlineStr"/>
-      <c r="L303" t="inlineStr"/>
       <c r="M303" t="n">
         <v>243</v>
       </c>
@@ -20108,8 +20089,6 @@
       <c r="P303" t="n">
         <v>3</v>
       </c>
-      <c r="Q303" t="inlineStr"/>
-      <c r="R303" t="inlineStr"/>
       <c r="S303" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -20158,9 +20137,6 @@
       <c r="I304" t="n">
         <v>404</v>
       </c>
-      <c r="J304" t="inlineStr"/>
-      <c r="K304" t="inlineStr"/>
-      <c r="L304" t="inlineStr"/>
       <c r="M304" t="n">
         <v>113</v>
       </c>
@@ -20173,8 +20149,6 @@
       <c r="P304" t="n">
         <v>1</v>
       </c>
-      <c r="Q304" t="inlineStr"/>
-      <c r="R304" t="inlineStr"/>
       <c r="S304" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -20249,8 +20223,6 @@
           <t>responses/20260713T105517Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
         </is>
       </c>
-      <c r="R305" t="inlineStr"/>
-      <c r="S305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -20320,8 +20292,6 @@
           <t>responses/20260713T105517Z/code/openai_gpt-oss-120b_free.java</t>
         </is>
       </c>
-      <c r="R306" t="inlineStr"/>
-      <c r="S306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -20365,9 +20335,6 @@
       <c r="I307" t="n">
         <v>429</v>
       </c>
-      <c r="J307" t="inlineStr"/>
-      <c r="K307" t="inlineStr"/>
-      <c r="L307" t="inlineStr"/>
       <c r="M307" t="n">
         <v>271</v>
       </c>
@@ -20380,8 +20347,6 @@
       <c r="P307" t="n">
         <v>3</v>
       </c>
-      <c r="Q307" t="inlineStr"/>
-      <c r="R307" t="inlineStr"/>
       <c r="S307" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -20456,8 +20421,6 @@
           <t>responses/20260713T105517Z/code/google_gemma-4-26b-a4b-it_free.java</t>
         </is>
       </c>
-      <c r="R308" t="inlineStr"/>
-      <c r="S308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -20527,8 +20490,6 @@
           <t>responses/20260713T105517Z/code/cohere_north-mini-code_free.java</t>
         </is>
       </c>
-      <c r="R309" t="inlineStr"/>
-      <c r="S309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -20598,8 +20559,6 @@
           <t>responses/20260713T105517Z/code/nvidia_nemotron-nano-9b-v2_free.java</t>
         </is>
       </c>
-      <c r="R310" t="inlineStr"/>
-      <c r="S310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -20669,8 +20628,6 @@
           <t>responses/20260713T105517Z/code/openai_gpt-oss-20b_free.java</t>
         </is>
       </c>
-      <c r="R311" t="inlineStr"/>
-      <c r="S311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -20740,8 +20697,6 @@
           <t>responses/20260713T105517Z/code/poolside_laguna-m.1_free.java</t>
         </is>
       </c>
-      <c r="R312" t="inlineStr"/>
-      <c r="S312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -20785,9 +20740,6 @@
       <c r="I313" t="n">
         <v>200</v>
       </c>
-      <c r="J313" t="inlineStr"/>
-      <c r="K313" t="inlineStr"/>
-      <c r="L313" t="inlineStr"/>
       <c r="M313" t="n">
         <v>120394</v>
       </c>
@@ -20800,9 +20752,1092 @@
       <c r="P313" t="n">
         <v>1</v>
       </c>
-      <c r="Q313" t="inlineStr"/>
-      <c r="R313" t="inlineStr"/>
-      <c r="S313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>21</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>404</v>
+      </c>
+      <c r="J314" t="inlineStr"/>
+      <c r="K314" t="inlineStr"/>
+      <c r="L314" t="inlineStr"/>
+      <c r="M314" t="n">
+        <v>262</v>
+      </c>
+      <c r="N314" t="n">
+        <v>0</v>
+      </c>
+      <c r="O314" t="n">
+        <v>0</v>
+      </c>
+      <c r="P314" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q314" t="inlineStr"/>
+      <c r="R314" t="inlineStr"/>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"This model is unavailable for free. The paid version is available now - use this slug instead: openai/gpt-oss-120b","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>21</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>429</v>
+      </c>
+      <c r="J315" t="inlineStr"/>
+      <c r="K315" t="inlineStr"/>
+      <c r="L315" t="inlineStr"/>
+      <c r="M315" t="n">
+        <v>208</v>
+      </c>
+      <c r="N315" t="n">
+        <v>0</v>
+      </c>
+      <c r="O315" t="n">
+        <v>0</v>
+      </c>
+      <c r="P315" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q315" t="inlineStr"/>
+      <c r="R315" t="inlineStr"/>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>21</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>429</v>
+      </c>
+      <c r="J316" t="inlineStr"/>
+      <c r="K316" t="inlineStr"/>
+      <c r="L316" t="inlineStr"/>
+      <c r="M316" t="n">
+        <v>182</v>
+      </c>
+      <c r="N316" t="n">
+        <v>0</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0</v>
+      </c>
+      <c r="P316" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q316" t="inlineStr"/>
+      <c r="R316" t="inlineStr"/>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>21</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>429</v>
+      </c>
+      <c r="J317" t="inlineStr"/>
+      <c r="K317" t="inlineStr"/>
+      <c r="L317" t="inlineStr"/>
+      <c r="M317" t="n">
+        <v>319</v>
+      </c>
+      <c r="N317" t="n">
+        <v>0</v>
+      </c>
+      <c r="O317" t="n">
+        <v>0</v>
+      </c>
+      <c r="P317" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q317" t="inlineStr"/>
+      <c r="R317" t="inlineStr"/>
+      <c r="S317" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>21</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>429</v>
+      </c>
+      <c r="J318" t="inlineStr"/>
+      <c r="K318" t="inlineStr"/>
+      <c r="L318" t="inlineStr"/>
+      <c r="M318" t="n">
+        <v>432</v>
+      </c>
+      <c r="N318" t="n">
+        <v>0</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0</v>
+      </c>
+      <c r="P318" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q318" t="inlineStr"/>
+      <c r="R318" t="inlineStr"/>
+      <c r="S318" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>21</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>404</v>
+      </c>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="inlineStr"/>
+      <c r="L319" t="inlineStr"/>
+      <c r="M319" t="n">
+        <v>94</v>
+      </c>
+      <c r="N319" t="n">
+        <v>0</v>
+      </c>
+      <c r="O319" t="n">
+        <v>0</v>
+      </c>
+      <c r="P319" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q319" t="inlineStr"/>
+      <c r="R319" t="inlineStr"/>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>21</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>429</v>
+      </c>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="inlineStr"/>
+      <c r="L320" t="inlineStr"/>
+      <c r="M320" t="n">
+        <v>452</v>
+      </c>
+      <c r="N320" t="n">
+        <v>0</v>
+      </c>
+      <c r="O320" t="n">
+        <v>0</v>
+      </c>
+      <c r="P320" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q320" t="inlineStr"/>
+      <c r="R320" t="inlineStr"/>
+      <c r="S320" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>21</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>cohere/north-mini-code:free</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>200</v>
+      </c>
+      <c r="J321" t="n">
+        <v>66</v>
+      </c>
+      <c r="K321" t="n">
+        <v>1156</v>
+      </c>
+      <c r="L321" t="n">
+        <v>1222</v>
+      </c>
+      <c r="M321" t="n">
+        <v>11515</v>
+      </c>
+      <c r="N321" t="n">
+        <v>5382</v>
+      </c>
+      <c r="O321" t="n">
+        <v>760</v>
+      </c>
+      <c r="P321" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/cohere_north-mini-code_free.java</t>
+        </is>
+      </c>
+      <c r="R321" t="inlineStr"/>
+      <c r="S321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>21</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>200</v>
+      </c>
+      <c r="J322" t="n">
+        <v>88</v>
+      </c>
+      <c r="K322" t="n">
+        <v>4839</v>
+      </c>
+      <c r="L322" t="n">
+        <v>4927</v>
+      </c>
+      <c r="M322" t="n">
+        <v>51019</v>
+      </c>
+      <c r="N322" t="n">
+        <v>19135</v>
+      </c>
+      <c r="O322" t="n">
+        <v>2202</v>
+      </c>
+      <c r="P322" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/nvidia_nemotron-3-nano-30b-a3b_free.java</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr"/>
+      <c r="S322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>21</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-12b-v2-vl:free</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>200</v>
+      </c>
+      <c r="J323" t="n">
+        <v>86</v>
+      </c>
+      <c r="K323" t="n">
+        <v>2747</v>
+      </c>
+      <c r="L323" t="n">
+        <v>2833</v>
+      </c>
+      <c r="M323" t="n">
+        <v>54196</v>
+      </c>
+      <c r="N323" t="n">
+        <v>12309</v>
+      </c>
+      <c r="O323" t="n">
+        <v>1342</v>
+      </c>
+      <c r="P323" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/nvidia_nemotron-nano-12b-v2-vl_free.java</t>
+        </is>
+      </c>
+      <c r="R323" t="inlineStr"/>
+      <c r="S323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>21</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>200</v>
+      </c>
+      <c r="J324" t="n">
+        <v>88</v>
+      </c>
+      <c r="K324" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L324" t="n">
+        <v>6088</v>
+      </c>
+      <c r="M324" t="n">
+        <v>74478</v>
+      </c>
+      <c r="N324" t="n">
+        <v>24986</v>
+      </c>
+      <c r="O324" t="n">
+        <v>2504</v>
+      </c>
+      <c r="P324" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q324" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/nvidia_nemotron-3-ultra-550b-a55b_free.java</t>
+        </is>
+      </c>
+      <c r="R324" t="inlineStr"/>
+      <c r="S324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>21</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>200</v>
+      </c>
+      <c r="J325" t="n">
+        <v>88</v>
+      </c>
+      <c r="K325" t="n">
+        <v>5890</v>
+      </c>
+      <c r="L325" t="n">
+        <v>5978</v>
+      </c>
+      <c r="M325" t="n">
+        <v>83128</v>
+      </c>
+      <c r="N325" t="n">
+        <v>20776</v>
+      </c>
+      <c r="O325" t="n">
+        <v>2365</v>
+      </c>
+      <c r="P325" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q325" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/nvidia_nemotron-3-super-120b-a12b_free.java</t>
+        </is>
+      </c>
+      <c r="R325" t="inlineStr"/>
+      <c r="S325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>21</v>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I326" t="n">
+        <v>200</v>
+      </c>
+      <c r="J326" t="n">
+        <v>86</v>
+      </c>
+      <c r="K326" t="n">
+        <v>2462</v>
+      </c>
+      <c r="L326" t="n">
+        <v>2548</v>
+      </c>
+      <c r="M326" t="n">
+        <v>88870</v>
+      </c>
+      <c r="N326" t="n">
+        <v>10488</v>
+      </c>
+      <c r="O326" t="n">
+        <v>1059</v>
+      </c>
+      <c r="P326" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q326" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/google_gemma-4-26b-a4b-it_free.java</t>
+        </is>
+      </c>
+      <c r="R326" t="inlineStr"/>
+      <c r="S326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>21</v>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I327" t="n">
+        <v>200</v>
+      </c>
+      <c r="J327" t="n">
+        <v>139</v>
+      </c>
+      <c r="K327" t="n">
+        <v>3996</v>
+      </c>
+      <c r="L327" t="n">
+        <v>4135</v>
+      </c>
+      <c r="M327" t="n">
+        <v>95182</v>
+      </c>
+      <c r="N327" t="n">
+        <v>16563</v>
+      </c>
+      <c r="O327" t="n">
+        <v>1862</v>
+      </c>
+      <c r="P327" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q327" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/code/openai_gpt-oss-20b_free.java</t>
+        </is>
+      </c>
+      <c r="R327" t="inlineStr"/>
+      <c r="S327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>21</v>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>poolside/laguna-m.1:free</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I328" t="n">
+        <v>200</v>
+      </c>
+      <c r="J328" t="n">
+        <v>81</v>
+      </c>
+      <c r="K328" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L328" t="n">
+        <v>6081</v>
+      </c>
+      <c r="M328" t="n">
+        <v>124507</v>
+      </c>
+      <c r="N328" t="n">
+        <v>0</v>
+      </c>
+      <c r="O328" t="n">
+        <v>0</v>
+      </c>
+      <c r="P328" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q328" t="inlineStr"/>
+      <c r="R328" t="inlineStr"/>
+      <c r="S328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>21</v>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Write a thread-safe, generic bounded blocking queue in Java (without using java.</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-nano-9b-v2:free</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>200</v>
+      </c>
+      <c r="J329" t="n">
+        <v>84</v>
+      </c>
+      <c r="K329" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L329" t="n">
+        <v>6084</v>
+      </c>
+      <c r="M329" t="n">
+        <v>223798</v>
+      </c>
+      <c r="N329" t="n">
+        <v>0</v>
+      </c>
+      <c r="O329" t="n">
+        <v>0</v>
+      </c>
+      <c r="P329" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q329" t="inlineStr"/>
+      <c r="R329" t="inlineStr"/>
+      <c r="S329" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20815,7 +21850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S313"/>
+  <dimension ref="A1:S329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40245,8 +41280,6 @@
           <t>responses/20260713T105517Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
         </is>
       </c>
-      <c r="R298" t="inlineStr"/>
-      <c r="S298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -40316,8 +41349,6 @@
           <t>responses/20260713T105517Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
         </is>
       </c>
-      <c r="R299" t="inlineStr"/>
-      <c r="S299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -40361,9 +41392,6 @@
       <c r="I300" t="n">
         <v>429</v>
       </c>
-      <c r="J300" t="inlineStr"/>
-      <c r="K300" t="inlineStr"/>
-      <c r="L300" t="inlineStr"/>
       <c r="M300" t="n">
         <v>221</v>
       </c>
@@ -40376,8 +41404,6 @@
       <c r="P300" t="n">
         <v>3</v>
       </c>
-      <c r="Q300" t="inlineStr"/>
-      <c r="R300" t="inlineStr"/>
       <c r="S300" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
@@ -40426,9 +41452,6 @@
       <c r="I301" t="n">
         <v>429</v>
       </c>
-      <c r="J301" t="inlineStr"/>
-      <c r="K301" t="inlineStr"/>
-      <c r="L301" t="inlineStr"/>
       <c r="M301" t="n">
         <v>236</v>
       </c>
@@ -40441,8 +41464,6 @@
       <c r="P301" t="n">
         <v>3</v>
       </c>
-      <c r="Q301" t="inlineStr"/>
-      <c r="R301" t="inlineStr"/>
       <c r="S301" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
@@ -40491,9 +41512,6 @@
       <c r="I302" t="n">
         <v>429</v>
       </c>
-      <c r="J302" t="inlineStr"/>
-      <c r="K302" t="inlineStr"/>
-      <c r="L302" t="inlineStr"/>
       <c r="M302" t="n">
         <v>199</v>
       </c>
@@ -40506,8 +41524,6 @@
       <c r="P302" t="n">
         <v>3</v>
       </c>
-      <c r="Q302" t="inlineStr"/>
-      <c r="R302" t="inlineStr"/>
       <c r="S302" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
@@ -40556,9 +41572,6 @@
       <c r="I303" t="n">
         <v>429</v>
       </c>
-      <c r="J303" t="inlineStr"/>
-      <c r="K303" t="inlineStr"/>
-      <c r="L303" t="inlineStr"/>
       <c r="M303" t="n">
         <v>188</v>
       </c>
@@ -40571,8 +41584,6 @@
       <c r="P303" t="n">
         <v>3</v>
       </c>
-      <c r="Q303" t="inlineStr"/>
-      <c r="R303" t="inlineStr"/>
       <c r="S303" t="inlineStr">
         <is>
           <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
@@ -40647,8 +41658,6 @@
           <t>responses/20260713T105517Z/text/poolside_laguna-m.1_free.md</t>
         </is>
       </c>
-      <c r="R304" t="inlineStr"/>
-      <c r="S304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -40692,9 +41701,6 @@
       <c r="I305" t="n">
         <v>404</v>
       </c>
-      <c r="J305" t="inlineStr"/>
-      <c r="K305" t="inlineStr"/>
-      <c r="L305" t="inlineStr"/>
       <c r="M305" t="n">
         <v>82</v>
       </c>
@@ -40707,8 +41713,6 @@
       <c r="P305" t="n">
         <v>1</v>
       </c>
-      <c r="Q305" t="inlineStr"/>
-      <c r="R305" t="inlineStr"/>
       <c r="S305" t="inlineStr">
         <is>
           <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
@@ -40783,8 +41787,6 @@
           <t>responses/20260713T105517Z/text/google_gemma-4-26b-a4b-it_free.md</t>
         </is>
       </c>
-      <c r="R306" t="inlineStr"/>
-      <c r="S306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -40854,8 +41856,6 @@
           <t>responses/20260713T105517Z/text/google_gemma-4-31b-it_free.md</t>
         </is>
       </c>
-      <c r="R307" t="inlineStr"/>
-      <c r="S307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -40925,8 +41925,6 @@
           <t>responses/20260713T105517Z/text/cohere_north-mini-code_free.md</t>
         </is>
       </c>
-      <c r="R308" t="inlineStr"/>
-      <c r="S308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -40996,8 +41994,6 @@
           <t>responses/20260713T105517Z/text/openai_gpt-oss-20b_free.md</t>
         </is>
       </c>
-      <c r="R309" t="inlineStr"/>
-      <c r="S309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -41067,8 +42063,6 @@
           <t>responses/20260713T105517Z/text/nvidia_nemotron-nano-9b-v2_free.md</t>
         </is>
       </c>
-      <c r="R310" t="inlineStr"/>
-      <c r="S310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -41138,8 +42132,6 @@
           <t>responses/20260713T105517Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
         </is>
       </c>
-      <c r="R311" t="inlineStr"/>
-      <c r="S311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -41183,9 +42175,6 @@
       <c r="I312" t="n">
         <v>200</v>
       </c>
-      <c r="J312" t="inlineStr"/>
-      <c r="K312" t="inlineStr"/>
-      <c r="L312" t="inlineStr"/>
       <c r="M312" t="n">
         <v>120424</v>
       </c>
@@ -41198,9 +42187,6 @@
       <c r="P312" t="n">
         <v>1</v>
       </c>
-      <c r="Q312" t="inlineStr"/>
-      <c r="R312" t="inlineStr"/>
-      <c r="S312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -41270,8 +42256,1090 @@
           <t>responses/20260713T105517Z/text/openai_gpt-oss-120b_free.md</t>
         </is>
       </c>
-      <c r="R313" t="inlineStr"/>
-      <c r="S313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>21</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>nousresearch/hermes-3-llama-3.1-405b:free</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>429</v>
+      </c>
+      <c r="J314" t="inlineStr"/>
+      <c r="K314" t="inlineStr"/>
+      <c r="L314" t="inlineStr"/>
+      <c r="M314" t="n">
+        <v>267</v>
+      </c>
+      <c r="N314" t="n">
+        <v>0</v>
+      </c>
+      <c r="O314" t="n">
+        <v>0</v>
+      </c>
+      <c r="P314" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q314" t="inlineStr"/>
+      <c r="R314" t="inlineStr"/>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"nousresearch/hermes-3-llama-3.1-405b:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice",</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>21</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-120b:free</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>404</v>
+      </c>
+      <c r="J315" t="inlineStr"/>
+      <c r="K315" t="inlineStr"/>
+      <c r="L315" t="inlineStr"/>
+      <c r="M315" t="n">
+        <v>85</v>
+      </c>
+      <c r="N315" t="n">
+        <v>0</v>
+      </c>
+      <c r="O315" t="n">
+        <v>0</v>
+      </c>
+      <c r="P315" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q315" t="inlineStr"/>
+      <c r="R315" t="inlineStr"/>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"This model is unavailable for free. The paid version is available now - use this slug instead: openai/gpt-oss-120b","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>21</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-next-80b-a3b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>429</v>
+      </c>
+      <c r="J316" t="inlineStr"/>
+      <c r="K316" t="inlineStr"/>
+      <c r="L316" t="inlineStr"/>
+      <c r="M316" t="n">
+        <v>215</v>
+      </c>
+      <c r="N316" t="n">
+        <v>0</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0</v>
+      </c>
+      <c r="P316" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q316" t="inlineStr"/>
+      <c r="R316" t="inlineStr"/>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-next-80b-a3b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>21</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-super-120b-a12b:free</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>200</v>
+      </c>
+      <c r="J317" t="n">
+        <v>73</v>
+      </c>
+      <c r="K317" t="n">
+        <v>462</v>
+      </c>
+      <c r="L317" t="n">
+        <v>535</v>
+      </c>
+      <c r="M317" t="n">
+        <v>31240</v>
+      </c>
+      <c r="N317" t="n">
+        <v>1057</v>
+      </c>
+      <c r="O317" t="n">
+        <v>168</v>
+      </c>
+      <c r="P317" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/text/nvidia_nemotron-3-super-120b-a12b_free.md</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr"/>
+      <c r="S317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>21</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct:free</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>429</v>
+      </c>
+      <c r="J318" t="inlineStr"/>
+      <c r="K318" t="inlineStr"/>
+      <c r="L318" t="inlineStr"/>
+      <c r="M318" t="n">
+        <v>233</v>
+      </c>
+      <c r="N318" t="n">
+        <v>0</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0</v>
+      </c>
+      <c r="P318" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q318" t="inlineStr"/>
+      <c r="R318" t="inlineStr"/>
+      <c r="S318" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"meta-llama/llama-3.3-70b-instruct:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>21</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>qwen/qwen3-coder:free</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>429</v>
+      </c>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="inlineStr"/>
+      <c r="L319" t="inlineStr"/>
+      <c r="M319" t="n">
+        <v>214</v>
+      </c>
+      <c r="N319" t="n">
+        <v>0</v>
+      </c>
+      <c r="O319" t="n">
+        <v>0</v>
+      </c>
+      <c r="P319" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q319" t="inlineStr"/>
+      <c r="R319" t="inlineStr"/>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"qwen/qwen3-coder:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Venice","is_byok":false,"ret</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>21</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>google/gemma-4-31b-it:free</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>429</v>
+      </c>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="inlineStr"/>
+      <c r="L320" t="inlineStr"/>
+      <c r="M320" t="n">
+        <v>222</v>
+      </c>
+      <c r="N320" t="n">
+        <v>0</v>
+      </c>
+      <c r="O320" t="n">
+        <v>0</v>
+      </c>
+      <c r="P320" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q320" t="inlineStr"/>
+      <c r="R320" t="inlineStr"/>
+      <c r="S320" t="inlineStr">
+        <is>
+          <t>HTTP 429: {"error":{"message":"Provider returned error","code":429,"metadata":{"raw":"google/gemma-4-31b-it:free is temporarily rate-limited upstream. Please retry shortly, or add your own key to accumulate your rate limits: https://openrouter.ai/settings/integrations","provider_name":"Google AI Studio","is_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>21</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>poolside/laguna-xs.2:free</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>404</v>
+      </c>
+      <c r="J321" t="inlineStr"/>
+      <c r="K321" t="inlineStr"/>
+      <c r="L321" t="inlineStr"/>
+      <c r="M321" t="n">
+        <v>140</v>
+      </c>
+      <c r="N321" t="n">
+        <v>0</v>
+      </c>
+      <c r="O321" t="n">
+        <v>0</v>
+      </c>
+      <c r="P321" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q321" t="inlineStr"/>
+      <c r="R321" t="inlineStr"/>
+      <c r="S321" t="inlineStr">
+        <is>
+          <t>HTTP 404: {"error":{"message":"No endpoints found for poolside/laguna-xs.2:free.","code":404},"user_id":"user_3FWWx2cLEsPQ6tm6LVPGgRET5mk"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>21</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>google/gemma-4-26b-a4b-it:free</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>200</v>
+      </c>
+      <c r="J322" t="n">
+        <v>56</v>
+      </c>
+      <c r="K322" t="n">
+        <v>1793</v>
+      </c>
+      <c r="L322" t="n">
+        <v>1849</v>
+      </c>
+      <c r="M322" t="n">
+        <v>38556</v>
+      </c>
+      <c r="N322" t="n">
+        <v>7602</v>
+      </c>
+      <c r="O322" t="n">
+        <v>1198</v>
+      </c>
+      <c r="P322" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/text/google_gemma-4-26b-a4b-it_free.md</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr"/>
+      <c r="S322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>21</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b:free</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>200</v>
+      </c>
+      <c r="J323" t="n">
+        <v>73</v>
+      </c>
+      <c r="K323" t="n">
+        <v>7626</v>
+      </c>
+      <c r="L323" t="n">
+        <v>7699</v>
+      </c>
+      <c r="M323" t="n">
+        <v>97478</v>
+      </c>
+      <c r="N323" t="n">
+        <v>26989</v>
+      </c>
+      <c r="O323" t="n">
+        <v>4116</v>
+      </c>
+      <c r="P323" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/text/nvidia_nemotron-3-ultra-550b-a55b_free.md</t>
+        </is>
+      </c>
+      <c r="R323" t="inlineStr"/>
+      <c r="S323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>21</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-nano-30b-a3b:free</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>200</v>
+      </c>
+      <c r="J324" t="n">
+        <v>73</v>
+      </c>
+      <c r="K324" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L324" t="n">
+        <v>8073</v>
+      </c>
+      <c r="M324" t="n">
+        <v>71647</v>
+      </c>
+      <c r="N324" t="n">
+        <v>17147</v>
+      </c>
+      <c r="O324" t="n">
+        <v>2482</v>
+      </c>
+      <c r="P324" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q324" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/text/nvidia_nemotron-3-nano-30b-a3b_free.md</t>
+        </is>
+      </c>
+      <c r="R324" t="inlineStr"/>
+      <c r="S324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2026-07-14T15:22:37.394319+00:00</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>21</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Write an in-depth, approximately 1000-line article on best practices in nonprofi</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>openai/gpt-oss-20b:free</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>200</v>
+      </c>
+      <c r="J325" t="n">
+        <v>122</v>
+      </c>
+      <c r="K325" t="n">
+        <v>4028</v>
+      </c>
+      <c r="L325" t="n">
+        <v>4150</v>
+      </c>
+      <c r="M325" t="n">
+        <v>76488</v>
+      </c>
+      <c r="N325" t="n">
+        <v>15403</v>
+      </c>
+      <c r="O325" t="n">
+        <v>2388</v>
+      </c>
+      <c r="P325" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q325" t="inlineStr">
+        <is>
+          <t>responses/20260714T152237Z/text/openai_gpt-oss-20b_free.md</t>
+        </is>
+      </c>
+      <c r="R325" t="inlineStr"/>
+      <c r="S325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>20260714T152237Z</t>
+        </is>
+      </c>
+      <c